<commit_message>
Kontrol turu: sütun başlıklarına klavye erişimi (tabindex), dil düzeltmeleri (hijyen, -malıdır), üretim zinciri depodan çalışır (küçük ham özetler eklendi), README
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -9501,7 +9501,7 @@
   <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="47" customWidth="1" min="1" max="1"/>
+    <col width="53" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -10243,7 +10243,7 @@
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Ticari hijyen (dispenser, el kurutma)</t>
+          <t>Ticari ıslak hacim donanımı (dispenser, el kurutma)</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
@@ -10262,7 +10262,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Banyomarka, profesyonel hijyen markaları</t>
+          <t>Banyomarka, profesyonel ıslak hacim markaları</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Rapor düzeni: insight'lar madde yapısı ve kalın rakam, notlar madde listesi, kısaltma balonları her paragrafta, alt başlık açıklamaları, alan adı logoları, uzun tablo eşiği, taşınma bölümü kaldırıldı, kök ifade, slug bağlantıları
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -1925,10 +1925,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1943,11 +1943,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Organik Kanal Performansı · Trafik hangi sayfa türlerine geliyor?
-Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır; Aralık 2025'te online.vitra.com.tr adreslerinin ana alan adına taşınması dönem içinde yer almaktadır.
+Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 10
 Sütun açıklamaları: Sayfa türü: Adres yapısına göre sayfa sınıfı; /c- ve kategori dizinleri kategori, -p-a kodlu adresler ürün sayfasıdır. | Sayfa: Dönemde en az bir gösterim almış sayfa sayısı (ilk 25.000 sayfa). | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam tık. | Pay: Sayfa türünün toplam tık içindeki payı. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
         </is>
@@ -2015,45 +2015,45 @@
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Ürün sayfaları</t>
+          <t>Diğer</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>7110</v>
+        <v>3621</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>489948</v>
+        <v>491593</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>15.8</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>5434587</v>
+        <v>37727037</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Eski online.vitra.com.tr adresleri</t>
+          <t>Ürün sayfaları</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>2499</v>
+        <v>7110</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>399074</v>
+        <v>489948</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>12.9</v>
+        <v>15.8</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>34108271</v>
+        <v>5434587</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>1.2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
@@ -2103,132 +2103,110 @@
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Diğer</t>
+          <t>Servis ve bayi</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1122</v>
+        <v>471</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>92519</v>
+        <v>71118</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>3618766</v>
+        <v>3955742</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Servis ve bayi</t>
+          <t>Koleksiyon sayfaları</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>471</v>
+        <v>189</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>71118</v>
+        <v>67240</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>3955742</v>
+        <v>1001585</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Koleksiyon sayfaları</t>
+          <t>Kurumsal</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>189</v>
+        <v>340</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>67240</v>
+        <v>24268</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>1001585</v>
+        <v>1490281</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>6.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Kurumsal</t>
+          <t>Katalog</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>340</v>
+        <v>41</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>24268</v>
+        <v>23441</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>0.8</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1490281</v>
+        <v>773671</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Katalog</t>
+          <t>Ürün teknik föyleri</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>41</v>
+        <v>2019</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>23441</v>
+        <v>13382</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>773671</v>
+        <v>216995</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Ürün teknik föyleri</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>13382</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>216995</v>
-      </c>
-      <c r="F15" s="9" t="n">
         <v>6.2</v>
       </c>
     </row>
@@ -2264,11 +2242,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="146" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Organik Kanal Performansı · Kategori bazında organik trafik
-Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır; Aralık 2025'te online.vitra.com.tr adreslerinin ana alan adına taşınması dönem içinde yer almaktadır.
+Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 10
 Sütun açıklamaları: Kategori: Kategori ve ürün sayfalarının adres yapısından türetilen ana kategori. | Sayfa: Kategoriye eşlenen sayfa sayısı. | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam tık. | Pay: Kategori ve ürün sayfaları toplamı içindeki pay. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
         </is>
@@ -2537,11 +2515,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Organik Kanal Performansı · En çok tık alan sayfalar · Tem-Eyl 2026
-Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır; Aralık 2025'te online.vitra.com.tr adreslerinin ana alan adına taşınması dönem içinde yer almaktadır.
+Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 10
 Sütun açıklamaları: Sayfa adresi: Sayfa adresi; bağlantı canlı sayfaya gider. | Tık · Tem-Eyl 2026: 1 Temmuz - 25 Eylül 2026 organik tık.</t>
         </is>
@@ -2740,11 +2718,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Organik Kanal Performansı · Cihaz ve ülke
-Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır; Aralık 2025'te online.vitra.com.tr adreslerinin ana alan adına taşınması dönem içinde yer almaktadır.
+Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 10
 Sütun açıklamaları: Kırılım: Search Console cihaz ve ülke boyutu. | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam. | Pay: Toplam tık içindeki pay. | CTR: Tık / gösterim.</t>
         </is>
@@ -2909,9 +2887,9 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · "vitra" ile başlayan aramalar
-Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 tohum ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
-Sütun açıklamaları: Tohum ifade: Google arama kutusuna yazılan ifade; öneriler bu ifadenin devamı olarak gelmektedir. | Autocomplete önerileri: Google'ın Türkiye, Türkçe, masaüstü Chrome için döndürdüğü ilk 10 tamamlama önerisi; sırası Google'ın sırasıdır.</t>
+Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
+Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
+Sütun açıklamaları: Kök ifade: Google arama kutusuna yazılan ifade; öneriler bu ifadenin devamı olarak gelmektedir. | Autocomplete önerileri: Google'ın Türkiye, Türkçe, masaüstü Chrome için döndürdüğü ilk 10 tamamlama önerisi; sırası Google'ın sırasıdır.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -2919,7 +2897,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Tohum ifade</t>
+          <t>Kök ifade</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -3128,9 +3106,9 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · Kategori ve rakip marka aramaları
-Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 tohum ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
-Sütun açıklamaları: Tohum ifade: Kategori veya rakip marka ile başlayan ifade. | Autocomplete önerileri: Google'ın döndürdüğü ilk 10 tamamlama önerisi.</t>
+Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
+Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
+Sütun açıklamaları: Kök ifade: Kategori veya rakip marka ile başlayan ifade. | Autocomplete önerileri: Google'ın döndürdüğü ilk 10 tamamlama önerisi.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -3138,7 +3116,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Tohum ifade</t>
+          <t>Kök ifade</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -3336,9 +3314,9 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · Öneri temaları
-Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 tohum ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
-Sütun açıklamaları: Öneri teması: Önerinin ifade kalıbına göre sınıfı. | Öneri: 49 tohum ifadeden dönen toplam öneri sayısı. | Pay: Toplam öneri içindeki pay.</t>
+Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
+Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
+Sütun açıklamaları: Öneri teması: Önerinin ifade kalıbına göre sınıfı. | Öneri: 49 kök ifadeden dönen toplam öneri sayısı. | Pay: Toplam öneri içindeki pay.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -3685,8 +3663,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · En çok tık getiren sorgular · Search Console
-Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 tohum ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
+Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
+Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
 Sütun açıklamaları: Sorgu: Kullanıcının Google'a yazdığı ifade. | Tık: 1 Haz 2025 - 25 Eyl 2026. | Gösterim: Aynı dönem. | CTR: Tık / gösterim. | Sıra: Ortalama sıra.</t>
         </is>
       </c>
@@ -17672,7 +17650,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Aksesuar setleri talebi daralmakta ( -%22,2 ); tek parça aksesuar aramaları sürmekte</t>
+          <t>Aksesuar setleri talebi daralmakta (-%22,2); tek parça aksesuar aramaları sürmekte</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -18350,7 +18328,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026</t>
+          <t>49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -18412,7 +18390,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>10 tohum grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
+          <t>10 kök ifade grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -18882,7 +18860,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Google Ads keyword ideas (keywords for keywords) · 10 tohum grubu, 52.973 kelime · Türkiye, Türkçe · Eyl 2022 - Ağu 2026</t>
+          <t>Google Ads keyword ideas (keywords for keywords) · 10 kök ifade grubu, 52.973 kelime · Türkiye, Türkçe · Eyl 2022 - Ağu 2026</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -18922,7 +18900,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Google Autocomplete · "vitra" ile başlayan 49 tohum ifade · Türkiye, Türkçe, masaüstü Chrome</t>
+          <t>Google Autocomplete · "vitra" ile başlayan 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Bölüm: Kanal Politikaları ve Keşif Kanalları (ödeme, teslimat, garanti, sosyal, Business Profile, Shopping blok); kaynak D23
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -55,14 +55,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46 Fiyat konumu" sheetId="46" state="visible" r:id="rId46"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="47 Satıcı yapısı, hizmet ve a" sheetId="47" state="visible" r:id="rId47"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="48 Trafik mıknatısı kategoril" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49 E-ticaret modelleri" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 Ürün keşfi ve dijital dene" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="51 Kanal rolleri" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="52 Hacimli ve ölçüye bağlı ür" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="53 Tamamlayıcı ürün kurgusu" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="54 Sonraki Adımlar" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55 Yöntem ve Kapsam" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49 Ödeme ve taksit koşulları" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50 Kargo, teslimat, iade ve m" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="51 Garanti, yedek parça ve se" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="52 Sosyal ve keşif kanalları" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="53 Google Business Profile m" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="54 E-ticaret modelleri" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="55 Ürün keşfi ve dijital dene" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="56 Kanal rolleri" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="57 Hacimli ve ölçüye bağlı ür" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="58 Tamamlayıcı ürün kurgusu" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="59 Sonraki Adımlar" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="60 Yöntem ve Kapsam" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="61" state="visible" r:id="rId61"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16230,258 +16235,310 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="118" customHeight="1">
+          <t>Kanal Politikaları ve Keşif Kanalları · Ödeme ve taksit koşulları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri
-Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 19 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 32 , 33 , 34 , 35 , 36 , 37 , 38
-Sütun açıklamaları: Oyuncu: İncelenen site. | Tip: İş modeli. | E-ticaret modeli: Ürün, kanal ve hizmetin nasıl bir araya getirildiği. | VitrA'ya uyarlanabilir nokta: VitrA'nın mevcut yapısına eklenebilecek unsur.</t>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Ödeme ve taksit koşulları
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 32
+Sütun açıklamaları: Site: Ödeme ve taksit sayfası okunan site; bağlantı ana sayfaya gider. | Taksit ve vade farksız koşul: Sitenin yardım, taksit veya ödeme rehberi sayfasındaki ifade; 29.09.2026. | Alışveriş kredisi: Sitede alışveriş kredisi veya mağaza kartı seçeneği. | Kapıda ödeme / havale: Kredi kartı dışındaki ödeme yolları. | Kurumsal fatura: Kurumsal fatura veya kurumsal kart seçeneği.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Oyuncu</t>
+          <t>Site</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Tip</t>
+          <t>Taksit ve vade farksız koşul</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>E-ticaret modeli</t>
+          <t>Alışveriş kredisi</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>VitrA'ya uyarlanabilir nokta</t>
+          <t>Kapıda ödeme / havale</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Kurumsal fatura</t>
         </is>
       </c>
     </row>
     <row r="5" ht="43" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Koçtaş</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Yapı market · TR</t>
+          <t>Şeritte tüm ürünlerde vade farksız 6 ay (eşiksiz); ürün tablosunda 12 taksite kadar, 8-12 çoğunlukla vade farklı; kampanyada 9 aya varan taksit</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Tüm banyo ve bitişik kategoriler tek tadilat sayfasında; montaj sepette ücretli; anahtar teslim tadilat mağazada; kampanyalar mağazaya özel</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Banyo yenilemesini ürün kategorisi değil "proje" olarak kurgulama</t>
+          <t>Yok (yalnızca kredi kartı)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Var (sepette)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>IKEA</t>
+          <t>koctas.com.tr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Mobilya perakendecisi · TR</t>
+          <t>Online 5.000 TL üzeri 7 taksite kadar vade farksız; vade farklı 9'a kadar</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Oda bazlı gezinme, hazır banyo setleri, ücretsiz planlayıcı, ücretli montaj, uzun vadeli alışveriş kredisi</t>
+          <t>Koçtaş Kart</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Oda ve set üzerinden gezinme; set fiyatının tek satırda gösterilmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Banyomarka</t>
+          <t>bauhaus.com.tr</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Banyo pureplayer · TR</t>
+          <t>2.500 TL ve üzeri anlaşmalı kartlarla vade farksız</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Çok markalı katalog, kombin sayfaları, çocuk, engelli ve genel kullanım alanı kategorileri, WhatsApp destek</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Kombin sayfası ve özel ihtiyaç kategorileri</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="43" customHeight="1">
+          <t>Havale / EFT</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Kurumsal kart</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Kale</t>
+          <t>ikea.com.tr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Banyo markası · TR</t>
+          <t>1.500 TL üzeri 3 taksit; IKEA Aile üyelerine 7.500 TL üzeri 6, 20.000 TL üzeri 9 taksit</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Marka sitesinde e-ticaret; montaj hizmetleri ve yedek parça sayfaları açılmış, 29.09.2026 itibarıyla ürün listelenmiyor; mutfak tezgahı ve yapı kimyasalı kategorileri</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Rakip marka da hizmet ve yedek parçayı e-ticarete taşımaya başlıyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>IKEA Kurumsal Kart</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Hepsiburada</t>
+          <t>shop.creavit.com.tr</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Pazaryeri · TR</t>
+          <t>Peşin fiyatına 6 ve 9 taksit ifadeleri birlikte</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Ürünle birlikte kurulum hizmeti sepete ekleniyor; iş ortağı firma randevu veriyor</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Pazaryeri mağazasında VitrA montaj hizmetinin ürünle birlikte listelenmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="43" customHeight="1">
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Victorian Plumbing</t>
+          <t>banyomarka.com</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Banyo pureplayer · İngiltere</t>
+          <t>Ürün kartında 4 taksit</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Komple banyo takımları (klozet + lavabo, genişletilmiş setlerde küvet, duşakabin ve dolap); 250 GBP üzeri siparişte %0 faizli finansman</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Koleksiyon bazlı komple banyo takımı ve sepet tutarına bağlı finansman</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>İstanbul içi kapıda nakit</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>BAUHAUS</t>
+          <t>banyoline.com</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Yapı market · Almanya</t>
+          <t>Şeritte peşin fiyatına 12 ay taksit</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Komple banyo sabit fiyatla: planlama, söküm, tesisat, seramik, montaj; proje koordinatörü</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Sabit fiyatlı yenileme paketi</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Home Depot</t>
+          <t>hepsiburada.com</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Yapı market · ABD</t>
+          <t>12 aya varan taksit (platform limiti)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Ücretsiz evde keşif, lisanslı yerel uygulayıcı, proje kredisi</t>
+          <t>Var</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Keşfin ürün alımına bağlı ücretsiz sunulması</t>
+          <t>Uygun ürünlerde kapıda nakit, üst limit 7.000 TL</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Mümkün</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Kohler</t>
+          <t>trendyol.com</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Üretici marka · ABD</t>
+          <t>Kategori, tutar ve kart tipine göre; her üründe taksit yok (arama özeti)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>"Reveal by Kohler": yetkili bayilerle duş ve küvet dönüşümü, bir günde kurulum, ömür boyu sınırlı garanti</t>
+          <t>Trendyol Kredi Pazaryeri</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Üretici markanın bayi ağıyla paket hizmet satması</t>
+          <t>Doğrulanamadı</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Mümkün</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16860,6 +16917,1202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Kargo, teslimat, iade ve montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Kargo, teslimat, iade ve montaj
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 32
+Sütun açıklamaları: Site: Teslimat, iade ve montaj sayfaları okunan site. | Ücretsiz kargo: Ücretsiz kargo eşiği. | Büyük ürün teslimat: Klozet, dolap, duşakabin gibi büyük ürünlerde teslimat süresi ve yöntemi. | İade: İade süresi ve büyük ürün koşulu. | Montaj: Montaj seçeneği, kapsamı ve fiyatı; 29.09.2026.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Ücretsiz kargo</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Büyük ürün teslimat</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>İade</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Eşiksiz ücretsiz kargo</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>3 iş günü içinde kargoya; ürün sayfasında tahmini tarih</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>30 gün (ürün sayfasında; iade rehberinde gün yazmıyor)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Sitede fiyatlı 7 kalem: klozet 2.750 TL, BM seti 4.000 TL, keşif 1.400 TL; 40.000 TL üzeri kampanyada ücretsiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>shop.creavit.com.tr</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>3.000 TL üzeri</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>5 iş günü içinde kargoya</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>30 gün</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>11 kalem: klozet 2.450 TL, armatür 1.750 TL, boy dolabı 1.400 TL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>bauhaus.com.tr</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1.000 TL ve üzeri (seçili ürün); 40.000 TL üzeri şehir içi nakliye</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>30 desi üstü lojistik firması; adalar kapsam dışı</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>14 gün; klozet takımında ambalaj açılmamış şartı</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Usta temini müşteri hizmetleri üzerinden</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>ikea.com.tr</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Eşik yok; kargo 299-799 TL, üstü %11</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Daire kapısına teslim</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>İnternet 14 gün, mağaza 30 gün</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Sepette montaj; bölgeye göre fiyat; 2 yıl kurulum garantisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>koctas.com.tr</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Doğrulanamadı (arama özeti 300-600 TL)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nakliye 4 gün içinde (arama özeti)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>14 gün</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>20 ilde montaj; seçili mobilyada ücretsiz; Ustabilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>banyoline.com</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Tüm alışverişlerde ücretsiz</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Bölgeye bağlı, 30 günü aşmaz</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>İptal ve iade formu</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>İstanbul'da ücretsiz montaj: VitrA Metropole Edge, Valarte, Nest Trendy, Sento, Root</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>hepsiburada.com</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Bulunamadı</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Mobilya birden fazla pakette, HepsiJET XL</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>14 gün, demonte ve orijinal kutu</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>69 ilde sepete eklenebilir montaj; klozet montajı 2.730 TL (Mr Usta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Alıcı eşiği doğrulanamadı</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Satıcının anlaşmalı taşıyıcısı</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>15 gün; montajı tamamlanmış ürün iade dışı</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayfasında ek montaj hizmeti; 30 gün içinde randevu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Garanti, yedek parça ve servis iletişimi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="174" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Garanti, yedek parça ve servis iletişimi
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 32
+Sütun açıklamaları: Marka: Garanti ve servis sayfaları okunan marka; bağlantı sitesine gider. | Garanti süresi: Sitede yazılı garanti süresi; "arama özeti" sayfa açılamadığı için arama sonucundan alındığını gösterir. | Yedek parça: Yedek parça sayfası, aracı veya listesi. | Servis ve iletişim: Servis randevu akışı, telefon ve anlık mesaj kanalı.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Marka</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Garanti süresi</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Yedek parça</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Servis ve iletişim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>VitrA</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayfalarında süre yazmıyor; V-Care 2 yıl (+2 yıl paket); ek garanti sayfası var</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı sayfa yok; gömme rezervuar montaj aksesuarları kategorisi</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Online servis randevusu, garanti talep formu, 0850 hattı; WhatsApp bulunamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Kale</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>SSG 10 yıl, armatür 5 yıl, musluk 2, duş ve gömme rezervuar 5; servis işçiliği 1 yıl</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı sayfa yok; kullanım kılavuzları</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yetkili servis sayfası, 0850 hattı, WhatsApp destek</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Creavit</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Seramik 12, gömme rezervuar 10, armatür 5 yıl (arama özeti)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Katalogda yedek parça listesi</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yetkili servis sayfası, e-mağaza hattı</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A.</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayfasında 20 yıl (Life lavabo bataryası)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayfasında yedek parça resmi</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Servis haritası, 444 hattı, WhatsApp</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Geberit</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Vitrifiyede ömür boyu; AquaClean 10 yıl parça bulunabilirliği (arama özeti)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Yedek parça ve bulunabilirlik sayfası</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Bayi ve servis sayfası, 0850 hattı</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Grohe</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Seçili ürünlerde 10 yıla kadar; 2 yıl (+1 kayıtla) ve 5 yıl</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Yedek parça bulucu; garanti kapsamında 48 saatte teslim</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Servis talebi formu, bayi bulucu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 32
+Sütun açıklamaları: Marka: Kanal büyüklükleri karşılaştırılan marka. | Instagram: Takipçi; profil girişe kapalı olduğu için Google sonuç özetinden, yaklaşık. "-" alınamadı. | YouTube: Abone, video ve toplam görüntüleme; kanal hakkında sayfası, 29.09.2026. | Pinterest: Profil takipçisi. | TikTok: Resmi hesap ve takipçi.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Marka</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>VitrA Türkiye</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>~144K</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>1,58 Mn · 402 video · 55,8 Mn</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1.478 + 3.825 (iki hesap)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Artema</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>~20K</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>4,75 B · 33 video · 19,7 Mn</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3.825 (ortak hesap)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Grohe (global kanal)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>75,1 B · 627 video · 21,9 Mn</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>10325</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Geberit Türkiye</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>~39K</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı TR kanalı yok</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A.</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>~24K</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı TR kanalı yok</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Creavit</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2,17 B · 227 video · 7,1 Mn</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>187</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>118 takipçi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Kale</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>948 · 577 video · 1,4 Mn</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>943</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 32
+Sütun açıklamaları: İl: Google Maps'te VitrA etiketli satış noktası profillerinin ili. | Profil: Tekil profil sayısı (cid ile). | Toplam yorum: Profillerin toplam yorum sayısı. | Ortalama puan: Yorum ağırlıklı ortalama puan.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>İl</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Profil</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Toplam yorum</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Ortalama puan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>3732</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>504</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>İzmir</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>461</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Muğla</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>533</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mersin</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Antalya</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>338</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>271</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Hatay</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="118" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri
+Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 19 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 33 , 34 , 35 , 36 , 37 , 38 , 39
+Sütun açıklamaları: Oyuncu: İncelenen site. | Tip: İş modeli. | E-ticaret modeli: Ürün, kanal ve hizmetin nasıl bir araya getirildiği. | VitrA'ya uyarlanabilir nokta: VitrA'nın mevcut yapısına eklenebilecek unsur.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Oyuncu</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>E-ticaret modeli</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>VitrA'ya uyarlanabilir nokta</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="43" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Yapı market · TR</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Tüm banyo ve bitişik kategoriler tek tadilat sayfasında; montaj sepette ücretli; anahtar teslim tadilat mağazada; kampanyalar mağazaya özel</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Banyo yenilemesini ürün kategorisi değil "proje" olarak kurgulama</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Mobilya perakendecisi · TR</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Oda bazlı gezinme, hazır banyo setleri, ücretsiz planlayıcı, ücretli montaj, uzun vadeli alışveriş kredisi</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Oda ve set üzerinden gezinme; set fiyatının tek satırda gösterilmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Banyomarka</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Banyo pureplayer · TR</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Çok markalı katalog, kombin sayfaları, çocuk, engelli ve genel kullanım alanı kategorileri, WhatsApp destek</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Kombin sayfası ve özel ihtiyaç kategorileri</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Kale</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Banyo markası · TR</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Marka sitesinde e-ticaret; montaj hizmetleri ve yedek parça sayfaları açılmış, 29.09.2026 itibarıyla ürün listelenmiyor; mutfak tezgahı ve yapı kimyasalı kategorileri</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka da hizmet ve yedek parçayı e-ticarete taşımaya başlıyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri · TR</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Ürünle birlikte kurulum hizmeti sepete ekleniyor; iş ortağı firma randevu veriyor</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri mağazasında VitrA montaj hizmetinin ürünle birlikte listelenmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="43" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Victorian Plumbing</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Banyo pureplayer · İngiltere</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Komple banyo takımları (klozet + lavabo, genişletilmiş setlerde küvet, duşakabin ve dolap); 250 GBP üzeri siparişte %0 faizli finansman</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Koleksiyon bazlı komple banyo takımı ve sepet tutarına bağlı finansman</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>BAUHAUS</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Yapı market · Almanya</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Komple banyo sabit fiyatla: planlama, söküm, tesisat, seramik, montaj; proje koordinatörü</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Sabit fiyatlı yenileme paketi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Yapı market · ABD</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Ücretsiz evde keşif, lisanslı yerel uygulayıcı, proje kredisi</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Keşfin ürün alımına bağlı ücretsiz sunulması</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Kohler</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Üretici marka · ABD</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>"Reveal by Kohler": yetkili bayilerle duş ve küvet dönüşümü, bir günde kurulum, ömür boyu sınırlı garanti</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Üretici markanın bayi ağıyla paket hizmet satması</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16882,7 +18135,7 @@
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · Ürün keşfi ve dijital deneyim örnekleri
 Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 19 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 32 , 33 , 34 , 35 , 36 , 37 , 38
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 19 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 33 , 34 , 35 , 36 , 37 , 38 , 39
 Sütun açıklamaları: Araç: Ürün keşfi ya da dijital deneyim aracı. | Örnek: Aracı kullanan oyuncular. | Ne sağlıyor?: Kullanıcıya sağladığı fayda. | VitrA'da: vitra.com.tr'deki karşılığı (29.09.2026). | Gözlem: Mevcut durum ve olası adım.</t>
         </is>
       </c>
@@ -17169,7 +18422,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17322,7 +18575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17541,7 +18794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17716,7 +18969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17785,7 +19038,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 16 , 34 , 35</t>
+          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 16 , 35 , 36</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -18005,7 +19258,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 16 , 32 , 33</t>
+          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 16 , 33 , 34</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -18159,7 +19412,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 36</t>
+          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 37</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -18209,1248 +19462,6 @@
       <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Karo trafiğinden çapraz satış</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Yöntem ve Kapsam · Tablo 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="90" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: Yöntem ve Kapsam
-Kapsam: Bu rapor, Inbound'un erişimindeki veri kaynaklarıyla hazırlanmıştır. VitrA'dan beklenen pazaryeri performansı, GA4 dönüşüm ve site içi arama raporları, iade ve çağrı merkezi verisi geldiğinde ilgili bölümler eklenecek ve öneriler güncellenecektir.
-Sütun açıklamaları: Veri kaynağı: Kullanılan kaynak. | Kapsam: Dönem, coğrafya ve örneklem. | Kullanıldığı bölüm: Verinin işlendiği bölüm. | Not: Ölçüm sınırı veya yöntem notu.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Veri kaynağı</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Kapsam</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Kullanıldığı bölüm</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Not</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="43" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads Keyword Planner</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2.420 kelime · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>03, 04, 05</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads benzer kelimeler için birleşik hacim döndürür; aynı hacimli yazım varyantları toplamda tekrar sayılmıştır ve toplamlar üst sınır olarak okunmalıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Google Search Console</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sorgu, cihaz, ülke</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>05, 06, 07</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Sayfa ve sorgu raporları ilk 25.000 satırla sınırlıdır; sayfa×gün tablosu 100.000 satır</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Google Autocomplete</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>07, 17</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Öneriler tek günlük anlık görüntüdür; sıralama Google'ın sırasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>YouTube arama</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>30 ifade · Türkiye · ilk sayfa · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>İzlenme sayıları video yayın tarihinden itibaren kümülatiftir</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Organik rakipler ve Batch Analysis · Türkiye · 27.09.2026</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek ziyaret sayısı değildir</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="56" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads keyword ideas</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>10 kök ifade grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>04, 10, 11, 12</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Kelimeler 58 temalı sözlükle sınıflandırılmış, gürültü ifadeleri ayıklanmış, aynı aylık seriyi taşıyan yazım varyantları tek sayılmıştır; tema toplamları yaklaşık büyüklük gösterir</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>vitra.com.tr ürün sitemap'i ve site incelemesi</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · Banyo Asistanı · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>10, 12, 16, 17</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Ürün sayısı renk ve ölçü varyantlarını ayrı sayar; model sayısı renk ekleri ayıklanarak yaklaşık hesaplanmıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Rakip kategori sitemap'leri</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline · Koçtaş tarayıcı ile</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>11, 16</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Kategori varlığı gözlemidir; ürün derinliği ve satış hacmi ölçülmemiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="43" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol arama sonuçları</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>13 tema, ilk 40-45 ürün · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>04, 10, 11</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Değerlendirme sayısı satış hacmine yaklaşık gösterge olarak kullanılmıştır; sonuç sırası kişiselleştirmeye bağlı olarak değişebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="43" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Rakip ve benzer oyuncuların siteleri</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Koçtaş, IKEA, Hepsiburada, Kale, Banyomarka, BAUHAUS, Home Depot, Kohler, Villeroy &amp; Boch, Duravit, hansgrohe, GROHE, Geberit, Victorian Plumbing</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>12, 16</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Hizmet ve kampanya koşulları erişim tarihindeki haliyle aktarılmıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Inbound sezonsallık ve rakip ürün analizi</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Haziran 2026 · Ahrefs content gap, 4.202 kelime, 7 rakip</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Dört ürün kümesi güncel veriyle yeniden ölçülmüştür</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Google arama sonuçları (DataForSEO SERP API)</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>109 kelime · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Sıralamalar tek günlük gözlemdir ve gün içinde değişebilir; AI Overview içeriği 31 bloğun 24'ünde alınabilmiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>YouTube arama ve yorumlar (genişletilmiş)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>68 ifade · Türkiye · ilk 20 sonuç · 33 videonun 2.218 yorumu · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Kanal türü ve yorum teması anahtar ifadelerle atanmıştır; bir yorum birden fazla temaya girebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer ve Keywords Explorer (marka siteleri)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>24 marka ve uzman site top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Sayfalar URL ve en iyi kelimeye göre temalara eşlenmiştir; listelenen sayfalar site toplamının %66-93'ünü kapsar</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer (pazaryeri ve yapı market)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>9 site, banyo kategori sayfaları ve kelimeleri · Türkiye · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol ve Hepsiburada tarayıcı incelemesi</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Kategori ağacı, arama önerileri, marka filtreleri, mağaza ve çok satan listeleri · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada'da her listede ilk sayfa (36 ürün) okunmuştur; sıralama kişiselleştirmeye bağlı olarak değişebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="43" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Kart harcamaları, kartlı ödeme endeksi, tüketici eğilimi, konut, banka kredileri, hane halkı beklentileri · 2024-2026</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Kart harcamaları nominaldir; reel karşılaştırma için kartlı ödeme endeksinin reel serisi kullanılmıştır</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kaynakça</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Raporun metnindeki üst simge numaraları bu listeye bağlanmaktadır.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Kaynak</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Adres</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Erişim</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS · banka ve kredi kartı harcamaları, sektörel haftalık akım (BKM)</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>https://evds3.tcmb.gov.tr</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS · Kartlı Ödeme Endeksi (nominal ve reel)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>https://evds3.tcmb.gov.tr</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS · Tüketici Eğilim Anketi (TÜİK-TCMB) · aylık</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>https://evds3.tcmb.gov.tr</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS · konut satış istatistikleri (TÜİK) ve Konut Fiyat Endeksi</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>https://evds3.tcmb.gov.tr</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS · Banka Kredileri Eğilim Anketi · üç aylık, net yüzde</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>https://evds3.tcmb.gov.tr</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads Keyword Planner · 2.420 kategori kelimesi · Türkiye, Türkçe · Eyl 2024 - Ağu 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>https://ads.google.com/home/tools/keyword-planner/</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>VitrA kategori kelime araştırması · 2.420 kelime, 8 ana / 64 alt kategori · Inbound, 2025</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol arama sonuçları · 13 tema, ilk 40-45 ürün (rezervuar iç takımı 150) · fiyat, marka, değerlendirme sayısı</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>https://www.trendyol.com</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads keyword ideas (keywords for keywords) · 10 kök ifade grubu, 52.973 kelime · Türkiye, Türkçe · Eyl 2022 - Ağu 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>https://ads.google.com/home/tools/keyword-planner/</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Google Search Console · sc-domain:vitra.com.tr · sayfa, sorgu, cihaz ve ülke kırılımı · 1 Haz 2025 - 25 Eyl 2026</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>https://search.google.com/search-console</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Google Autocomplete · "vitra" ile başlayan 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.google.com.tr</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Google arama sonuçları (DataForSEO SERP API) · 109 kategori kelimesi, ilk 20 organik sonuç, AI Overview ve SERP özellikleri · Türkiye, Türkçe, mobil · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.google.com.tr</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>YouTube arama sonuçları · 30 kategori, montaj ve tamir ifadesi · Türkiye · ilk 20 sonuç</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Macit Tesisat · "VitrA gömme klozet tamiri çok basit" · YouTube</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=a1i0pneZhdw</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>YouTube arama sonuçları ve yorumlar · 68 arama ifadesi, 560 kanal, 2.218 yorum · Türkiye · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="43" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>vitra.com.tr ürün sitemap'i (7.804 adres), kategori, hizmet ve ürün sayfaları, Banyo Asistanı akışı</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>https://www.vitra.com.tr/sitemaps/sitemap-products.xml · https://www.vitra.com.tr/c-montaj-hizmeti · https://www.vitra.com.tr/kesif-hizmeti/kesif-hizmeti-p-etic_kesif</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="69" customHeight="1">
-      <c r="A21" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Rakip kategori sitemap'leri · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bauhaus.com.tr/google/sitemap/category · https://www.ikea.com.tr/sitemap/kategori.sitemap.xml · https://www.tekzen.com.tr/sitemap/categories/0.xml · https://www.banyomarka.com/xml/sitemap/category.xml · https://www.kale.com.tr/sitemap-category.xml</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Inbound · VitrA sezonsallık ve banyo mobilyası fırsat çalışması, rakip analizi ve ürün fırsatları · Haziran 2026</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Koçtaş · Banyo Tadilatı sayfası</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>https://www.koctas.com.tr/banyo-tadilati</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Koçtaş · Montaj hizmetleri ve banyo kampanyası koşulları</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>https://www.koctas.com.tr/hizmetlerimiz · https://www.koctas.com.tr/banyo-kampanyasi</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>IKEA Türkiye · Banyo, montaj hizmeti ve taksit bilgisi</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>https://www.ikea.com.tr/odalar/banyo · https://www.ikea.com.tr/montaj-hizmeti</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada · Kurulum hizmeti</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hepsiburada.com/staticPage/12413</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Kale · Montaj hizmetleri ve yedek parça sayfaları</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>https://www.kale.com.tr/montaj-hizmetleri · https://www.kale.com.tr/yedek-parcalar</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>BAUHAUS Almanya · Komplettbad-Service</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bauhaus.info/service/leistungen/montageservice/komplettbad</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>The Home Depot · Bathroom remodeling</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>https://www.homedepot.com/services/c/bathroom-remodel/d9843b7cb</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Reveal by KOHLER · Shower and bath remodel</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>https://reveal.kohler.com/en</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer · organik rakipler ve toplu alan adı metrikleri · Türkiye</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>https://ahrefs.com/site-explorer</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer ve Keywords Explorer · 24 marka ve uzman e-ticaret sitesi top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>https://ahrefs.com/site-explorer · https://ahrefs.com/keywords-explorer</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="43" customHeight="1">
-      <c r="A33" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Ahrefs Site Explorer · pazaryeri ve yapı market kategori sayfaları (Trendyol, Hepsiburada, Koçtaş, Akakçe, IKEA, Cimri, Amazon, Bauhaus, n11) · top pages ve organic keywords · Türkiye · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>https://ahrefs.com/site-explorer</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol · banyo, vitrifiye ve armatür kategori ağacı, arama önerileri, mağaza ve çok satan listeleri · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>https://www.trendyol.com/banyo-yapi-malzemeleri-x-c105718 · https://www.trendyol.com/magaza/vitra-m-144409</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada · banyo kategori listeleri, marka filtreleri, satıcı ve hizmet ürünleri (ilk sayfa, 36 ürün) · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hepsiburada.com</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Duravit · Bathroom planner</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>hansgrohe · Spare parts search</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>GROHE · Spare Parts Finder</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Geberit · AquaClean evde deneme</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="43" customHeight="1">
-      <c r="A41" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Banyomarka · Batarya ve musluk kombinleri</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>https://www.banyomarka.com/batarya-musluk-kombinleri</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Erişim 28.09.2026</t>
         </is>
       </c>
     </row>
@@ -19925,6 +19936,1268 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Yöntem ve Kapsam · Tablo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Yöntem ve Kapsam
+Kapsam: Bu rapor, Inbound'un erişimindeki veri kaynaklarıyla hazırlanmıştır. VitrA'dan beklenen pazaryeri performansı, GA4 dönüşüm ve site içi arama raporları, iade ve çağrı merkezi verisi geldiğinde ilgili bölümler eklenecek ve öneriler güncellenecektir.
+Sütun açıklamaları: Veri kaynağı: Kullanılan kaynak. | Kapsam: Dönem, coğrafya ve örneklem. | Kullanıldığı bölüm: Verinin işlendiği bölüm. | Not: Ölçüm sınırı veya yöntem notu.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Veri kaynağı</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kapsam</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Kullanıldığı bölüm</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="43" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads Keyword Planner</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.420 kelime · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>03, 04, 05</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads benzer kelimeler için birleşik hacim döndürür; aynı hacimli yazım varyantları toplamda tekrar sayılmıştır ve toplamlar üst sınır olarak okunmalıdır</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Google Search Console</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sorgu, cihaz, ülke</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>05, 06, 07</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sayfa ve sorgu raporları ilk 25.000 satırla sınırlıdır; sayfa×gün tablosu 100.000 satır</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Google Autocomplete</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>07, 17</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Öneriler tek günlük anlık görüntüdür; sıralama Google'ın sırasıdır</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>30 ifade · Türkiye · ilk sayfa · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>İzlenme sayıları video yayın tarihinden itibaren kümülatiftir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Organik rakipler ve Batch Analysis · Türkiye · 27.09.2026</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek ziyaret sayısı değildir</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads keyword ideas</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>10 kök ifade grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>04, 10, 11, 12</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Kelimeler 58 temalı sözlükle sınıflandırılmış, gürültü ifadeleri ayıklanmış, aynı aylık seriyi taşıyan yazım varyantları tek sayılmıştır; tema toplamları yaklaşık büyüklük gösterir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr ürün sitemap'i ve site incelemesi</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · Banyo Asistanı · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>10, 12, 16, 17</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayısı renk ve ölçü varyantlarını ayrı sayar; model sayısı renk ekleri ayıklanarak yaklaşık hesaplanmıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Rakip kategori sitemap'leri</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline · Koçtaş tarayıcı ile</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>11, 16</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Kategori varlığı gözlemidir; ürün derinliği ve satış hacmi ölçülmemiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol arama sonuçları</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>13 tema, ilk 40-45 ürün · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>04, 10, 11</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Değerlendirme sayısı satış hacmine yaklaşık gösterge olarak kullanılmıştır; sonuç sırası kişiselleştirmeye bağlı olarak değişebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="43" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Rakip ve benzer oyuncuların siteleri</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş, IKEA, Hepsiburada, Kale, Banyomarka, BAUHAUS, Home Depot, Kohler, Villeroy &amp; Boch, Duravit, hansgrohe, GROHE, Geberit, Victorian Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>12, 16</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Hizmet ve kampanya koşulları erişim tarihindeki haliyle aktarılmıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Inbound sezonsallık ve rakip ürün analizi</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Haziran 2026 · Ahrefs content gap, 4.202 kelime, 7 rakip</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Dört ürün kümesi güncel veriyle yeniden ölçülmüştür</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Google arama sonuçları (DataForSEO SERP API)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>109 kelime · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Sıralamalar tek günlük gözlemdir ve gün içinde değişebilir; AI Overview içeriği 31 bloğun 24'ünde alınabilmiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama ve yorumlar (genişletilmiş)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>68 ifade · Türkiye · ilk 20 sonuç · 33 videonun 2.218 yorumu · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Kanal türü ve yorum teması anahtar ifadelerle atanmıştır; bir yorum birden fazla temaya girebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer ve Keywords Explorer (marka siteleri)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>24 marka ve uzman site top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Sayfalar URL ve en iyi kelimeye göre temalara eşlenmiştir; listelenen sayfalar site toplamının %66-93'ünü kapsar</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer (pazaryeri ve yapı market)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>9 site, banyo kategori sayfaları ve kelimeleri · Türkiye · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol ve Hepsiburada tarayıcı incelemesi</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Kategori ağacı, arama önerileri, marka filtreleri, mağaza ve çok satan listeleri · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada'da her listede ilk sayfa (36 ürün) okunmuştur; sıralama kişiselleştirmeye bağlı olarak değişebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="43" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Kart harcamaları, kartlı ödeme endeksi, tüketici eğilimi, konut, banka kredileri, hane halkı beklentileri · 2024-2026</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Kart harcamaları nominaldir; reel karşılaştırma için kartlı ödeme endeksinin reel serisi kullanılmıştır</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kaynakça</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Raporun metnindeki üst simge numaraları bu listeye bağlanmaktadır.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kaynak</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Adres</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Erişim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS · banka ve kredi kartı harcamaları, sektörel haftalık akım (BKM)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>https://evds3.tcmb.gov.tr</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS · Kartlı Ödeme Endeksi (nominal ve reel)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>https://evds3.tcmb.gov.tr</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS · Tüketici Eğilim Anketi (TÜİK-TCMB) · aylık</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>https://evds3.tcmb.gov.tr</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS · konut satış istatistikleri (TÜİK) ve Konut Fiyat Endeksi</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>https://evds3.tcmb.gov.tr</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS · Banka Kredileri Eğilim Anketi · üç aylık, net yüzde</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>https://evds3.tcmb.gov.tr</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads Keyword Planner · 2.420 kategori kelimesi · Türkiye, Türkçe · Eyl 2024 - Ağu 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>https://ads.google.com/home/tools/keyword-planner/</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>VitrA kategori kelime araştırması · 2.420 kelime, 8 ana / 64 alt kategori · Inbound, 2025</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol arama sonuçları · 13 tema, ilk 40-45 ürün (rezervuar iç takımı 150) · fiyat, marka, değerlendirme sayısı</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.trendyol.com</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads keyword ideas (keywords for keywords) · 10 kök ifade grubu, 52.973 kelime · Türkiye, Türkçe · Eyl 2022 - Ağu 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>https://ads.google.com/home/tools/keyword-planner/</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Google Search Console · sc-domain:vitra.com.tr · sayfa, sorgu, cihaz ve ülke kırılımı · 1 Haz 2025 - 25 Eyl 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>https://search.google.com/search-console</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Google Autocomplete · "vitra" ile başlayan 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com.tr</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Google arama sonuçları (DataForSEO SERP API) · 109 kategori kelimesi, ilk 20 organik sonuç, AI Overview ve SERP özellikleri · Türkiye, Türkçe, mobil · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com.tr</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama sonuçları · 30 kategori, montaj ve tamir ifadesi · Türkiye · ilk 20 sonuç</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Macit Tesisat · "VitrA gömme klozet tamiri çok basit" · YouTube</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=a1i0pneZhdw</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama sonuçları ve yorumlar · 68 arama ifadesi, 560 kanal, 2.218 yorum · Türkiye · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="43" customHeight="1">
+      <c r="A20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr ürün sitemap'i (7.804 adres), kategori, hizmet ve ürün sayfaları, Banyo Asistanı akışı</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vitra.com.tr/sitemaps/sitemap-products.xml · https://www.vitra.com.tr/c-montaj-hizmeti · https://www.vitra.com.tr/kesif-hizmeti/kesif-hizmeti-p-etic_kesif</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="69" customHeight="1">
+      <c r="A21" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Rakip kategori sitemap'leri · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bauhaus.com.tr/google/sitemap/category · https://www.ikea.com.tr/sitemap/kategori.sitemap.xml · https://www.tekzen.com.tr/sitemap/categories/0.xml · https://www.banyomarka.com/xml/sitemap/category.xml · https://www.kale.com.tr/sitemap-category.xml</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Inbound · VitrA sezonsallık ve banyo mobilyası fırsat çalışması, rakip analizi ve ürün fırsatları · Haziran 2026</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş · Banyo Tadilatı sayfası</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.koctas.com.tr/banyo-tadilati</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş · Montaj hizmetleri ve banyo kampanyası koşulları</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.koctas.com.tr/hizmetlerimiz · https://www.koctas.com.tr/banyo-kampanyasi</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>IKEA Türkiye · Banyo, montaj hizmeti ve taksit bilgisi</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ikea.com.tr/odalar/banyo · https://www.ikea.com.tr/montaj-hizmeti</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada · Kurulum hizmeti</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hepsiburada.com/staticPage/12413</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Kale · Montaj hizmetleri ve yedek parça sayfaları</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kale.com.tr/montaj-hizmetleri · https://www.kale.com.tr/yedek-parcalar</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>BAUHAUS Almanya · Komplettbad-Service</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bauhaus.info/service/leistungen/montageservice/komplettbad</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>The Home Depot · Bathroom remodeling</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>https://www.homedepot.com/services/c/bathroom-remodel/d9843b7cb</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Reveal by KOHLER · Shower and bath remodel</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>https://reveal.kohler.com/en</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer · organik rakipler ve toplu alan adı metrikleri · Türkiye</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>https://ahrefs.com/site-explorer</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer ve Keywords Explorer · 24 marka ve uzman e-ticaret sitesi top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>https://ahrefs.com/site-explorer · https://ahrefs.com/keywords-explorer</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="43" customHeight="1">
+      <c r="A33" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer · pazaryeri ve yapı market kategori sayfaları (Trendyol, Hepsiburada, Koçtaş, Akakçe, IKEA, Cimri, Amazon, Bauhaus, n11) · top pages ve organic keywords · Türkiye · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>https://ahrefs.com/site-explorer</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol · banyo, vitrifiye ve armatür kategori ağacı, arama önerileri, mağaza ve çok satan listeleri · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.trendyol.com/banyo-yapi-malzemeleri-x-c105718 · https://www.trendyol.com/magaza/vitra-m-144409</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada · banyo kategori listeleri, marka filtreleri, satıcı ve hizmet ürünleri (ilk sayfa, 36 ürün) · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hepsiburada.com</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="95" customHeight="1">
+      <c r="A36" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Kanal politikaları taraması · vitra.com.tr, Koçtaş, Bauhaus, IKEA, Creavit, Banyomarka, Banyoline, Hepsiburada, Trendyol, Kale, E.C.A., Geberit, Grohe yardım, ödeme, teslimat, iade, garanti ve servis sayfaları · sosyal profiller · Google Maps ve SERP (DataForSEO) · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vitra.com.tr/odeme-rehberi · https://www.vitra.com.tr/teslimat-rehberi · https://www.vitra.com.tr/garanti-hizmetleri · https://www.koctas.com.tr/taksitler · https://www.bauhaus.com.tr/taksit-secenekleri · https://www.ikea.com.tr/odeme-secenekleri · https://www.banyoline.com/montaj-hizmeti · https://www.grohe.com/tr-TR/servis-destek/garanti</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Duravit · Bathroom planner</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>hansgrohe · Spare parts search</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>GROHE · Spare Parts Finder</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Geberit · AquaClean evde deneme</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="43" customHeight="1">
+      <c r="A42" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Banyomarka · Batarya ve musluk kombinleri</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>https://www.banyomarka.com/batarya-musluk-kombinleri</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Akakçe ve Cimri: 29 VitrA ürününde satıcı sayısı ve en düşük fiyat, kategori görünümü (Chrome okuması); kaynak D27; KISIT notu güncellendi
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -71,19 +71,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="62 Trendyol ve Hepsiburada ço" sheetId="62" state="visible" r:id="rId62"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="63 VitrA ürünlerinde kanal fi" sheetId="63" state="visible" r:id="rId63"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="64 Ürün grubuna göre fark med" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="65 Ödeme ve taksit koşulları" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="66 Kargo, teslimat, iade ve m" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="67 Garanti, yedek parça ve se" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="68 Sosyal ve keşif kanalları" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="69 Google Business Profile m" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="70 E-ticaret modelleri" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="71 Ürün keşfi ve dijital dene" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="72 Kanal rolleri" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="73 Hacimli ve ölçüye bağlı ür" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="74 Tamamlayıcı ürün kurgusu" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="75 Sonraki Adımlar" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="76 Yöntem ve Kapsam" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="65 Akakçe ve Cimri 29 VitrA " sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="66 Fiyat karşılaştırma sitele" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="67 Ödeme ve taksit koşulları" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="68 Kargo, teslimat, iade ve m" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="69 Garanti, yedek parça ve se" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="70 Sosyal ve keşif kanalları" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="71 Google Business Profile m" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="72 E-ticaret modelleri" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="73 Ürün keşfi ve dijital dene" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="74 Kanal rolleri" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="75 Hacimli ve ölçüye bağlı ür" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="76 Tamamlayıcı ürün kurgusu" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="77 Sonraki Adımlar" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="78 Yöntem ve Kapsam" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="79" state="visible" r:id="rId79"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17920,11 +17922,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="230" customHeight="1">
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Ürün tipi ve mecra bazında fiyat bandı
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün tipi: Google Shopping kelimelerinin eşlendiği ürün tipi; tüm markalar birlikte. | Trendyol: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Hepsiburada: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Amazon TR: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Koçtaş: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Bağımsız mağaza: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | VitrA Online: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Tüm mecralar: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir.</t>
         </is>
@@ -18556,11 +18558,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · En ucuz ve en pahalı mecra
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün tipi: Ürün tipi. | En düşük medyanlı mecra: Çok markalı mecralar arasında (en az 5 ilan) medyan fiyatı en düşük olan; resmi marka mağazaları hariç. | Medyan: TL. | En yüksek medyanlı mecra: Medyan fiyatı en yüksek çok markalı mecra. | Medyan: TL.</t>
         </is>
@@ -18905,11 +18907,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA ve Artema ilanlarında mecra farkı
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün tipi: Yalnızca başlığında VitrA veya Artema geçen ilanlar. | VitrA Online medyan (ilan): vitra.com.tr mağazasının Shopping ilanlarında medyan fiyat (TL) ve ilan sayısı. | Trendyol: Mecra medyanının VitrA Online medyanına göre farkı (ilan sayısı). Model karışımı aynı değildir; yön göstergesidir. | Hepsiburada: Aynı fark. | Koçtaş: Aynı fark. | Bağımsız mağaza: Aynı fark.</t>
         </is>
@@ -19114,11 +19116,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="202" customHeight="1">
+    <row r="2" ht="216" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Aynı ürünün satıcıları: 24 VitrA ve Artema listesi
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün listesi: Google Shopping'de aynı ürünü satan satıcıların toplandığı liste; VitrA ve Artema ürün adı aramalarından. | Satıcı: Listede görünen satıcı sayısı; 10 değeri "10 ve üzeri" anlamına gelir. | En ucuz satıcı (mecra): Listede en düşük toplam fiyatı veren satıcı ve mecra türü. | Min: TL. | Medyan: TL. | Maks: TL. | VitrA Online fiyat (sıra): Resmi mağazanın listedeki fiyatı ve fiyat sırası; "listede yok" ilk 10 satıcı arasında bulunmadığını gösterir. | VitrA Online / en düşük: Resmi mağaza fiyatının listedeki en düşük fiyata göre farkı.</t>
         </is>
@@ -20019,11 +20021,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Aynı ürünün satıcıları: 24 VitrA ve Artema listesi
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Mecra: Satıcı dökümündeki mecra türü. | Görüldüğü liste: 24 ürün listesinin kaçında satıcı olarak görünüyor. | En ucuz olduğu liste: Kaç listede en düşük fiyatı veriyor. | En düşük fiyata medyan fark: Mecranın fiyatının listedeki en düşük fiyata göre medyan farkı.</t>
         </is>
@@ -20709,11 +20711,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Marka payı
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Marka: İlan başlığında geçen marka; başlığında marka geçmeyen ilanlar (%65) dışarıdadır. | Listeleme: 27 kategori kelimesinin ilk 120 sonucundaki listeleme sayısı (3.240 satır). | Pay (ilk 120): Tüm listelemeler içindeki pay. | Pay (ilk 10): Yalnızca ilk 10 sonuç içindeki pay.</t>
         </is>
@@ -20933,11 +20935,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="146" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA Online'ın göründüğü kelimeler
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Kategori kelimesi: VitrA Online'ın Shopping sonuçlarında göründüğü 12 kelime; 15 kelimede hiç görünmüyor. | Listeleme: İlk 120 sonuçtaki VitrA Online ilanı. | En iyi sıra: İlanın en iyi sırası.</t>
         </is>
@@ -21153,11 +21155,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="230" customHeight="1">
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Trendyol ve Hepsiburada çok satan listeleri: 14 kategori
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Kategori: Pazaryerinde "çok satan" sıralamasının ilk 36 ürünü; 29.09.2026. | TY medyan (TL): Trendyol ilk 36 ürünün medyan fiyatı. | HB medyan (TL): Hepsiburada ilk 36 ürünün medyan fiyatı; dört kategoride arama sonucu kullanıldığı için aksesuar ağırlıklıdır. | TY 3P / 36: Trendyol'da üçüncü taraf satıcı listelemesi sayısı. | HB 3P / 36: Hepsiburada'da üçüncü taraf satıcı listelemesi; kalan marka mağazası ve Hepsiburada'nın kendi satışıdır. | TY en yüksek değerlendirme payı: Trendyol ilk 36'da değerlendirme sayısı payı en yüksek marka. | HB en yüksek değerlendirme payı: Hepsiburada ilk 36'da değerlendirme payı en yüksek marka. | VitrA + Artema TY: İlk 36'daki VitrA ve Artema ürün sayısı ve değerlendirme payı; "-" yer almıyor. | VitrA + Artema HB: Aynı ölçü, Hepsiburada.</t>
         </is>
@@ -21857,11 +21859,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="230" customHeight="1">
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA ürünlerinde kanal fiyat farkı: 29 ürün
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün: vitra.com.tr ürün sayfası; bağlantı canlı sayfaya gider. | Kod: Ürün kodu (SKU); eşleşme başlıkta kod geçen listelemelerle yapılmıştır. | Grup: Ürün grubu. | vitra.com.tr: Ürün sayfasındaki liste fiyatı (TL); sepette %10-15 ek indirim etiketi ayrıca vardır. | TY VitrA mağazası: Trendyol'daki VitrA mağazasının liste fiyatı; "-" listelenmemiş. | TY en düşük 3P (satıcı): Trendyol'da üçüncü taraf satıcıların en düşük fiyatı ve satıcı adı. | HB buybox (satıcı): Hepsiburada'da "sepete ekle" düğmesini kazanan satıcının fiyatı. | Koçtaş: Koçtaş'taki fiyat; 16 eşleşmenin tamamı üçüncü taraf satıcı listelemesidir. | En ucuz kanal: Liste fiyatı en düşük kanal. | Fark: vitra.com.tr liste fiyatından en ucuz kanala düşüş oranı. | vitra.com.tr stok: Gözlem anında ürün sayfasındaki stok durumu.</t>
         </is>
@@ -23442,11 +23444,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Ürün grubuna göre fark medyanı
-Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Cimri ve Akakçe bot koruması nedeniyle yalnızca sınırlı okunabilmiştir. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
 Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
 Sütun açıklamaları: Ürün grubu: Birden fazla kanalda fiyatı bulunan ürünlerin grubu. | Ürün sayısı: Karşılaştırılan ürün sayısı. | Fark medyanı: vitra.com.tr liste fiyatına göre en ucuz kanalın altında kalma oranının medyanı.</t>
         </is>
@@ -23584,6 +23586,1642 @@
 </file>
 
 <file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Akakçe ve Cimri: 29 VitrA ürününde satıcı sayısı ve en düşük fiyat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="230" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Akakçe ve Cimri: 29 VitrA ürününde satıcı sayısı ve en düşük fiyat
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Sütun açıklamaları: Ürün: VitrA veya Artema ürünü. | Kod: Ürün kodu; Akakçe ve Cimri kayıtları kodla eşlenmiştir. | Grup: Ürün grubu. | vitra.com.tr: Ürün sayfasındaki liste fiyatı (TL), 29.09.2026. | Akakçe satıcı: Akakçe'nin ürün için listelediği toplam fiyat (satıcı) sayısı. | Akakçe en düşük: Kargo dahil en düşük fiyat (TL), 30.09.2026. | En düşük fiyatın mecrası / satıcısı: Akakçe'de en düşük fiyatı veren pazaryeri ve o pazaryerindeki satıcı. | Akakçe medyan: Listelenen ilk 16 satıcının medyan fiyatı (TL). | Fark: vitra.com.tr liste fiyatından Akakçe en düşük fiyata düşüş; eksi değer vitra.com.tr'nin daha düşük olduğunu gösterir. | Cimri en düşük (fiyat sayısı): Cimri kategori kartındaki en düşük fiyat ve fiyat sayısı; "-" Cimri'de kod eşleşmesi yok.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Ürün</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kod</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Grup</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe satıcı</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe en düşük</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>En düşük fiyatın mecrası / satıcısı</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe medyan</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Fark</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Cimri en düşük (fiyat sayısı)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Integra Asma klozet</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>7041B003-0090</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Asma klozet</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>12027</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>10251</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Pttavm / Evdema</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>11139</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>10.251 (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>S50 Asma Klozet</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>5618L003-0850</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Asma klozet</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>8663</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>7308</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>n11 / evdema</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>8677</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>7.525 (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Sento Asma Klozet</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>7748B003-0559</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Asma klozet</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>14767</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>11814</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Amazon Türkiye</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>15671</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>S20 Asma Klozet</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>5505L003-0868</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Asma klozet</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>6455</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>7655</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada / Evdema</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>7655</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>-18.6</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>S20 Tezgahaltı Lavabo</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>5473B003-0618</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Lavabo</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>4913</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>5232</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş / Evdema</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>5813</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>S20 Lavabo</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>5501L003-0001</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Lavabo</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>4791</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>4020</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş / Evdeniste</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>5236</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Sento Lavabo Dolabı</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>60785</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Banyo mobilyası (lavabo dolabı)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>32596</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>40430</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş / Banyoatelier</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>40430</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>-24</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>28.000 (3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mia Boy Dolabı</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>66166</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Banyo mobilyası (boy dolabı)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>9992</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>9992</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada / VitrA</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>9992</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>9.892 (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Mia Banyo Dolabı Seti</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>67093</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Banyo mobilyası (lavabo dolabı)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>13881</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada / Damla Yapıı</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Mia Banyo Dolabı Seti</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>75102</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Banyo mobilyası (lavabo dolabı)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>12387</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>12870</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Pttavm / Hace Yapı Malzemeleri</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>13248</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Solid S Lavabo Bataryası</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>A42484</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (lavabo bataryası)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>5016</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>3821</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>4600</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Shift T10 Lavabo Bataryası</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>A43715</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (lavabo bataryası)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>4707</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>2989</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>5061</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Flow Round Lavabo Bataryası</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>A42923</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (lavabo bataryası)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>4707</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>2813</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş / Banyoline</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>3284</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>2.970 (8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Flow Round Banyo Bataryası</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>A43057</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (banyo bataryası)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>7112</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>3749</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>n11 / bodrum-akel</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>4524</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>3.749 (13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Minimax S Banyo Bataryası</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>A41994</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (banyo bataryası)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>5907</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>n11 / banyoom</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>4191</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>AquaHeat Termostatik Duş Bataryası</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>A47055EXPS</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (termostatik batarya)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>13892</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>6946</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada / VitrA</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>8168</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Filtreli Ara Musluk</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>A45200</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (ara musluk)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>427</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>324</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>n11 / enarhome</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>373</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Filtreli Çamaşır Musluğu</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>A45228</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Armatür (çamaşır musluğu)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>427</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>338</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>idefix / DMR YAPI MARKET</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>427</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>V8 Gömme Rezervuar Seti</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>800-1896</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Gömme rezervuar seti</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>8385</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>6056</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>idefix / Evdeniste</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>6254</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>V-Fix Prime 8cm Asma Klozetler için Gömm</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>768-1851-01</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Gömme rezervuar seti</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>5730</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>4985</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Amazon Türkiye / BANYOME</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>4.985 (5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Universal Klozet Kapağı</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>121-003-909</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Klozet kapağı</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1720</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Acarlaronline.net / Acarlaronline.net</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>1578</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>1.427 (14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Universal Klozet Kapağı</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>109-003-909</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Klozet kapağı</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1720</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>1176</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Pttavm / Evre Yapı</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>1420</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>1.199 (16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Universal Klozet Kapağı</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>84-003-009</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Klozet kapağı</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2612</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>1998</v>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>idefix / snn.yapımalzemeleri</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>2399</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>1.998 (5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>İç Takım</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>330B1314</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>İç takım</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>896</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>675</v>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>990</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="39" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Fiyat karşılaştırma sitelerinde kategori görünümü</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="216" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Fiyat karşılaştırma sitelerinde kategori görünümü
+Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Sütun açıklamaları: Kategori: Akakçe ve Cimri kategori sayfası. | Akakçe ürün: Kategorideki toplam ürün; "-" sayfada okunamadı. | Akakçe medyan (ilk 32): Popülerlik sırasındaki ilk 32 ürünün en düşük fiyat medyanı (TL). | Akakçe ilk 3 marka: İlk 32 üründe en çok ürünü olan markalar. | Ek fiyat medyanı: Ürün başına ek satıcı sayısı medyanı (ilk 32). | Cimri ürün: Cimri kategori sayfasının bildirdiği toplam ürün. | Cimri medyan (ilk 32): İlk 32 ürünün en düşük fiyat medyanı (TL). | Cimri marka sırası: Cimri'nin marka filtresindeki ilk 3 marka (ürün sayısına göre). | Cimri mağaza sırası: Cimri'nin mağaza filtresindeki ilk 4 mağaza.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe ürün</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe medyan (ilk 32)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Akakçe ilk 3 marka</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Ek fiyat medyanı</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Cimri ürün</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Cimri medyan (ilk 32)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Cimri marka sırası</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Cimri mağaza sırası</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Klozet</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1747</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>7308</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Creavit, VitrA, Bocchi</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>937</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>6481</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Creavit, VitrA, Serel</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, PttAVM, idefix, Yapıdeko</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Klozet kapağı</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1012</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>VitrA, Nkp, Visam</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>3477</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1080</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>VitrA, Visam, Nkp</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, PttAVM, idefix, Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Lavabo</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>4943</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>5190</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Turkuaz, İsvea, Bocchi</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>5001</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>3608</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Turkuaz, Cerastyle, Creavit</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, PttAVM, idefix, Koçtaş</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Banyo dolabı</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>4680</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Karen, Teta, Kenzlife</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>3814</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>5158</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Kenzlife, Teta Home, Orka</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, PttAVM, Koçtaş, Trendyol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Duşakabin</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>7066</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Durul, Monaqua, Teknesiz</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>18213</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>5990</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Durul, Sanica, Teknoduş</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş, Hepsiburada, idefix, PttAVM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Banyo bataryası</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>6105</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>3995</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Artema, E.C.A., Creavit</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>1582</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>3809</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A, Artema, GPD</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, idefix, PttAVM, Koçtaş</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Lavabo bataryası</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>3725</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Artema, E.C.A., Grohe</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>3047</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>2847</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A, Artema, GPD</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, idefix, PttAVM, Koçtaş</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Duş seti</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>3316</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Artema, E.C.A., Creavit</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>4888</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>3368</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A, Tema, Artema</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, idefix, PttAVM, Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Rezervuar</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>347</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>4250</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>VitrA, Visam, Geberit</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Gömme rezervuar</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>145</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>3892</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>VitrA, Visam, Serel</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada, PttAVM, idefix, Amazon</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Banyo aynası</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>2111</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Creavit, Nuun, Özlider</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>981</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>5390</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Buffer, Artema, Creavit</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş, PttAVM, Hepsiburada, idefix</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23611,7 +25249,7 @@
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Ödeme ve taksit koşulları
 Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 35
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
 Sütun açıklamaları: Site: Ödeme ve taksit sayfası okunan site; bağlantı ana sayfaya gider. | Taksit ve vade farksız koşul: Sitenin yardım, taksit veya ödeme rehberi sayfasındaki ifade; 29.09.2026. | Alışveriş kredisi: Sitede alışveriş kredisi veya mağaza kartı seçeneği. | Kapıda ödeme / havale: Kredi kartı dışındaki ödeme yolları. | Kurumsal fatura: Kurumsal fatura veya kurumsal kart seçeneği.</t>
         </is>
       </c>
@@ -23898,7 +25536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23926,7 +25564,7 @@
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Kargo, teslimat, iade ve montaj
 Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 35
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
 Sütun açıklamaları: Site: Teslimat, iade ve montaj sayfaları okunan site. | Ücretsiz kargo: Ücretsiz kargo eşiği. | Büyük ürün teslimat: Klozet, dolap, duşakabin gibi büyük ürünlerde teslimat süresi ve yöntemi. | İade: İade süresi ve büyük ürün koşulu. | Montaj: Montaj seçeneği, kapsamı ve fiyatı; 29.09.2026.</t>
         </is>
       </c>
@@ -24186,7 +25824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24213,7 +25851,7 @@
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Garanti, yedek parça ve servis iletişimi
 Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 35
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
 Sütun açıklamaları: Marka: Garanti ve servis sayfaları okunan marka; bağlantı sitesine gider. | Garanti süresi: Sitede yazılı garanti süresi; "arama özeti" sayfa açılamadığı için arama sonucundan alındığını gösterir. | Yedek parça: Yedek parça sayfası, aracı veya listesi. | Servis ve iletişim: Servis randevu akışı, telefon ve anlık mesaj kanalı.</t>
         </is>
       </c>
@@ -24373,454 +26011,6 @@
         <is>
           <t>Servis talebi formu, bayi bulucu</t>
         </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="160" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 35
-Sütun açıklamaları: Marka: Kanal büyüklükleri karşılaştırılan marka. | Instagram: Takipçi; profil girişe kapalı olduğu için Google sonuç özetinden, yaklaşık. "-" alınamadı. | YouTube: Abone, video ve toplam görüntüleme; kanal hakkında sayfası, 29.09.2026. | Pinterest: Profil takipçisi. | TikTok: Resmi hesap ve takipçi.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Marka</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Pinterest</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>VitrA Türkiye</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>~144K</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>1,58 Mn · 402 video · 55,8 Mn</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>1.478 + 3.825 (iki hesap)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Artema</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>~20K</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>4,75 B · 33 video · 19,7 Mn</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>3.825 (ortak hesap)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Grohe (global kanal)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>75,1 B · 627 video · 21,9 Mn</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>10325</v>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Geberit Türkiye</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>~39K</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Ayrı TR kanalı yok</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>E.C.A.</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>~24K</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Ayrı TR kanalı yok</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Creavit</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>2,17 B · 227 video · 7,1 Mn</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>187</v>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>118 takipçi</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Kale</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>948 · 577 video · 1,4 Mn</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>943</v>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Yok</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="160" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 35
-Sütun açıklamaları: İl: Google Maps'te VitrA etiketli satış noktası profillerinin ili. | Profil: Tekil profil sayısı (cid ile). | Toplam yorum: Profillerin toplam yorum sayısı. | Ortalama puan: Yorum ağırlıklı ortalama puan.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>İl</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Profil</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Toplam yorum</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Ortalama puan</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>İstanbul</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>64</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>3732</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Ankara</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>504</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>İzmir</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>461</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Muğla</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>533</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Mersin</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>125</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>4.6</v>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Antalya</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>338</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Bursa</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>271</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Hatay</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>87</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>4.5</v>
       </c>
     </row>
   </sheetData>
@@ -25228,6 +26418,454 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Sütun açıklamaları: Marka: Kanal büyüklükleri karşılaştırılan marka. | Instagram: Takipçi; profil girişe kapalı olduğu için Google sonuç özetinden, yaklaşık. "-" alınamadı. | YouTube: Abone, video ve toplam görüntüleme; kanal hakkında sayfası, 29.09.2026. | Pinterest: Profil takipçisi. | TikTok: Resmi hesap ve takipçi.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Marka</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>VitrA Türkiye</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>~144K</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>1,58 Mn · 402 video · 55,8 Mn</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1.478 + 3.825 (iki hesap)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Artema</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>~20K</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>4,75 B · 33 video · 19,7 Mn</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3.825 (ortak hesap)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Grohe (global kanal)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>75,1 B · 627 video · 21,9 Mn</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>10325</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Geberit Türkiye</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>~39K</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı TR kanalı yok</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>E.C.A.</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>~24K</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Ayrı TR kanalı yok</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Creavit</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2,17 B · 227 video · 7,1 Mn</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>187</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>118 takipçi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Kale</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>948 · 577 video · 1,4 Mn</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>943</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Sütun açıklamaları: İl: Google Maps'te VitrA etiketli satış noktası profillerinin ili. | Profil: Tekil profil sayısı (cid ile). | Toplam yorum: Profillerin toplam yorum sayısı. | Ortalama puan: Yorum ağırlıklı ortalama puan.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>İl</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Profil</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Toplam yorum</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Ortalama puan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>3732</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>504</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>İzmir</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>461</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Muğla</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>533</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mersin</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Antalya</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>338</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>271</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Hatay</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -25249,7 +26887,7 @@
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri
 Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 36 , 37 , 38 , 39 , 40 , 41 , 42
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 37 , 38 , 39 , 40 , 41 , 42 , 43
 Sütun açıklamaları: Oyuncu: İncelenen site. | Tip: İş modeli. | E-ticaret modeli: Ürün, kanal ve hizmetin nasıl bir araya getirildiği. | VitrA'ya uyarlanabilir nokta: VitrA'nın mevcut yapısına eklenebilecek unsur.</t>
         </is>
       </c>
@@ -25485,7 +27123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25513,7 +27151,7 @@
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · Ürün keşfi ve dijital deneyim örnekleri
 Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 36 , 37 , 38 , 39 , 40 , 41 , 42
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 37 , 38 , 39 , 40 , 41 , 42 , 43
 Sütun açıklamaları: Araç: Ürün keşfi ya da dijital deneyim aracı. | Örnek: Aracı kullanan oyuncular. | Ne sağlıyor?: Kullanıcıya sağladığı fayda. | VitrA'da: vitra.com.tr'deki karşılığı (29.09.2026). | Gözlem: Mevcut durum ve olası adım.</t>
         </is>
       </c>
@@ -25800,7 +27438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25953,7 +27591,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26172,7 +27810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26347,7 +27985,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26416,7 +28054,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 17 , 38 , 39</t>
+          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 17 , 39 , 40</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -26526,7 +28164,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 16 , 35</t>
+          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 16 , 36</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -26570,7 +28208,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>VitrA Online Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 33 , 35</t>
+          <t>VitrA Online Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 33 , 36</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -26592,7 +28230,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 35</t>
+          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 36</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -26724,7 +28362,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 17 , 36 , 37</t>
+          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 17 , 37 , 38</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -26878,7 +28516,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 40</t>
+          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 41</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -26939,13 +28577,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -27394,38 +29032,58 @@
     <row r="24" ht="43" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Site politika sayfaları, sosyal profiller, Google Maps ve SERP</t>
+          <t>Akakçe ve Cimri</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>13 site ve markanın ödeme, teslimat, iade, garanti ve servis sayfaları; 7 markanın sosyal hesapları; 103 Maps sorgusu; 15 + 10 kelime SERP · 29.09.2026</t>
+          <t>29 SKU arama ve ürün sayfası, 12 + 10 kategori sayfası · Chrome · 30.09.2026</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Bot korumalı sayfalarda değer arama özetinden alınmış ve işaretlenmiştir; Instagram ve TikTok sayıları yaklaşıktır</t>
+          <t>Akakçe satıcı listesi ilk 16 satıcıyla sınırlıdır; Cimri ürün sayfalarında satıcı listesi alınamadığı için kart düzeyi kullanılmıştır</t>
         </is>
       </c>
     </row>
     <row r="25" ht="43" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
+          <t>Site politika sayfaları, sosyal profiller, Google Maps ve SERP</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>13 site ve markanın ödeme, teslimat, iade, garanti ve servis sayfaları; 7 markanın sosyal hesapları; 103 Maps sorgusu; 15 + 10 kelime SERP · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Bot korumalı sayfalarda değer arama özetinden alınmış ve işaretlenmiştir; Instagram ve TikTok sayıları yaklaşıktır</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="43" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>TCMB EVDS</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Kart harcamaları, kartlı ödeme endeksi, tüketici eğilimi, konut, banka kredileri, hane halkı beklentileri · 2024-2026</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C26" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Kart harcamaları nominaldir; reel karşılaştırma için kartlı ödeme endeksinin reel serisi kullanılmıştır</t>
         </is>
@@ -27439,13 +29097,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -28173,18 +29831,18 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="95" customHeight="1">
+    <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="n">
         <v>35</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Kanal politikaları taraması · vitra.com.tr, Koçtaş, Bauhaus, IKEA, Creavit, Banyomarka, Banyoline, Hepsiburada, Trendyol, Kale, E.C.A., Geberit, Grohe yardım, ödeme, teslimat, iade, garanti ve servis sayfaları · sosyal profiller · Google Maps ve SERP (DataForSEO) · 29.09.2026</t>
+          <t>Akakçe arama, ürün ve kategori sayfaları (29 SKU, 12 kategori) · Cimri kategori ve marka sayfaları (10 kategori) · 30.09.2026</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/odeme-rehberi · https://www.vitra.com.tr/teslimat-rehberi · https://www.vitra.com.tr/garanti-hizmetleri · https://www.koctas.com.tr/taksitler · https://www.bauhaus.com.tr/taksit-secenekleri · https://www.ikea.com.tr/odeme-secenekleri · https://www.banyoline.com/montaj-hizmeti · https://www.grohe.com/tr-TR/servis-destek/garanti</t>
+          <t>https://www.akakce.com/klozet.html · https://www.cimri.com/klozet</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -28193,18 +29851,18 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
+    <row r="40" ht="95" customHeight="1">
       <c r="A40" s="6" t="n">
         <v>36</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
+          <t>Kanal politikaları taraması · vitra.com.tr, Koçtaş, Bauhaus, IKEA, Creavit, Banyomarka, Banyoline, Hepsiburada, Trendyol, Kale, E.C.A., Geberit, Grohe yardım, ödeme, teslimat, iade, garanti ve servis sayfaları · sosyal profiller · Google Maps ve SERP (DataForSEO) · 29.09.2026</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
+          <t>https://www.vitra.com.tr/odeme-rehberi · https://www.vitra.com.tr/teslimat-rehberi · https://www.vitra.com.tr/garanti-hizmetleri · https://www.koctas.com.tr/taksitler · https://www.bauhaus.com.tr/taksit-secenekleri · https://www.ikea.com.tr/odeme-secenekleri · https://www.banyoline.com/montaj-hizmeti · https://www.grohe.com/tr-TR/servis-destek/garanti</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -28219,12 +29877,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Duravit · Bathroom planner</t>
+          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
+          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -28239,12 +29897,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>hansgrohe · Spare parts search</t>
+          <t>Duravit · Bathroom planner</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
+          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -28259,12 +29917,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>GROHE · Spare Parts Finder</t>
+          <t>hansgrohe · Spare parts search</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
+          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -28279,12 +29937,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Geberit · AquaClean evde deneme</t>
+          <t>GROHE · Spare Parts Finder</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
+          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -28293,18 +29951,18 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="43" customHeight="1">
+    <row r="45" ht="30" customHeight="1">
       <c r="A45" s="6" t="n">
         <v>41</v>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
+          <t>Geberit · AquaClean evde deneme</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -28313,21 +29971,41 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
+    <row r="46" ht="43" customHeight="1">
       <c r="A46" s="6" t="n">
         <v>42</v>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
+          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
           <t>Banyomarka · Batarya ve musluk kombinleri</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>https://www.banyomarka.com/batarya-musluk-kombinleri</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Erişim 28.09.2026</t>
         </is>

</xml_diff>

<commit_message>
Tarayıcı doğrulaması: Cimri 19 ürün 110 teklif fiyat tablosuna, politika hücreleri sayfadan doğrulandı ve düzeltildi (Koçtaş kargo eşiği, teslimat, taksit), Şikayetvar marka yanıtı bulgusu, HB 2-3. sayfa notu; kaynak D28
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -9174,7 +9174,7 @@
         <is>
           <t>Bölüm: Katalog ve Talep Eşleşmesi
 Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. İkinci bölümde aynı temaların Trendyol'daki görünümü (fiyat bandı, öne çıkan satıcılar, VitrA varlığı) incelenmiştir.
-Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 8 , 9 , 17
+Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 8 , 9 , 18
 Sütun açıklamaları: Grup: Tema grubu. | Tema: Genişletilmiş kelime evreninde tanımlanan ürün teması. | Aylık talep: Eyl 2025 - Ağu 2026 aylık ortalama arama hacmi; yazım varyantları tek sayılmıştır. | 3 yıllık değişim: Eyl 22 - Ağu 23 ile Eyl 25 - Ağu 26 ortalamaları arasındaki değişim. | VitrA ürün: vitra.com.tr ürün sitemap'inde temaya eşlenen ürün adresi sayısı; renk ve ölçü varyantları ayrı sayılır. | Model: Renk ekleri ayıklanmış tekil ürün adı sayısı (yaklaşık). | Durum: VitrA kataloğunda temanın karşılığı: Var, Kısmi (sınırlı derinlik), Yok. | Not: Katalog ve pazaryeri gözlemi.</t>
         </is>
       </c>
@@ -10373,7 +10373,7 @@
         <is>
           <t>Bölüm: Katalog ve Talep Eşleşmesi · Pazaryerindeki görünüm: Trendyol
 Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. İkinci bölümde aynı temaların Trendyol'daki görünümü (fiyat bandı, öne çıkan satıcılar, VitrA varlığı) incelenmiştir.
-Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 8 , 9 , 17
+Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 8 , 9 , 18
 Sütun açıklamaları: Trendyol araması: Trendyol arama kutusuna yazılan ifade. | İncelenen ürün: İncelenen ilk sonuç sayısı. | Medyan fiyat (TL): İncelenen ürünlerin medyan satış fiyatı; havlupanda yalnız ısıtıcılı havlupanlar, iç takımda jenerik ürünler. | VitrA / Artema ürün: İlk sonuçlarda VitrA veya Artema markalı ürün sayısı. | En çok değerlendirme alan: Değerlendirme sayısı en yüksek ürünün markası, fiyatı ve değerlendirme sayısı; satış hacmi göstergesi olarak kullanılmıştır. | Gözlem: Sonuç sayfasının genel görünümü.</t>
         </is>
       </c>
@@ -10807,7 +10807,7 @@
         <is>
           <t>Bölüm: Yeni Kategori ve Segment Fırsatları
 Kapsam: Genişletilmiş kelime evreni (52.973 kelime) VitrA'nın bugünkü kategori ağacının dışına taşan temaları da kapsayacak şekilde sınıflandırılmıştır. Aşağıdaki tablo VitrA kataloğunda bulunmayan ya da sınırlı derinlikte bulunan temaları; talebi, rakipte kimin sattığını, VitrA'ya uyumu ve olası satış modelini birlikte göstermektedir. Haziran 2026 sezonsallık çalışmasındaki dört ürün kümesi (yedek parça, evye, arıtmalı batarya, universal akıllı kapak) bu tabloda güncel veriyle yeniden ölçülmüştür.
-Kaynak: Google Ads Keyword Planner genişletilmiş evren (48 ay) · vitra.com.tr ürün sitemap'i · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline kategori sitemap'leri · Trendyol arama sonuçları · Inbound VitrA sezonsallık ve rakip ürün analizi (Haziran 2026) · 28.09.2026 8 , 9 , 17 , 18 , 19
+Kaynak: Google Ads Keyword Planner genişletilmiş evren (48 ay) · vitra.com.tr ürün sitemap'i · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline kategori sitemap'leri · Trendyol arama sonuçları · Inbound VitrA sezonsallık ve rakip ürün analizi (Haziran 2026) · 28.09.2026 8 , 9 , 18 , 19 , 20
 Sütun açıklamaları: Tema: VitrA kataloğunda bulunmayan ya da sınırlı derinlikte bulunan ürün teması. | Aylık talep: Eyl 2025 - Ağu 2026 aylık ortalama arama hacmi; yazım varyantları tek sayılmıştır. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | 3 yıllık değişim: Eyl 22 - Ağu 23 ile Eyl 25 - Ağu 26 ortalamaları arasındaki değişim. | VitrA: VitrA kataloğundaki karşılık. | Rakipte kim satıyor?: Rakip sitelerin kategori ağaçları, Trendyol sonuçları ve Inbound'un Haziran 2026 rakip ürün analizi. | VitrA'ya uyum: Yakın: VitrA veya Artema üretim yetkinliğine bitişik · Orta: tamamlayıcı, iş ortağıyla sunulabilir · Uzak: marka ve kanal açısından uzak. | Model önerisi: Temanın vitra.com.tr'de nasıl sunulabileceği; 3P = üçüncü taraf satıcı. | Örnek aramalar: Temanın en yüksek hacimli aramaları.</t>
         </is>
       </c>
@@ -12293,7 +12293,7 @@
         <is>
           <t>Bölüm: Set, Komple Banyo ve Ürün + Hizmet · VitrA'nın mevcut hizmet kalemleri
 Kapsam: VitrA'nın bugün sunduğu set, montaj, keşif ve danışmanlık kurgusu site üzerinde incelenmiş; talep verisi ve rakip modelleriyle karşılaştırılmıştır.
-Kaynak: vitra.com.tr hizmet ve ürün sayfaları (29.09.2026) · Google Search Console · Google Ads Keyword Planner · rakip siteler ve kampanya sayfaları 9 , 10 , 17 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27
+Kaynak: vitra.com.tr hizmet ve ürün sayfaları (29.09.2026) · Google Search Console · Google Ads Keyword Planner · rakip siteler ve kampanya sayfaları 9 , 10 , 18 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 28
 Sütun açıklamaları: Hizmet: vitra.com.tr'de ürün olarak satılan hizmet kalemi. | Fiyat (TL): 29.09.2026 itibarıyla sitedeki fiyat. | Kapsam: Hizmet sayfasındaki kapsam açıklamasının özeti. Tüm montajlarda eski ürünün sökümü ve imhası dahil, 1 yıl servis garantisi; ilave tesisat malzemesi ve silikon ayrıca ücretlendirilir.</t>
         </is>
       </c>
@@ -12491,7 +12491,7 @@
         <is>
           <t>Bölüm: Set, Komple Banyo ve Ürün + Hizmet · Rakip ve benzer modeller
 Kapsam: VitrA'nın bugün sunduğu set, montaj, keşif ve danışmanlık kurgusu site üzerinde incelenmiş; talep verisi ve rakip modelleriyle karşılaştırılmıştır.
-Kaynak: vitra.com.tr hizmet ve ürün sayfaları (29.09.2026) · Google Search Console · Google Ads Keyword Planner · rakip siteler ve kampanya sayfaları 9 , 10 , 17 , 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27
+Kaynak: vitra.com.tr hizmet ve ürün sayfaları (29.09.2026) · Google Search Console · Google Ads Keyword Planner · rakip siteler ve kampanya sayfaları 9 , 10 , 18 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 28
 Sütun açıklamaları: Oyuncu: İncelenen marka veya perakendeci. | Set ve paket: Ürünlerin birlikte sunulma biçimi. | Hizmet: Montaj, keşif ve tadilat hizmetleri. | VitrA ile fark: VitrA'nın mevcut kurgusuna göre ayrışan nokta.</t>
         </is>
       </c>
@@ -12735,7 +12735,7 @@
         <is>
           <t>Bölüm: Rakip Görünürlüğü ve Kanal Ölçeği · Aynı aramalarda görünen siteler
 Kapsam: Benchmark seti üç halkadan oluşmaktadır: vitra.com.tr ile aynı aramalarda görünen organik rakipler, banyo sektörünün marka siteleri ve ürünün satıldığı pazaryeri ile yapı market kanalları. Ölçüm Ahrefs Türkiye verisiyle yapılmıştır; organik trafik değerleri tahmindir.
-Kaynak: Ahrefs Site Explorer · organik rakipler ve Batch Analysis · Türkiye · alt alan adları dahil · 27.09.2026 28
+Kaynak: Ahrefs Site Explorer · organik rakipler ve Batch Analysis · Türkiye · alt alan adları dahil · 27.09.2026 29
 Sütun açıklamaları: Alan adı: vitra.com.tr ile aynı kelimelerde sıralanan alan adı; Ahrefs organik rakipler raporu, Türkiye. | Tip: Sitenin iş modeli. | Ortak kelime: İki sitenin birlikte sıralandığı kelime sayısı. | VitrA kelimelerine oranı: Ortak kelime / vitra.com.tr'nin toplam sıralanan kelimesi (7.428). | Rakibin kelimesi: Rakibin Türkiye'de sıralandığı toplam kelime. | Organik trafik: Ahrefs tahmini aylık organik ziyaret. | DR: Domain Rating, 0-100.</t>
         </is>
       </c>
@@ -13227,7 +13227,7 @@
         <is>
           <t>Bölüm: Rakip Görünürlüğü ve Kanal Ölçeği · Kanal ölçeği: pazaryeri, yapı market, pureplayer ve marka siteleri
 Kapsam: Benchmark seti üç halkadan oluşmaktadır: vitra.com.tr ile aynı aramalarda görünen organik rakipler, banyo sektörünün marka siteleri ve ürünün satıldığı pazaryeri ile yapı market kanalları. Ölçüm Ahrefs Türkiye verisiyle yapılmıştır; organik trafik değerleri tahmindir.
-Kaynak: Ahrefs Site Explorer · organik rakipler ve Batch Analysis · Türkiye · alt alan adları dahil · 27.09.2026 28
+Kaynak: Ahrefs Site Explorer · organik rakipler ve Batch Analysis · Türkiye · alt alan adları dahil · 27.09.2026 29
 Sütun açıklamaları: Alan adı: Ahrefs Batch Analysis, Türkiye, alt alan adları dahil. | Tip: Sitenin iş modeli. | DR: Domain Rating. | Organik kelime: Türkiye'de sıralanan kelime sayısı. | İlk 3: İlk üç sırada yer alan kelime sayısı. | Organik trafik: Tahmini aylık organik ziyaret. | Paid trafik: Tahmini aylık Google Ads ziyareti. | Paid kelime: Reklam verilen kelime sayısı.</t>
         </is>
       </c>
@@ -13917,7 +13917,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Tema bazında VitrA ve en yüksek rakip
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 29
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 30
 Sütun açıklamaları: Tema: Top pages sayfalarının URL ve en iyi kelimesine göre eşlendiği kategori teması. | vitra.com.tr: Temaya eşlenen VitrA sayfalarının Ahrefs tahmini aylık organik trafiği. | En yüksek rakip: Temada en yüksek trafiği alan marka ya da uzman site. | Rakip trafiği: Rakibin tema trafiği. | Durum: VitrA ile en yüksek rakibin karşılaştırması.</t>
         </is>
       </c>
@@ -14458,7 +14458,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Kategori baş kelimeleri: hacim, potansiyel ve VitrA sırası
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 29
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 30
 Sütun açıklamaları: Baş kelime: Kategori baş kelimesi. | Aylık hacim: Ahrefs Keywords Explorer, Türkiye. | Trafik potansiyeli: Bu kelimede 1. sıradaki sayfanın tüm kelimelerinden aldığı tahmini aylık trafik (Ahrefs TP). | VitrA sırası: Google TR mobil SERP, 29.09.2026; "-" ilk 20'de yok.</t>
         </is>
       </c>
@@ -14804,7 +14804,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Rehber içerik: rakiplerin trafik aldığı konular
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 29
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 30
 Sütun açıklamaları: Rehber konusu: Rakiplerin rehber sayfalarından organik trafik aldığı konu. | Rakip sayfaları (aylık trafik): Ahrefs tahmini aylık organik trafik. | VitrA karşılığı: vitra.com.tr /ilham-veren-fikirler içindeki karşılık ve trafiği.</t>
         </is>
       </c>
@@ -15015,7 +15015,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Marka arama talebi
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 29
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 12 , 30
 Sütun açıklamaları: Marka araması: Aranan marka ifadesi. | Aylık hacim: Ahrefs, son 12 ay ortalaması, Türkiye. | Son 12 ay / önceki 12 ay: Ekim 2025 - Eylül 2026 ile Eylül 2024 - Ağustos 2025 aylık serilerinin toplam değişimi.</t>
         </is>
       </c>
@@ -15258,7 +15258,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Banyo trafiği hangi sitelerde?
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Site: Pazaryeri, perakendeci veya fiyat karşılaştırma sitesi. | Banyo ana kategorileri: Banyo, SSG, BM, armatür ve yıkanma sayfalarının Ahrefs tahmini aylık organik trafiği; sorgu satır sınırı nedeniyle alt sınırdır. | SSG: Klozet, lavabo, bide, pisuvar, rezervuar, klozet kapağı ve iç takım sayfaları. | BM: Banyo dolabı, lavabo dolabı, boy dolabı, ayna, çamaşır makinesi dolabı ve tezgah sayfaları. | Bitişik: Evye, mutfak bataryası, seramik, boy aynası, şofben gibi banyoya bitişik sayfalar. | En çok trafik alan sayfa: Banyonun ana kategorilerinde en yüksek trafikli adres.</t>
         </is>
       </c>
@@ -15576,7 +15576,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Alt kategori trafiği: Trendyol ve Hepsiburada
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Alt kategori: Sayfaların URL ve en iyi kelimesine göre sınıflandığı banyo alt kategorisi. | Grup: Ana: VitrA'nın sattığı banyo kategorileri · bitişik: banyoyla birlikte alınan ama VitrA'nın sınırlı sattığı kategoriler. | Trendyol trafik: Ahrefs tahmini aylık organik trafik. | Hepsiburada trafik: Ahrefs tahmini aylık organik trafik. | Trendyol'da en çok trafik getiren kelime: Kelime, aylık hacim ve Trendyol'un sırası.</t>
         </is>
       </c>
@@ -16431,7 +16431,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Kategori yapısı ve VitrA'nın listeleme payı
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Kategori: Pazaryerindeki kategori. | Trendyol ürün: Kategori sayfasının gösterdiği sonuç sayısı, 29.09.2026. | VitrA Trendyol: Kategori ve marka filtresiyle VitrA (ve Artema) listeleme sayısı. | Trendyol payı: VitrA listelemesinin kategori içindeki payı. | Hepsiburada ürün: Kategori sonuç sayısı; 10.000 üzeri "10.000+" olarak gösterilir. | VitrA Hepsiburada: Marka filtreli sonuç sayısı; "-" okunmadı. | Hepsiburada payı: VitrA listelemesinin kategori içindeki payı.</t>
         </is>
       </c>
@@ -16869,7 +16869,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Çok satanlarda kim önde?
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Kategori: Çok satan sıralamasının okunduğu kategori veya arama. | Trendyol: çok satanlarda öne çıkan: "En Çok Satan" sıralamasının ilk 36 ürününde değerlendirme payı en yüksek markalar. | VitrA Trendyol: İlk 36 içindeki VitrA ürün sayısı ve değerlendirme payı. | Hepsiburada: çok satanlarda öne çıkan: "Çok satanlar" sıralamasının ilk 36 ürününde öne çıkan markalar. | VitrA Hepsiburada: İlk 36 içindeki VitrA (Artema) ürün sayısı ve değerlendirme toplamı.</t>
         </is>
       </c>
@@ -17266,7 +17266,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Fiyat konumu
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Kategori: Fiyat karşılaştırılan kategori. | Trendyol kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Trendyol: VitrA marka filtresindeki çok satan ilk 36'nın medyanı, TL. | Hepsiburada kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Hepsiburada: VitrA marka filtreli ilk 36 medyanı, TL. | VitrA / kategori: VitrA medyanının kategori medyanına oranı (iki pazaryeri aralığı).</t>
         </is>
       </c>
@@ -17498,7 +17498,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Satıcı yapısı, hizmet ve arama önerileri
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Kök: Arama kutusuna yazılan ifade. | Trendyol önerileri: Arama kutusunun sıraladığı öneriler (kategori ve marka önerileri dahil). | Hepsiburada önerileri: Arama kutusunun öneri servisi; marka sayacı parantez içinde.</t>
         </is>
       </c>
@@ -17643,7 +17643,7 @@
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Trafik mıknatısı kategoriler
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
-Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 30 , 31 , 32
+Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
 Sütun açıklamaları: Kategori: Düşük fiyatlı, trafik getiren ve çapraz satışa uygun kategori. | 10 site toplamı: Trendyol, Hepsiburada, n11, Amazon, Koçtaş, Bauhaus, IKEA, Tekzen, Akakçe ve Cimri'de Ahrefs tahmini aylık organik trafik toplamı. | Trendyol: Aylık tahmini organik trafik. | Hepsiburada: Aylık tahmini organik trafik. | Koçtaş: Aylık tahmini organik trafik.</t>
         </is>
       </c>
@@ -17927,7 +17927,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Ürün tipi ve mecra bazında fiyat bandı
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün tipi: Google Shopping kelimelerinin eşlendiği ürün tipi; tüm markalar birlikte. | Trendyol: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Hepsiburada: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Amazon TR: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Koçtaş: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Bağımsız mağaza: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | VitrA Online: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir. | Tüm mecralar: Mecradaki ilanların medyan fiyatı (TL) ve ilan adedi; en az 3 ilan. Marka ve model karışımından etkilenir.</t>
         </is>
       </c>
@@ -18563,7 +18563,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · En ucuz ve en pahalı mecra
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün tipi: Ürün tipi. | En düşük medyanlı mecra: Çok markalı mecralar arasında (en az 5 ilan) medyan fiyatı en düşük olan; resmi marka mağazaları hariç. | Medyan: TL. | En yüksek medyanlı mecra: Medyan fiyatı en yüksek çok markalı mecra. | Medyan: TL.</t>
         </is>
       </c>
@@ -18912,7 +18912,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA ve Artema ilanlarında mecra farkı
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün tipi: Yalnızca başlığında VitrA veya Artema geçen ilanlar. | VitrA Online medyan (ilan): vitra.com.tr mağazasının Shopping ilanlarında medyan fiyat (TL) ve ilan sayısı. | Trendyol: Mecra medyanının VitrA Online medyanına göre farkı (ilan sayısı). Model karışımı aynı değildir; yön göstergesidir. | Hepsiburada: Aynı fark. | Koçtaş: Aynı fark. | Bağımsız mağaza: Aynı fark.</t>
         </is>
       </c>
@@ -19121,7 +19121,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Aynı ürünün satıcıları: 24 VitrA ve Artema listesi
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün listesi: Google Shopping'de aynı ürünü satan satıcıların toplandığı liste; VitrA ve Artema ürün adı aramalarından. | Satıcı: Listede görünen satıcı sayısı; 10 değeri "10 ve üzeri" anlamına gelir. | En ucuz satıcı (mecra): Listede en düşük toplam fiyatı veren satıcı ve mecra türü. | Min: TL. | Medyan: TL. | Maks: TL. | VitrA Online fiyat (sıra): Resmi mağazanın listedeki fiyatı ve fiyat sırası; "listede yok" ilk 10 satıcı arasında bulunmadığını gösterir. | VitrA Online / en düşük: Resmi mağaza fiyatının listedeki en düşük fiyata göre farkı.</t>
         </is>
       </c>
@@ -20026,7 +20026,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Aynı ürünün satıcıları: 24 VitrA ve Artema listesi
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Mecra: Satıcı dökümündeki mecra türü. | Görüldüğü liste: 24 ürün listesinin kaçında satıcı olarak görünüyor. | En ucuz olduğu liste: Kaç listede en düşük fiyatı veriyor. | En düşük fiyata medyan fark: Mecranın fiyatının listedeki en düşük fiyata göre medyan farkı.</t>
         </is>
       </c>
@@ -20716,7 +20716,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Marka payı
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Marka: İlan başlığında geçen marka; başlığında marka geçmeyen ilanlar (%65) dışarıdadır. | Listeleme: 27 kategori kelimesinin ilk 120 sonucundaki listeleme sayısı (3.240 satır). | Pay (ilk 120): Tüm listelemeler içindeki pay. | Pay (ilk 10): Yalnızca ilk 10 sonuç içindeki pay.</t>
         </is>
       </c>
@@ -20940,7 +20940,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA Online'ın göründüğü kelimeler
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Kategori kelimesi: VitrA Online'ın Shopping sonuçlarında göründüğü 12 kelime; 15 kelimede hiç görünmüyor. | Listeleme: İlk 120 sonuçtaki VitrA Online ilanı. | En iyi sıra: İlanın en iyi sırası.</t>
         </is>
       </c>
@@ -21160,7 +21160,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Trendyol ve Hepsiburada çok satan listeleri: 14 kategori
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Kategori: Pazaryerinde "çok satan" sıralamasının ilk 36 ürünü; 29.09.2026. | TY medyan (TL): Trendyol ilk 36 ürünün medyan fiyatı. | HB medyan (TL): Hepsiburada ilk 36 ürünün medyan fiyatı; dört kategoride arama sonucu kullanıldığı için aksesuar ağırlıklıdır. | TY 3P / 36: Trendyol'da üçüncü taraf satıcı listelemesi sayısı. | HB 3P / 36: Hepsiburada'da üçüncü taraf satıcı listelemesi; kalan marka mağazası ve Hepsiburada'nın kendi satışıdır. | TY en yüksek değerlendirme payı: Trendyol ilk 36'da değerlendirme sayısı payı en yüksek marka. | HB en yüksek değerlendirme payı: Hepsiburada ilk 36'da değerlendirme payı en yüksek marka. | VitrA + Artema TY: İlk 36'daki VitrA ve Artema ürün sayısı ve değerlendirme payı; "-" yer almıyor. | VitrA + Artema HB: Aynı ölçü, Hepsiburada.</t>
         </is>
       </c>
@@ -21864,7 +21864,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · VitrA ürünlerinde kanal fiyat farkı: 29 ürün
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün: vitra.com.tr ürün sayfası; bağlantı canlı sayfaya gider. | Kod: Ürün kodu (SKU); eşleşme başlıkta kod geçen listelemelerle yapılmıştır. | Grup: Ürün grubu. | vitra.com.tr: Ürün sayfasındaki liste fiyatı (TL); sepette %10-15 ek indirim etiketi ayrıca vardır. | TY VitrA mağazası: Trendyol'daki VitrA mağazasının liste fiyatı; "-" listelenmemiş. | TY en düşük 3P (satıcı): Trendyol'da üçüncü taraf satıcıların en düşük fiyatı ve satıcı adı. | HB buybox (satıcı): Hepsiburada'da "sepete ekle" düğmesini kazanan satıcının fiyatı. | Koçtaş: Koçtaş'taki fiyat; 16 eşleşmenin tamamı üçüncü taraf satıcı listelemesidir. | En ucuz kanal: Liste fiyatı en düşük kanal. | Fark: vitra.com.tr liste fiyatından en ucuz kanala düşüş oranı. | vitra.com.tr stok: Gözlem anında ürün sayfasındaki stok durumu.</t>
         </is>
       </c>
@@ -23449,7 +23449,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Ürün grubuna göre fark medyanı
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Ürün grubu: Birden fazla kanalda fiyatı bulunan ürünlerin grubu. | Ürün sayısı: Karşılaştırılan ürün sayısı. | Fark medyanı: vitra.com.tr liste fiyatına göre en ucuz kanalın altında kalma oranının medyanı.</t>
         </is>
       </c>
@@ -23603,7 +23603,7 @@
     <col width="39" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -23613,13 +23613,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="230" customHeight="1">
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Akakçe ve Cimri: 29 VitrA ürününde satıcı sayısı ve en düşük fiyat
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
-Sütun açıklamaları: Ürün: VitrA veya Artema ürünü. | Kod: Ürün kodu; Akakçe ve Cimri kayıtları kodla eşlenmiştir. | Grup: Ürün grubu. | vitra.com.tr: Ürün sayfasındaki liste fiyatı (TL), 29.09.2026. | Akakçe satıcı: Akakçe'nin ürün için listelediği toplam fiyat (satıcı) sayısı. | Akakçe en düşük: Kargo dahil en düşük fiyat (TL), 30.09.2026. | En düşük fiyatın mecrası / satıcısı: Akakçe'de en düşük fiyatı veren pazaryeri ve o pazaryerindeki satıcı. | Akakçe medyan: Listelenen ilk 16 satıcının medyan fiyatı (TL). | Fark: vitra.com.tr liste fiyatından Akakçe en düşük fiyata düşüş; eksi değer vitra.com.tr'nin daha düşük olduğunu gösterir. | Cimri en düşük (fiyat sayısı): Cimri kategori kartındaki en düşük fiyat ve fiyat sayısı; "-" Cimri'de kod eşleşmesi yok.</t>
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
+Sütun açıklamaları: Ürün: VitrA veya Artema ürünü. | Kod: Ürün kodu; Akakçe ve Cimri kayıtları kodla eşlenmiştir. | Grup: Ürün grubu. | vitra.com.tr: Ürün sayfasındaki liste fiyatı (TL), 29.09.2026. | Akakçe satıcı: Akakçe'nin ürün için listelediği toplam fiyat (satıcı) sayısı. | Akakçe en düşük: Kargo dahil en düşük fiyat (TL), 30.09.2026. | En düşük fiyatın mecrası / satıcısı: Akakçe'de en düşük fiyatı veren pazaryeri ve o pazaryerindeki satıcı. | Akakçe medyan: Listelenen ilk 16 satıcının medyan fiyatı (TL). | Fark: vitra.com.tr liste fiyatından Akakçe en düşük fiyata düşüş; eksi değer vitra.com.tr'nin daha düşük olduğunu gösterir. | Cimri en düşük (teklif): Cimri ürün sayfasındaki en düşük teklif (TL) ve teklif sayısı, 30.09.2026; "-" Cimri'de kod eşleşmesi yok ya da yalnızca paket kaydı var.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -23680,7 +23680,7 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Cimri en düşük (fiyat sayısı)</t>
+          <t>Cimri en düşük (teklif)</t>
         </is>
       </c>
     </row>
@@ -23722,7 +23722,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>10.251 (2)</t>
+          <t>10.251 (1)</t>
         </is>
       </c>
     </row>
@@ -23890,7 +23890,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.232 (1)</t>
         </is>
       </c>
     </row>
@@ -23932,7 +23932,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.121 (1)</t>
         </is>
       </c>
     </row>
@@ -24092,7 +24092,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12.263 (1)</t>
         </is>
       </c>
     </row>
@@ -24134,7 +24134,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.821 (4)</t>
         </is>
       </c>
     </row>
@@ -24218,7 +24218,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>2.970 (8)</t>
+          <t>2.970 (10)</t>
         </is>
       </c>
     </row>
@@ -24680,7 +24680,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>753 (9)</t>
         </is>
       </c>
     </row>
@@ -24724,7 +24724,7 @@
         <is>
           <t>Bölüm: Fiyat ve Satıcı Manzarası: Shopping, Trendyol, Hepsiburada · Fiyat karşılaştırma sitelerinde kategori görünümü
 Kapsam: Google Shopping'de 27 kategori ve 3 marka kelimesinin ilk 120 sonucu (3.600 ilan) ile 12 VitrA ve Artema ürün adının satıcı dökümü (24 liste) alınmıştır; Akakçe ürün ve kategori sayfaları ile Cimri kategori ve marka sayfaları ayrıca okunmuştur. Fiyatlar 29.09.2026 tarihli anlık değerlerdir ve günlük değişebilir; mecra medyanları marka ve model karışımından etkilenir, aynı ürün üzerinden kıyas yalnızca satıcı dökümünde yapılmıştır.
-Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 33
+Kaynak: Google Shopping (DataForSEO merchant/google/products ve merchant/google/sellers) · 30 kelime × 120 ilan, 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026 · Akakçe ve Cimri sınırlı okuma 34
 Sütun açıklamaları: Kategori: Akakçe ve Cimri kategori sayfası. | Akakçe ürün: Kategorideki toplam ürün; "-" sayfada okunamadı. | Akakçe medyan (ilk 32): Popülerlik sırasındaki ilk 32 ürünün en düşük fiyat medyanı (TL). | Akakçe ilk 3 marka: İlk 32 üründe en çok ürünü olan markalar. | Ek fiyat medyanı: Ürün başına ek satıcı sayısı medyanı (ilk 32). | Cimri ürün: Cimri kategori sayfasının bildirdiği toplam ürün. | Cimri medyan (ilk 32): İlk 32 ürünün en düşük fiyat medyanı (TL). | Cimri marka sırası: Cimri'nin marka filtresindeki ilk 3 marka (ürün sayısına göre). | Cimri mağaza sırası: Cimri'nin mağaza filtresindeki ilk 4 mağaza.</t>
         </is>
       </c>
@@ -25232,7 +25232,7 @@
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
@@ -25248,8 +25248,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Ödeme ve taksit koşulları
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuş, bot korumalı sayfalardaki değerler 30.09.2026'da tarayıcıda açılarak doğrulanmış ve düzeltilmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 37
 Sütun açıklamaları: Site: Ödeme ve taksit sayfası okunan site; bağlantı ana sayfaya gider. | Taksit ve vade farksız koşul: Sitenin yardım, taksit veya ödeme rehberi sayfasındaki ifade; 29.09.2026. | Alışveriş kredisi: Sitede alışveriş kredisi veya mağaza kartı seçeneği. | Kapıda ödeme / havale: Kredi kartı dışındaki ödeme yolları. | Kurumsal fatura: Kurumsal fatura veya kurumsal kart seçeneği.</t>
         </is>
       </c>
@@ -25312,7 +25312,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="43" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>koctas.com.tr</t>
@@ -25320,7 +25320,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Online 5.000 TL üzeri 7 taksite kadar vade farksız; vade farklı 9'a kadar</t>
+          <t>Yardım sayfasında 10.000 TL ve üzeri vade farksız (World 2-7 taksit); taksitler sayfasında 5.000 TL eşiği yazıyor, iki sayfa tutarsız</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -25330,7 +25330,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Yok</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -25509,17 +25509,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Kategori, tutar ve kart tipine göre; her üründe taksit yok (arama özeti)</t>
+          <t>Taksit yapılabilen ürünlerde seçenek sunuluyor; her üründe yok</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Trendyol Kredi Pazaryeri</t>
+          <t>Alışveriş kredisi: 500 TL üzeri sepette 36 aya kadar</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Doğrulanamadı</t>
+          <t>Yok (kapıda ödeme ve havale yok)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -25547,8 +25547,8 @@
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="57" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -25563,8 +25563,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Kargo, teslimat, iade ve montaj
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuş, bot korumalı sayfalardaki değerler 30.09.2026'da tarayıcıda açılarak doğrulanmış ve düzeltilmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 37
 Sütun açıklamaları: Site: Teslimat, iade ve montaj sayfaları okunan site. | Ücretsiz kargo: Ücretsiz kargo eşiği. | Büyük ürün teslimat: Klozet, dolap, duşakabin gibi büyük ürünlerde teslimat süresi ve yöntemi. | İade: İade süresi ve büyük ürün koşulu. | Montaj: Montaj seçeneği, kapsamı ve fiyatı; 29.09.2026.</t>
         </is>
       </c>
@@ -25708,7 +25708,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="17" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>koctas.com.tr</t>
@@ -25716,22 +25716,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Doğrulanamadı (arama özeti 300-600 TL)</t>
+          <t>300 TL ve üzeri; altı 49,90 TL</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Nakliye 4 gün içinde (arama özeti)</t>
+          <t>Ürün sayfasındaki tarih aralığı; 30 desi üstü lojistikle kata teslim, altı apartman kapısına</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>14 gün</t>
+          <t>14 gün; iade kodu 7 gün; montajı yapılmış demonte ürün ve ambalajı açılmış klozet takımı iade dışı</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>20 ilde montaj; seçili mobilyada ücretsiz; Ustabilir</t>
+          <t>Koçtaş ve Koçtaş Fix illerinde ücretli montaj, 2 yıl işçilik garantisi; söküm ek ücretli</t>
         </is>
       </c>
     </row>
@@ -25770,26 +25770,26 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Bulunamadı</t>
+          <t>Eşik herkese açık sayfada yok; Bugün Kapında 54,90 TL, Yarın Kapında 49,90 TL (Premium ücretsiz)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Mobilya birden fazla pakette, HepsiJET XL</t>
+          <t>Mobilya birden fazla pakette, HepsiJET XL; büyük ürün iadesi adresten randevuyla</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>14 gün, demonte ve orijinal kutu</t>
+          <t>14 gün, demonte ve orijinal kutu; Kapında İade ücretsiz</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>69 ilde sepete eklenebilir montaj; klozet montajı 2.730 TL (Mr Usta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
+          <t>69 ilde sepete eklenebilir montaj; klozet montajı 2.730 TL (Mr Usta); tekrar kurulumda servis bedeli</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>trendyol.com</t>
@@ -25797,17 +25797,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Alıcı eşiği doğrulanamadı</t>
+          <t>Genel eşik yok; standart kargo 59,99 TL, "kargo bedava" etiketli ürünlerde ücretsiz</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Satıcının anlaşmalı taşıyıcısı</t>
+          <t>30 desi üstü lojistikle (Horoz, Ceva) kata teslim</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>15 gün; montajı tamamlanmış ürün iade dışı</t>
+          <t>15 gün; kurulum gerektiren ürün yetkili servis dışında açılırsa iade dışı</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -25850,8 +25850,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Garanti, yedek parça ve servis iletişimi
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuş, bot korumalı sayfalardaki değerler 30.09.2026'da tarayıcıda açılarak doğrulanmış ve düzeltilmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 37
 Sütun açıklamaları: Marka: Garanti ve servis sayfaları okunan marka; bağlantı sitesine gider. | Garanti süresi: Sitede yazılı garanti süresi; "arama özeti" sayfa açılamadığı için arama sonucundan alındığını gösterir. | Yedek parça: Yedek parça sayfası, aracı veya listesi. | Servis ve iletişim: Servis randevu akışı, telefon ve anlık mesaj kanalı.</t>
         </is>
       </c>
@@ -25925,7 +25925,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Creavit</t>
@@ -25933,12 +25933,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Seramik 12, gömme rezervuar 10, armatür 5 yıl (arama özeti)</t>
+          <t>SSG için 12 yıl, armatür için 2 yıl garanti belgesi (PDF)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Katalogda yedek parça listesi</t>
+          <t>Sitede yedek parça girişi bulunamadı</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -25977,12 +25977,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Vitrifiyede ömür boyu; AquaClean 10 yıl parça bulunabilirliği (arama özeti)</t>
+          <t>Garanti koşulları PDF olarak medya merkezinde; süre sayfada yazmıyor</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Yedek parça ve bulunabilirlik sayfası</t>
+          <t>Ayrı sayfa yok; bayi ve yetkili servis üzerinden</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -26439,8 +26439,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Sosyal ve keşif kanalları
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuş, bot korumalı sayfalardaki değerler 30.09.2026'da tarayıcıda açılarak doğrulanmış ve düzeltilmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 37
 Sütun açıklamaları: Marka: Kanal büyüklükleri karşılaştırılan marka. | Instagram: Takipçi; profil girişe kapalı olduğu için Google sonuç özetinden, yaklaşık. "-" alınamadı. | YouTube: Abone, video ve toplam görüntüleme; kanal hakkında sayfası, 29.09.2026. | Pinterest: Profil takipçisi. | TikTok: Resmi hesap ve takipçi.</t>
         </is>
       </c>
@@ -26693,8 +26693,8 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Politikaları ve Keşif Kanalları · Google Business Profile: mağaza ve servis noktaları
-Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuştur; bot korumalı sayfalarda değerler arama sonucu özetinden alınmış ve "arama özeti" olarak işaretlenmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
-Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 36
+Kapsam: VitrA'nın ve rakiplerinin kamuya açık ödeme, teslimat, iade, montaj ve garanti koşulları ile sosyal kanal, Google Business Profile ve Google Shopping görünürlüğü karşılaştırılmıştır. Sayfalar 29.09.2026 tarihinde okunmuş, bot korumalı sayfalardaki değerler 30.09.2026'da tarayıcıda açılarak doğrulanmış ve düzeltilmiştir. "Bulunamadı" bilginin sayfada görünmediğini gösterir, bulunmadığı anlamına gelmeyebilir.
+Kaynak: Site yardım, ödeme, teslimat, iade, garanti ve servis sayfaları (29.09.2026) · YouTube ve Pinterest profil sayfaları · Google sonuç özetleri (Instagram, TikTok) · Google Maps (DataForSEO, 103 sorgu) · Google TR mobil ve masaüstü SERP (DataForSEO, 15 + 10 kelime) 37
 Sütun açıklamaları: İl: Google Maps'te VitrA etiketli satış noktası profillerinin ili. | Profil: Tekil profil sayısı (cid ile). | Toplam yorum: Profillerin toplam yorum sayısı. | Ortalama puan: Yorum ağırlıklı ortalama puan.</t>
         </is>
       </c>
@@ -26887,7 +26887,7 @@
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri
 Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 37 , 38 , 39 , 40 , 41 , 42 , 43
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 21 , 22 , 23 , 24 , 25 , 26 , 27 , 28 , 38 , 39 , 40 , 41 , 42 , 43 , 44
 Sütun açıklamaları: Oyuncu: İncelenen site. | Tip: İş modeli. | E-ticaret modeli: Ürün, kanal ve hizmetin nasıl bir araya getirildiği. | VitrA'ya uyarlanabilir nokta: VitrA'nın mevcut yapısına eklenebilecek unsur.</t>
         </is>
       </c>
@@ -27151,7 +27151,7 @@
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · Ürün keşfi ve dijital deneyim örnekleri
 Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
-Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 20 , 21 , 22 , 23 , 24 , 25 , 26 , 27 , 37 , 38 , 39 , 40 , 41 , 42 , 43
+Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 21 , 22 , 23 , 24 , 25 , 26 , 27 , 28 , 38 , 39 , 40 , 41 , 42 , 43 , 44
 Sütun açıklamaları: Araç: Ürün keşfi ya da dijital deneyim aracı. | Örnek: Aracı kullanan oyuncular. | Ne sağlıyor?: Kullanıcıya sağladığı fayda. | VitrA'da: vitra.com.tr'deki karşılığı (29.09.2026). | Gözlem: Mevcut durum ve olası adım.</t>
         </is>
       </c>
@@ -27465,7 +27465,7 @@
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Kanal rolleri
 Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
-Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 17
+Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 18
 Sütun açıklamaları: Kanal: Satış kanalı. | Bugünkü rol: Bu çalışmadaki gözlemlere dayalı mevcut konum; VitrA'nın panel verisiyle doğrulanacaktır. | Önerilen rol: Kanalın büyüme planında üstlenebileceği rol. | Öne çıkarılabilecek ürün grubu: Talep ve ihtiyaç verisine göre kanalda öne çıkarılabilecek grup.</t>
         </is>
       </c>
@@ -27618,7 +27618,7 @@
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Hacimli ve ölçüye bağlı ürünlerde etkileşim modeli
 Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
-Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 17
+Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 18
 Sütun açıklamaları: Bileşen: Hacimli ve ölçüye bağlı üründe karar öncesi belirsizliği azaltan unsur. | VitrA'da bugün: vitra.com.tr üzerindeki mevcut uygulama (29.09.2026). | Durum: Var, Kısmi (sınırlı kapsam), Yok. | Geliştirme alanı: Mevcut yapının üzerine eklenebilecek adım.</t>
         </is>
       </c>
@@ -27837,7 +27837,7 @@
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Tamamlayıcı ürün kurgusu
 Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
-Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 17
+Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 6 , 8 , 10 , 11 , 18
 Sütun açıklamaları: Ürün grubu: VitrA'nın üretmediği veya sınırlı ürettiği, kategori satın almasıyla birlikte ihtiyaç duyulan grup. | Talep sinyali: Kelime araştırması, autocomplete veya Search Console'daki ifade. | Bugün nerede satılıyor?: Kullanıcının bu ürünü bulduğu kanal; rakip site incelemesine göre. | Model önerisi: vitra.com.tr için değerlendirilebilecek satış modeli.</t>
         </is>
       </c>
@@ -28054,7 +28054,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 17 , 39 , 40</t>
+          <t>İç takım ve yedek parça aramaları aylık 117K; eski yedek parça sayfası ayda ~300 tık alıyordu ve bugün tek ürünlü kategoriye yönleniyor; Trendyol'da VitrA iç takımda ilk sırada 8 , 9 , 10 , 18 , 40 , 41</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -28076,7 +28076,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Montaj, keşif, ücretsiz montajlı mobilya ve Banyo Asistanı mevcut ama ayrı sunuluyor; tasarım ve tadilat aramaları büyüyor; Koçtaş, BAUHAUS ve Kohler proje satışına geçmiş 9 , 17 , 20 , 25 , 27</t>
+          <t>Montaj, keşif, ücretsiz montajlı mobilya ve Banyo Asistanı mevcut ama ayrı sunuluyor; tasarım ve tadilat aramaları büyüyor; Koçtaş, BAUHAUS ve Kohler proje satışına geçmiş 9 , 18 , 21 , 26 , 28</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -28098,7 +28098,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Duşakabin talebi aylık 297K; duşakabin ürün sayfasında montaj ya da keşif seçeneği bulunmuyor 9 , 17</t>
+          <t>Duşakabin talebi aylık 297K; duşakabin ürün sayfasında montaj ya da keşif seçeneği bulunmuyor 9 , 18</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -28120,7 +28120,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Üst bantta "vade farksız 6 ay", Banyo Asistanı'nda "9 taksit"; kullanıcı "vitra 9 taksit" ve "vitra taksit seçenekleri" arıyor 11 , 17</t>
+          <t>Üst bantta "vade farksız 6 ay", Banyo Asistanı'nda "9 taksit"; kullanıcı "vitra 9 taksit" ve "vitra taksit seçenekleri" arıyor 11 , 18</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -28142,7 +28142,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>BM aramalarının %9,5'i perakendeci adıyla yapılıyor; Trendyol'da banyo dolabı medyanı 3.249 TL, VitrA 14.462 TL; Hepsiburada'da VitrA ürünlerinin %69'u üçüncü taraf satıcıda 8 , 9 , 28 , 31 , 32</t>
+          <t>BM aramalarının %9,5'i perakendeci adıyla yapılıyor; Trendyol'da banyo dolabı medyanı 3.249 TL, VitrA 14.462 TL; Hepsiburada'da VitrA ürünlerinin %69'u üçüncü taraf satıcıda 8 , 9 , 29 , 32 , 33</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -28164,7 +28164,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 16 , 36</t>
+          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 16 , 37</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -28186,7 +28186,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>29 üründen 19'unda en ucuz kanal pazaryeri (medyan %24,7); Trendyol'da VitrA mağazasıyla birlikte bulunan 6 üründe 3P daha ucuz; Hepsiburada'da aynı ürün için birden fazla katalog kaydı 33 , 34</t>
+          <t>29 üründen 19'unda en ucuz kanal pazaryeri (medyan %24,7); Trendyol'da VitrA mağazasıyla birlikte bulunan 6 üründe 3P daha ucuz; Hepsiburada'da aynı ürün için birden fazla katalog kaydı 34 , 35</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -28208,7 +28208,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>VitrA Online Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 33 , 36</t>
+          <t>VitrA Online Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 34 , 37</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -28230,7 +28230,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 36</t>
+          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 37</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -28252,7 +28252,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Banyo dolabı aylık 60.000 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; banyo bataryası ve taharet musluğunda VitrA ilk 20'de yok; baş kelimelerin çoğunda KD 0-2 12 , 29</t>
+          <t>Banyo dolabı aylık 60.000 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; banyo bataryası ve taharet musluğunda VitrA ilk 20'de yok; baş kelimelerin çoğunda KD 0-2 12 , 30</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -28274,7 +28274,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Hela taşı 64,4K arama / 1 ürün, havlupan 50,7K arama / 2 ürün, çamaşır makinesi dolabı 103K arama / 29 ürün ama Trendyol ilk 40'ta yok 8 , 9 , 17</t>
+          <t>Hela taşı 64,4K arama / 1 ürün, havlupan 50,7K arama / 2 ürün, çamaşır makinesi dolabı 103K arama / 29 ürün ama Trendyol ilk 40'ta yok 8 , 9 , 18</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -28296,7 +28296,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 8 , 9 , 19</t>
+          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 8 , 9 , 20</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -28318,7 +28318,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 560K; Trendyol'da armatür markası yok 8 , 9 , 19</t>
+          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 560K; Trendyol'da armatür markası yok 8 , 9 , 20</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -28340,7 +28340,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Yaşlı ve engelli ürünleri aylık 29,4K (YoY +%8,1 ); ürünler katalogda var ama tek sayfada toplanmıyor 9 , 17</t>
+          <t>Yaşlı ve engelli ürünleri aylık 29,4K (YoY +%8,1 ); ürünler katalogda var ama tek sayfada toplanmıyor 9 , 18</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -28362,7 +28362,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 17 , 37 , 38</t>
+          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 9 , 18 , 38 , 39</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -28406,7 +28406,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Rakip rehberler tıkanıklık, koku, su kaçırma ve fayans hesabından trafik alıyor (Creavit 1.416, Kalekim 2.675); "klozet yaptırmak kaç TL", "klozet kapakları standart mı" soruları SERP'te; VitrA 24 AI Overview'un 7'sinde kaynak 12 , 29</t>
+          <t>Rakip rehberler tıkanıklık, koku, su kaçırma ve fayans hesabından trafik alıyor (Creavit 1.416, Kalekim 2.675); "klozet yaptırmak kaç TL", "klozet kapakları standart mı" soruları SERP'te; VitrA 24 AI Overview'un 7'sinde kaynak 12 , 30</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -28428,7 +28428,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 16 ayda 36.458 tık almış 10 , 17</t>
+          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 16 ayda 36.458 tık almış 10 , 18</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -28494,7 +28494,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 9 , 20</t>
+          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 9 , 21</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -28516,7 +28516,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 41</t>
+          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 6 , 42</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 21.000 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 29</t>
+          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 21.000 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 30</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -29037,7 +29037,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>29 SKU arama ve ürün sayfası, 12 + 10 kategori sayfası · Chrome · 30.09.2026</t>
+          <t>29 SKU arama ve ürün sayfası, 12 + 10 kategori sayfası, Cimri 19 ürün sayfası · Chrome · 30.09.2026</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
@@ -29045,11 +29045,11 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Akakçe satıcı listesi ilk 16 satıcıyla sınırlıdır; Cimri ürün sayfalarında satıcı listesi alınamadığı için kart düzeyi kullanılmıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="43" customHeight="1">
+          <t>Akakçe satıcı listesi ilk 16 satıcıyla sınırlıdır; Cimri arama sayfası engelli, 10 SKU eşleşmemiştir; paket ve set kayıtları fiyat kıyasına alınmamıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="56" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Site politika sayfaları, sosyal profiller, Google Maps ve SERP</t>
@@ -29065,7 +29065,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Bot korumalı sayfalarda değer arama özetinden alınmış ve işaretlenmiştir; Instagram ve TikTok sayıları yaklaşıktır</t>
+          <t>Bot korumalı sayfalar 30.09.2026'da tarayıcıda açılarak doğrulanmıştır (31 hücre: 14 doğrulandı, 10 kısmen, 4 yeni, 1 düzeltildi, 2 bulunamadı); Instagram ve TikTok sayıları yaklaşıktır</t>
         </is>
       </c>
     </row>
@@ -29103,7 +29103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -29471,18 +29471,18 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="43" customHeight="1">
+    <row r="21" ht="82" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>vitra.com.tr ürün sitemap'i (7.804 adres), kategori, hizmet ve ürün sayfaları, Banyo Asistanı akışı</t>
+          <t>Tarayıcı doğrulaması (Chrome, 30.09.2026) · Cimri ürün sayfaları (19 ürün, 110 teklif) · Koçtaş, Trendyol, n11, Amazon TR ve Hepsiburada yardım sayfaları · Creavit, Geberit ve Duravit garanti ve servis sayfaları · Şikayetvar şikayet ve marka sayfaları · Hepsiburada çok satan 2-3. sayfa</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/sitemaps/sitemap-products.xml · https://www.vitra.com.tr/c-montaj-hizmeti · https://www.vitra.com.tr/kesif-hizmeti/kesif-hizmeti-p-etic_kesif</t>
+          <t>https://www.koctas.com.tr/myaccount/faq · https://www.trendyol.com/yardim/iade · https://www.n11.com/destek-merkezi · https://www.amazon.com.tr/gp/help/customer/display.html?nodeId=GNWCU626A4NXEEGJ · https://www.creavit.com.tr/dokumanlar/ · https://www.duravit.com.tr/servis_hizmeti/faqs.tr-tr.html</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -29491,18 +29491,18 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="69" customHeight="1">
+    <row r="22" ht="43" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Rakip kategori sitemap'leri · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline</t>
+          <t>vitra.com.tr ürün sitemap'i (7.804 adres), kategori, hizmet ve ürün sayfaları, Banyo Asistanı akışı</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>https://www.bauhaus.com.tr/google/sitemap/category · https://www.ikea.com.tr/sitemap/kategori.sitemap.xml · https://www.tekzen.com.tr/sitemap/categories/0.xml · https://www.banyomarka.com/xml/sitemap/category.xml · https://www.kale.com.tr/sitemap-category.xml</t>
+          <t>https://www.vitra.com.tr/sitemaps/sitemap-products.xml · https://www.vitra.com.tr/c-montaj-hizmeti · https://www.vitra.com.tr/kesif-hizmeti/kesif-hizmeti-p-etic_kesif</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -29511,18 +29511,18 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="69" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Inbound · VitrA sezonsallık ve banyo mobilyası fırsat çalışması, rakip analizi ve ürün fırsatları · Haziran 2026</t>
+          <t>Rakip kategori sitemap'leri · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
+          <t>https://www.bauhaus.com.tr/google/sitemap/category · https://www.ikea.com.tr/sitemap/kategori.sitemap.xml · https://www.tekzen.com.tr/sitemap/categories/0.xml · https://www.banyomarka.com/xml/sitemap/category.xml · https://www.kale.com.tr/sitemap-category.xml</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -29537,12 +29537,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Koçtaş · Banyo Tadilatı sayfası</t>
+          <t>Inbound · VitrA sezonsallık ve banyo mobilyası fırsat çalışması, rakip analizi ve ürün fırsatları · Haziran 2026</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>https://www.koctas.com.tr/banyo-tadilati</t>
+          <t>https://github.com/erdogan1ozdemir/vitra-sezon-tr</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -29557,12 +29557,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Koçtaş · Montaj hizmetleri ve banyo kampanyası koşulları</t>
+          <t>Koçtaş · Banyo Tadilatı sayfası</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://www.koctas.com.tr/hizmetlerimiz · https://www.koctas.com.tr/banyo-kampanyasi</t>
+          <t>https://www.koctas.com.tr/banyo-tadilati</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -29577,12 +29577,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>IKEA Türkiye · Banyo, montaj hizmeti ve taksit bilgisi</t>
+          <t>Koçtaş · Montaj hizmetleri ve banyo kampanyası koşulları</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>https://www.ikea.com.tr/odalar/banyo · https://www.ikea.com.tr/montaj-hizmeti</t>
+          <t>https://www.koctas.com.tr/hizmetlerimiz · https://www.koctas.com.tr/banyo-kampanyasi</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -29597,12 +29597,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Hepsiburada · Kurulum hizmeti</t>
+          <t>IKEA Türkiye · Banyo, montaj hizmeti ve taksit bilgisi</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>https://www.hepsiburada.com/staticPage/12413</t>
+          <t>https://www.ikea.com.tr/odalar/banyo · https://www.ikea.com.tr/montaj-hizmeti</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -29617,12 +29617,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Kale · Montaj hizmetleri ve yedek parça sayfaları</t>
+          <t>Hepsiburada · Kurulum hizmeti</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>https://www.kale.com.tr/montaj-hizmetleri · https://www.kale.com.tr/yedek-parcalar</t>
+          <t>https://www.hepsiburada.com/staticPage/12413</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -29637,12 +29637,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>BAUHAUS Almanya · Komplettbad-Service</t>
+          <t>Kale · Montaj hizmetleri ve yedek parça sayfaları</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>https://www.bauhaus.info/service/leistungen/montageservice/komplettbad</t>
+          <t>https://www.kale.com.tr/montaj-hizmetleri · https://www.kale.com.tr/yedek-parcalar</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -29657,12 +29657,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>The Home Depot · Bathroom remodeling</t>
+          <t>BAUHAUS Almanya · Komplettbad-Service</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>https://www.homedepot.com/services/c/bathroom-remodel/d9843b7cb</t>
+          <t>https://www.bauhaus.info/service/leistungen/montageservice/komplettbad</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -29677,12 +29677,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Reveal by KOHLER · Shower and bath remodel</t>
+          <t>The Home Depot · Bathroom remodeling</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>https://reveal.kohler.com/en</t>
+          <t>https://www.homedepot.com/services/c/bathroom-remodel/d9843b7cb</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -29697,12 +29697,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer · organik rakipler ve toplu alan adı metrikleri · Türkiye</t>
+          <t>Reveal by KOHLER · Shower and bath remodel</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>https://ahrefs.com/site-explorer</t>
+          <t>https://reveal.kohler.com/en</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -29717,12 +29717,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer ve Keywords Explorer · 24 marka ve uzman e-ticaret sitesi top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
+          <t>Ahrefs Site Explorer · organik rakipler ve toplu alan adı metrikleri · Türkiye</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>https://ahrefs.com/site-explorer · https://ahrefs.com/keywords-explorer</t>
+          <t>https://ahrefs.com/site-explorer</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -29731,18 +29731,18 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="43" customHeight="1">
+    <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="n">
         <v>30</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer · pazaryeri ve yapı market kategori sayfaları (Trendyol, Hepsiburada, Koçtaş, Akakçe, IKEA, Cimri, Amazon, Bauhaus, n11) · top pages ve organic keywords · Türkiye · 28.09.2026</t>
+          <t>Ahrefs Site Explorer ve Keywords Explorer · 24 marka ve uzman e-ticaret sitesi top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>https://ahrefs.com/site-explorer</t>
+          <t>https://ahrefs.com/site-explorer · https://ahrefs.com/keywords-explorer</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -29751,18 +29751,18 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
+    <row r="35" ht="43" customHeight="1">
       <c r="A35" s="6" t="n">
         <v>31</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Trendyol · banyo, vitrifiye ve armatür kategori ağacı, arama önerileri, mağaza ve çok satan listeleri · 29.09.2026</t>
+          <t>Ahrefs Site Explorer · pazaryeri ve yapı market kategori sayfaları (Trendyol, Hepsiburada, Koçtaş, Akakçe, IKEA, Cimri, Amazon, Bauhaus, n11) · top pages ve organic keywords · Türkiye · 28.09.2026</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>https://www.trendyol.com/banyo-yapi-malzemeleri-x-c105718 · https://www.trendyol.com/magaza/vitra-m-144409</t>
+          <t>https://ahrefs.com/site-explorer</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -29777,12 +29777,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Hepsiburada · banyo kategori listeleri, marka filtreleri, satıcı ve hizmet ürünleri (ilk sayfa, 36 ürün) · 29.09.2026</t>
+          <t>Trendyol · banyo, vitrifiye ve armatür kategori ağacı, arama önerileri, mağaza ve çok satan listeleri · 29.09.2026</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>https://www.hepsiburada.com</t>
+          <t>https://www.trendyol.com/banyo-yapi-malzemeleri-x-c105718 · https://www.trendyol.com/magaza/vitra-m-144409</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -29791,18 +29791,18 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="43" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="6" t="n">
         <v>33</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Google Shopping (DataForSEO merchant/google/products ve sellers) · 27 kategori + 3 marka kelimesi, ilk 120 ilan; 12 VitrA ve Artema ürünü için 24 satıcı listesi · Türkiye · 29.09.2026 · Akakçe ve Cimri sınırlı okuma</t>
+          <t>Hepsiburada · banyo kategori listeleri, marka filtreleri, satıcı ve hizmet ürünleri (ilk sayfa, 36 ürün) · 29.09.2026</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>https://shopping.google.com · https://www.akakce.com · https://www.cimri.com</t>
+          <t>https://www.hepsiburada.com</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -29817,12 +29817,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Trendyol ve Hepsiburada çok satan listeleri (14 kategori × 36 ürün, 1.008 kayıt) · 29 VitrA ve Artema ürününde vitra.com.tr, Trendyol, Hepsiburada ve Koçtaş liste fiyatı · 29.09.2026</t>
+          <t>Google Shopping (DataForSEO merchant/google/products ve sellers) · 27 kategori + 3 marka kelimesi, ilk 120 ilan; 12 VitrA ve Artema ürünü için 24 satıcı listesi · Türkiye · 29.09.2026 · Akakçe ve Cimri sınırlı okuma</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>https://www.trendyol.com/magaza/vitra-m-144409 · https://www.hepsiburada.com · https://www.koctas.com.tr</t>
+          <t>https://shopping.google.com · https://www.akakce.com · https://www.cimri.com</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -29831,18 +29831,18 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
+    <row r="39" ht="43" customHeight="1">
       <c r="A39" s="6" t="n">
         <v>35</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Akakçe arama, ürün ve kategori sayfaları (29 SKU, 12 kategori) · Cimri kategori ve marka sayfaları (10 kategori) · 30.09.2026</t>
+          <t>Trendyol ve Hepsiburada çok satan listeleri (14 kategori × 36 ürün, 1.008 kayıt) · 29 VitrA ve Artema ürününde vitra.com.tr, Trendyol, Hepsiburada ve Koçtaş liste fiyatı · 29.09.2026</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.akakce.com/klozet.html · https://www.cimri.com/klozet</t>
+          <t>https://www.trendyol.com/magaza/vitra-m-144409 · https://www.hepsiburada.com · https://www.koctas.com.tr</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -29851,18 +29851,18 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="95" customHeight="1">
+    <row r="40" ht="30" customHeight="1">
       <c r="A40" s="6" t="n">
         <v>36</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Kanal politikaları taraması · vitra.com.tr, Koçtaş, Bauhaus, IKEA, Creavit, Banyomarka, Banyoline, Hepsiburada, Trendyol, Kale, E.C.A., Geberit, Grohe yardım, ödeme, teslimat, iade, garanti ve servis sayfaları · sosyal profiller · Google Maps ve SERP (DataForSEO) · 29.09.2026</t>
+          <t>Akakçe arama, ürün ve kategori sayfaları (29 SKU, 12 kategori) · Cimri kategori ve marka sayfaları (10 kategori) · 30.09.2026</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/odeme-rehberi · https://www.vitra.com.tr/teslimat-rehberi · https://www.vitra.com.tr/garanti-hizmetleri · https://www.koctas.com.tr/taksitler · https://www.bauhaus.com.tr/taksit-secenekleri · https://www.ikea.com.tr/odeme-secenekleri · https://www.banyoline.com/montaj-hizmeti · https://www.grohe.com/tr-TR/servis-destek/garanti</t>
+          <t>https://www.akakce.com/klozet.html · https://www.cimri.com/klozet</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -29871,18 +29871,18 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
+    <row r="41" ht="95" customHeight="1">
       <c r="A41" s="6" t="n">
         <v>37</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
+          <t>Kanal politikaları taraması · vitra.com.tr, Koçtaş, Bauhaus, IKEA, Creavit, Banyomarka, Banyoline, Hepsiburada, Trendyol, Kale, E.C.A., Geberit, Grohe yardım, ödeme, teslimat, iade, garanti ve servis sayfaları · sosyal profiller · Google Maps ve SERP (DataForSEO) · 29.09.2026</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
+          <t>https://www.vitra.com.tr/odeme-rehberi · https://www.vitra.com.tr/teslimat-rehberi · https://www.vitra.com.tr/garanti-hizmetleri · https://www.koctas.com.tr/taksitler · https://www.bauhaus.com.tr/taksit-secenekleri · https://www.ikea.com.tr/odeme-secenekleri · https://www.banyoline.com/montaj-hizmeti · https://www.grohe.com/tr-TR/servis-destek/garanti</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -29897,12 +29897,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Duravit · Bathroom planner</t>
+          <t>Villeroy &amp; Boch · 3D online bathroom planner</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
+          <t>https://www.villeroy-boch.co.uk/r/bathroom-ideas/planning/bathroom-planner-online/</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -29917,12 +29917,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>hansgrohe · Spare parts search</t>
+          <t>Duravit · Bathroom planner</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
+          <t>https://www.duravit.com/en-us/service/bathroom-planner/</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -29937,12 +29937,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>GROHE · Spare Parts Finder</t>
+          <t>hansgrohe · Spare parts search</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
+          <t>https://www.hansgrohe-usa.com/service/spare-parts-search</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -29957,12 +29957,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Geberit · AquaClean evde deneme</t>
+          <t>GROHE · Spare Parts Finder</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
+          <t>https://www.grohe.com/en-GB/service-support/spare-parts-finder</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -29971,18 +29971,18 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="43" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="n">
         <v>42</v>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
+          <t>Geberit · AquaClean evde deneme</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+          <t>https://www.geberit.de/badezimmerprodukte/wcs-urinale/dusch-wcs-geberit-aquaclean/testen/</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -29991,21 +29991,41 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1">
+    <row r="47" ht="43" customHeight="1">
       <c r="A47" s="6" t="n">
         <v>43</v>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
+          <t>Victorian Plumbing · Bathroom suites ve finansman</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>https://www.victorianplumbing.co.uk/bathroom-suites · https://www.victorianplumbing.co.uk/help-and-customer-service/bathroom-finance</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 28.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
           <t>Banyomarka · Batarya ve musluk kombinleri</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>https://www.banyomarka.com/batarya-musluk-kombinleri</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Erişim 28.09.2026</t>
         </is>

</xml_diff>

<commit_message>
Düzen ve veri güncellemeleri: aylık ortalama etiketleri, autocomplete hacim rozetleri, sıralanabilir ve kopyalanabilir tablolar, sola bitişik içindekiler, başlık ve vurgu stilleri
- Talep ve ihtiyaç tablolarında "Oca-Ağu 2026" başlıkları "2026 aylık ort." olarak netleştirildi (değerler zaten aylık ortalamaydı)
- Autocomplete kelimelerine Google Ads 2026 aylık ortalama hacim rozeti (714 kelime, DataForSEO)
- Tüm tablolarda sütun başlığına tıklayarak sıralama ve tablo üstünde kopyalama düğmesi (TSV + HTML)
- İçindekiler sola bitişik, içerik alanı genişletildi; h2 gradient alt çizgi, h3 vurgu zemini; alt başlık açıklamaları tam genişlik
- Insight metinlerinde marka adları kalın, üstünlük ifadeleri coral vurgu
- Katalog ve derin bölümlerinde en çok değerlendirilen ürün: marka bağlantılı, fiyat ve değerlendirme ayrı sütun; "Çok satanlarda kim önde?" tablosu yapılandırıldı

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -783,7 +783,7 @@
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -796,13 +796,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: İhtiyaç Dili: Kullanıcı Ne Arıyor?
 Kapsam: Aynı kelime seti, kullanıcının hangi ihtiyaçla aradığına göre yeniden sınıflandırılmıştır. Kategori adıyla yapılan jenerik aramaların dışında kalan altı ihtiyaç sınıfı, e-ticaret sayfalarının hangi soruya cevap vermesi gerektiğini göstermektedir.
 Kaynak: Google Ads Keyword Planner (ihtiyaç sınıfları, Oca-Ağu 2025 ve 2026) · Google Search Console, sc-domain:vitra.com.tr, 1 Haz 2025 - 25 Eyl 2026, ilk 25.000 sorgu 6 , 10
-Sütun açıklamaları: İhtiyaç sınıfı: Kelimenin taşıdığı ihtiyaç; ifade kalıplarına göre sınıflandırılmıştır, markalı kelimeler dışarıda tutulmuştur. | Tanım: Sınıfa giren ifade kalıpları. | Kelime: Sınıftaki kelime sayısı. | Oca-Ağu 2026: Ocak - Ağustos 2026 aylık ortalama hacim toplamı. | Pay: Sınıfın toplam markasız hacim içindeki payı. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | Örnek: Sınıfın en yüksek hacimli kelimeleri.</t>
+Sütun açıklamaları: İhtiyaç sınıfı: Kelimenin taşıdığı ihtiyaç; ifade kalıplarına göre sınıflandırılmıştır, markalı kelimeler dışarıda tutulmuştur. | Tanım: Sınıfa giren ifade kalıpları. | Kelime: Sınıftaki kelime sayısı. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi (sınıftaki kelimelerin toplamı). | Pay: Sınıfın toplam markasız hacim içindeki payı. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | Örnek: Sınıfın en yüksek hacimli kelimeleri.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2026</t>
+          <t>2026 aylık ort.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1070,7 +1070,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -1086,13 +1086,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: İhtiyaç Dili: Kullanıcı Ne Arıyor? · Kategori bazında ihtiyaç dağılımı
 Kapsam: Aynı kelime seti, kullanıcının hangi ihtiyaçla aradığına göre yeniden sınıflandırılmıştır. Kategori adıyla yapılan jenerik aramaların dışında kalan altı ihtiyaç sınıfı, e-ticaret sayfalarının hangi soruya cevap vermesi gerektiğini göstermektedir.
 Kaynak: Google Ads Keyword Planner (ihtiyaç sınıfları, Oca-Ağu 2025 ve 2026) · Google Search Console, sc-domain:vitra.com.tr, 1 Haz 2025 - 25 Eyl 2026, ilk 25.000 sorgu 6 , 10
-Sütun açıklamaları: Kategori: Ana kategori. | Markasız hacim: Oca-Ağu 2026 aylık ortalama, markalı kelimeler hariç. | Fiyat: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Tasarım ve fikir: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Seçim ve karşılaştırma: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Ölçü ve teknik: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Montaj: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Tamir ve bakım: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026.</t>
+Sütun açıklamaları: Kategori: Ana kategori. | Markasız hacim · 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama, markalı kelimeler hariç. | Fiyat: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Tasarım ve fikir: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Seçim ve karşılaştırma: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Ölçü ve teknik: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Montaj: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026. | Tamir ve bakım: Sınıfın kategori hacmi içindeki payı, Oca-Ağu 2026.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Markasız hacim</t>
+          <t>Markasız hacim · 2026 aylık ort.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -2904,7 +2904,7 @@
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2915,13 +2915,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="146" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · "vitra" ile başlayan aramalar
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
 Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
-Sütun açıklamaları: Kök ifade: Google arama kutusuna yazılan ifade; öneriler bu ifadenin devamı olarak gelmektedir. | Autocomplete önerileri: Google'ın Türkiye, Türkçe, masaüstü Chrome için döndürdüğü ilk 10 tamamlama önerisi; sırası Google'ın sırasıdır.</t>
+Sütun açıklamaları: Kök ifade: Google arama kutusuna yazılan ifade; öneriler bu ifadenin devamı olarak gelmektedir. | Autocomplete önerileri · 2026 aylık ort. hacim: Google'ın Türkiye, Türkçe, masaüstü Chrome için döndürdüğü ilk 10 tamamlama önerisi; sırası Google'ın sırasıdır. Rozet: Ocak - Ağustos 2026 aylık ortalama arama hacmi (Google Ads); rozeti olmayan kelime için hacim dönmemiştir.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -2934,131 +2934,131 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Autocomplete önerileri</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="43" customHeight="1">
+          <t>Autocomplete önerileri · 2026 aylık ort. hacim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>vitra</t>
+          <t>vitra 33,1K</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>vitra klozet vitra kayseri vitra gömme rezervuar vitra klozet fiyatları vitra seramik vitra banyo dolabı vitra klozet kapağı vitra lavabo vitra tuvalet taşı vitra duş seti</t>
+          <t>vitra klozet 11,0K vitra kayseri 96 vitra gömme rezervuar 13,4K vitra klozet fiyatları 2,3K vitra seramik 4,5K vitra banyo dolabı 4,5K vitra klozet kapağı 4,1K vitra lavabo 2,9K vitra tuvalet taşı 728 vitra duş seti 2,1K</t>
         </is>
       </c>
     </row>
     <row r="6" ht="69" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>vitra klozet</t>
+          <t>vitra klozet 11,0K</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>vitra klozet fiyatları vitra klozet kapağı vitra klozet modelleri vitra klozet takımı vitra klozet fiyatları koçtaş vitra klozet kapağı menteşesi vitra klozet iç takımı vitra klozet su kaçırıyor vitra klozet takımı fiyatları vitra klozet şamandırası</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="82" customHeight="1">
+          <t>vitra klozet fiyatları 2,3K vitra klozet kapağı 4,1K vitra klozet modelleri 760 vitra klozet takımı 549 vitra klozet fiyatları koçtaş 381 vitra klozet kapağı menteşesi 820 vitra klozet iç takımı 962 vitra klozet su kaçırıyor 40 vitra klozet takımı fiyatları 269 vitra klozet şamandırası 149</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>vitra gömme rezervuar</t>
+          <t>vitra gömme rezervuar 13,4K</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>vitra gömme rezervuar iç takımı vitra gömme rezervuar seti vitra gömme rezervuar fiyatları vitra gömme rezervuar şamandıra vitra gömme rezervuar contası vitra gömme rezervuar ölçüleri vitra gömme rezervuar şamandıra suyu kesmiyor vitra gömme rezervuar montajı vitra gömme rezervuar boşaltma grubu vitra gömme rezervuar kapağı</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="69" customHeight="1">
+          <t>vitra gömme rezervuar iç takımı 3,4K vitra gömme rezervuar seti 1,7K vitra gömme rezervuar fiyatları 820 vitra gömme rezervuar şamandıra 622 vitra gömme rezervuar contası 1,0K vitra gömme rezervuar ölçüleri 388 vitra gömme rezervuar şamandıra suyu kesmiyor 386 vitra gömme rezervuar montajı 395 vitra gömme rezervuar boşaltma grubu 370 vitra gömme rezervuar kapağı 549</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="82" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>vitra banyo dolabı</t>
+          <t>vitra banyo dolabı 4,5K</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>vitra banyo dolabı seti vitra banyo dolabı modelleri vitra banyo dolabı fiyatları vitra banyo dolabı duvara montajı vitra banyo dolabı 100 cm vitra banyo dolabı 80 cm vitra banyo dolabı takımı vitra banyo dolabı koçtaş vitra banyo dolabı 60 cm vitra banyo dolabı montajı</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1">
+          <t>vitra banyo dolabı seti 334 vitra banyo dolabı modelleri 565 vitra banyo dolabı fiyatları 119 vitra banyo dolabı duvara montajı vitra banyo dolabı 100 cm 40 vitra banyo dolabı 80 cm 66 vitra banyo dolabı takımı 31 vitra banyo dolabı koçtaş 25 vitra banyo dolabı 60 cm 20 vitra banyo dolabı montajı 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="69" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>vitra batarya</t>
+          <t>vitra batarya 925</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>vitra batarya fiyatları vitra batarya banyo vitra batarya mutfak vitra batarya seti vitra batarya modelleri vitra batarya kartuşu vitra batarya yedek parça vitra batarya lavabo vitra batarya garanti süresi vitra batarya süzgeci</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="69" customHeight="1">
+          <t>vitra batarya fiyatları 98 vitra batarya banyo 140 vitra batarya mutfak 101 vitra batarya seti 32 vitra batarya modelleri 28 vitra batarya kartuşu 22 vitra batarya yedek parça vitra batarya lavabo 24 vitra batarya garanti süresi vitra batarya süzgeci</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="82" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>vitra duşakabin</t>
+          <t>vitra duşakabin 1,1K</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>vitra duşakabin fiyatları vitra duşakabin koçtaş vitra duşakabin modelleri ve fiyatları vitra duşakabin teknesi vitra duşakabin tekerleği vitra duşakabin gider kapağı vitra duşakabin yedek parça vitra duşakabin modelleri vitra duşakabin dwg vitra duşakabin 100x100</t>
+          <t>vitra duşakabin fiyatları 232 vitra duşakabin koçtaş 48 vitra duşakabin modelleri ve fiyatları 96 vitra duşakabin teknesi 19 vitra duşakabin tekerleği 22 vitra duşakabin gider kapağı 19 vitra duşakabin yedek parça 15 vitra duşakabin modelleri 378 vitra duşakabin dwg vitra duşakabin 100x100 35</t>
         </is>
       </c>
     </row>
     <row r="11" ht="82" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>vitra akıllı klozet</t>
+          <t>vitra akıllı klozet 381</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>vitra akıllı klozet fiyatları vitra akıllı klozet kapağı vitra akıllı klozet kapağı fiyatları vitra akıllı klozet kullanım kılavuzu vitra akıllı klozet video vitra akıllı klozet taharet musluğu vitra akıllı klozet özellikleri vitra akıllı klozet montajı vitra akıllı klozet arızaları vitra akıllı klozet elektrik bağlantısı</t>
+          <t>vitra akıllı klozet fiyatları 118 vitra akıllı klozet kapağı 101 vitra akıllı klozet kapağı fiyatları 11 vitra akıllı klozet kullanım kılavuzu 10 vitra akıllı klozet video 5 vitra akıllı klozet taharet musluğu vitra akıllı klozet özellikleri 8 vitra akıllı klozet montajı 10 vitra akıllı klozet arızaları vitra akıllı klozet elektrik bağlantısı</t>
         </is>
       </c>
     </row>
     <row r="12" ht="82" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>vitra klozet kapağı</t>
+          <t>vitra klozet kapağı 4,1K</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>vitra klozet kapağı menteşesi vitra klozet kapağı montajı vitra klozet kapağı nasıl sökülür vitra klozet kapağı fiyatları vitra klozet kapağı nasıl takılır vitra klozet kapağı parçaları vitra klozet kapağı yavaş kapanan vitra klozet kapağı damper seti vitra klozet kapağı menteşe seti vitra klozet kapağı damperi</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="56" customHeight="1">
+          <t>vitra klozet kapağı menteşesi 820 vitra klozet kapağı montajı 209 vitra klozet kapağı nasıl sökülür 236 vitra klozet kapağı fiyatları 260 vitra klozet kapağı nasıl takılır 104 vitra klozet kapağı parçaları 144 vitra klozet kapağı yavaş kapanan 128 vitra klozet kapağı damper seti vitra klozet kapağı menteşe seti 62 vitra klozet kapağı damperi 159</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="69" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>vitra servis</t>
+          <t>vitra servis 2,6K</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>vitra servis kayseri vitra servis yedek parça vitra servis ücreti vitra servis numarası vitra servis istanbul vitra servis müşteri hizmetleri vitra servis iletişim vitra servis ankara vitra servis en yakın vitra servis randevu</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="69" customHeight="1">
+          <t>vitra servis kayseri 41 vitra servis yedek parça 504 vitra servis ücreti 34 vitra servis numarası 39 vitra servis istanbul 165 vitra servis müşteri hizmetleri vitra servis iletişim 14 vitra servis ankara 114 vitra servis en yakın vitra servis randevu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="82" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>vitra yedek parça</t>
+          <t>vitra yedek parça 392</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>vitra yedek parça fiyat listesi vitra yedek parça online satış vitra yedek parça listesi vitra yedek parça servis vitra yedek parça satış noktaları vitra yedek parça kataloğu vitra yedek parça istanbul vitra yedek parça izmir vitra yedek parça bursa vitra yedek parça ankara</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="56" customHeight="1">
+          <t>vitra yedek parça fiyat listesi 58 vitra yedek parça online satış 92 vitra yedek parça listesi 60 vitra yedek parça servis 21 vitra yedek parça satış noktaları 116 vitra yedek parça kataloğu 10 vitra yedek parça istanbul 50 vitra yedek parça izmir 15 vitra yedek parça bursa vitra yedek parça ankara</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="69" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>vitra bayi</t>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>vitra bayileri vitra bayi kayseri vitra bayii vitra bayileri istanbul vitra bayilik vitra bayilik şartları vitra bayi izmir vitra bayileri istanbul avrupa yakası vitra bayileri ankara vitra bayileri istanbul anadolu yakası</t>
+          <t>vitra bayileri 1,0K vitra bayi kayseri vitra bayii 1,0K vitra bayileri istanbul 82 vitra bayilik 1,0K vitra bayilik şartları 26 vitra bayi izmir vitra bayileri istanbul avrupa yakası 69 vitra bayileri ankara 44 vitra bayileri istanbul anadolu yakası 94</t>
         </is>
       </c>
     </row>
@@ -3085,24 +3085,24 @@
     <row r="17" ht="43" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>vitra indirim</t>
+          <t>vitra indirim 14</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>vitra indirim kodu vitra indirimli ürünler vitra klozet indirim vitra 45 indirim vitra indirimleri vitra online indirim kodu</t>
+          <t>vitra indirim kodu vitra indirimli ürünler 10 vitra klozet indirim 9 vitra 45 indirim vitra indirimleri vitra online indirim kodu</t>
         </is>
       </c>
     </row>
     <row r="18" ht="69" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>vitra outlet</t>
+          <t>vitra outlet 56</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>vitra outlet tuzla vitra outlet mağazaları vitra outlet banyo dolabı vitra outlet mağazaları istanbul yakınında vitra outlet online vitra outlet istanbul vitra outlet bozüyük vitra outlet mağazaları kadıköy yakınında vitra outlet zaandam vitra outlet weil am rhein</t>
+          <t>vitra outlet tuzla 10 vitra outlet mağazaları 118 vitra outlet banyo dolabı vitra outlet mağazaları istanbul yakınında 26 vitra outlet online 8 vitra outlet istanbul 11 vitra outlet bozüyük 10 vitra outlet mağazaları kadıköy yakınında vitra outlet zaandam 0 vitra outlet weil am rhein 0</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3123,7 @@
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -3134,13 +3134,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · Kategori ve rakip marka aramaları
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
 Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 10 , 11
-Sütun açıklamaları: Kök ifade: Kategori veya rakip marka ile başlayan ifade. | Autocomplete önerileri: Google'ın döndürdüğü ilk 10 tamamlama önerisi.</t>
+Sütun açıklamaları: Kök ifade: Kategori veya rakip marka ile başlayan ifade. | Autocomplete önerileri · 2026 aylık ort. hacim: Google'ın döndürdüğü ilk 10 tamamlama önerisi; rozet Ocak - Ağustos 2026 aylık ortalama arama hacmidir (Google Ads).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -3153,103 +3153,103 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Autocomplete önerileri</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="56" customHeight="1">
+          <t>Autocomplete önerileri · 2026 aylık ort. hacim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="69" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>klozet</t>
+          <t>klozet 49,5K</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>klozet fiyatları klozet kapağı klozet şamandırası klozet takımı klozet taharet musluğu klozet modelleri klozet kapağı fiyatları klozet iç takım klozet fiyatları kayseri klozet kapağı menteşesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
+          <t>klozet fiyatları 65,6K klozet kapağı 35,9K klozet şamandırası 7,3K klozet takımı 12,8K klozet taharet musluğu 4,5K klozet modelleri 7,3K klozet kapağı fiyatları 6,5K klozet iç takım 9,4K klozet fiyatları kayseri 65 klozet kapağı menteşesi 4,5K</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="69" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı</t>
+          <t>banyo dolabı 95,4K</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı fiyatları banyo dolabı lavabolu banyo dolabı seti banyo dolabı kayseri banyo dolabı ölçüleri banyo dolabı plastik banyo dolabı takımı banyo dolabı aynalı banyo dolabı modelleri küçük banyo dolabı modelleri fiyatları</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="69" customHeight="1">
+          <t>banyo dolabı fiyatları 6,8K banyo dolabı lavabolu 3,6K banyo dolabı seti 3,3K banyo dolabı kayseri 36 banyo dolabı ölçüleri 1,2K banyo dolabı plastik 940 banyo dolabı takımı 2,3K banyo dolabı aynalı 875 banyo dolabı modelleri küçük 270 banyo dolabı modelleri fiyatları 895</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="82" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>gömme rezervuar</t>
+          <t>gömme rezervuar 16,0K</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>gömme rezervuar iç takımı gömme rezervuar ölçüleri gömme rezervuar şamandıra gömme rezervuar fiyatları gömme rezervuar montajı gömme rezervuar su kaçırıyor gömme rezervuar şamandıra ayarı gömme rezervuar taharet musluğu gömme rezervuar tamiri gömme rezervuar şamandıra suyu kesmiyor</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
+          <t>gömme rezervuar iç takımı 4,7K gömme rezervuar ölçüleri 1,6K gömme rezervuar şamandıra 820 gömme rezervuar fiyatları 1,4K gömme rezervuar montajı 1,1K gömme rezervuar su kaçırıyor 812 gömme rezervuar şamandıra ayarı 156 gömme rezervuar taharet musluğu 760 gömme rezervuar tamiri 1,2K gömme rezervuar şamandıra suyu kesmiyor 508</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="69" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>duşakabin</t>
+          <t>duşakabin 92,9K</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>duşakabin fiyatları duşakabin modelleri duşakabin kayseri duşakabin tekerleği duşakabin cam filmi duşakabin camı duşakabin temizliği duşakabin fiyatları kayseri duşakabin silikonu duşakabin ölçüleri</t>
+          <t>duşakabin fiyatları 56,4K duşakabin modelleri 43,9K duşakabin kayseri 184 duşakabin tekerleği 9,7K duşakabin cam filmi 1,4K duşakabin camı 6,5K duşakabin temizliği 5,0K duşakabin fiyatları kayseri 54 duşakabin silikonu 2,2K duşakabin ölçüleri 1,9K</t>
         </is>
       </c>
     </row>
     <row r="9" ht="69" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>akıllı klozet</t>
+          <t>akıllı klozet 2,5K</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>akıllı klozet kapağı akıllı klozet fiyatları akıllı klozet kapağı fiyatları akıllı klozet türkiye akıllı klozet nedir akıllı klozet vitra akıllı klozet özellikleri akıllı klozet kapağı vitra akıllı klozet modelleri akıllı klozet kapağı tamiri</t>
+          <t>akıllı klozet kapağı 941 akıllı klozet fiyatları 554 akıllı klozet kapağı fiyatları 146 akıllı klozet türkiye 48 akıllı klozet nedir 48 akıllı klozet vitra 56 akıllı klozet özellikleri 31 akıllı klozet kapağı vitra 12 akıllı klozet modelleri akıllı klozet kapağı tamiri</t>
         </is>
       </c>
     </row>
     <row r="10" ht="69" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>klozet montaj</t>
+          <t>klozet montaj 1,2K</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>klozet montajı klozet montaj aparatı klozet montajı nasıl yapılır klozet montaj vidası klozet montaj ücreti klozet montaj ölçüleri klozet montaj aparatı ve körüklü kada klozet montaj aparatı koçtaş klozet montaj seti klozet montajı nasıl yapılır video</t>
+          <t>klozet montajı 1,2K klozet montaj aparatı 902 klozet montajı nasıl yapılır 535 klozet montaj vidası 639 klozet montaj ücreti 86 klozet montaj ölçüleri 149 klozet montaj aparatı ve körüklü kada 90 klozet montaj aparatı koçtaş 74 klozet montaj seti 101 klozet montajı nasıl yapılır video 32</t>
         </is>
       </c>
     </row>
     <row r="11" ht="69" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>klozet tamir</t>
+          <t>klozet tamir 1,3K</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>klozet tamiri klozet tamir takımı klozet tamiri nasıl yapılır klozet tamir takımı fiyatları klozet tamiri fiyat klozet tamirini kim yapar klozet tamir seti klozet tamir takımı değişimi klozet tamir takımı nasıl değişir klozet tamiri kiracıya mı ait</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="69" customHeight="1">
+          <t>klozet tamiri 1,3K klozet tamir takımı 426 klozet tamiri nasıl yapılır 185 klozet tamir takımı fiyatları 54 klozet tamiri fiyat 31 klozet tamirini kim yapar 49 klozet tamir seti 24 klozet tamir takımı değişimi 18 klozet tamir takımı nasıl değişir 8 klozet tamiri kiracıya mı ait 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="82" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı montaj</t>
+          <t>banyo dolabı montaj 290</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı montajı banyo dolabı montaj ölçüleri banyo dolabı montaj aparatı banyo dolabı montaj ücreti banyo dolabı montaj dahil banyo dolabı montaj yüksekliği banyo dolabı montajı nasıl yapılır banyo dolabı montaj vidası banyo dolabı montaj ustası banyo dolabı montaj videosu</t>
+          <t>banyo dolabı montajı 290 banyo dolabı montaj ölçüleri 170 banyo dolabı montaj aparatı 56 banyo dolabı montaj ücreti 4 banyo dolabı montaj dahil 16 banyo dolabı montaj yüksekliği banyo dolabı montajı nasıl yapılır 75 banyo dolabı montaj vidası banyo dolabı montaj ustası banyo dolabı montaj videosu</t>
         </is>
       </c>
     </row>
@@ -3261,55 +3261,55 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>klozet taktırma klozet taktırma fiyatı klozet takımı tekzen klozet taktırma ücreti</t>
+          <t>klozet taktırma klozet taktırma fiyatı klozet takımı tekzen 8 klozet taktırma ücreti</t>
         </is>
       </c>
     </row>
     <row r="14" ht="69" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>banyo yenileme</t>
+          <t>banyo yenileme 2,1K</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>banyo yenileme maliyeti banyo yenileme maliyeti 2026 banyo yenileme modelleri banyo yenileme fikirleri banyo yenileme videoları banyo yenileme malzemeleri banyo yenileme pinterest banyo yenileme örnekleri banyo yenileme kendin yap banyo yenileme izmir</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="56" customHeight="1">
+          <t>banyo yenileme maliyeti 434 banyo yenileme maliyeti 2026 262 banyo yenileme modelleri 264 banyo yenileme fikirleri 381 banyo yenileme videoları 11 banyo yenileme malzemeleri 14 banyo yenileme pinterest banyo yenileme örnekleri banyo yenileme kendin yap 16 banyo yenileme izmir 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="69" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>artema</t>
+          <t>artema 6,2K</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>artema mutfak bataryası artema banyo bataryası artema lavabo bataryası artema duş seti artema taharet musluğu artema musluk artema servis kayseri artema kayseri artema batarya artema duş başlığı</t>
+          <t>artema mutfak bataryası 7,2K artema banyo bataryası 5,3K artema lavabo bataryası 4,1K artema duş seti 3,0K artema taharet musluğu 1,7K artema musluk 1,6K artema servis kayseri 15 artema kayseri artema batarya 1,8K artema duş başlığı 1,2K</t>
         </is>
       </c>
     </row>
     <row r="16" ht="82" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>creavit klozet</t>
+          <t>creavit klozet 3,8K</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>creavit klozet kapağı creavit klozet kapağı menteşesi creavit klozet fiyatları creavit klozet kapağı nasıl sökülür creavit klozet kapağı parçaları creavit klozet şamandırası nasıl takılır creavit klozet kapağı montajı creavit klozet iç takımı creavit klozet montajı creavit klozet kapağı amortisörü</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="69" customHeight="1">
+          <t>creavit klozet kapağı 2,5K creavit klozet kapağı menteşesi 535 creavit klozet fiyatları 330 creavit klozet kapağı nasıl sökülür 209 creavit klozet kapağı parçaları 339 creavit klozet şamandırası nasıl takılır 132 creavit klozet kapağı montajı 75 creavit klozet iç takımı 165 creavit klozet montajı 80 creavit klozet kapağı amortisörü 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="82" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>kale klozet</t>
+          <t>kale klozet 2,0K</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>kale klozet kapağı kale klozet fiyatları kale klozet kapağı nasıl sökülür kale klozet iç takımı kale klozet şamandıra tamiri kale klozet modelleri kale klozet yetkili servis kale klozet kapağı fiyatları kale klozet kapağı montajı kale klozet kapağı damperi</t>
+          <t>kale klozet kapağı 2,1K kale klozet fiyatları 870 kale klozet kapağı nasıl sökülür 255 kale klozet iç takımı 308 kale klozet şamandıra tamiri 149 kale klozet modelleri 166 kale klozet yetkili servis 281 kale klozet kapağı fiyatları 134 kale klozet kapağı montajı 68 kale klozet kapağı damperi 131</t>
         </is>
       </c>
     </row>
@@ -7133,8 +7133,8 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
@@ -7152,7 +7152,7 @@
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Ana kategori düzeyinde değişim
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
 Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 6 , 7
-Sütun açıklamaları: Kategori: VitrA kategori ağacındaki ana kategori; 2.420 kelime 8 ana kategoriye dağıtılmıştır. | Kelime: Kategoriye atanan kelime sayısı. | Oca-Ağu 2025: Ocak - Ağustos 2025 aylık ortalama arama hacmi toplamı, Google Keyword Planner, Türkiye. | Oca-Ağu 2026: Ocak - Ağustos 2026 aylık ortalama arama hacmi toplamı; aynı takvim aylarını kapsar. | YoY: İki pencere arasındaki yüzde değişim; mevsimsellikten arındırılmıştır. | Pay: Kategorinin 2026 penceresindeki toplam hacim içindeki payı.</t>
+Sütun açıklamaları: Kategori: VitrA kategori ağacındaki ana kategori; 2.420 kelime 8 ana kategoriye dağıtılmıştır. | Kelime: Kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi (kategorideki kelimelerin toplamı, aya bölünmüş), Google Keyword Planner, Türkiye. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi; aynı takvim aylarını kapsar. | YoY: İki pencere arasındaki yüzde değişim; mevsimsellikten arındırılmıştır. | Pay: Kategorinin 2026 penceresindeki toplam hacim içindeki payı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -7174,12 +7174,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2025</t>
+          <t>2025 aylık ort.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2026</t>
+          <t>2026 aylık ort.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -10359,15 +10359,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="51" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -10377,13 +10379,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="188" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Katalog ve Talep Eşleşmesi · Pazaryerindeki görünüm: Trendyol
 Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. İkinci bölümde aynı temaların Trendyol'daki görünümü (fiyat bandı, öne çıkan satıcılar, VitrA varlığı) incelenmiştir.
 Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 8 , 9 , 18
-Sütun açıklamaları: Trendyol araması: Trendyol arama kutusuna yazılan ifade. | İncelenen ürün: İncelenen ilk sonuç sayısı. | Medyan fiyat (TL): İncelenen ürünlerin medyan satış fiyatı; havlupanda yalnız ısıtıcılı havlupanlar, iç takımda jenerik ürünler. | VitrA / Artema ürün: İlk sonuçlarda VitrA veya Artema markalı ürün sayısı. | En çok değerlendirme alan: Değerlendirme sayısı en yüksek ürünün markası, fiyatı ve değerlendirme sayısı; satış hacmi göstergesi olarak kullanılmıştır. | Gözlem: Sonuç sayfasının genel görünümü.</t>
+Sütun açıklamaları: Trendyol araması: Trendyol arama kutusuna yazılan ifade. | İncelenen ürün: İncelenen ilk sonuç sayısı. | Medyan fiyat (TL): İncelenen ürünlerin medyan satış fiyatı; havlupanda yalnız ısıtıcılı havlupanlar, iç takımda jenerik ürünler. | VitrA / Artema ürün: İlk sonuçlarda VitrA veya Artema markalı ürün sayısı. | En çok değerlendirilen marka: İlk sonuçlarda değerlendirme sayısı en yüksek ürünün markası; bağlantı Trendyol'da marka + arama ifadesiyle yapılan aramaya gider. | Fiyat (TL): Bu ürünün satış fiyatı, 29.09.2026. | Değerlendirme sayısı: Bu ürünün değerlendirme sayısı; satış hacmi göstergesi olarak kullanılmıştır. | Gözlem: Sonuç sayfasının genel görünümü.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -10391,6 +10393,8 @@
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
       <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -10415,10 +10419,20 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>En çok değerlendirme alan</t>
+          <t>En çok değerlendirilen marka</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Fiyat (TL)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Değerlendirme sayısı</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Gözlem</t>
         </is>
@@ -10441,10 +10455,16 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Irmak · 1.390 TL · 3.141</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+          <t>Irmak</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1390</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>3141</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>İlk 45 sonucun tamamına yakını düz paket mobilya markaları (MOBİLİQUE, Bofigo, KZY, Montenero, FURNICI); lavabolu set tek VitrA ürünü 14.462 TL</t>
         </is>
@@ -10469,10 +10489,16 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Asil Krom (çelik) · 2.300 TL · 429</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+          <t>Asil Krom (çelik)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>429</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>RealStone listelemelerin yaklaşık yarısı; değerlendirme sayıları düşük, kategori pazaryerinde henüz olgunlaşmamış</t>
         </is>
@@ -10497,10 +10523,16 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Saban · 599 TL · 2.887</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+          <t>Saban</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>599</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>2887</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Bebek ürünü markaları ve jenerik satıcılar; klozet markası yok</t>
         </is>
@@ -10523,10 +10555,16 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>hakersan · 342 TL · 681</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+          <t>hakersan</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>342</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>681</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>VitrA listelemelerin yaklaşık %22'si ve ilk sırada; jenerik iç takımlar 280-480 TL bandında ve daha fazla değerlendirme alıyor</t>
         </is>
@@ -10551,10 +10589,16 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ESMOPA MOBİLYA · 4.799 TL · 2.495</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+          <t>ESMOPA MOBİLYA</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>4799</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>2495</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>40 sonucun 14'ü MOBİLİQUE, 7'si Bofigo; PVC ve suya dayanıklı gövde vurgusu</t>
         </is>
@@ -10579,10 +10623,16 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Moonlife Mobilya · 4.473 TL · 1.472</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+          <t>Moonlife Mobilya</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>4473</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>1472</v>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>VitrA sitede 29 çamaşır makinesi dolabı listeliyor, Trendyol ilk 40 sonuçta görünmüyor</t>
         </is>
@@ -10605,10 +10655,16 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>SUEL HOUSE · 490 TL · 2.277</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+          <t>SUEL HOUSE</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>490</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>2277</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Dekorasyon ve ayna atölyesi markaları; VitrA tek ürün, pazar medyanının yaklaşık 8 katı fiyatta</t>
         </is>
@@ -10633,10 +10689,16 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Arya · 2.420 TL · 3.359</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>3359</v>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Arıtma cihazı markaları ve jenerik satıcılar; armatür markası (VitrA, Artema, Eca, Grohe) ilk 40'ta yok</t>
         </is>
@@ -10659,10 +10721,16 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>KUMTEL · 2.129 TL · 1.289</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
+          <t>KUMTEL</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>2129</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>1289</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Sonuçların yaklaşık yarısı havlupan değil, düşük fiyatlı havluluk ve askı; ısıtıcılı havlupanda Eca, Toprak, DG Therm, Termofer</t>
         </is>
@@ -10685,10 +10753,16 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Seval Su Armatürleri · 120 TL · 30</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+          <t>Seval Su Armatürleri</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Değerlendirme sayıları düşük (en yüksek 30); jenerik kartuşlar 120-350 TL, Artema ve Eca orijinal kartuşları 465-735 TL</t>
         </is>
@@ -10713,10 +10787,16 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Genel Markalar · 819 TL · 180</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+          <t>Genel Markalar</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>819</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Sonuçların çoğu medikal tedarikçiler (MEDİKALCİM, Medikaltec, MEDİLABS); değerlendirme çok az, kategori pazaryerinde oturmamış</t>
         </is>
@@ -10739,10 +10819,16 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Genel Markalar · 1.125 TL · 252</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
+          <t>Genel Markalar</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>1125</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>252</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Paslanmaz çelik üreticileri ve jenerik satıcılar; banyo markası olarak yalnız VitrA tek ürünle var</t>
         </is>
@@ -10767,10 +10853,16 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>VitrA Arkitekt asma klozet + gömme rezervuar seti · 11.999 TL · 86</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
+          <t>VitrA Arkitekt asma klozet + gömme rezervuar seti</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>11999</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>86</v>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Aramada klozet + rezervuar + kapak setleri öne çıkıyor; klozet, lavabo ve dolabı birlikte sunan komple banyo seti ilk 40 sonuçta yok. İDEVİT seti montaj parçalarını (taharet musluğu, hortum, iç takım) pakete dahil ediyor</t>
         </is>
@@ -10778,7 +10870,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11921,8 +12013,8 @@
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -11939,7 +12031,7 @@
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Büyüyen alt kategoriler
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
 Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 6 , 7
-Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | Oca-Ağu 2025: Ocak - Ağustos 2025 aylık ortalama hacim toplamı. | Oca-Ağu 2026: Ocak - Ağustos 2026 aylık ortalama hacim toplamı. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
+Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -11966,12 +12058,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2025</t>
+          <t>2025 aylık ort.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2026</t>
+          <t>2026 aylık ort.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -16055,8 +16147,8 @@
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -16073,7 +16165,7 @@
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Daralan alt kategoriler
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
 Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 6 , 7
-Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | Oca-Ağu 2025: Ocak - Ağustos 2025 aylık ortalama hacim toplamı. | Oca-Ağu 2026: Ocak - Ağustos 2026 aylık ortalama hacim toplamı. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
+Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -16100,12 +16192,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2025</t>
+          <t>2025 aylık ort.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Oca-Ağu 2026</t>
+          <t>2026 aylık ort.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -16856,14 +16948,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -16873,19 +16970,24 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="174" customHeight="1">
+    <row r="2" ht="216" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Çok satanlarda kim önde?
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
 Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 31 , 32 , 33
-Sütun açıklamaları: Kategori: Çok satan sıralamasının okunduğu kategori veya arama. | Trendyol: çok satanlarda öne çıkan: "En Çok Satan" sıralamasının ilk 36 ürününde değerlendirme payı en yüksek markalar. | VitrA Trendyol: İlk 36 içindeki VitrA ürün sayısı ve değerlendirme payı. | Hepsiburada: çok satanlarda öne çıkan: "Çok satanlar" sıralamasının ilk 36 ürününde öne çıkan markalar. | VitrA Hepsiburada: İlk 36 içindeki VitrA (Artema) ürün sayısı ve değerlendirme toplamı.</t>
+Sütun açıklamaları: Kategori: Çok satan sıralamasının okunduğu kategori veya arama. | Trendyol lider marka: "En Çok Satan" sıralamasının ilk 36 ürününde değerlendirme payı en yüksek marka. | Lider payı (TY): Lider markanın ilk 36'daki değerlendirme payı. | VitrA ürün (TY ilk 36): İlk 36 içindeki VitrA (Artema) ürün sayısı; 0 = listede yok. | VitrA değ. payı (TY): VitrA ürünlerinin ilk 36'daki değerlendirme payı. | Hepsiburada lider marka: "Çok satanlar" sıralamasının ilk 36 ürününde öne çıkan marka. | Lider değ. (HB): Lider markanın ilk 36'daki toplam değerlendirme sayısı; "-" okunmadı. | VitrA ürün (HB ilk 36): İlk 36 içindeki VitrA (Artema) ürün sayısı; 0 = listede yok. | VitrA değ. (HB): VitrA ürünlerinin ilk 36'daki toplam değerlendirme sayısı. | Not: İkinci ve üçüncü markalar, okuma yöntemi.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -16895,22 +16997,47 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Trendyol: çok satanlarda öne çıkan</t>
+          <t>Trendyol lider marka</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>VitrA Trendyol</t>
+          <t>Lider payı (TY)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Hepsiburada: çok satanlarda öne çıkan</t>
+          <t>VitrA ürün (TY ilk 36)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>VitrA Hepsiburada</t>
+          <t>VitrA değ. payı (TY)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Hepsiburada lider marka</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Lider değ. (HB)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>VitrA ürün (HB ilk 36)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>VitrA değ. (HB)</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Not</t>
         </is>
       </c>
     </row>
@@ -16922,22 +17049,35 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Turavit %38, Turkuaz %11, Seramiksan %9</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>3 ürün · %3</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Turkuaz 536, Creavit 224 değ.</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>9 ürün · 147 değ.</t>
+          <t>Turavit</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Turkuaz</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>536</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>147</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>2. Turkuaz %11, 3. Seramiksan %9</t>
         </is>
       </c>
     </row>
@@ -16949,22 +17089,35 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Visam %21, ELİTRA %20, Saban %16</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>1 ürün · %2,6</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>NKP 5.354, Visam 1.495 değ.</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>8 ürün · 1.038 değ.</t>
+          <t>Visam</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>NKP</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>5354</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>1038</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>ELİTRA %20, Saban %16; HB'de Visam 1.495</t>
         </is>
       </c>
     </row>
@@ -16976,22 +17129,37 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Turkuaz %56 (13 ürün)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>1 ürün · %0,5</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Turkuaz 14 ürün, 1.221 değ.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>ilk 36'da yok</t>
+          <t>Turkuaz</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Turkuaz</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1221</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Turkuaz 13 ürün; HB'de 14 ürün</t>
         </is>
       </c>
     </row>
@@ -17003,22 +17171,35 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Visam %27</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>9 ürün · %16</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Visam 8 ürün, 1.962 değ.</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>8 ürün · 2.248 değ.</t>
+          <t>Visam</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Visam</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>1962</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>2248</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>HB'de Visam 8 ürün</t>
         </is>
       </c>
     </row>
@@ -17030,22 +17211,41 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>KAREN BANYO %47, ÖZCEDEN %26</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>ilk 24'te yok</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Aeka, Mowo Home (arama)</t>
-        </is>
+          <t>KAREN BANYO</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ilk 36'da yok</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Aeka</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>ÖZCEDEN %26; HB listesi arama sonucudur (Aeka, Mowo Home)</t>
         </is>
       </c>
     </row>
@@ -17067,12 +17267,33 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Dmz Home Concept 8 ürün</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Mia 3 ürün · 402 değ.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Dmz Home Concept</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>402</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>HB'de Dmz Home Concept 8 ürün; VitrA Mia</t>
         </is>
       </c>
     </row>
@@ -17084,22 +17305,43 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>sepet ve organizer ağırlıklı (Bofigo)</t>
+          <t>Bofigo</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>yok</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Remaks, Bofigo</t>
-        </is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>yok</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Remaks</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Liste sepet ve düzenleyici ağırlıklı; HB'de Bofigo da var</t>
         </is>
       </c>
     </row>
@@ -17111,26 +17353,43 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>SUEL HOUSE %48</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>yok</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
+          <t>SUEL HOUSE</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>ER-KA DİZAYN</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>1 ürün · 5 değ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Lavabo bataryası</t>
@@ -17138,26 +17397,43 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Genel Markalar %30, Sardıcı %16</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Artema ilk 10'da yok</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Creavit 6, Sardıcı 6, ECA 4 ürün</t>
-        </is>
+          <t>Genel Markalar</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Artema 4 ürün · 200 değ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Creavit</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Sardıcı %16; HB'de Creavit 6, Sardıcı 6, ECA 4 ürün; Artema Trendyol ilk 10'da yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Eviye bataryası</t>
@@ -17165,22 +17441,39 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>KUSTAR %48</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Artema ilk 10'da yok</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Artema 6, Sardıcı 4 ürün</t>
-        </is>
+          <t>KUSTAR</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Artema 6 ürün · 1.269 değ.</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Artema</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>1269</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>HB'de Artema 6, Sardıcı 4 ürün; Artema Trendyol ilk 10'da yok</t>
         </is>
       </c>
     </row>
@@ -17192,22 +17485,41 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Durul %93</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>yok</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Durul 27/36 ürün</t>
-        </is>
+          <t>Durul</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>yok</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Durul</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>HB'de Durul 27/36 ürün</t>
         </is>
       </c>
     </row>
@@ -17219,28 +17531,47 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>NOY %21, Kaşbaşı Home %16</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>yok</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Berev 13 ürün</t>
-        </is>
+          <t>NOY</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>yok</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Berev</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Kaşbaşı Home %16; HB'de Berev 13 ürün</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19628,13 +19959,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="188" customHeight="1">
+    <row r="2" ht="202" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · En çok değerlendirilen ürünler
 Kapsam: Trendyol (42 kategori), Hepsiburada (40), Akakçe (42 sayfa ve 8 VitrA marka sayfası) ve Cimri'de (30) çok satan ya da popülerlik sıralamasının ilk iki sayfası ile Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağazasının kategori sayfaları okunmuştur; toplam 9.000'den fazla pazaryeri ve 2.500'den fazla mağaza ürün satırı. Kategoriler VitrA'nın hedef gamı (SSG, rezervuar, mobilya, armatür, yıkanma) ve hedef dışı bitişik kesitler olarak ayrılmıştır. Değerlendirme sayısı satış hacminin yaklaşık göstergesidir; fiyatlar 30.09.2026 tarihli liste fiyatlarıdır. Kale fiyat göstermediği, IKEA TR ürün listesi vermediği için kapsam dışıdır.
 Kaynak: Trendyol, Hepsiburada, Akakçe ve Cimri kategori listeleri (ilk 2 sayfa) · Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağaza kategori sayfaları · Chrome · 30.09.2026 34
-Sütun açıklamaları: Kategori: Kategori. | Kanal: Pazaryeri. | En çok değerlendirilen ürün: Çok satan ilk 72 ürün içinde değerlendirme sayısı en yüksek ürün. | Marka: Ürünün markası. | Fiyat (TL): Liste fiyatı, 30.09.2026. | Değerlendirme sayısı: Değerlendirme sayısı. | Puan: Ortalama puan (5 üzerinden).</t>
+Sütun açıklamaları: Kategori: Kategori. | Kanal: Pazaryeri. | En çok değerlendirilen ürün: Çok satan ilk 72 ürün içinde değerlendirme sayısı en yüksek ürün. | Marka: Ürünün markası; bağlantı pazaryerinde marka + ürün adıyla aramaya gider. | Fiyat (TL): Liste fiyatı, 30.09.2026. | Değerlendirme sayısı: Değerlendirme sayısı. | Puan: Ortalama puan (5 üzerinden).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -41275,7 +41606,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>https://www.vitra.com.tr/c-canak-lavabolar · https://www.vitra.com.tr/c-dus-uniteleri · https://www.vitra.com.tr/c-kampanyali-urunler · https://www.trendyol.com/sr?q=s%C3%BCrg%C3%BCl%C3%BC%20el%20du%C5%9Fu%20tak%C4%B1m%C4%B1&amp;sst=BEST_SELLER · https://www.hepsiburada.com/ara?q=ankastre%20stop%20valf&amp;siralama=coksatan · https://www.akakce.com/arama/?q=%C3%A7anak%20lavabo · https://www.cimri.com/arama?q=ayakl%C4%B1%20klozet · https://www.koctas.com.tr/search?q=%C3%A7anak%20lavabo&amp;sort=bestseller-desc · https://www.banyomarka.com/arama?q=s%C3%BCrg%C3%BCl%C3%BC%20el%20du%C5%9Fu%20tak%C4%B1m%C4%B1</t>
+          <t>https://www.vitra.com.tr/c-canak-lavabolar · https://www.vitra.com.tr/c-dus-uniteleri · https://www.vitra.com.tr/c-kampanyali-urunler · https://www.trendyol.com/sr?q=s%C3%BCrg%C3%BCl%C3%BC%20el%20du%C5%9Fu%20tak%C4%B1m%C4%B1&amp;sst=BEST_SELLER · https://www.hepsiburada.com/ara?q=ankastre%20stop%20valf&amp;siralama=coksatan · https://www.akakce.com/klozet/ayakli-klozet.html · https://www.cimri.com/arama?q=ayakl%C4%B1%20klozet · https://www.koctas.com.tr/search?q=%C3%A7anak%20lavabo&amp;sort=bestseller-desc · https://www.banyomarka.com/arama?q=s%C3%BCrg%C3%BCl%C3%BC%20el%20du%C5%9Fu%20tak%C4%B1m%C4%B1</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Dil ve düzen: hero sadeleşti, meta cümleler kaldırıldı, kat oranları açıklayıcı, madde listelerinde vurgu, bulgu kartı düzeni
- Hero'dan açıklama paragrafı ve sürüm/dönem çipleri kaldırıldı; Özet'in meta girişi kaldırıldı
- 'Bu bölüm', 'Bu rapor', 'İkinci bölümde', 'Aşağıdaki tablo' tipi yapı anlatan cümleler doğrudan olgu cümlelerine çevrildi
- Kat oranları sadeleşti ve açıklandı (2,0-6,1x → 2-6 kat, ne neye oranlanıyor yazıldı; 1,66/1,99 → 1,7/2; 2-2,7 → 2-3; 4,1x/2,0x → 4/2 kat)
- Kritik tespit, not ve bulgu kartı maddelerinde sayılar, markalar ve üstünlük ifadeleri otomatik vurgulanıyor; EN blok çevirisi için madde metni ayrı sarmalayıcıda
- Bulgu kartlarında 'Bulgu 01' etiketi ile başlığın üst üste binmesi giderildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -650,7 +650,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Makro Ortam ve Ödeme Gücü · Kart harcamaları: banyo ile ilişkili sektörler
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket eden bir karar alanıdır. Bu bölümde TCMB EVDS üzerinden kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları izlenmektedir; kategori talebindeki daralma (Bölüm 03) bu ortamla birlikte okunmalıdır.
+Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Harcama kalemi: BKM ve TCMB'nin haftalık sektörel kart harcama akımı; haftalar takvim ayına toplanmıştır. | Oca-Ağu 2025: Ocak - Ağustos 2025 toplam kart harcaması, milyar TL, nominal. | Oca-Ağu 2026: Ocak - Ağustos 2026 toplam kart harcaması, milyar TL, nominal. | Değişim: İki pencere arasındaki nominal yüzde değişim; enflasyon etkisi arındırılmamıştır.</t>
         </is>
@@ -813,7 +813,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: SSG ve BM: Derin Talep İncelemesi · Kullanıcı hangi özellikle arıyor? SSG
-Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. İkinci bölümde aynı segmentlerin genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı ölçülmüştür.
+Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. Genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı da ölçülmüştür.
 Kaynak: Google Ads Keyword Planner · temel set 2.420 kelime 48 ay (Eyl 2022 - Ağu 2026) · genişletilmiş kelime evreni (keywords for keywords, 52.973 kelime) · Türkiye, Türkçe · 28.09.2026 7 , 10
 Sütun açıklamaları: Boyut: Arama ifadesinde geçen özellik grubu. | Arama özelliği: İfadede geçen özellik; bir kelime birden fazla özelliğe girebilir. | Aylık hacim: Eyl 2025 - Ağu 2026 aylık ortalama; genişletilmiş kelime evreni, yazım varyantları tek sayılmıştır. | Pay: Segmentin toplam arama hacmi içindeki pay. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | Örnek: Özelliğin en yüksek hacimli kelimeleri.</t>
         </is>
@@ -2082,11 +2082,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="76" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Yöntem ve Kapsam
-Kapsam: Bu rapor, Inbound'un erişimindeki veri kaynaklarıyla hazırlanmıştır. VitrA'dan beklenen pazaryeri performansı, GA4 dönüşüm ve site içi arama raporları, iade ve çağrı merkezi verisi geldiğinde ilgili bölümler eklenecek ve öneriler güncellenecektir.
+Kapsam: Veri kaynakları, dönemleri ve yöntem notları aşağıdadır. GA4 dönüşüm ve site içi arama raporları, iade ve çağrı merkezi verisi bu sürüme dahil değildir.
 Sütun açıklamaları: Veri kaynağı: Kullanılan kaynak. | Kapsam: Dönem, coğrafya ve örneklem. | Kullanıldığı bölüm: Verinin işlendiği bölüm. | Not: Ölçüm sınırı veya yöntem notu.</t>
         </is>
       </c>
@@ -3690,7 +3690,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: SSG ve BM: Derin Talep İncelemesi · Kullanıcı hangi özellikle arıyor? BM
-Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. İkinci bölümde aynı segmentlerin genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı ölçülmüştür.
+Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. Genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı da ölçülmüştür.
 Kaynak: Google Ads Keyword Planner · temel set 2.420 kelime 48 ay (Eyl 2022 - Ağu 2026) · genişletilmiş kelime evreni (keywords for keywords, 52.973 kelime) · Türkiye, Türkçe · 28.09.2026 7 , 10
 Sütun açıklamaları: Boyut: Arama ifadesinde geçen özellik grubu. | Arama özelliği: İfadede geçen özellik; bir kelime birden fazla özelliğe girebilir. | Aylık hacim: Eyl 2025 - Ağu 2026 aylık ortalama; genişletilmiş kelime evreni, yazım varyantları tek sayılmıştır. | Pay: Segmentin toplam arama hacmi içindeki pay. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | Örnek: Özelliğin en yüksek hacimli kelimeleri.</t>
         </is>
@@ -6604,7 +6604,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Makro Ortam ve Ödeme Gücü · Konut hareketliliği ve kredi koşulları
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket eden bir karar alanıdır. Bu bölümde TCMB EVDS üzerinden kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları izlenmektedir; kategori talebindeki daralma (Bölüm 03) bu ortamla birlikte okunmalıdır.
+Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Gösterge: TCMB EVDS'den alınan seri. | Değer: Belirtilen dönem için değer. | Karşılaştırma: Bir önceki dönem veya bir yıl önceki değer. | Okuma: Banyo kategorisi açısından kısa yorum.</t>
         </is>
@@ -10237,7 +10237,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket eden bir karar alanıdır. Bu bölümde TCMB EVDS üzerinden kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları izlenmektedir; kategori talebindeki daralma (Bölüm 03) bu ortamla birlikte okunmalıdır.
+Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Yıllık yenileme oranı: Konutların yılda yüzde kaçında banyonun yenilendiği varsayımı; Türkiye için ölçülmüş bir oran bulunmadığından senaryo olarak verilmiştir. | Karşılığı: Oranın ima ettiği ortalama yenileme döngüsü; Almanya'da yenilenmemiş banyoların ortalama yaşı 19,5 yıldır (VDS, 2017). | Yenilenen banyo (milyon): 26,6 milyon hane × oran × konut başına 1,1-1,3 banyo. | Yeni konut banyosu (milyon): Yılda 0,4-0,6 milyon iskanlı daire × 1,1-1,3 banyo. | Toplam (milyon banyo / yıl): Yenileme ve yeni konut toplamı.</t>
         </is>
@@ -12516,7 +12516,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Katalog ve Talep Eşleşmesi
-Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. İkinci bölümde aynı temaların Trendyol'daki görünümü (fiyat bandı, öne çıkan satıcılar, VitrA varlığı) incelenmiştir.
+Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. Aynı temaların Trendyol'daki fiyat bandı, öne çıkan satıcıları ve VitrA varlığı da karşılaştırılmıştır.
 Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 9 , 10 , 19
 Sütun açıklamaları: Grup: Tema grubu. | Tema: Genişletilmiş kelime evreninde tanımlanan ürün teması. | Aylık talep: Eyl 2025 - Ağu 2026 aylık ortalama arama hacmi; yazım varyantları tek sayılmıştır. | 3 yıllık değişim: Eyl 22 - Ağu 23 ile Eyl 25 - Ağu 26 ortalamaları arasındaki değişim. | VitrA ürün: vitra.com.tr ürün sitemap'inde temaya eşlenen ürün adresi sayısı; renk ve ölçü varyantları ayrı sayılır. | Model: Renk ekleri ayıklanmış tekil ürün adı sayısı (yaklaşık). | Durum: VitrA kataloğunda temanın karşılığı: Var, Kısmi (sınırlı derinlik), Yok. | Not: Katalog ve pazaryeri gözlemi.</t>
         </is>
@@ -13712,7 +13712,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket eden bir karar alanıdır. Bu bölümde TCMB EVDS üzerinden kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları izlenmektedir; kategori talebindeki daralma (Bölüm 03) bu ortamla birlikte okunmalıdır.
+Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Gösterge: Tahminde kullanılan girdi. | Değer: Kaynaktaki değer. | Kaynak ve not: Kaynak ve ölçüm türü.</t>
         </is>
@@ -13886,7 +13886,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Katalog ve Talep Eşleşmesi · Pazaryerindeki görünüm: Trendyol
-Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. İkinci bölümde aynı temaların Trendyol'daki görünümü (fiyat bandı, öne çıkan satıcılar, VitrA varlığı) incelenmiştir.
+Kapsam: vitra.com.tr ürün sitemap'indeki 7.804 ürün adresi temalara eşlenerek her temadaki katalog derinliği arama talebiyle karşılaştırılmıştır. Aynı temaların Trendyol'daki fiyat bandı, öne çıkan satıcıları ve VitrA varlığı da karşılaştırılmıştır.
 Kaynak: vitra.com.tr ürün sitemap'i (7.804 adres) ve kategori sayfaları · Google Ads Keyword Planner genişletilmiş evren · Trendyol arama sonuçları (Apify) · 28.09.2026 9 , 10 , 19
 Sütun açıklamaları: Trendyol araması: Trendyol arama kutusuna yazılan ifade. | İncelenen ürün: İncelenen ilk sonuç sayısı. | Medyan fiyat (TL): İncelenen ürünlerin medyan satış fiyatı; havlupanda yalnız ısıtıcılı havlupanlar, iç takımda jenerik ürünler. | VitrA / Artema ürün: İlk sonuçlarda VitrA veya Artema markalı ürün sayısı. | En çok değerlendirilen marka: İlk sonuçlarda değerlendirme sayısı en yüksek ürünün markası; bağlantı ürün sayfasını yeni sekmede açar. | Fiyat (TL): Bu ürünün satış fiyatı, 29.09.2026. | Değerlendirme sayısı: Bu ürünün değerlendirme sayısı; satış hacmi göstergesi olarak kullanılmıştır. | Gözlem: Sonuç sayfasının genel görünümü.</t>
         </is>
@@ -14410,7 +14410,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Yeni Kategori ve Segment Fırsatları
-Kapsam: Genişletilmiş kelime evreni (52.973 kelime) VitrA'nın bugünkü kategori ağacının dışına taşan temaları da kapsayacak şekilde sınıflandırılmıştır. Aşağıdaki tablo VitrA kataloğunda bulunmayan ya da sınırlı derinlikte bulunan temaları; talebi, rakipte kimin sattığını, VitrA'ya uyumu ve olası satış modelini birlikte göstermektedir. Haziran 2026 sezonsallık çalışmasındaki dört ürün kümesi (yedek parça, evye, arıtmalı batarya, universal akıllı kapak) bu tabloda güncel veriyle yeniden ölçülmüştür.
+Kapsam: Genişletilmiş kelime evreni (52.973 kelime) VitrA'nın bugünkü kategori ağacının dışına taşan temaları da kapsayacak şekilde sınıflandırılmıştır. VitrA kataloğunda bulunmayan ya da sınırlı derinlikte bulunan temalar için talep, rakipte kimin sattığı, VitrA'ya uyum ve olası satış modeli birlikte değerlendirilmiştir; Haziran 2026 sezonsallık çalışmasındaki dört ürün kümesi (yedek parça, evye, arıtmalı batarya, universal akıllı kapak) güncel veriyle yeniden ölçülmüştür.
 Kaynak: Google Ads Keyword Planner genişletilmiş evren (48 ay) · vitra.com.tr ürün sitemap'i · Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline kategori sitemap'leri · Trendyol arama sonuçları · Inbound VitrA sezonsallık ve rakip ürün analizi (Haziran 2026) · 28.09.2026 9 , 10 , 19 , 20 , 21
 Sütun açıklamaları: Tema: VitrA kataloğunda bulunmayan ya da sınırlı derinlikte bulunan ürün teması. | Aylık talep: Eyl 2025 - Ağu 2026 aylık ortalama arama hacmi; yazım varyantları tek sayılmıştır. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi. | 3 yıllık değişim: Eyl 22 - Ağu 23 ile Eyl 25 - Ağu 26 ortalamaları arasındaki değişim. | VitrA: VitrA kataloğundaki karşılık. | Rakipte kim satıyor?: Rakip sitelerin kategori ağaçları, Trendyol sonuçları ve Inbound'un Haziran 2026 rakip ürün analizi. | VitrA'ya uyum: Yakın: VitrA veya Artema üretim yetkinliğine bitişik · Orta: tamamlayıcı, iş ortağıyla sunulabilir · Uzak: marka ve kanal açısından uzak. | Model önerisi: Temanın vitra.com.tr'de nasıl sunulabileceği; 3P = üçüncü taraf satıcı. | Örnek aramalar: Temanın en yüksek hacimli aramaları.</t>
         </is>
@@ -20647,13 +20647,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Fiyat konumu
 Kapsam: Pazaryerleri üç kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; tarayıcı ile Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
 Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 32 , 33 , 34
-Sütun açıklamaları: Kategori: Fiyat karşılaştırılan kategori. | Trendyol kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Trendyol: VitrA marka filtresindeki çok satan ilk 36'nın medyanı, TL. | Hepsiburada kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Hepsiburada: VitrA marka filtreli ilk 36 medyanı, TL. | VitrA / kategori: VitrA medyanının kategori medyanına oranı (iki pazaryeri aralığı).</t>
+Sütun açıklamaları: Kategori: Fiyat karşılaştırılan kategori. | Trendyol kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Trendyol: VitrA marka filtresindeki çok satan ilk 36'nın medyanı, TL. | Hepsiburada kategori medyanı: Çok satan ilk 36 ürünün medyan fiyatı, TL. | VitrA Hepsiburada: VitrA marka filtreli ilk 36 medyanı, TL. | VitrA / kategori: VitrA ürünlerinin medyan fiyatının, kategorinin çok satan ürünlerinin medyan fiyatına oranı; iki pazaryeri aralığı, yuvarlanmıştır.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -20714,7 +20714,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2,0-2,1x</t>
+          <t>~2x</t>
         </is>
       </c>
     </row>
@@ -20740,7 +20740,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2,7-3,3x</t>
+          <t>~3x</t>
         </is>
       </c>
     </row>
@@ -20764,7 +20764,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2,8-4,2x</t>
+          <t>3-4x</t>
         </is>
       </c>
     </row>
@@ -20788,7 +20788,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>2,5-6,1x</t>
+          <t>2,5-6x</t>
         </is>
       </c>
     </row>
@@ -20814,7 +20814,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>1,7-3,2x</t>
+          <t>2-3x</t>
         </is>
       </c>
     </row>
@@ -20846,7 +20846,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>1,4-1,5x</t>
+          <t>~1,5x</t>
         </is>
       </c>
     </row>
@@ -38053,7 +38053,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: SSG ve BM: Derin Talep İncelemesi · SSG: ürün tipi düzeyinde değişim
-Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. İkinci bölümde aynı segmentlerin genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı ölçülmüştür.
+Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. Genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı da ölçülmüştür.
 Kaynak: Google Ads Keyword Planner · temel set 2.420 kelime 48 ay (Eyl 2022 - Ağu 2026) · genişletilmiş kelime evreni (keywords for keywords, 52.973 kelime) · Türkiye, Türkçe · 28.09.2026 7 , 10
 Sütun açıklamaları: Alt kategori: VitrA kategori ağacındaki alt kategori. | Ürün tipi: Alt kategorinin altındaki ürün tipi; "Genel" alt kategori adıyla yapılan aramalardır. | Eyl 22 - Ağu 23: Eylül 2022 - Ağustos 2023 aylık ortalama arama hacmi. | Eyl 25 - Ağu 26: Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | 3 yıllık değişim: İki 12 aylık pencerenin ortalamaları arasındaki yüzde değişim. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi.</t>
         </is>
@@ -44391,7 +44391,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: SSG ve BM: Derin Talep İncelemesi · BM: ürün tipi düzeyinde değişim
-Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. İkinci bölümde aynı segmentlerin genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı ölçülmüştür.
+Kapsam: Seramik sağlık gereçleri (SSG: klozet, lavabo, bide, pisuvar, rezervuar) ve banyo mobilyası (BM) için talep dört yıllık aylık seriyle, ürün tipi düzeyinde incelenmiştir. Genişletilmiş kelime evreninde kullanıcının hangi tip, ölçü, renk, özellik ve bağlamla aradığı da ölçülmüştür.
 Kaynak: Google Ads Keyword Planner · temel set 2.420 kelime 48 ay (Eyl 2022 - Ağu 2026) · genişletilmiş kelime evreni (keywords for keywords, 52.973 kelime) · Türkiye, Türkçe · 28.09.2026 7 , 10
 Sütun açıklamaları: Alt kategori: VitrA kategori ağacındaki alt kategori. | Ürün tipi: Alt kategorinin altındaki ürün tipi; "Genel" alt kategori adıyla yapılan aramalardır. | Eyl 22 - Ağu 23: Eylül 2022 - Ağustos 2023 aylık ortalama arama hacmi. | Eyl 25 - Ağu 26: Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | 3 yıllık değişim: İki 12 aylık pencerenin ortalamaları arasındaki yüzde değişim. | YoY: Oca-Ağu 2026 / Oca-Ağu 2025 yüzde değişimi.</t>
         </is>
@@ -46028,7 +46028,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · E-ticaret modelleri
-Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
+Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. Ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte karşılaştırılmıştır.
 Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 22 , 23 , 24 , 25 , 26 , 27 , 28 , 29 , 42 , 43 , 44 , 45 , 46 , 47 , 48
 Sütun açıklamaları: Oyuncu: İncelenen site. | Tip: İş modeli. | E-ticaret modeli: Ürün, kanal ve hizmetin nasıl bir araya getirildiği. | VitrA'ya uyarlanabilir nokta: VitrA'nın mevcut yapısına eklenebilecek unsur.</t>
         </is>
@@ -46292,7 +46292,7 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Benchmark: E-Ticaret Modelleri ve Dijital Deneyim · Ürün keşfi ve dijital deneyim örnekleri
-Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. İkinci tabloda ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte verilmiştir.
+Kapsam: Türkiye'den yapı market, mobilya perakendecisi, pureplayer, marka ve pazaryeri; yurt dışından banyo pureplayer'ı, yapı market ve üretici marka modelleri incelenmiştir. Ürün keşfi ve dijital deneyim araçları VitrA'daki karşılıklarıyla birlikte karşılaştırılmıştır.
 Kaynak: Rakip ve benzer oyuncuların web siteleri, hizmet ve kampanya sayfaları · 28.09.2026 22 , 23 , 24 , 25 , 26 , 27 , 28 , 29 , 42 , 43 , 44 , 45 , 46 , 47 , 48
 Sütun açıklamaları: Araç: Ürün keşfi ya da dijital deneyim aracı. | Örnek: Aracı kullanan oyuncular. | Ne sağlıyor?: Kullanıcıya sağladığı fayda. | VitrA'da: vitra.com.tr'deki karşılığı (29.09.2026). | Gözlem: Mevcut durum ve olası adım.</t>
         </is>
@@ -46602,11 +46602,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="118" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Kanal rolleri
-Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
+Kapsam: VitrA bugün Banyo Asistanı, montaj ve keşif hizmetleri ve ürün sayfası bilgileriyle kanal içinde etkileşim sunmaktadır; aşağıdaki kanal rolleri ve etkileşim modeli bu yapının üzerine kurulmuştur.
 Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 7 , 9 , 11 , 12 , 19
 Sütun açıklamaları: Kanal: Satış kanalı. | Bugünkü rol: Bu çalışmadaki gözlemlere dayalı mevcut konum; VitrA'nın panel verisiyle doğrulanacaktır. | Önerilen rol: Kanalın büyüme planında üstlenebileceği rol. | Öne çıkarılabilecek ürün grubu: Talep ve ihtiyaç verisine göre kanalda öne çıkarılabilecek grup.</t>
         </is>
@@ -46755,11 +46755,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="118" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Hacimli ve ölçüye bağlı ürünlerde etkileşim modeli
-Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
+Kapsam: VitrA bugün Banyo Asistanı, montaj ve keşif hizmetleri ve ürün sayfası bilgileriyle kanal içinde etkileşim sunmaktadır; aşağıdaki kanal rolleri ve etkileşim modeli bu yapının üzerine kurulmuştur.
 Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 7 , 9 , 11 , 12 , 19
 Sütun açıklamaları: Bileşen: Hacimli ve ölçüye bağlı üründe karar öncesi belirsizliği azaltan unsur. | VitrA'da bugün: vitra.com.tr üzerindeki mevcut uygulama (29.09.2026). | Durum: Var, Kısmi (sınırlı kapsam), Yok. | Geliştirme alanı: Mevcut yapının üzerine eklenebilecek adım.</t>
         </is>
@@ -46974,11 +46974,11 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kanal Rolleri ve Etkileşim Modeli · Tamamlayıcı ürün kurgusu
-Kapsam: Bu bölüm, talep ve davranış verisinin kanal rollerine ve etkileşim modeline nasıl çevrilebileceğini ele almaktadır. VitrA'nın bugün sunduğu uygulamalar (Banyo Asistanı, montaj ve keşif hizmetleri, ürün sayfası bilgileri) incelenmiş; öneriler bu yapının üzerine kurulmuştur. Pazaryeri ve GA4 verisi geldiğinde güncellenecektir.
+Kapsam: VitrA bugün Banyo Asistanı, montaj ve keşif hizmetleri ve ürün sayfası bilgileriyle kanal içinde etkileşim sunmaktadır; aşağıdaki kanal rolleri ve etkileşim modeli bu yapının üzerine kurulmuştur.
 Kaynak: vitra.com.tr ürün, hizmet ve kategori sayfaları (29.09.2026) · Google Keyword Planner, Search Console, Autocomplete · Trendyol arama sonuçları 7 , 9 , 11 , 12 , 19
 Sütun açıklamaları: Ürün grubu: VitrA'nın üretmediği veya sınırlı ürettiği, kategori satın almasıyla birlikte ihtiyaç duyulan grup. | Talep sinyali: Kelime araştırması, autocomplete veya Search Console'daki ifade. | Bugün nerede satılıyor?: Kullanıcının bu ürünü bulduğu kanal; rakip site incelemesine göre. | Model önerisi: vitra.com.tr için değerlendirilebilecek satış modeli.</t>
         </is>

</xml_diff>

<commit_message>
Talep grafiği 2023'ten, açılır kelime listeleri, SERP doğrulaması, gruplu autocomplete tablosu
- Kategori talebi aylık serisi Oca 2023 - Ağu 2026; yıllar ayrı renkte, her yılın peak ve base ayı etiketli; grafik balonunda ay adı
- Kategori ve alt kategori tablolarında ok simgesi ilgili en yüksek hacimli kelimeleri açılır pencerede gösteriyor
- Kim sıralanıyor, VitrA nerede ve YouTube bölümlerinde kelime listesi açılır pencereleri
- VitrA'nın görünmediği kelimeler Search Console ve Google (google.com.tr) ile doğrulandı; ilk 5 alan adı sütunu
- Kategori ve rakip marka aramaları: 52 kök ifade, 6 grup, 16 rakip marka kök ifadesi; hacim rozeti aralığı düzeltildi
- Hacim hücreleri ekranda yuvarlanmış (21,6K), kopyalama ve Excel'de tam sayı
- Kısa ara başlık notları tam cümleye çevrildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -31,7 +31,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 En çok tık getiren sorgula" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Kim sıralanıyor" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 VitrA nerede" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 VitrA'nın görünmediği yüks" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 Yüksek hacimli kelimelerde" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26 SERP özellikleri ve AI Ove" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27 YouTube Montaj, Tamir ve " sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28 Kimler görünür" sheetId="28" state="visible" r:id="rId28"/>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Banyo dolabı aylık 60.000 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; banyo bataryası ve taharet musluğunda VitrA ilk 20'de yok; baş kelimelerin çoğunda KD 0-2 13 , 31</t>
+          <t>Banyo dolabı aylık 60.000 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; taharet musluğunda VitrA ilk sayfada yok, banyo ve lavabo bataryasında 3. sırada; baş kelimelerin çoğunda KD 0-2 13 , 31</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -6379,12 +6379,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · "vitra" ile başlayan aramalar
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 11 , 12
+Kaynak: Google Autocomplete · 49 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
 Sütun açıklamaları: Kök ifade: Google arama kutusuna yazılan ifade; öneriler bu ifadenin devamı olarak gelmektedir. | Autocomplete önerileri · 2026 aylık ort. hacim: Google'ın Türkiye, Türkçe, masaüstü Chrome için döndürdüğü ilk 10 tamamlama önerisi; sırası Google'ın sırasıdır. Rozet: Ocak - Ağustos 2026 aylık ortalama arama hacmi (Google Ads); rozeti olmayan kelime için hacim dönmemiştir.</t>
         </is>
       </c>
@@ -6769,11 +6769,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -6783,24 +6784,30 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · Kategori ve rakip marka aramaları
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 11 , 12
-Sütun açıklamaları: Kök ifade: Kategori veya rakip marka ile başlayan ifade. | Autocomplete önerileri · 2026 aylık ort. hacim: Google'ın döndürdüğü ilk 10 tamamlama önerisi; rozet Ocak - Ağustos 2026 aylık ortalama arama hacmidir (Google Ads).</t>
+Kaynak: Google Autocomplete · 49 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
+Sütun açıklamaları: Grup: Kök ifadenin türü: kategori, montaj ve tamir, yenileme ve tasarım, fiyat ve ödeme, rakip marka, perakendeci. | Kök ifade: Google arama kutusuna yazılan ifade; rozet Ocak - Ağustos 2026 aylık ortalama arama hacmidir (Google Ads). Grup içinde hacme göre sıralanmıştır. | Autocomplete önerileri · 2026 aylık ort. hacim: Google'ın Türkiye, Türkçe, Chrome için döndürdüğü ilk 10 tamamlama önerisi (30 Eyl 2026); sırası Google'ın sırasıdır. Rozet Ocak - Ağustos 2026 aylık ortalama arama hacmidir.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
+          <t>Grup</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>Kök ifade</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Autocomplete önerileri · 2026 aylık ort. hacim</t>
         </is>
@@ -6809,162 +6816,890 @@
     <row r="5" ht="69" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>klozet 49,5K</t>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>klozet fiyatları 65,6K klozet kapağı 35,9K klozet şamandırası 7,3K klozet takımı 12,8K klozet taharet musluğu 4,5K klozet modelleri 7,3K klozet kapağı fiyatları 6,5K klozet iç takım 9,4K klozet fiyatları kayseri 65 klozet kapağı menteşesi 4,5K</t>
+          <t>banyo dolabı 95,4K</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı fiyatları 6,8K banyo dolabı lavabolu 3,6K banyo dolabı seti 3,3K banyo dolabı kayseri 36 banyo dolabı ölçüleri 1,2K banyo dolabı takımı 2,3K banyo dolabı plastik 940 banyo dolabı aynalı 875 banyo dolabı modelleri fiyatları 895 banyo dolabı modelleri küçük 270</t>
         </is>
       </c>
     </row>
     <row r="6" ht="69" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı 95,4K</t>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı fiyatları 6,8K banyo dolabı lavabolu 3,6K banyo dolabı seti 3,3K banyo dolabı kayseri 36 banyo dolabı ölçüleri 1,2K banyo dolabı plastik 940 banyo dolabı takımı 2,3K banyo dolabı aynalı 875 banyo dolabı modelleri küçük 270 banyo dolabı modelleri fiyatları 895</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="82" customHeight="1">
+          <t>duşakabin 92,9K</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>duşakabin fiyatları 56,4K duşakabin modelleri 43,9K duşakabin kayseri 184 duşakabin tekerleği 9,7K duşakabin cam filmi 1,4K duşakabin camı 6,5K duşakabin temizliği 5,0K duşakabin fiyatları kayseri 54 duşakabin silikonu 2,2K duşakabin ölçüleri 1,9K</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="69" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>klozet 49,5K</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>klozet fiyatları 65,6K klozet kapağı 35,9K klozet şamandırası 7,3K klozet takımı 12,8K klozet taharet musluğu 4,5K klozet modelleri 7,3K klozet kapağı fiyatları 6,5K klozet iç takım 9,4K klozet fiyatları kayseri 65 klozet kapağı menteşesi 4,5K</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>lavabo 41,4K</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>lavabo açıcı 24,0K lavabo bataryası 23,4K lavabo gider borusu 12,5K lavabo fiyatları 5,5K lavabo modelleri 9,5K lavabo dolabı 8,1K lavabo sifonu 6,3K lavabo süzgeci 5,2K lavabolu banyo dolabı 6,6K lavabo altı dolap 5,3K</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="82" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>banyo bataryası 38,6K</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>banyo bataryası fiyatları 8,1K banyo bataryası duş seti 1,9K banyo bataryası tamiri 1,3K banyo bataryası fiyatları en ucuz 1,2K banyo bataryası nasıl takılır 404 banyo bataryası kartuş değişimi 319 banyo bataryası duş yönlendirici tamiri banyo bataryası su kaçırıyor 124 banyo bataryası parçaları 728 banyo bataryası tesisat ölçüleri 152</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="82" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>klozet kapağı 35,9K</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>klozet kapağı fiyatları 6,5K klozet kapağı menteşesi 4,5K klozet kapağı nasıl sökülür 820 klozet kapağı montajı 895 klozet kapağı vidası 2,5K klozet kapağı a101 611 klozet kapağı nasıl değiştirilir 639 klozet kapağı amortisörü tamiri 576 klozet kapağı örtüsü 1,8K klozet kapağı montaj vidası 720</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="95" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>lavabo bataryası 23,4K</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>lavabo bataryası fiyatları 3,2K lavabo bataryası sıcak soğuk 1,0K lavabo bataryası sökme anahtarı 764 lavabo bataryası nasıl sökülür 424 lavabo bataryası sıcak soğuk en ucuz 524 lavabo bataryası nasıl takılır 315 lavabo bataryası sıcak soğuk fiyatları 384 lavabo bataryası modelleri 142 lavabo bataryası içi nasıl sökülür 82 lavabo bataryası eca 236</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="69" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>duş seti 17,7K</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>duş seti fiyatları 2,9K duş seti parçaları 404 duş seti montajı 306 duş seti yönlendirici 329 duş seti modelleri 265 duş seti yönlendirici tamiri duş seti siyah 235 duş seti nasıl takılır 62 duş seti eca 151 duş seti nasıl sökülür 59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="82" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
           <t>gömme rezervuar 16,0K</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>gömme rezervuar iç takımı 4,7K gömme rezervuar ölçüleri 1,6K gömme rezervuar şamandıra 820 gömme rezervuar fiyatları 1,4K gömme rezervuar montajı 1,1K gömme rezervuar su kaçırıyor 812 gömme rezervuar şamandıra ayarı 156 gömme rezervuar taharet musluğu 760 gömme rezervuar tamiri 1,2K gömme rezervuar şamandıra suyu kesmiyor 508</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="69" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin 92,9K</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin fiyatları 56,4K duşakabin modelleri 43,9K duşakabin kayseri 184 duşakabin tekerleği 9,7K duşakabin cam filmi 1,4K duşakabin camı 6,5K duşakabin temizliği 5,0K duşakabin fiyatları kayseri 54 duşakabin silikonu 2,2K duşakabin ölçüleri 1,9K</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="69" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>akıllı klozet 2,5K</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>akıllı klozet kapağı 941 akıllı klozet fiyatları 554 akıllı klozet kapağı fiyatları 146 akıllı klozet türkiye 48 akıllı klozet nedir 48 akıllı klozet vitra 56 akıllı klozet özellikleri 31 akıllı klozet kapağı vitra 12 akıllı klozet modelleri akıllı klozet kapağı tamiri</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="69" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>klozet montaj 1,2K</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>klozet montajı 1,2K klozet montaj aparatı 902 klozet montajı nasıl yapılır 535 klozet montaj vidası 639 klozet montaj ücreti 86 klozet montaj ölçüleri 149 klozet montaj aparatı ve körüklü kada 90 klozet montaj aparatı koçtaş 74 klozet montaj seti 101 klozet montajı nasıl yapılır video 32</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="69" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>klozet tamir 1,3K</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>klozet tamiri 1,3K klozet tamir takımı 426 klozet tamiri nasıl yapılır 185 klozet tamir takımı fiyatları 54 klozet tamiri fiyat 31 klozet tamirini kim yapar 49 klozet tamir seti 24 klozet tamir takımı değişimi 18 klozet tamir takımı nasıl değişir 8 klozet tamiri kiracıya mı ait 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="82" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>banyo dolabı montaj 290</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>banyo dolabı montajı 290 banyo dolabı montaj ölçüleri 170 banyo dolabı montaj aparatı 56 banyo dolabı montaj ücreti 4 banyo dolabı montaj dahil 16 banyo dolabı montaj yüksekliği banyo dolabı montajı nasıl yapılır 75 banyo dolabı montaj vidası banyo dolabı montaj ustası banyo dolabı montaj videosu</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>klozet taksit</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>klozet taktırma klozet taktırma fiyatı klozet takımı tekzen 8 klozet taktırma ücreti</t>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>gömme rezervuar iç takımı 4,7K gömme rezervuar ölçüleri 1,6K gömme rezervuar fiyatları 1,4K gömme rezervuar şamandıra 820 gömme rezervuar montajı 1,1K gömme rezervuar su kaçırıyor 812 gömme rezervuar taharet musluğu 760 gömme rezervuar tamiri 1,2K gömme rezervuar şamandıra suyu kesmiyor 508 gömme rezervuar kapağı 800</t>
         </is>
       </c>
     </row>
     <row r="14" ht="69" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>banyo yenileme 2,1K</t>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>banyo yenileme maliyeti 434 banyo yenileme maliyeti 2026 262 banyo yenileme modelleri 264 banyo yenileme fikirleri 381 banyo yenileme videoları 11 banyo yenileme malzemeleri 14 banyo yenileme pinterest banyo yenileme örnekleri banyo yenileme kendin yap 16 banyo yenileme izmir 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="69" customHeight="1">
+          <t>havlupan 14,4K</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>havlupan fiyatları 5,0K havlupan petek 2,1K havlupan ölçüleri 1,1K havlupan modelleri 704 havlupan vanası 585 havlupan askısı 598 havlupan montajı 405 havlupan petek fiyatları 481 havlupan fiyatları koçtaş 102 havlupan montaj seti 238</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="82" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>artema 6,2K</t>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>artema mutfak bataryası 7,2K artema banyo bataryası 5,3K artema lavabo bataryası 4,1K artema duş seti 3,0K artema taharet musluğu 1,7K artema musluk 1,6K artema servis kayseri 15 artema kayseri artema batarya 1,8K artema duş başlığı 1,2K</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="82" customHeight="1">
+          <t>banyo aksesuar 9,9K</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>banyo aksesuarları 9,9K banyo aksesuar seti 1,9K banyo aksesuarları kayseri banyo aksesuar modelleri 258 banyo aksesuarları trendyol 159 banyo aksesuarı montaj duvara bağlantı aparatı 168 banyo aksesuarları ikea 82 banyo aksesuar seti krom 80 banyo aksesuarları süsleri 114 banyo aksesuarları yapışkanlı 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="69" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>creavit klozet 3,8K</t>
+          <t>Kategori</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>creavit klozet kapağı 2,5K creavit klozet kapağı menteşesi 535 creavit klozet fiyatları 330 creavit klozet kapağı nasıl sökülür 209 creavit klozet kapağı parçaları 339 creavit klozet şamandırası nasıl takılır 132 creavit klozet kapağı montajı 75 creavit klozet iç takımı 165 creavit klozet montajı 80 creavit klozet kapağı amortisörü 70</t>
+          <t>lavabo dolabı 8,1K</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>lavabo dolabı modelleri 3,2K lavabo dolabı aynalı 446 lavabo dolabı yüksekliği 38 lavabo dolabı fiyatları 471 lavabo dolabı ölçüleri 219 lavabo dolabı a101 94 lavabo dolabı montajı 42 lavabo dolabı yerden yüksekliği 30 lavabo dolabı seti 151 lavabo dolabı takımı 156</t>
         </is>
       </c>
     </row>
     <row r="17" ht="82" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>asma klozet 7,0K</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>asma klozet fiyatları 2,6K asma klozet montajı 675 asma klozet ölçüleri 935 asma klozet taharet çubuğu 392 asma klozet alttan su kaçırıyor 401 asma klozet montajı nasıl yapılır 462 asma klozet taharet çubuğu nasıl değiştirilir 346 asma klozet montaj seti 355 asma klozet ve gömme rezervuar fiyatları 330 asma klozet modelleri 364</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="69" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>çanak lavabo 7,0K</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>çanak lavabo modelleri 1,9K çanak lavabo bataryası 1,7K çanak lavabo ölçüleri 330 çanak lavabolu banyo dolabı 688 çanak lavabo fiyatları 235 çanak lavabo dolabı 364 çanak lavabo banyo dolabı 688 çanak lavabo yüksekliği 88 çanak lavabo altı dolap 136 çanak lavabo dolap modelleri 221</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="69" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Kategori</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>akıllı klozet 2,5K</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>akıllı klozet kapağı 941 akıllı klozet fiyatları 554 akıllı klozet kapağı fiyatları 146 akıllı klozet türkiye 48 akıllı klozet nedir 48 akıllı klozet vitra 56 akıllı klozet özellikleri 31 akıllı klozet kapağı vitra 12 akıllı klozet modelleri akıllı klozet kapağı tamiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>klozet su kaçırıyor 1,8K</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>klozet su kaçırıyorsa çok basit tamiri 1,6K klozet su kaçırıyor ne yapmalıyım 588 klozet su kaçırıyor nasıl tamir edilir 708 klozet su kaçırıyor neden 16 klozet su kaçırıyor tamiri nasıl yapılır 4 klozet su kaçırıyor gömme 11 klozet su kaçırıyor nasıl yapılır 10 klozet su kaçırıyor sebebi nedir klozet su kaçırıyor su faturası klozet su kaçırıyor şamandıra 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="69" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>klozet tamir 1,3K</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>klozet tamiri 1,3K klozet tamir takımı 426 klozet tamiri nasıl yapılır 185 klozet tamir takımı fiyatları 54 klozet tamiri fiyat 31 klozet tamirini kim yapar 49 klozet tamir seti 24 klozet tamir takımı değişimi 18 klozet tamir takımı nasıl değişir 8 klozet tamiri kiracıya mı ait 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="69" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>klozet montaj 1,2K</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>klozet montajı 1,2K klozet montaj aparatı 902 klozet montajı nasıl yapılır 535 klozet montaj vidası 639 klozet montaj ücreti 86 klozet montaj ölçüleri 149 klozet montaj aparatı ve körüklü kada 90 klozet montaj aparatı koçtaş 74 klozet montaj seti 101 klozet montajı nasıl yapılır video 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="82" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>gömme rezervuar tamiri 1,2K</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>gömme rezervuar tamiri nasıl yapılır 85 gömme rezervuar tamiri vitra 12 gömme rezervuar tamiri kale gömme rezervuar tamiri visam gömme rezervuar tamiri kime aittir gömme rezervuar tamiri ankara gömme rezervuar tamiri serel gömme rezervuar tamiri fiyatları 10 gömme rezervuar tamiri izmir creavit gömme rezervuar tamiri 111</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="82" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>rezervuar tamiri 311</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>rezervuar tamiri nasıl yapılır 29 rezervuar tamiri nasıl gömme rezervuar tamiri 1,2K gömme rezervuar tamiri nasıl yapılır 85 klozet rezervuar tamiri 35 tuvalet rezervuar tamiri 31 rezervuar şamandıra tamiri 26 kapalı rezervuar tamiri 12 vitra rezervuar tamiri 15 gömme rezervuar tamiri vitra 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="82" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Montaj ve tamir</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı montaj 290</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı montajı 290 banyo dolabı montaj ölçüleri 170 banyo dolabı montaj aparatı 56 banyo dolabı montaj ücreti 4 banyo dolabı montaj dahil 16 banyo dolabı montaj yüksekliği banyo dolabı montajı nasıl yapılır 75 banyo dolabı montaj vidası banyo dolabı montaj ustası banyo dolabı montaj videosu</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="82" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme ve tasarım</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>banyo dekorasyon 6,4K</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>banyo dekorasyon fikirleri 911 banyo dekorasyon ürünleri 459 banyo dekorasyon modelleri 449 banyo dekorasyonları 6,4K banyo dekorasyonu örnekleri 371 banyo dekorasyonu pinterest 149 banyo dekorasyon aksesuar 144 banyo dekorasyon fikirleri pinterest 34 banyo dekorasyon fiyatları 51 banyo dekorasyon resimleri 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="69" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme ve tasarım</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>banyo tasarım 4,5K</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>banyo tasarımları 4,5K banyo tasarımı 4,5K banyo tasarım modelleri 359 banyo tasarımları pinterest 159 banyo tasarım programı 132 banyo tasarımı yap 120 banyo tasarım programı ücretsiz 164 banyo tasarımı yapay zeka 24 banyo tasarım fikirleri 156 banyo tasarım örnekleri 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="82" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme ve tasarım</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>banyo yenileme 2,1K</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>banyo yenileme maliyeti 434 banyo yenileme maliyeti 2026 262 banyo yenileme modelleri 264 banyo yenileme fikirleri 381 banyo yenileme fiyatları 188 banyo yenileme videoları 11 banyo yenilemek ne kadar tutar 35 banyo yenileme malzemeleri 14 banyo yenileme ücreti 12 banyo yenileme ne kadar tutar 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="82" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme ve tasarım</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>banyo tadilat 1,9K</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>banyo tadilatı 1,9K banyo tadilatı ne kadar tutar 174 banyo tadilatı ne kadar tutar 2026 101 banyo tadilat modelleri 212 banyo tadilat örnekleri 199 banyo tadilat fikirleri 82 banyo tadilatı kaç gün sürer 70 banyo tadilat görselleri 14 banyo tadilatında dikkat edilmesi gerekenler 15 banyo tadilatı ne kadar sürer 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="69" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme ve tasarım</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>küçük banyo 284</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>küçük banyo modelleri 2,3K küçük banyo tasarımları 1,7K küçük banyo dolabı 1,3K küçük banyo dekorasyonu 1,1K küçük banyo dolap modelleri 550 küçük banyo fayans modelleri 3,0K küçük banyo raf modelleri küçük banyo lavabosu 290 küçük banyo hamam modelleri 345 küçük banyo lavabo modelleri 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="82" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat ve ödeme</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>klozet fiyatları 65,6K</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>klozet fiyatları kayseri 65 klozet fiyatları ne kadar 1,1K klozet fiyatları turkuaz 45 klozet fiyatları koçtaş 339 klozet fiyatları en ucuz 211 klozet fiyatları vitra 364 klozet fiyatları ikinci el 22 klozet fiyatları 2026 18 klozet fiyatları alttan çıkışlı 75 klozet fiyatları ve modelleri 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="82" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat ve ödeme</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>duşakabin fiyatları 56,4K</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>duşakabin fiyatları kayseri 54 duşakabin fiyatları ne kadar 718 duşakabin fiyatları 2026 132 duşakabin fiyatları koçtaş 249 duşakabin fiyatları tekneli 128 duşakabin fiyatları ve modelleri 71 duşakabin fiyatları 90x90 99 duşakabin fiyatları plastik 60 duşakabin fiyatları mika 98 duşakabin fiyatları 100x100 89</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="82" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat ve ödeme</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı fiyatları 6,8K</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı fiyatları en ucuz 39 banyo dolabı fiyatları ve modelleri 16 banyo dolabı fiyatları koçtaş 46 banyo dolabı fiyatları cimri banyo dolabı fiyatları trendyol 28 banyo dolabı fiyatları 2026 banyo dolabı fiyatları ankara 31 banyo dolabı fiyatları plastik banyo dolabı fiyatları bauhaus 10 banyo dolabı fiyatları lavabolu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="82" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat ve ödeme</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>banyo tadilat fiyatları 496</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>banyo tadilat fiyatları 2026 banyo tadilat fiyatları 2025 9 banyo tadilat fiyatları ankara 21 banyo tadilat fiyatları izmir 8 banyo tadilat fiyatları adana banyo tadilat fiyatları istanbul 10 koçtaş banyo tadilat fiyatları 255 komple banyo tadilat fiyatları 26 banyo tuvalet tadilat fiyatları 32 mutfak banyo tadilat fiyatları 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat ve ödeme</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>klozet taksit</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>klozet taktırma klozet taktırma fiyatı klozet takımı tekzen 8 klozet taktırma ücreti</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="69" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>artema 6,2K</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>artema mutfak bataryası 7,2K artema banyo bataryası 5,3K artema lavabo bataryası 4,1K artema duş seti 3,0K artema servis kayseri 15 artema kayseri artema batarya 1,8K artema musluk 1,6K artema taharet musluğu 1,7K artema duş başlığı 1,2K</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="82" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>orka banyo dolabı 5,5K</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>orka banyo dolabı modelleri 229 orka banyo dolabı 80 cm 178 orka banyo dolabı montajı 35 orka banyo dolabı fiyatları 282 orka banyo dolabı satış noktaları 111 orka banyo dolabı katalog 70 orka banyo dolabı 100 cm 106 orka banyo dolabı modelleri fiyatı 16 orka banyo dolabı koçtaş 135 orka banyo dolabı 65 cm 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="95" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>geberit gömme rezervuar 4,0K</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>geberit gömme rezervuar iç takımı 611 geberit gömme rezervuar fiyatları 364 geberit gömme rezervuar montajı 119 geberit gömme rezervuar seti 132 geberit gömme rezervuar kapağı 138 geberit gömme rezervuar iç takımı değiştirme 90 geberit gömme rezervuar yedek parça 88 geberit gömme rezervuar ölçüleri 96 geberit gömme rezervuar iç takımı montajı 72 geberit gömme rezervuar iç takımı fiyatları 82</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="82" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>creavit klozet 3,8K</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>creavit klozet kapağı 2,5K creavit klozet kapağı menteşesi 535 creavit klozet fiyatları 330 creavit klozet kapağı nasıl sökülür 209 creavit klozet kapağı parçaları 339 creavit klozet şamandırası nasıl takılır 132 creavit klozet kapağı montajı 75 creavit klozet iç takımı 165 creavit klozet montajı 80 creavit klozet kapağı amortisörü 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="69" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>eca batarya 3,8K</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>eca batarya modelleri 60 eca batarya fiyatları 1,2K eca batarya kartuşu 384 eca batarya mutfak 526 eca batarya yedek parçaları 286 eca batarya banyo 241 eca batarya seti 201 eca batarya kartuşu koçtaş 220 eca batarya yetkili servis 90 eca batarya satış noktaları 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="69" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>grohe batarya 2,8K</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>grohe batarya fiyatları 120 grohe batarya banyo 89 grohe batarya mutfak 98 grohe batarya yedek parça 51 grohe batarya nerenin malı 15 grohe batarya kartuşu 75 grohe batarya kartuş değişimi 38 grohe batarya kartuş fiyatı 44 grohe batarya seti 34 grohe batarya montajı 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="82" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>serel klozet 2,4K</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>serel klozet kapağı 2,5K serel klozet fiyatları 479 serel klozet kapağı menteşesi 508 serel klozet iç takımı 549 serel klozet takımı 129 serel klozet takımı fiyatları 120 serel klozet kapağı nasıl sökülür 102 serel klozet kapağı parçaları 130 serel klozet kapağı montajı 82 serel klozet şamandıra ayarı nasıl yapılır 88</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="82" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>turkuaz klozet 2,3K</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>turkuaz klozet fiyatları 952 turkuaz klozet kapağı 622 turkuaz klozet takımı 108 turkuaz klozet modelleri 196 turkuaz klozet takımı fiyatları 131 turkuaz klozet şamandırası 46 turkuaz klozet iç takımı 162 turkuaz klozet montajı 44 turkuaz klozet kapağı fiyatları 68 turkuaz klozet kapağı damperi 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="82" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
           <t>kale klozet 2,0K</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>kale klozet kapağı 2,1K kale klozet fiyatları 870 kale klozet kapağı nasıl sökülür 255 kale klozet iç takımı 308 kale klozet şamandıra tamiri 149 kale klozet modelleri 166 kale klozet yetkili servis 281 kale klozet kapağı fiyatları 134 kale klozet kapağı montajı 68 kale klozet kapağı damperi 131</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="82" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>kale banyo dolabı 1,9K</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>kale banyo dolabı fiyatları 171 kale banyo dolabı modelleri 130 kale banyo dolabı takımı 24 kale banyo dolabı 80 cm 46 kale banyo dolabı 100 cm 50 kale banyo dolabı çekmecesi nasıl sökülür kale banyo dolabı koçtaş 116 kale banyo dolabı 60 cm kale banyo dolabı 65 cm 16 kale banyo dolabı katalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="82" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>hansgrohe duş seti 1,1K</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>hansgrohe duş seti montajı 26 hansgrohe duş seti fiyat 38 hansgrohe duş seti ankastre 16 hansgrohe duş seti bronz hansgrohe duş seti gold hansgrohe duş seti siyah hansgrohe ankastre duş seti montajı 62 hansgrohe termostatik duş seti 42 hansgrohe crometta duş seti 19 hansgrohe ankastre duş seti fiyat 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="69" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>idevit klozet 1,1K</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>idevit klozet kapağı 671 idevit klozet fiyatları 200 idevit klozet kapağı menteşesi 172 idevit klozet kapağı koçtaş 40 idevit klozet iç takım 59 idevit klozet montajı 20 idevit klozet takımı 42 idevit klozet yedek parça 35 idevit klozet rezervuar fiyatları 45 idevit klozet duvara sıfır 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="82" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>duravit klozet 985</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>duravit klozet kapağı 1,1K duravit klozet fiyatları 121 duravit klozet kapağı menteşesi 96 duravit klozet modelleri 38 duravit klozet kapağı koçtaş 39 duravit klozet yedek parça 58 duravit klozet iç takımı 36 duravit klozet kapağı montajı 18 duravit klozet kapağı nasıl sökülür 25 duravit klozet taharet ucu 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="69" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>isvea klozet 330</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>isvea klozet kapağı 724 ısvea klozet 639 isvea klozet kapağı menteşesi 196 isvea klozet montajı 52 isvea klozet yorumları 48 isvea klozet fiyatları 91 isvea klozet yedek parça 51 isvea klozet kapağı montaj vidası 50 isvea klozet kapağı montajı 49 isvea klozet taharet çubuğu</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="82" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>ideal standard klozet 212</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>ideal standard klozet kapağı 230 ideal standard klozet kapağı menteşesi ideal standard klozet duvara sıfır ideal standard klozet kapağı montajı 12 ideal standard klozet kapağı sökme ıdeal standard klozet iç takımı ideal standard klozet taharet musluğu ideal standard klozetas 1 ideal standard klozeto dangtis ideal standard asma klozet 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="69" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Rakip marka</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>roca klozet 58</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>roca klozet kapağı 42 roca klozet fiyatları 12 roca klozetas 0 roca klozeto dangtis roca kale klozet kapağı 346 roca kale klozet 148 roca kale klozet kapağı koçtaş 90 roca kale klozet kapağı fiyat 51 roca kale klozet kapağı ölçüleri 35 roca kale klozet fiyat 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="69" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Perakendeci</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>ikea banyo dolabı 7,9K</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>ikea banyo dolabı seti 249 ikea banyo dolabı lavabolu 32 ikea banyo dolabı plastik 28 ikea banyo dolabı takımı 24 ikea banyo dolabı tasarla 14 ikea banyo dolabı kirli sepetli 18 ikea banyo dolabı kurulumu ikea banyo dolabı ve lavabo ikea banyo dolabı ayağı ikea banyo dolabı düzenleyici 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="82" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Perakendeci</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>bauhaus banyo dolabı 3,4K</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>bauhaus banyo dolabı fiyatları 318 bauhaus banyo dolabı takımı 216 bauhaus banyo dolabı modelleri 60 bauhaus banyo dolabı plastik 38 bauhaus banyo dolabı lavabolu 10 bauhaus banyo dolabı modelleri ve fiyatları 9 bauhaus banyo dolabı 100 cm bauhaus banyo dolabı montajı 10 bauhaus banyo dolabı ve lavabo fiyatları 11 bauhaus banyo dolabı 60 cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="82" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Perakendeci</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>koçtaş klozet 2,3K</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>koçtaş klozet fiyatları 2,1K koçtaş klozet kapağı 1,0K koçtaş klozet kapağı fiyatları 325 koçtaş klozet takımı 284 koçtaş klozet fırçası 22 koçtaş klozet iç takımı 58 koçtaş klozet fırçası çöp kovası ikili set 82 koçtaş klozet modelleri 39 koçtaş klozet takımı fiyatları 75 koçtaş klozet kapağı menteşesi 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="82" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Perakendeci</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>trendyol banyo dolabı 1,3K</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>trendyol banyo dolabı fiyatları 540 trendyol banyo dolabı beyaz 561 trendyol banyo dolabı plastik 88 trendyol banyo dolabı modelleri 56 trendyol banyo dolabı takımı 10 trendyol banyo dolabı aynalı 8 trendyol banyo dolabı lavabolu 11 trendyol banyo dolabı düzenleyici trendyol banyo dolabı kirli sepetli trendyol banyo dolabı modelleri ve fiyatları</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="43" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Perakendeci</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>tekzen klozet 58</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>tekzen klozet fiyatları 415 tekzen klozet kapağı 42 tekzen klozet rezervuar 8 tekzen klozet modelleri 6 tekzen klozet takımı 26</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6991,12 +7726,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · Öneri temaları
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 11 , 12
+Kaynak: Google Autocomplete · 49 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
 Sütun açıklamaları: Öneri teması: Önerinin ifade kalıbına göre sınıfı. | Öneri: 49 kök ifadeden dönen toplam öneri sayısı. | Pay: Toplam öneri içindeki pay.</t>
         </is>
       </c>
@@ -7155,12 +7890,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118" customHeight="1">
+    <row r="2" ht="132" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka Aramaları ve Autocomplete · En çok tık getiren sorgular · Search Console
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 49 kök ifade için Türkiye, Türkçe, masaüstü Chrome sonuçları alınmıştır.
-Kaynak: Google Autocomplete · 49 kök ifade · Türkiye, Türkçe, masaüstü Chrome · 28.09.2026 · Google Search Console sorgu raporu 11 , 12
+Kaynak: Google Autocomplete · 49 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
 Sütun açıklamaları: Sorgu: Kullanıcının Google'a yazdığı ifade. | Tık: 1 Haz 2025 - 25 Eyl 2026. | Gösterim: Aynı dönem. | CTR: Tık / gösterim. | Sıra: Ortalama sıra.</t>
         </is>
       </c>
@@ -7607,12 +8342,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · Kim sıralanıyor?
 Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir; 19 kelimede ilk çekim eksik sonuç döndürdüğü için bu kelimeler yeniden çekilmiştir.
-Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · hacim Keyword Planner 10 , 13
+Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr gizli sekme kontrolü, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
 Sütun açıklamaları: Alan adı: Google TR mobil ilk 10 organik sonuçta görünen alan adı. | İlk 10 (kelime): 109 kelimeden kaçında ilk 10'da. | İlk 3 (kelime): Kaç kelimede ilk 3'te. | Ort. sıra: Görüldüğü kelimelerdeki en iyi sıranın ortalaması. | SSG / BM / Armatür / Bitişik: Tema bazında ilk 10'da görüldüğü kelime sayısı (tema büyüklükleri 16 / 15 / 13 / 24).</t>
         </is>
       </c>
@@ -7977,14 +8712,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -7994,19 +8730,20 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · VitrA nerede?
 Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir; 19 kelimede ilk çekim eksik sonuç döndürdüğü için bu kelimeler yeniden çekilmiştir.
-Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · hacim Keyword Planner 10 , 13
-Sütun açıklamaları: Tema: Kelime grubu. | Kelime: Temadaki kelime sayısı. | VitrA ilk 3: vitra.com.tr'nin ilk 3'te olduğu kelime sayısı. | VitrA ilk 10: İlk 10'da olduğu kelime sayısı. | İlk 20'de yok: vitra.com.tr'nin ilk 20'de görünmediği kelime sayısı.</t>
+Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr gizli sekme kontrolü, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Sütun açıklamaları: Tema: Kelime grubu; ok simgesi temadaki kelimeleri ve metriklerini açar. | Kelime: Temadaki kelime sayısı. | VitrA ilk 3 (SERP): 29.09.2026 mobil gözlemde vitra.com.tr'nin ilk 3'te olduğu kelime sayısı. | VitrA ilk 10 (SERP): Aynı gözlemde ilk 10'da olduğu kelime sayısı. | VitrA ilk 10 (Search Console): Search Console'da 26.06 - 25.09.2026 ortalama sırası 10 ve altında olan kelime sayısı; tüm cihazlar. | SERP'te ilk 20'de yok: Tek günlük gözlemde vitra.com.tr'nin ilk 20'de görünmediği kelime sayısı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -8021,24 +8758,29 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>VitrA ilk 3</t>
+          <t>VitrA ilk 3 (SERP)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>VitrA ilk 10</t>
+          <t>VitrA ilk 10 (SERP)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>İlk 20'de yok</t>
+          <t>VitrA ilk 10 (Search Console)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>SERP'te ilk 20'de yok</t>
         </is>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>SSG</t>
+          <t>SSG ↗</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
@@ -8051,13 +8793,16 @@
         <v>14</v>
       </c>
       <c r="E5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>BM ↗</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -8070,13 +8815,16 @@
         <v>11</v>
       </c>
       <c r="E6" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Armatür ve duş</t>
+          <t>Armatür ve duş ↗</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
@@ -8089,13 +8837,16 @@
         <v>5</v>
       </c>
       <c r="E7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Yıkanma</t>
+          <t>Yıkanma ↗</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -8108,13 +8859,16 @@
         <v>5</v>
       </c>
       <c r="E8" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Bitişik ürünler</t>
+          <t>Bitişik ürünler ↗</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -8127,13 +8881,16 @@
         <v>3</v>
       </c>
       <c r="E9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="6" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Hizmet ve ilham</t>
+          <t>Hizmet ve ilham ↗</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -8148,11 +8905,14 @@
       <c r="E10" s="6" t="n">
         <v>10</v>
       </c>
+      <c r="F10" s="6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Karo</t>
+          <t>Karo ↗</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -8165,13 +8925,16 @@
         <v>3</v>
       </c>
       <c r="E11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Soru ve karar</t>
+          <t>Soru ve karar ↗</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -8184,13 +8947,16 @@
         <v>5</v>
       </c>
       <c r="E12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Marka</t>
+          <t>Marka ↗</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
@@ -8205,10 +8971,13 @@
       <c r="E13" s="6" t="n">
         <v>5</v>
       </c>
+      <c r="F13" s="6" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8220,32 +8989,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Google Arama Sonuçları ve AI Overview · VitrA'nın görünmediği yüksek hacimli kelimeler</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="118" customHeight="1">
+          <t>Google Arama Sonuçları ve AI Overview · Yüksek hacimli kelimelerde VitrA'nın yeri: SERP, Search Console ve Google kontrolü</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="202" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Google Arama Sonuçları ve AI Overview · VitrA'nın görünmediği yüksek hacimli kelimeler
+          <t>Bölüm: Google Arama Sonuçları ve AI Overview · Yüksek hacimli kelimelerde VitrA'nın yeri: SERP, Search Console ve Google kontrolü
 Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir; 19 kelimede ilk çekim eksik sonuç döndürdüğü için bu kelimeler yeniden çekilmiştir.
-Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · hacim Keyword Planner 10 , 13
-Sütun açıklamaları: Arama kelimesi: vitra.com.tr'nin ilk 20'de görünmediği kelime. | Aylık hacim: Keyword Planner 12 aylık ortalama. | SERP lideri: Organik 1. sıradaki alan adı.</t>
+Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr gizli sekme kontrolü, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Sütun açıklamaları: Arama kelimesi: 29.09.2026 mobil SERP gözleminde vitra.com.tr'nin ilk 20'de görünmediği kelime. | Aylık hacim: Keyword Planner 12 aylık ortalama. | Search Console ort. sıra: vitra.com.tr'nin 26.06 - 25.09.2026 ortalama sırası, tüm cihazlar; "-" gösterim yok. | Search Console tık: Aynı dönemde bu kelimeden gelen tık. | Google sırası (30.09): google.com.tr, gizli sekme, oturumsuz, 30.09.2026; ilk sayfadaki organik sonuçlar arasında vitra.com.tr'nin sırası; "-" ilk sayfada yok. | İlk 5 alan adı (30.09): Aynı Google kontrolünde ilk beş organik sonucun alan adı. | Durum: VitrA'nın 30.09.2026 Google ilk sayfasındaki varlığı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -8260,11 +9037,31 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>SERP lideri</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
+          <t>Search Console ort. sıra</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Search Console tık</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Google sırası (30.09)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>İlk 5 alan adı (30.09)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>su arıtma cihazı</t>
@@ -8275,11 +9072,29 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>aquabella.com.tr · sumosuaritma.com · trendyol.com · rainwater.com.tr · eksisozluk.com</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>termosifon</t>
@@ -8288,13 +9103,29 @@
       <c r="B6" s="6" t="n">
         <v>61500</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
+      <c r="C6" s="8" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · sahibinden.com · arcelik.com.tr · hepsiburada.com</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>banyo bataryası</t>
@@ -8303,13 +9134,27 @@
       <c r="B7" s="6" t="n">
         <v>39267</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
+      <c r="C7" s="8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1148</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · vitra.com.tr · hepsiburada.com · banyomarka.com</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>taharet musluğu</t>
@@ -8318,13 +9163,29 @@
       <c r="B8" s="6" t="n">
         <v>37417</v>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>akakce.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
+      <c r="C8" s="8" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · hepsiburada.com · eca.com.tr · akakce.com · koctas.com.tr</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>tesisatçı</t>
@@ -8333,13 +9194,29 @@
       <c r="B9" s="6" t="n">
         <v>36800</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>armut.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
+      <c r="C9" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>armut.com · ozyurttesisat.com · tr.wikipedia.org · kariyer.net · eksisozluk.com</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>şofben</t>
@@ -8350,11 +9227,29 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · akakce.com · hepsiburada.com · donanimhaber.com</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>jakuzi</t>
@@ -8363,13 +9258,27 @@
       <c r="B11" s="6" t="n">
         <v>28967</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>jakuzicenter.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
+      <c r="C11" s="8" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>313</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>jakuzicenter.com · trendyol.com · atlasjakuzi.com · sahibinden.com · vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>banyo paspası</t>
@@ -8380,11 +9289,29 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · irya.com · lcw.com · chakra.com.tr · boyner.com.tr</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>dolap kulpu</t>
@@ -8393,13 +9320,29 @@
       <c r="B13" s="6" t="n">
         <v>24242</v>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
+      <c r="C13" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · evnepa.com · koctas.com.tr · hepsiburada.com · bellamaison.com</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>mutfak tezgahı</t>
@@ -8408,13 +9351,29 @@
       <c r="B14" s="6" t="n">
         <v>24242</v>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>koctas.com.tr</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
+      <c r="C14" s="8" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>koctas.com.tr · trendyol.com · kale.com.tr · ikea.com.tr · lnyapi.com</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>lavabo bataryası</t>
@@ -8423,13 +9382,27 @@
       <c r="B15" s="6" t="n">
         <v>23833</v>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
+      <c r="C15" s="8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>736</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · vitra.com.tr · shop.creavit.com.tr · hepsiburada.com</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>fayans fiyatları</t>
@@ -8438,13 +9411,29 @@
       <c r="B16" s="6" t="n">
         <v>23425</v>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>koctas.com.tr</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1">
+      <c r="C16" s="8" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>koctas.com.tr · trendyol.com · sahibinden.com · toptanseramik.net · yerevdekor.com</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>banyo seti</t>
@@ -8453,13 +9442,29 @@
       <c r="B17" s="6" t="n">
         <v>23017</v>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="17" customHeight="1">
+      <c r="C17" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>121</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · primanova.com.tr · linens.com.tr · shop.okyanushome.com · madamecoco.com</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>çamaşır sepeti</t>
@@ -8470,11 +9475,29 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · hepsiburada.com · sese.com.tr · englishhome.com</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>evye</t>
@@ -8483,13 +9506,27 @@
       <c r="B19" s="6" t="n">
         <v>18783</v>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1">
+      <c r="C19" s="8" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>238</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · ankastredunyasi.com · koctas.com.tr · schnelle.com.tr · ankastresepetim.com</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>havlupan</t>
@@ -8498,13 +9535,29 @@
       <c r="B20" s="6" t="n">
         <v>16642</v>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="17" customHeight="1">
+      <c r="C20" s="8" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>181</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · hammamonline.com · hepsiburada.com · koctas.com.tr · eca.com.tr</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>derz dolgu</t>
@@ -8515,11 +9568,29 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="17" customHeight="1">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · koctas.com.tr · kalekim.com · banyome.com · tr.weber</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>banyo rafı</t>
@@ -8528,13 +9599,29 @@
       <c r="B22" s="6" t="n">
         <v>10708</v>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="17" customHeight="1">
+      <c r="C22" s="8" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · ikea.com.tr · koctas.com.tr · hepsiburada.com · amazon.com.tr</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>gömme rezervuar iç takımı</t>
@@ -8543,13 +9630,29 @@
       <c r="B23" s="6" t="n">
         <v>4650</v>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>akakce.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="17" customHeight="1">
+      <c r="C23" s="8" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>hepsiburada.com · trendyol.com · koctas.com.tr · banyoline.com · bauhaus.com.tr</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>granit evye</t>
@@ -8558,13 +9661,29 @@
       <c r="B24" s="6" t="n">
         <v>4667</v>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>ankastredunyasi.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="17" customHeight="1">
+      <c r="C24" s="8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>ankastredunyasi.com · acarlaronline.net · hepsiburada.com · trendyol.com · teka.com</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>klozet kapağı menteşesi</t>
@@ -8573,13 +9692,29 @@
       <c r="B25" s="6" t="n">
         <v>4483</v>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17" customHeight="1">
+      <c r="C25" s="8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>hepsiburada.com · vimaryapi.com.tr · trendyol.com · kombitesisatmarket.com · cimri.com</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>geberit gömme rezervuar</t>
@@ -8588,13 +9723,29 @@
       <c r="B26" s="6" t="n">
         <v>3933</v>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>trendyol.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="17" customHeight="1">
+      <c r="C26" s="8" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>geberit.com.tr · trendyol.com · banyomarka.com · koctas.com.tr · akakce.com</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>creavit klozet</t>
@@ -8603,13 +9754,29 @@
       <c r="B27" s="6" t="n">
         <v>3800</v>
       </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>creavit.com.tr</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="17" customHeight="1">
+      <c r="C27" s="8" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>shop.creavit.com.tr · trendyol.com · creavit.com.tr · koctas.com.tr · sikayetvar.com</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>kanalsız klozet</t>
@@ -8618,15 +9785,29 @@
       <c r="B28" s="6" t="n">
         <v>2025</v>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>bauhaus.com.tr</t>
+      <c r="C28" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>trendyol.com · shop.creavit.com.tr · hepsiburada.com · vitra.com.tr · koctas.com.tr</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>İlk sayfada</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8654,12 +9835,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="132" customHeight="1">
+    <row r="2" ht="146" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · SERP özellikleri ve AI Overview
 Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir; 19 kelimede ilk çekim eksik sonuç döndürdüğü için bu kelimeler yeniden çekilmiştir.
-Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · hacim Keyword Planner 10 , 13
+Kaynak: Google TR mobil SERP · DataForSEO · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr gizli sekme kontrolü, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
 Sütun açıklamaları: SERP özelliği: Arama sonuç sayfasında organik sonuç dışındaki blok. | Kelime (pay): 109 kelimeden kaçında görüldüğü. | SSG / BM / Armatür / Bitişik: Tema bazında görüldüğü kelime sayısı. | En yoğun olduğu temalar: En yüksek görülme oranı.</t>
         </is>
       </c>
@@ -17690,13 +18871,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Kategori baş kelimeleri: hacim, potansiyel ve VitrA sırası
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
 Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil SERP (DataForSEO, 29.09.2026) 13 , 31
-Sütun açıklamaları: Baş kelime: Kategori baş kelimesi. | Aylık hacim: Ahrefs Keywords Explorer, Türkiye. | Trafik potansiyeli: Bu kelimede 1. sıradaki sayfanın tüm kelimelerinden aldığı tahmini aylık trafik (Ahrefs TP). | VitrA sırası: Google TR mobil SERP, 29.09.2026; "-" ilk 20'de yok.</t>
+Sütun açıklamaları: Baş kelime: Kategori baş kelimesi. | Aylık hacim: Ahrefs Keywords Explorer, Türkiye. | Trafik potansiyeli: Bu kelimede 1. sıradaki sayfanın tüm kelimelerinden aldığı tahmini aylık trafik (Ahrefs TP). | VitrA sırası: Google TR mobil SERP, 29.09.2026; "-" ilk 20'de yok. * Tek günlük ölçümde ilk 20 dışında görünen, 30.09.2026 google.com.tr gizli sekme kontrolünde ve Search Console'da (ort. 4,2) 3. sırada olan kelime.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -17869,7 +19050,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3*</t>
         </is>
       </c>
     </row>
@@ -18475,7 +19656,7 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -18490,13 +19671,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Ana kategori düzeyinde değişim
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
-Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
-Sütun açıklamaları: Kategori: VitrA kategori ağacındaki ana kategori; 2.420 kelime 8 ana kategoriye dağıtılmıştır. | Kelime: Kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi (kategorideki kelimelerin toplamı, aya bölünmüş), Google Keyword Planner, Türkiye. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi; aynı takvim aylarını kapsar. | YoY: İki pencere arasındaki yüzde değişim; mevsimsellikten arındırılmıştır. | Pay: Kategorinin 2026 penceresindeki toplam hacim içindeki payı.</t>
+Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Oca 2023 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
+Sütun açıklamaları: Kategori: VitrA kategori ağacındaki ana kategori; 2.420 kelime 8 ana kategoriye dağıtılmıştır. Ok simgesi kategorideki en yüksek hacimli 50 kelimeyi açar. | Kelime: Kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi (kategorideki kelimelerin toplamı, aya bölünmüş), Google Keyword Planner, Türkiye. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi; aynı takvim aylarını kapsar. | YoY: İki pencere arasındaki yüzde değişim; mevsimsellikten arındırılmıştır. | Pay: Kategorinin 2026 penceresindeki toplam hacim içindeki payı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -18540,7 +19721,7 @@
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Banyo Mobilyaları</t>
+          <t>Banyo Mobilyaları ↗</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
@@ -18562,7 +19743,7 @@
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Vitrifiyeler</t>
+          <t>Vitrifiyeler ↗</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -18584,7 +19765,7 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Armatürler</t>
+          <t>Armatürler ↗</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
@@ -18606,7 +19787,7 @@
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Yıkanma Alanları</t>
+          <t>Yıkanma Alanları ↗</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -18628,7 +19809,7 @@
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Karo Seramik Ürünleri</t>
+          <t>Karo Seramik Ürünleri ↗</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -18650,7 +19831,7 @@
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Banyo Aksesuarları</t>
+          <t>Banyo Aksesuarları ↗</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -18672,7 +19853,7 @@
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Duşlar</t>
+          <t>Duşlar ↗</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -18694,7 +19875,7 @@
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Rezervuarlar</t>
+          <t>Rezervuarlar ↗</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -24006,7 +25187,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -24025,7 +25206,7 @@
         <is>
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Büyüyen alt kategoriler
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
-Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
+Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Oca 2023 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
 Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
         </is>
       </c>
@@ -24075,7 +25256,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Balkon, Teras &amp; Bahçe Karo Seramikleri</t>
+          <t>Balkon, Teras &amp; Bahçe Karo Seramikleri ↗</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -24099,7 +25280,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Duşlar</t>
+          <t>Duşlar ↗</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -24123,7 +25304,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Banyo Karo Seramikleri</t>
+          <t>Banyo Karo Seramikleri ↗</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -24147,7 +25328,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Ankastre Duş Yönlendiriciler</t>
+          <t>Ankastre Duş Yönlendiriciler ↗</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -24171,7 +25352,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Banyo Mobilyaları</t>
+          <t>Banyo Mobilyaları ↗</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -24195,7 +25376,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Klozetler</t>
+          <t>Klozetler ↗</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -24219,7 +25400,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Banyo Tezgahları</t>
+          <t>Banyo Tezgahları ↗</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -24243,7 +25424,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Duş Kanalları</t>
+          <t>Duş Kanalları ↗</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -24267,7 +25448,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Duş Tekneleri</t>
+          <t>Duş Tekneleri ↗</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -24291,7 +25472,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Armatür Tamamlayıcı Ürünleri</t>
+          <t>Armatür Tamamlayıcı Ürünleri ↗</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -24315,7 +25496,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Tuvalet Fırçaları</t>
+          <t>Tuvalet Fırçaları ↗</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -24339,7 +25520,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Duvar Karoları</t>
+          <t>Duvar Karoları ↗</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -34871,7 +36052,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -34890,7 +36071,7 @@
         <is>
           <t>Bölüm: Kategori Talebi ve Dönemsel Değişim · Daralan alt kategoriler
 Kapsam: Talep tabanı, VitrA kategori ağacına eşlenmiş 2.420 arama kelimesidir; hacimler Google Keyword Planner'dan Eylül 2024 - Ağustos 2026 dönemi için aylık olarak alınmıştır. Karşılaştırma, aynı takvim aylarını kapsayan Ocak - Ağustos pencereleri üzerinden yapılmaktadır.
-Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Eyl 2024 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
+Kaynak: Google Ads Keyword Planner · Türkiye, Türkçe · 2.420 kelime · aylık hacim Oca 2023 - Ağu 2026 · kategori eşlemesi Inbound kelime araştırması (2025) 7 , 8
 Sütun açıklamaları: Ana kategori: Alt kategorinin bağlı olduğu ana kategori. | Alt kategori: VitrA kategori ağacındaki alt kategori. | Kelime: Alt kategoriye atanan kelime sayısı. | 2025 aylık ort.: Ocak - Ağustos 2025 aylık ortalama arama hacmi. | 2026 aylık ort.: Ocak - Ağustos 2026 aylık ortalama arama hacmi. | YoY: İki pencere arasındaki yüzde değişim. Tabloya aylık 3.000 ve üzeri hacimli alt kategoriler alınmıştır.</t>
         </is>
       </c>
@@ -34940,7 +36121,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Lavabo Dolapları</t>
+          <t>Lavabo Dolapları ↗</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -34964,7 +36145,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Banyo Aksesuar Setleri</t>
+          <t>Banyo Aksesuar Setleri ↗</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -34988,7 +36169,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Bideler</t>
+          <t>Bideler ↗</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -35012,7 +36193,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Banyo Aynaları</t>
+          <t>Banyo Aynaları ↗</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -35036,7 +36217,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Banyo Aksesuarları</t>
+          <t>Banyo Aksesuarları ↗</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -35060,7 +36241,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Banyo Set Modülleri</t>
+          <t>Banyo Set Modülleri ↗</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -35084,7 +36265,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Tuvalet Kağıtlıkları</t>
+          <t>Tuvalet Kağıtlıkları ↗</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -35108,7 +36289,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Banyo Mobilya Tamamlayıcıları</t>
+          <t>Banyo Mobilya Tamamlayıcıları ↗</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -35132,7 +36313,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Duş Başlıkları</t>
+          <t>Duş Başlıkları ↗</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -35156,7 +36337,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Duş Tamamlayıcı Ürünleri</t>
+          <t>Duş Tamamlayıcı Ürünleri ↗</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -35180,7 +36361,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Banyo Dolapları</t>
+          <t>Banyo Dolapları ↗</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -35204,7 +36385,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Duş Setleri</t>
+          <t>Duş Setleri ↗</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">

</xml_diff>

<commit_message>
GEO bölümü fırsat odaklı sadeleştirildi; ayrıntılı plan rapordan çıkarıldı
- Bölüm adı: AI Arama ve GEO Fırsatları
- Durum grafiği + altı fırsat kartı; soru sorguları açılır tabloda
- Sonraki Adımlar'da GEO maddeleri 3 genel maddeye indirildi; Özet maddesi fırsat diliyle

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -109,13 +109,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100 Kanal rolleri" sheetId="100" state="visible" r:id="rId100"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="101 Hacimli ve ölçüye bağlı" sheetId="101" state="visible" r:id="rId101"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="102 Tamamlayıcı ürün kurgusu" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="103 Rehber içerik hangi" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="104 Soru sorgularında sıra ve" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="105 AI Overview odaklı içerik" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="106 Marka ve entity" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="107 Sonraki Adımlar" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="108 Yöntem ve Kapsam" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="103 Sonraki Adımlar" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="104 Yöntem ve Kapsam" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="105" state="visible" r:id="rId105"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1918,1282 +1914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="47" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Rehber içerik: hangi konular trafik alıyor?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="216" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Rehber içerik: hangi konular trafik alıyor?
-Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek üç unsura bağlıdır: soruyu doğrudan cevaplayan sayfa, markanın ansiklopedik kayıtlarda tutarlı tanımlanması ve markadan site dışında söz edilmesi. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli Wikidata ve Wikipedia kayıtlarına dayanmaktadır.
-Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 109 kelime, 29.09.2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 39 , 50 , 51 , 52
-Sütun açıklamaları: İçerik grubu: Sayfa adresindeki konuya göre yapılan gruplama. | Sayfa: Dönemde en az 5 tık alan sayfa sayısı. | Tık: 1 Eki 2025 - 25 Eyl 2026 organik tık. | Tık payı: Rehber içeriklerin toplam tıkı içindeki pay. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim. | En çok tık alan sayfa: Grubun en çok tık alan sayfası; bağlantı canlı sayfayı açar.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>İçerik grubu</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Sayfa</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Tık</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Tık payı</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Gösterim</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>CTR</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>En çok tık alan sayfa</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Tamir, temizlik ve bakım</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>16906</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>1411680</v>
-      </c>
-      <c r="F5" s="9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Dusakabin temizligi nasil yapilir (8.623)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Montaj ve kurulum</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>11433</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>1283613</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Gomme rezervuar montaji nasil yapilir (2.497)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Seçim, ölçü ve "nedir" rehberleri</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>31087</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>2233198</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>En kullanisli evye hangisi (12.719)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Planlama ve tadilat</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>1788</v>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>104439</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Banyo tadilatina nereden baslamali (772)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Dekorasyon, trend ve karo modelleri</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>17953</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>22.3</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>1477719</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Ahsap gorunumlu seramik modelleri (5.765)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Sürdürülebilirlik ve kurumsal</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>1209</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>123615</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Herkes icin tasarim (694)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Soru sorgularında sıra ve tık</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="188" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Soru sorgularında sıra ve tık
-Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek üç unsura bağlıdır: soruyu doğrudan cevaplayan sayfa, markanın ansiklopedik kayıtlarda tutarlı tanımlanması ve markadan site dışında söz edilmesi. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli Wikidata ve Wikipedia kayıtlarına dayanmaktadır.
-Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 109 kelime, 29.09.2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 39 , 50 , 51 , 52
-Sütun açıklamaları: Sorgu: Search Console'da vitra.com.tr'nin gösterim aldığı soru biçimli sorgu; "nasıl" ve "su kaçır" içeren sorgulardan gösterime göre seçilmiştir. | Gösterim: 1 Eki 2025 - 25 Eyl 2026 gösterim. | Tık: Aynı dönemde tık. | CTR: Tık / gösterim. | Ort. sıra: Gösterim ağırlıklı ortalama sıra, tüm cihazlar.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Sorgu</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Gösterim</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Tık</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>CTR</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Ort. sıra</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>42119</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>197</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>4.8</v>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>gömme klozet su kaçırıyorsa çok basit tamiri</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>32934</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>410</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin nasıl temizlenir</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>17275</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>445</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>2.58</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>amortisörlü klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>10004</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>4.9</v>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>gömme rezervuar su kaçırıyor</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>9302</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>üstten vidalı klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>9188</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>eski tip klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>7667</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>tezgah üstü musluk nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>6838</v>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>51</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>basmalı rezervuar iç takımı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>6302</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>banyo batarya contası nasıl değiştirilir</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>6291</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin kireci nasıl temizlenir</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>5919</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>54</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin montajı nasıl yapılır</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>5855</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>68</v>
-      </c>
-      <c r="D16" s="9" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>4.3</v>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>bide nasıl kullanılır</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>5828</v>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>103</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>yavaş kapanan klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>5428</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="D18" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>4.8</v>
-      </c>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>banyo bataryası nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>5274</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>46</v>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>klozet su kaçırıyorsa çok basit tamiri</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>5225</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>lavabo bataryası nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>4366</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>5.7</v>
-      </c>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>klozet kapağı nasıl değiştirilir</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>4353</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="D22" s="9" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>duş başlığı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>3545</v>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="D23" s="9" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>gömme rezervuar montajı nasıl yapılır</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n">
-        <v>3051</v>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>vitra rezervuar iç takımı montajı nasıl yapılır</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>2822</v>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>63</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="E25" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet105.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · AI Overview odaklı içerik planı: destek sayfaları ve rehber içerik</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="216" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · AI Overview odaklı içerik planı: destek sayfaları ve rehber içerik
-Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek üç unsura bağlıdır: soruyu doğrudan cevaplayan sayfa, markanın ansiklopedik kayıtlarda tutarlı tanımlanması ve markadan site dışında söz edilmesi. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli Wikidata ve Wikipedia kayıtlarına dayanmaktadır.
-Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 109 kelime, 29.09.2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 39 , 50 , 51 , 52
-Sütun açıklamaları: Öncelik: Talep, mevcut görünürlük ve satış sonrası etkisi birlikte değerlendirilerek verilen sıra. | Konu kümesi: Aynı ihtiyacı karşılayan soru grubu. | Sayfa tipi: Konunun karşılanacağı sayfa: destek sayfası, rehber yazı ya da kategori sayfasında soru-cevap. | Kullanıcı soruları: PAA kutusu, Search Console ve Autocomplete'ten örnek sorular; kullanıcının yazdığı biçimde. | Dayanak: Konuyu öne çıkaran bulgu.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Öncelik</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Konu kümesi</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Sayfa tipi</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Kullanıcı soruları</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Dayanak</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="69" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Gömme rezervuar ve iç takım arızaları: su kaçırma, su doldurmama, iç takım, şamandıra ve kumanda paneli değişimi</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Destek sayfası; model ve rezervuar tipine göre alt başlıklar</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>VitrA gömme rezervuar neden su doldurmuyor? Klozet iç takım değişimi ne kadar? basmalı rezervuar iç takımı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>"gömme klozet su kaçırıyorsa çok basit tamiri" 32,9K gösterim, CTR %1,2; sitedeki tek tamir yazısı 6.653 tık, 615K gösterim; "gömme rezervuar iç takımı" AI Overview'unda kaynaklar trendyol.com, youtube.com, koctas.com.tr, bauhaus.com.tr, VitrA yok 13 , 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Klozet kapağı montajı ve uyumluluk: kapak tipine göre montaj, hangi kapak hangi klozete uyar</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Destek sayfası; ürün sayfalarında klozet koduna göre uyumlu kapak tablosu</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Klozet kapakları standart mı? amortisörlü klozet kapağı nasıl takılır eski tip klozet kapağı nasıl takılır</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Kapak montajı soran 6 sorgu toplam 78,8K gösterim, 390 tık (CTR %0,50); ortalama sıra 4,8-5,9 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="43" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Batarya bakımı ve parça değişimi: conta, kartuş, kireç, damlatma ve montaj</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Destek sayfası; armatür ürün sayfalarından bağlantı</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>banyo batarya contası nasıl değiştirilir tezgah üstü musluk nasıl takılır lavabo bataryası nasıl takılır</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Conta değişimi 6,3K, tezgah üstü musluk montajı 6,8K gösterim; YouTube'da batarya ve kartuş konuları 7,0M izlenme ve VitrA kanal videosu yok 16 , 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Ölçü ve yerleşim: klozet, lavabo, banyo dolabı ve duşakabin ölçüleri, montaj yükseklikleri</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Rehber yazı; kategori sayfalarında kısa soru-cevap</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Klozet duvardan kaç cm uzakta olmalı? Banyo dolabı yüksekliği kaç santim olmalı? 80'lik banyo dolabının ölçüleri nedir?</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>"klozet ölçüleri" AI Overview'unda VitrA kaynak gösterilmektedir; "80 cm banyo dolabı" AI Overview'unda kaynaklar koctas.com.tr, banyomega.com, trendyol.com, hepsiburada.com, VitrA yok 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Seçim karşılaştırmaları: gömme mi dış rezervuar mı, kanallı mı kanalsız mı, suya dayanıklı dolap malzemesi</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Rehber yazı; karşılaştırma tablosuyla</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Gömme rezervuar mantıklı mı? Kanallı klozet mi iyi kanalsız mı? MDF banyo dolabı suya dayanıklı mı?</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>"gömme rezervuar mı dış rezervuar mı" AI Overview'unda kaynaklar youtube.com, instagram.com, banyome.com, facebook.com; VitrA bu sorguda 14. sırada. "suya dayanıklı banyo dolabı" AI Overview'unda kaynaklar Trendyol ve Instagram 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Marka soruları: VitrA ve Artema ilişkisi, menşei, kalite ve garanti</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Kurumsal soru-cevap sayfası; Wikidata ve Wikipedia güncellemeleriyle birlikte</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>VitrA ve Artema aynı marka mı? Artema hangi ülkenin markası? VitrA iyi marka mı?</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Bu sorular PAA kutusunda çıkmaktadır; Artema'nın Wikidata ve Wikipedia kaydı bulunmamaktadır 13 , 51</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="43" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Yedek parça, garanti ve servis: parça bulma, garanti süresi, servis ücreti ve başvuru adımları</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Destek sayfası; ürün sayfalarından ve yedek parça kategorisinden bağlantı</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>vitra servis vitra yedek parça Klozet değişimini kim yapar?</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça teması %17,8 (Nis - Eyl 2026); ürün sayfalarında garanti süresi bulunmamaktadır 17 , 19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="43" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Montaj ücreti ve işçilik: ürün bazında montaj kapsamı ve fiyatı</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Montaj hizmeti sayfasında soru-cevap bölümü</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Klozet montajı kaç TL? Klozet yaptırmak kaç TL? Bir banyo tadilatı ne kadara mal olur?</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>"klozet montaj ücreti" AI Overview'unda kaynaklar gigbi.com, hepsiburada.com, armut.com; VitrA'da 11 fiyatlı montaj kalemi bulunmaktadır 13 , 19</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="43" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Temizlik ve bakım: duşakabin, klozet ve batarya temizliği, kireç</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Mevcut yazıların soru-cevap bölümüyle güncellenmesi; ürün sayfalarına bakım bağlantısı</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>duşakabin kireci nasıl temizlenir Klozet nasıl temizlenir? duşakabin camı nasıl temizlenir</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Duşakabin temizliği yazısı 8.623 tık ile ikinci en çok tık alan rehber içeriktir; "duşakabin kireci nasıl temizlenir" 5,9K gösterim, sıra 6,2 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="43" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Erişilebilir ve çocuk banyosu: engelli klozeti ölçüleri, tutunma barları, çocuk klozeti</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Rehber yazı; erişilebilir banyo kategori sayfasıyla birlikte</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Engelli klozetinin farkı nedir? Engelli tuvaletinin ölçüleri nelerdir? Klozet adaptörü ne işe yarar?</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>"engelli klozet" AI Overview'unda kaynaklar banyomarka.com, hepsiburada.com, creavit.com.tr, eca.com.tr, turkuazseramik.com.tr; VitrA yok 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="43" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Alt kategori açılımı: sayfası olmayan ya da farklı adla duran kesitler</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Kategori sayfası ve kısa soru-cevap</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>sıva üstü banyo bataryası fotoselli batarya jakuzi ayaklı lavabo</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryerlerinde ayrı kategori olarak aranan bu kesitlerin vitra.com.tr'de karşılık gelen sayfası bulunmamakta ya da farklı adla durmaktadır 35 , 36</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="43" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Ürün tanımları ve bitişik ürünler: "nedir" yazılarının güncellenmesi, havlupan ve ısıtmalı kapak rehberleri</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Mevcut yazıların güncellenmesi; yeni rehber yazı</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Pisuvar nedir? Şamandıra nedir ne işe yarar? Elektrikli havlupan banyoyu ısıtır mı?</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Bide nedir yazısı 3.200 tık; "pisuvar" AI Overview'unda VitrA kaynak gösterilmektedir; "şamandıra" ve "elektrikli havlupan" AI Overview'larında VitrA yok 13 , 50</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:E2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet106.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Marka ve entity tutarlılığı: Wikidata ve Wikipedia</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="202" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Bölüm: AI Aramada Görünürlük: İçerik, Entity ve Site Dışı Sinyaller · Marka ve entity tutarlılığı: Wikidata ve Wikipedia
-Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek üç unsura bağlıdır: soruyu doğrudan cevaplayan sayfa, markanın ansiklopedik kayıtlarda tutarlı tanımlanması ve markadan site dışında söz edilmesi. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli Wikidata ve Wikipedia kayıtlarına dayanmaktadır.
-Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 109 kelime, 29.09.2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 39 , 50 , 51 , 52
-Sütun açıklamaları: Kayıt: Markanın yapay zeka modelleri ve arama motorlarınca okunan kaydı; bağlantı kaydı açar. | Mevcut durum (02.10.2026): Kaydın 2 Ekim 2026 tarihli durumu. | Önerilen güncelleme: Kaydı vitra.com.tr ve kurumsal bilgiyle tutarlı hale getirecek düzenleme.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Kayıt</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Mevcut durum (02.10.2026)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Önerilen güncelleme</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="56" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Wikidata · Q7937213</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Wikipedia maddelerine bağlı ana kayıt; resmi web sitesi alanında vitra.com.tr yerine ilgisiz bir alan adı kayıtlı; kuruluş yılı 1942; Instagram, YouTube, LinkedIn ve Facebook alanları boş; X hesabı iki yazımla</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Resmi web sitesinin vitra.com.tr olarak düzeltilmesi; sosyal hesap alanlarının eklenmesi; ürün grubu, üst kuruluş ve Artema ilişkisinin kaynakla girilmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Wikidata · Q127325081</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Aynı şirket için ikinci kayıt; web sitesi vitra.com.tr; Wikipedia bağlantısı yok</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>İki kaydın tek kayıtta birleştirilmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Wikipedia TR · VitrA</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Kısa madde (2.031 bayt); son düzenleme 17.12.2025; ürün grupları, Artema ve güncel üretim bilgisi yer almıyor</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Bağımsız yayınlara dayanan genişletme: ürün grupları, üretim, Artema ilişkisi, tasarım ödülleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Wikipedia EN · VitrA (sanitaryware)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>6.619 bayt; son düzenleme 31.08.2026</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Ürün gamı ve Artema bilgisinin güncel tutulması</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="43" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Artema</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Wikidata ve Wikipedia'da kayıt bulunmuyor; "Artema hangi ülkenin markası?" ve "VitrA ve Artema aynı marka mı?" soruları PAA kutusunda çıkıyor</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Wikidata kaydının açılması (üst kuruluş, web sitesi, ürün grubu); VitrA maddesinde Artema bölümü; sitede marka ilişkisini anlatan sayfa</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>vitra.com.tr · llms.txt</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Kurumsal metin "1958 yılında kurulan VitrA" ifadesini kullanıyor; Wikipedia ve Wikidata 1942'yi gösteriyor</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Kuruluş tarihi için tek anlatının belirlenmesi ve tüm kayıtlarda aynı biçimde yer alması</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet107.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3375,7 +2096,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="82" customHeight="1">
+    <row r="11" ht="56" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
@@ -3383,21 +2104,21 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Destek merkezi: gömme rezervuar ve iç takım arızaları, klozet kapağı montajı ve uyumluluğu, batarya bakımı, yedek parça, garanti ve servis sayfaları</t>
+          <t>AI aramada görünürlük için sorun çözen içerik: arıza, montaj, uyumluluk ve garanti konularında destek sayfaları; ölçü, seçim ve marka sorularında rehber içerik</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Destek bölümünde 5 sayfa var (SSS, ödeme, teslimat, işlem, değişim-iade); montaj, tamir ve temizlik yazıları rehber sayfalarının %17'sini oluşturup tıklarının %35'ini alıyor; "gömme klozet su kaçırıyorsa çok basit tamiri" 32,9K gösterim, kapak montajı soran 6 sorgu 78,8K gösterim ve CTR %0,50 17 , 50 , 52</t>
+          <t>Rehber sayfalarında tıkların %35'i montaj, tamir ve temizlik yazılarından geliyor; destek bölümünde bu konularda sayfa yok; soru sorgularında site ilk sayfada ama CTR %0,93; VitrA 24 AI Overview'un 7'sinde kaynak 13 , 17 , 50</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Tamir anında trafik, AI Overview'da kaynak gösterilme ve satış sonrası başvurunun siteye dönmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="56" customHeight="1">
+          <t>AI yanıtlarında kaynak gösterilme, tamir anında trafik ve satış sonrası başvurunun siteye dönmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="43" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Öncelik 1</t>
@@ -3405,17 +2126,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Wikidata kayıtlarının düzeltilmesi: iki VitrA kaydının birleştirilmesi, resmi web sitesinin vitra.com.tr olarak girilmesi, sosyal hesaplar ve kuruluş bilgisi; Artema için kayıt açılması</t>
+          <t>Marka ve entity tutarlılığı: Wikidata ve Wikipedia kayıtlarının VitrA ve Artema için güncel ve tutarlı hale getirilmesi</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Ana kayıtta (Q7937213) resmi web sitesi alanında ilgisiz bir alan adı kayıtlı; ikinci kayıt (Q127325081) ayrı duruyor; Artema'nın kaydı yok; kurumsal metin 1958, ansiklopedik kayıtlar 1942 kuruluş yılını gösteriyor 51 , 52</t>
+          <t>Wikidata'da iki ayrı VitrA kaydı var ve ana kayıtta resmi web sitesi vitra.com.tr'yi göstermiyor; Artema'nın kaydı yok 51</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Yapay zeka yanıtlarında markanın doğru ve tek kayıtla tanımlanması</t>
+          <t>AI yanıtlarında markanın doğru tanımlanması</t>
         </is>
       </c>
     </row>
@@ -3537,7 +2258,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Google Merchant Center feed'inin tüm kategorileri kapsaması, başlıklarda kategori kelimesi; ölçü, model kodu, uyumlu parça, garanti ve montaj bilgisi (AI alışveriş yanıtları için)</t>
+          <t>Google Merchant Center feed'inin tüm kategorileri kapsaması, başlıklarda kategori kelimesi; AI alışveriş yanıtları için zengin ürün bilgisi</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3683,7 +2404,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="82" customHeight="1">
+    <row r="25" ht="43" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
@@ -3691,21 +2412,21 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>AI Overview odaklı rehber içerik planı: ölçü ve yerleşim, seçim karşılaştırmaları, marka soruları, erişilebilir banyo, montaj ücreti; mevcut yüksek trafikli yazıların soru-cevap bölümüyle güncellenmesi; kategori ve ürün sayfalarında kısa soru-cevap blokları</t>
+          <t>Site dışı sinyaller: Şikayetvar yanıtları, YouTube tamir içerikleri ve rehber sitelerinde uzman içerik</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>VitrA 24 AI Overview'un 7'sinde kaynak; "80 cm banyo dolabı", "gömme rezervuar mı dış rezervuar mı", "engelli klozet" ve "klozet montaj ücreti" AI Overview'larında kaynaklar pazaryerleri, rakip markalar ve rehber siteleri; rakip rehberler tıkanıklık, koku, su kaçırma ve fayans hesabından trafik alıyor (Creavit 1.416, Kalekim 2.675) 13 , 31 , 50</t>
+          <t>Şikayetvar puanı 18; en çok izlenen 14 tamir ve kurulum konusunda VitrA kanal videosu yok; AI Overview kaynakları arasında markadan bağımsız rehber siteleri var 13 , 16 , 17</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Karar ve tamir sorularında kaynak gösterilme; organik trafikte konu çeşitliliği</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="56" customHeight="1">
+          <t>Markanın site dışında anılması ve AI yanıtlarında kaynak çeşitliliği</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="43" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Öncelik 2</t>
@@ -3713,87 +2434,87 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Wikipedia: Türkçe VitrA maddesinin bağımsız kaynaklarla genişletilmesi, Artema bölümü; düzenlemelerin tartışma sayfası üzerinden önerilmesi</t>
+          <t>Banyo Asistanı'nın bayi ağına genişletilmesi ve adımlarının GA4'te ölçülmesi</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Türkçe madde 2.031 bayt ve son düzenleme 17.12.2025; "VitrA ve Artema aynı marka mı?" ve "Artema hangi ülkenin markası?" PAA kutusunda çıkıyor; Wikipedia 4 AI Overview bloğunda kaynak 13 , 51</t>
+          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 1 Haziran 2025 - 25 Eylül 2026 döneminde 36.458 tık almıştır 11 , 19</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Marka sorularında tutarlı cevap</t>
+          <t>Lead'in satışa dönmesi</t>
         </is>
       </c>
     </row>
     <row r="27" ht="43" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Şikayetvar yanıt standardı: yedek parça, montaj ve garanti şikayetlerine standart yanıt ve ilgili destek sayfasına bağlantı, çözülen kayıtların kapatılması</t>
+          <t>Granit ve çelik evye + mutfak bataryası seti</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>VitrA puanı 18, son 1 yıl çözüm oranı %18; yedek parça teması %8,1'den %17,8'e, montaj ve usta %27,0'dan %48,5'e (Eki 2024 - Mar 2025 → Nis - Eyl 2026) 17</t>
+          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 9 , 10 , 21</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Marka güvenilirliği sorularında daha dengeli kaynak</t>
+          <t>Mutfakta set satışı</t>
         </is>
       </c>
     </row>
     <row r="28" ht="43" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Rehber ve topluluk sitelerinde uzman içerik ve konuk yazı: ölçü, seçim ve bakım konularında VitrA'nın kaynak olarak anılması</t>
+          <t>Arıtmalı batarya ve filtre aboneliği</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>AI Overview kaynakları arasında Banyome (5), Yapılır (4), Banyomega (3) ve Ekşi Sözlük (2) gibi markadan bağımsız siteler bulunuyor 13</t>
+          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 560K; Trendyol'da arıtmalı batarya aramasının ilk 40 sonucunda armatür markası bulunmamaktadır 9 , 10 , 21</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Site dışı anılma ve AI yanıtlarında kaynak çeşitliliği</t>
+          <t>Tekrarlı gelir</t>
         </is>
       </c>
     </row>
     <row r="29" ht="43" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Banyo Asistanı'nın bayi ağına genişletilmesi ve adımlarının GA4'te ölçülmesi</t>
+          <t>Banyo planlayıcının (V-Design) yeniden devreye alınması ve Banyo Asistanı'na bağlanması</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 1 Haziran 2025 - 25 Eylül 2026 döneminde 36.458 tık almıştır 11 , 19</t>
+          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 10 , 19 , 43 , 44</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Lead'in satışa dönmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="43" customHeight="1">
+          <t>Ürün keşfinden lead'e geçiş</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
@@ -3801,21 +2522,21 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Granit ve çelik evye + mutfak bataryası seti</t>
+          <t>Tamamlayıcı ürünlerde üçüncü taraf satıcı modelinin montaj malzemesi ve yapı kimyasalında test edilmesi</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 9 , 10 , 21</t>
+          <t>Yapıştırıcı, derz ve su yalıtımı aramaları YoY +%12,8 ; montaj parçaları yapı marketten tamamlanıyor 10 , 12</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Mutfakta set satışı</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="43" customHeight="1">
+          <t>Sepet bütünlüğü</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
@@ -3823,17 +2544,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Arıtmalı batarya ve filtre aboneliği</t>
+          <t>Ledli ayna, aydınlatma ve koleksiyon uyumlu havlupan derinliği</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 560K; Trendyol'da arıtmalı batarya aramasının ilk 40 sonucunda armatür markası bulunmamaktadır 9 , 10 , 21</t>
+          <t>Ledli ayna ve aydınlatma aramaları üç yılda +%13,1 ; Trendyol'da ledli ayna medyanı 1.650 TL 9 , 10</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Tekrarlı gelir</t>
+          <t>BM setine bağlı ek satış</t>
         </is>
       </c>
     </row>
@@ -3845,21 +2566,21 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Banyo planlayıcının (V-Design) yeniden devreye alınması ve Banyo Asistanı'na bağlanması</t>
+          <t>Yenileme paketinde iş ortağı ürünleri (şofben, termosifon, tekstil, düzenleme)</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>"banyo tasarım" aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 10 , 19 , 43 , 44</t>
+          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 10 , 22</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Ürün keşfinden lead'e geçiş</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="56" customHeight="1">
+          <t>Tadilat sepetinin tamamlanması</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
@@ -3867,21 +2588,21 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>llms.txt'nin destek, montaj, yedek parça, garanti ve Artema bölümleriyle genişletilmesi; rehber site haritasındaki şablon adreslerin temizlenmesi; sayfaların sade metin sürümlerinin altyapıyla birlikte değerlendirilmesi</t>
+          <t>V-Care için deneyim modeli ve universal akıllı kapağın izlenmesi</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>llms.txt'deki 83 bağlantının 3'ü rehber içeriğe, 1'i destek sayfasına gidiyor; sitemap-ilham.xml'de 2 doldurulmamış şablon adresi ve 1 tekrar 52</t>
+          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 7 , 47</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Yapay zeka araçlarının destek ve rehber içeriğe ulaşması</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
+          <t>Premium segmentte dönüşüm</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="43" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
@@ -3889,21 +2610,21 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Tamamlayıcı ürünlerde üçüncü taraf satıcı modelinin montaj malzemesi ve yapı kimyasalında test edilmesi</t>
+          <t>Satın alan müşteriye ürün ömrüne göre yenileme ve yedek parça hatırlatması; olumsuz deneyim sonrası tekrar sipariş oranının izlenmesi</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Yapıştırıcı, derz ve su yalıtımı aramaları YoY +%12,8 ; montaj parçaları yapı marketten tamamlanıyor 10 , 12</t>
+          <t>Konut tamiratı niyeti yükselmekte, ipotekli konut satışları artmaktadır; mevcut müşteri tabanı yenileme adayı olarak değerlendirilebilir 3 , 4</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Sepet bütünlüğü</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
+          <t>Yaşam boyu değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
           <t>Öncelik 3</t>
@@ -3911,103 +2632,15 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Ledli ayna, aydınlatma ve koleksiyon uyumlu havlupan derinliği</t>
+          <t>Karo, mutfak tezgahı ve yapı kimyasalında kategori genişlemesinin değerlendirilmesi</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Ledli ayna ve aydınlatma aramaları üç yılda +%13,1 ; Trendyol'da ledli ayna medyanı 1.650 TL 9 , 10</t>
+          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 21.000 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 31</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>BM setine bağlı ek satış</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="43" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Yenileme paketinde iş ortağı ürünleri (şofben, termosifon, tekstil, düzenleme)</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 10 , 22</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Tadilat sepetinin tamamlanması</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>V-Care için deneyim modeli ve universal akıllı kapağın izlenmesi</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 7 , 47</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Premium segmentte dönüşüm</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="43" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Satın alan müşteriye ürün ömrüne göre yenileme ve yedek parça hatırlatması; olumsuz deneyim sonrası tekrar sipariş oranının izlenmesi</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Konut tamiratı niyeti yükselmekte, ipotekli konut satışları artmaktadır; mevcut müşteri tabanı yenileme adayı olarak değerlendirilebilir 3 , 4</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Yaşam boyu değer</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="56" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Karo, mutfak tezgahı ve yapı kimyasalında kategori genişlemesinin değerlendirilmesi</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 21.000 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 31</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Karo trafiğinden çapraz satış</t>
         </is>
@@ -4021,7 +2654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet108.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4623,7 +3256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet109.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet105.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Hacimler Keyword Planner'a geçti, SSG/BM ve şikayet grafikleri yenilendi, grup etiketleri, açıklama vurguları
- Kategori baş kelimeleri, marka arama talebi ve pazaryeri kelimelerinde Ahrefs hacmi yerine Google Keyword Planner; SEOmonitor rakipleri marka tablosuna eklendi
- SSG/BM ürün tipi grafikleri: değişim yüzdesi ve iki dönem hacmi sekmeleri
- Aylık şikayet serisine Kale, Creavit, Bocchi, Geberit ve E.C.A. eklendi; lejanttan aç/kapa
- YouTube, pazaryeri, rakip ve Similarweb tablolarında renkli grup etiketleri
- Similarweb grafiğinde %5 ve üzeri paylar etiketli
- GSC tablolarında click; autocomplete başlığı; kanal rollerinde yapı market satırı çıkarıldı
- Alt başlık açıklamalarında önemli ifadeler vurgulu, tablolarda VitrA satırı vurgulu
- Enleri ve model kodu açıklamalarına liste ve eşleşme sayıları

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -27,7 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Cihaz ve ülke" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 &quot;vitra&quot; ile başlayan" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Kategori ve rakip marka" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Öneri temaları" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Autocomplete önerilerinin" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 En çok tık getiren sorgular" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Kim sıralanıyor" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 VitrA nerede" sheetId="24" state="visible" r:id="rId24"/>
@@ -2595,10 +2595,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -2709,28 +2709,6 @@
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Klozet takımı, banyo dolabı, duşakabin, küvet</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="43" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Yapı market (Koçtaş, Bauhaus, Tekzen)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Kategori aramalarında VitrA ile en çok ortak kelimeye sahip kanal; "vitra klozet fiyatları koçtaş" gibi aramalar mevcut</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Tamamlayıcı ürün ve montaj hizmetiyle birlikte satış</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Klozet, lavabo, batarya, montaj malzemesi</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3535,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Banyo dolabı aylık 60.000 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; taharet musluğunda VitrA ilk sayfada yok, banyo ve lavabo bataryasında 3. sırada; baş kelimelerin çoğunda KD 0-2 13 , 32</t>
+          <t>Banyo dolabı aylık 98.625 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; taharet musluğunda VitrA ilk sayfada yok, banyo ve lavabo bataryasında 3. sırada; baş kelimelerin çoğunda KD 0-2 13 , 32</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -3887,7 +3865,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 21.000 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 32</t>
+          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 24.242 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 32</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -4236,7 +4214,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="43" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Ahrefs Site Explorer ve Keywords Explorer (marka siteleri)</t>
@@ -4244,7 +4222,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>24 marka ve uzman site top pages, 69 baş kelime, 18 marka araması · Türkiye · 28.09.2026</t>
+          <t>24 marka ve uzman site top pages ve 69 baş kelimenin sıralama verisi · Türkiye · 28.09.2026; bu bölümdeki arama hacimleri Google Keyword Planner (Eyl 2024 - Ağu 2026)</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
@@ -6920,7 +6898,7 @@
           <t>Bölüm: İhtiyaç Dili: Kullanıcı Ne Arıyor? · Sitenin fiilen aldığı trafik: Search Console sorguları
 Kapsam: Aynı kelime seti, kullanıcının hangi ihtiyaçla aradığına göre yeniden sınıflandırılmıştır. Kategori adıyla yapılan jenerik aramaların dışında kalan altı ihtiyaç sınıfı, e-ticaret sayfalarının hangi soruya cevap vermesi gerektiğini göstermektedir.
 Kaynak: Google Ads Keyword Planner (ihtiyaç sınıfları, Oca-Ağu 2025 ve 2026) · Google Search Console, sc-domain:vitra.com.tr, 1 Haz 2025 - 25 Eyl 2026, ilk 25.000 sorgu 7 , 11
-Sütun açıklamaları: Marka: Sorgunun "vitra" veya "artema" içerip içermediği. | İhtiyaç sınıfı: Sorgunun ifade kalıbına göre sınıfı. | Tık: Google Search Console, 1 Haz 2025 - 25 Eyl 2026, ilk 25.000 sorgu. | Pay: Sınıfın toplam tık içindeki payı. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim. | Örnek: Sınıfın en çok tık alan sorguları.</t>
+Sütun açıklamaları: Marka: Sorgunun "vitra" veya "artema" içerip içermediği. | İhtiyaç sınıfı: Sorgunun ifade kalıbına göre sınıfı. | Click: Google Search Console, 1 Haz 2025 - 25 Eyl 2026, ilk 25.000 sorgu. | Pay: Sınıfın toplam tık içindeki payı. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim. | Örnek: Sınıfın en çok tık alan sorguları.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -6943,7 +6921,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tık</t>
+          <t>Click</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -7469,7 +7447,7 @@
           <t>Bölüm: Organik Kanal Performansı · Trafik hangi sayfa türlerine geliyor?
 Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 11
-Sütun açıklamaları: Sayfa türü: Adres yapısına göre sayfa sınıfı; /c- ve kategori dizinleri kategori, -p- ve -sku- kodlu adresler (eski adres yapısı dahil) ürün sayfasıdır. | Sayfa: Dönemde en az bir gösterim almış tekil sayfa sayısı (ilk 25.000 adres); sayfalama ve filtre parametreli adresler ana sayfayla tek sayfa sayılmıştır. | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam tık. | Pay: Sayfa türünün toplam tık içindeki payı. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
+Sütun açıklamaları: Sayfa türü: Adres yapısına göre sayfa sınıfı; /c- ve kategori dizinleri kategori, -p- ve -sku- kodlu adresler (eski adres yapısı dahil) ürün sayfasıdır. | Sayfa: Dönemde en az bir gösterim almış tekil sayfa sayısı (ilk 25.000 adres); sayfalama ve filtre parametreli adresler ana sayfayla tek sayfa sayılmıştır. | Click: 1 Haz 2025 - 25 Eyl 2026 toplam click. | Pay: Sayfa türünün toplam tık içindeki payı. | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -7491,7 +7469,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tık</t>
+          <t>Click</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -7791,7 +7769,7 @@
           <t>Bölüm: Organik Kanal Performansı · Kategori bazında organik trafik
 Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 11
-Sütun açıklamaları: Kategori: Kategori, ürün, koleksiyon ve eski online.vitra.com.tr sayfalarının adres yapısından türetilen ana kategori. | Sayfa: Kategoriye eşlenen tekil sayfa sayısı; sayfalama ve filtre parametreli adresler tek sayılmıştır. | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam tık. | Tık payı: Kategoriye eşlenen sayfaların (kategori, ürün, koleksiyon, teknik föy ve eski online.vitra.com.tr adresleri) toplam tıkı içindeki pay. | Talep payı: Kategorinin Oca-Ağu 2026 arama talebindeki payı (Bölüm 03, 2.342 kelime). | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
+Sütun açıklamaları: Kategori: Kategori, ürün, koleksiyon ve eski online.vitra.com.tr sayfalarının adres yapısından türetilen ana kategori. | Sayfa: Kategoriye eşlenen tekil sayfa sayısı; sayfalama ve filtre parametreli adresler tek sayılmıştır. | Click: 1 Haz 2025 - 25 Eyl 2026 toplam click. | Click payı: Kategoriye eşlenen sayfaların (kategori, ürün, koleksiyon, teknik föy ve eski online.vitra.com.tr adresleri) toplam click'i içindeki pay. | Talep payı: Kategorinin Oca-Ağu 2026 arama talebindeki payı (Bölüm 03, 2.342 kelime). | Gösterim: Aynı dönemde gösterim. | CTR: Tık / gösterim.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -7814,12 +7792,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tık</t>
+          <t>Click</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Tık payı</t>
+          <t>Click payı</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -8083,7 +8061,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -8099,7 +8077,7 @@
           <t>Bölüm: Organik Kanal Performansı · En çok tık alan sayfalar · Tem-Eyl 2026
 Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 11
-Sütun açıklamaları: Sayfa adresi: Sayfa adresi; bağlantı canlı sayfaya gider. | Tık · Tem-Eyl 2026: 1 Temmuz - 25 Eylül 2026 organik tık.</t>
+Sütun açıklamaları: Sayfa adresi: Sayfa adresi; bağlantı canlı sayfaya gider. | Click · Tem-Eyl 2026: 1 Temmuz - 25 Eylül 2026 organik click.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -8112,7 +8090,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Tık · Tem-Eyl 2026</t>
+          <t>Click · Tem-Eyl 2026</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8280,7 @@
           <t>Bölüm: Organik Kanal Performansı · Cihaz ve ülke
 Kapsam: Search Console verisi, vitra.com.tr'nin Google'dan aldığı trafiğin hangi sayfa türlerine ve kategorilere geldiğini göstermektedir. Dönem 1 Haziran 2025 - 25 Eylül 2026'dır. Veri alan adı düzeyindeki mülkten (sc-domain:vitra.com.tr) alınmıştır; vitra.com.tr'nin tüm alt alan adları ve adresleri tek toplam olarak kapsanmaktadır.
 Kaynak: Google Search Console · sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sayfa×gün, cihaz×gün ve ülke boyutları · 28.09.2026 11
-Sütun açıklamaları: Kırılım: Search Console cihaz ve ülke boyutu. | Tık: 1 Haz 2025 - 25 Eyl 2026 toplam. | Pay: Toplam tık içindeki pay. | CTR: Tık / gösterim.</t>
+Sütun açıklamaları: Kırılım: Search Console cihaz ve ülke boyutu. | Click: 1 Haz 2025 - 25 Eyl 2026 toplam. | Pay: Toplam tık içindeki pay. | CTR: Tık / gösterim.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -8317,7 +8295,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Tık</t>
+          <t>Click</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -9804,14 +9782,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Marka Aramaları ve Autocomplete · Öneri temaları</t>
+          <t>Marka Aramaları ve Autocomplete · Autocomplete önerilerinin tema oranı</t>
         </is>
       </c>
     </row>
     <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Marka Aramaları ve Autocomplete · Öneri temaları
+          <t>Bölüm: Marka Aramaları ve Autocomplete · Autocomplete önerilerinin tema oranı
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 66 kök ifade için Türkiye, Türkçe, masaüstü Chrome önerileri alınmıştır: "vitra" ile başlayan 14 kök ifade (28 Eylül 2026) ve kategori, hizmet, fiyat, rakip marka ve perakendeci için 52 kök ifade (30 Eylül 2026). Karolar ve tema dağılımı bu iki setteki 625 öneriye dayanmaktadır.
 Kaynak: Google Autocomplete · "vitra" ile başlayan 14 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, masaüstü Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
 Sütun açıklamaları: Öneri teması: Önerinin ifade kalıbına göre sınıfı. | Öneri: Tablolarda yer alan 66 kök ifadeden dönen tekil öneri sayısı (kök ifade başına en fazla 10; iki kök ifadede dönen öneri bir kez sayılmıştır). | Pay: Toplam öneri içindeki pay.</t>
@@ -9978,7 +9956,7 @@
           <t>Bölüm: Marka Aramaları ve Autocomplete · En çok tık getiren sorgular · Search Console
 Kapsam: Google'ın arama kutusunda önerdiği tamamlamalar, gerçek kullanıcı aramalarından türetildiği için markadan ne beklendiğini en doğrudan gösteren kaynaklardan biridir. 66 kök ifade için Türkiye, Türkçe, masaüstü Chrome önerileri alınmıştır: "vitra" ile başlayan 14 kök ifade (28 Eylül 2026) ve kategori, hizmet, fiyat, rakip marka ve perakendeci için 52 kök ifade (30 Eylül 2026). Karolar ve tema dağılımı bu iki setteki 625 öneriye dayanmaktadır.
 Kaynak: Google Autocomplete · "vitra" ile başlayan 14 kök ifade (28.09.2026) ve 52 kategori, hizmet, fiyat, rakip marka ve perakendeci kök ifadesi (30 Eyl 2026) · Türkiye, Türkçe, masaüstü Chrome · Google Ads hacim · Google Search Console sorgu raporu 11 , 12
-Sütun açıklamaları: Sorgu: Kullanıcının Google'a yazdığı ifade. | Tık: 1 Haz 2025 - 25 Eyl 2026. | Gösterim: Aynı dönem. | CTR: Tık / gösterim. | Sıra: Ortalama sıra.</t>
+Sütun açıklamaları: Sorgu: Kullanıcının Google'a yazdığı ifade. | Click: 1 Haz 2025 - 25 Eyl 2026. | Gösterim: Aynı dönem. | CTR: Tık / gösterim. | Sıra: Ortalama sıra.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -9994,7 +9972,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Tık</t>
+          <t>Click</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -11077,7 +11055,7 @@
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -11096,7 +11074,7 @@
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · Tek günlük gözlemde VitrA'nın ilk 20'de görünmediği kelimeler: SERP, Search Console ve Google kontrolü
 Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
 Kaynak: Google TR mobil sonuç sayfası · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
-Sütun açıklamaları: Arama kelimesi: 29.09.2026 mobil SERP gözleminde vitra.com.tr'nin ilk 20'de görünmediği kelime. | Aylık hacim: Google Keyword Planner, Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | Search Console ort. sıra: vitra.com.tr'nin bu sorgudaki 26.06 - 25.09.2026 ortalama sırası (sorgu düzeyinde, tüm cihazlar); "-" sorgu raporda yok. | Search Console tık: Aynı dönemde bu kelimeden gelen tık. | Google sırası (30.09): google.com.tr, oturumsuz arama, 30.09.2026; ilk sayfadaki organik sonuçlar arasında vitra.com.tr'nin sırası; "-" ilk sayfada yok. | İlk 5 sonuç (30.09): Aynı Google kontrolünde ilk beş organik sonucun alan adı, sırasıyla; "-" alan adı okunamayan sonuç. | Durum: VitrA'nın 30.09.2026 Google ilk sayfasındaki varlığı.</t>
+Sütun açıklamaları: Arama kelimesi: 29.09.2026 mobil SERP gözleminde vitra.com.tr'nin ilk 20'de görünmediği kelime. | Aylık hacim: Google Keyword Planner, Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | Search Console ort. sıra: vitra.com.tr'nin bu sorgudaki 26.06 - 25.09.2026 ortalama sırası (sorgu düzeyinde, tüm cihazlar); "-" sorgu raporda yok. | Search Console click: Aynı dönemde bu kelimeden gelen click. | Google sırası (30.09): google.com.tr, oturumsuz arama, 30.09.2026; ilk sayfadaki organik sonuçlar arasında vitra.com.tr'nin sırası; "-" ilk sayfada yok. | İlk 5 sonuç (30.09): Aynı Google kontrolünde ilk beş organik sonucun alan adı, sırasıyla; "-" alan adı okunamayan sonuç. | Durum: VitrA'nın 30.09.2026 Google ilk sayfasındaki varlığı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -11124,7 +11102,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Search Console tık</t>
+          <t>Search Console click</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -22761,7 +22739,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Tema bazında VitrA ve en yüksek rakip
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026; trafik tahmini) · arama hacimleri Google Keyword Planner (TR, Eyl 2024 - Ağu 2026) · SEOmonitor rakip listesi · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
 Sütun açıklamaları: Tema: Top pages sayfalarının URL ve en iyi kelimesine göre eşlendiği kategori teması. | vitra.com.tr: Temaya eşlenen VitrA sayfalarının Ahrefs tahmini aylık organik trafiği. | En yüksek marka / uzman site rakibi: Temada en yüksek trafiği alan marka ya da uzman site; pazaryerleri ve yapı marketler karşılaştırmaya dahil değildir. | Rakip trafiği: Rakibin tema trafiği. | Durum: VitrA ile en yüksek marka / uzman site rakibinin karşılaştırması.</t>
         </is>
       </c>
@@ -23297,13 +23275,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="174" customHeight="1">
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Kategori baş kelimeleri: hacim, potansiyel ve VitrA sırası
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
-Sütun açıklamaları: Baş kelime: Kategori baş kelimesi. | Aylık hacim: Ahrefs Keywords Explorer, Türkiye; Bölüm 16'daki pazaryeri kelime hacimleri farklı bir Ahrefs raporundan geldiği için küçük farklar gösterebilir. | Trafik potansiyeli: Bu kelimede 1. sıradaki sayfanın tüm kelimelerinden aldığı tahmini aylık trafik (Ahrefs TP). | VitrA sırası: Google TR mobil SERP, 29.09.2026; "-" ilk 20'de yok. * 30.09.2026 Google kontrolüne ve Search Console ortalama sırasına (4,2) göre.</t>
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026; trafik tahmini) · arama hacimleri Google Keyword Planner (TR, Eyl 2024 - Ağu 2026) · SEOmonitor rakip listesi · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
+Sütun açıklamaları: Baş kelime: Kategori baş kelimesi. | Aylık hacim: Google Keyword Planner, Türkiye, Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | Trafik potansiyeli: Bu kelimede 1. sıradaki sayfanın tüm kelimelerinden aldığı tahmini aylık trafik (Ahrefs TP). | VitrA sırası: Google TR mobil SERP, 29.09.2026; "-" ilk 20'de yok. * 30.09.2026 Google kontrolüne ve Search Console ortalama sırasına (4,2) göre.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -23339,7 +23317,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>60000</v>
+        <v>98625</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>24000</v>
@@ -23355,7 +23333,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>59000</v>
+        <v>95375</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>5600</v>
@@ -23367,17 +23345,17 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>duş başlığı</t>
+          <t>lavabo</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>43000</v>
+        <v>55483</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2000</v>
+        <v>18000</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
@@ -23387,7 +23365,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>39000</v>
+        <v>50417</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>31000</v>
@@ -23399,119 +23377,119 @@
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>taharet musluğu</t>
+          <t>duş başlığı</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>32000</v>
+        <v>42133</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2200</v>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2000</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>lavabo</t>
+          <t>banyo bataryası</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>28000</v>
+        <v>39267</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>18000</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>1</v>
+        <v>8000</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>3*</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>çamaşır makinesi dolabı</t>
+          <t>klozet kapağı</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>27000</v>
+        <v>38167</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>4100</v>
+        <v>11000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>klozet kapağı</t>
+          <t>taharet musluğu</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>27000</v>
+        <v>37417</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>11000</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>6</v>
+        <v>2200</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>banyo bataryası</t>
+          <t>çamaşır makinesi dolabı</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>24000</v>
+        <v>33450</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>3*</t>
-        </is>
+        <v>4100</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>banyo modelleri</t>
+          <t>dolap kulpu</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>24000</v>
+        <v>24242</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>5</v>
+        <v>19000</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>dolap kulpu</t>
+          <t>banyo modelleri</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>22000</v>
+        <v>20283</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>19000</v>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>7700</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -23521,7 +23499,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>17000</v>
+        <v>18850</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>18000</v>
@@ -23537,7 +23515,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>15000</v>
+        <v>15625</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>3300</v>
@@ -23553,7 +23531,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>11000</v>
+        <v>13450</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>6200</v>
@@ -23571,7 +23549,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>10000</v>
+        <v>13000</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>9800</v>
@@ -23583,35 +23561,35 @@
     <row r="20" ht="17" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>banyo aynası</t>
+          <t>kartuş</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>7500</v>
+        <v>12042</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>5600</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>6</v>
+        <v>4200</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>kartuş</t>
+          <t>banyo aynası</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>6600</v>
+        <v>10267</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>4200</v>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5600</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -23927,7 +23905,7 @@
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Rehber içerik: rakiplerin trafik aldığı konular
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026; trafik tahmini) · arama hacimleri Google Keyword Planner (TR, Eyl 2024 - Ağu 2026) · SEOmonitor rakip listesi · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
 Sütun açıklamaları: Rehber konusu: Rakiplerin rehber sayfalarından organik trafik aldığı konu. | Rakip: Konuda trafik alan rakip siteler. | Rakip trafiği: Rakip rehber sayfalarının toplam Ahrefs tahmini aylık organik trafiği. | VitrA sayfası: vitra.com.tr /ilham-veren-fikirler içindeki karşılık. | VitrA trafiği: VitrA rehber sayfasının Ahrefs tahmini aylık organik trafiği.</t>
         </is>
       </c>
@@ -24194,10 +24172,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
   </cols>
@@ -24209,13 +24187,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Marka ve Uzman Sitelerde Kategori Trafiği · Marka arama talebi
 Kapsam: Marka ve uzman e-ticaret sitelerinin (Kale, Creavit, E.C.A., Geberit, Duravit, Banyomarka, Banyoline, Yapımanya, Yerevdekor, Balneom, Kalekim, seramik markaları ve diğerleri) en yüksek trafikli sayfaları Ahrefs ile çekilmiş, kategori temalarına eşlenmiş ve vitra.com.tr ile karşılaştırılmıştır. Değerler Ahrefs tahmini aylık organik trafiktir; listelenen sayfalar site toplamının %66-93'ünü kapsamaktadır.
-Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026) · Ahrefs Keywords Explorer ve SERP overview · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
-Sütun açıklamaları: Marka araması: Aranan marka ifadesi. | Aylık hacim: Ahrefs, son 12 ay ortalaması, Türkiye. | Son 12 ay / önceki 12 ay: Eylül 2025 - Ağustos 2026 ile Eylül 2024 - Ağustos 2025 aylık serilerinin toplam değişimi. * "eca" hacminin önemli bölümü kombi ve klima aramalarından gelmektedir.</t>
+Kaynak: Ahrefs Site Explorer top pages (TR, 28.09.2026; trafik tahmini) · arama hacimleri Google Keyword Planner (TR, Eyl 2024 - Ağu 2026) · SEOmonitor rakip listesi · Google TR mobil sonuç sayfası (29.09.2026) 13 , 32
+Sütun açıklamaları: Marka araması: Aranan marka ifadesi; "SEOmonitor rakibi" etiketi kampanyada doğrudan rakip olarak tanımlı siteleri gösterir. Perakendecilerde banyo ile birlikte yapılan aramalar alınmıştır. | Aylık hacim: Google Keyword Planner, Türkiye, Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | Son 12 ay / önceki 12 ay: Eylül 2025 - Ağustos 2026 ile Eylül 2024 - Ağustos 2025 aylık arama toplamlarının değişimi (Google Keyword Planner).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -24241,92 +24219,92 @@
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>VitrA</t>
+          <t>Kale * · SEOmonitor rakibi</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>30000</v>
+        <v>60208</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>E.C.A. *</t>
+          <t>VitrA</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>16000</v>
+        <v>34950</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Bien</t>
+          <t>E.C.A. **</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>5.4</v>
+        <v>20825</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>-13.3</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Artema</t>
+          <t>Bien</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>5200</v>
+        <v>12367</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Bocchi</t>
+          <t>Creavit · SEOmonitor rakibi</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>4800</v>
+        <v>9000</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2.1</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Creavit</t>
+          <t>Bocchi</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>4700</v>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>-0.9</v>
+        <v>7050</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>15.6</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Grohe</t>
+          <t>Artema</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>4400</v>
+        <v>6425</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
@@ -24336,88 +24314,166 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>3000</v>
+        <v>6425</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>4.1</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Hansgrohe</t>
+          <t>Grohe</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>2900</v>
+        <v>5717</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>7.4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Turkuaz Seramik</t>
+          <t>Hansgrohe</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>1800</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0.1</v>
+        <v>5350</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Duravit</t>
+          <t>Turkuaz Seramik</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C15" s="10" t="n">
-        <v>-0.6</v>
+        <v>3558</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>18.9</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Visam</t>
+          <t>Duravit</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>1200</v>
+        <v>2775</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>7.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Serel</t>
+          <t>Visam</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>-2.5</v>
+        <v>2375</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>12.6</v>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>Serel</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>1850</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Banyomarka · SEOmonitor rakibi</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>1575</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>IKEA banyo · SEOmonitor rakibi</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>1375</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>-8.300000000000001</v>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>Kale banyo</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
-        <v>800</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>-3</v>
+      <c r="B21" s="6" t="n">
+        <v>1110</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>-3.5</v>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Banyomega · SEOmonitor rakibi</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>416</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Banyoline · SEOmonitor rakibi</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>327</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>-31.2</v>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Bauhaus banyo · SEOmonitor rakibi</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>-2.4</v>
       </c>
     </row>
   </sheetData>
@@ -24760,7 +24816,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -24770,13 +24826,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="174" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryerleri: Kategori Yapısı ve Çok Satanlar · Alt kategori trafiği: Trendyol ve Hepsiburada
 Kapsam: Pazaryerleri iki kaynakla incelenmiştir: Ahrefs ile Trendyol, Hepsiburada ve sekiz perakende ve karşılaştırma sitesinin banyo kategorilerinden aldığı organik trafik; site üzerinde Trendyol ve Hepsiburada'nın kategori yapısı, çok satan sıralamaları, marka filtreleri ve arama önerileri. Değerlendirme sayısı satış adedine yaklaşık bir gösterge olarak kullanılmıştır.
 Kaynak: Ahrefs Site Explorer top pages ve organic keywords (TR, 28.09.2026) · Trendyol ve Hepsiburada kategori, çok satan, marka filtresi ve arama önerisi sayfaları (tarayıcı, 29.09.2026) 33 , 34 , 35
-Sütun açıklamaları: Alt kategori: Sayfaların URL ve en iyi kelimesine göre sınıflandığı banyo alt kategorisi. | Grup: Ana: VitrA'nın sattığı banyo kategorileri · bitişik: banyoyla birlikte alınan ama VitrA'nın sınırlı sattığı kategoriler. | Trendyol trafik: Ahrefs tahmini aylık organik trafik. | Hepsiburada trafik: Ahrefs tahmini aylık organik trafik. | Trendyol'da en çok trafik getiren kelime: Kelime, aylık hacim ve Trendyol'un sırası.</t>
+Sütun açıklamaları: Alt kategori: Sayfaların URL ve en iyi kelimesine göre sınıflandığı banyo alt kategorisi. | Grup: Ana: VitrA'nın sattığı banyo kategorileri · bitişik: banyoyla birlikte alınan ama VitrA'nın sınırlı sattığı kategoriler. | Trendyol trafik: Ahrefs tahmini aylık organik trafik. | Hepsiburada trafik: Ahrefs tahmini aylık organik trafik. | Trendyol'da en çok trafik getiren kelime: Kelime, aylık arama hacmi (Google Keyword Planner, Eyl 2025 - Ağu 2026 ortalaması) ve Trendyol'un sırası.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -24830,7 +24886,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>boy aynası (27.000 · 1. sıra)</t>
+          <t>boy aynası (- · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24853,7 +24909,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>mutfak musluğu (8.100 · 1. sıra)</t>
+          <t>mutfak musluğu (12.550 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24876,7 +24932,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>banyo dolabı (64.000 · 1. sıra)</t>
+          <t>banyo dolabı (98.625 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24899,7 +24955,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>duşakabin (66.000 · 1. sıra)</t>
+          <t>duşakabin (95.375 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24922,7 +24978,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>çamaşır ve kurutma makinesi dolabı (6.800 · 1. sıra)</t>
+          <t>çamaşır ve kurutma makinesi dolabı (10.625 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24945,7 +25001,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>60 120 fayans (1.700 · 1. sıra)</t>
+          <t>60 120 fayans (2.733 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24968,7 +25024,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>banyo seti (13.000 · 1. sıra)</t>
+          <t>banyo seti (23.017 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -24991,7 +25047,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>duş başlığı (45.000 · 3. sıra)</t>
+          <t>duş başlığı (42.133 · 3. sıra)</t>
         </is>
       </c>
     </row>
@@ -25014,7 +25070,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>mutfak bataryası (24.000 · 1. sıra)</t>
+          <t>mutfak bataryası (36.800 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25037,7 +25093,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>klozet (41.000 · 2. sıra)</t>
+          <t>klozet (50.417 · 2. sıra)</t>
         </is>
       </c>
     </row>
@@ -25060,7 +25116,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>abdest lavabosu (4.800 · 1. sıra)</t>
+          <t>abdest lavabosu (9.967 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25083,7 +25139,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>lavabo gider borusu (7.100 · 1. sıra)</t>
+          <t>lavabo gider borusu (11.333 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25106,7 +25162,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>banyo paspası (15.000 · 1. sıra)</t>
+          <t>banyo paspası (26.717 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25129,7 +25185,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>klozet kapağı (29.000 · 1. sıra)</t>
+          <t>klozet kapağı (38.167 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25152,7 +25208,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>en kullanışlı tezgah arası (2.700 · 2. sıra)</t>
+          <t>en kullanışlı tezgah arası (2.108 · 2. sıra)</t>
         </is>
       </c>
     </row>
@@ -25175,7 +25231,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>termosifon (33.000 · 2. sıra)</t>
+          <t>termosifon (61.500 · 2. sıra)</t>
         </is>
       </c>
     </row>
@@ -25198,7 +25254,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>banyo havalandırma fanı (3.300 · 1. sıra)</t>
+          <t>banyo havalandırma fanı (4.650 · 1. sıra)</t>
         </is>
       </c>
     </row>
@@ -25221,7 +25277,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>klozet şamandırası (5.000 · 2. sıra)</t>
+          <t>klozet şamandırası (7.750 · 2. sıra)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SERP 107 kelime (hacimsiz 2 kelime çıktı), GEO'ya AI yanıt verisi, 4 veri seti alt sayfası ve üst bar butonları
- serp_ozet.py: SERP rakamları tek hesaptan; seçim yöntemi lede'de
- GEO: ChatGPT, Gemini ve AI Overview yanıtlarında VitrA, kaynak alan adları, satın alma ve montaj soruları
- alt_veri.py: arama sonuçları, kelime evreni, pazaryeri taraması, YouTube alt sayfaları
- Okunabilirlik: h2/h3 punto, turuncu madde imleri, önemli ifadeler bold, açıklamalar

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
+++ b/VitrA_E-Ticaret_Buyume_Firsatlari.xlsx
@@ -114,9 +114,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="105 Kanal rolleri" sheetId="105" state="visible" r:id="rId105"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="106 Hacimli ve ölçüye bağlı" sheetId="106" state="visible" r:id="rId106"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="107 Tamamlayıcı ürün kurgusu" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="108 Sonraki Adımlar" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="109 Yöntem ve Kapsam" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="108 Yapay zeka yanıtlarında" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="109 Yapay zeka yanıtlarında en" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="110 Satın alma ve montaj" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="111 Sonraki Adımlar" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="112 Yöntem ve Kapsam" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaynakça" sheetId="113" state="visible" r:id="rId113"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -650,15 +653,15 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Makro Ortam ve Ödeme Gücü · Kart harcamaları: banyo ile ilişkili sektörler</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="160" customHeight="1">
+          <t>Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Kart harcamaları: banyo ile ilişkili sektörler</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="188" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Makro Ortam ve Ödeme Gücü · Kart harcamaları: banyo ile ilişkili sektörler
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
+          <t>Bölüm: Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Kart harcamaları: banyo ile ilişkili sektörler
+Kapsam: Bu bölüm, banyo ürünlerine olan talebi etkileyen genel ekonomik koşulları özetlemektedir: insanların kartla ne kadar harcadığı, ekonomiye güvenleri ve evlerini tamir ettirme niyetleri, konut alım-satımı ve bankaların kredi verme koşulları. Banyo yenilemesi ertelenebilen bir harcama olduğu için bu göstergeler, kategori aramalarındaki daralmanın (Bölüm 03) arka planını açıklamaya yardımcı olur. Veriler Türkiye Cumhuriyet Merkez Bankası'nın veri sisteminden (TCMB EVDS) alınmıştır.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Harcama kalemi: BKM ve TCMB'nin haftalık sektörel kart harcama akımı; haftalar takvim ayına toplanmıştır. | Oca-Ağu 2025 (milyar TL): Ocak - Ağustos 2025 toplam kart harcaması, milyar TL, nominal. | Oca-Ağu 2026 (milyar TL): Ocak - Ağustos 2026 toplam kart harcaması, milyar TL, nominal. | Değişim: İki pencere arasındaki nominal yüzde değişim; enflasyon etkisi arındırılmamıştır.</t>
         </is>
@@ -3120,763 +3123,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sonraki Adımlar · Tablo 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="104" customHeight="1">
+          <t>AI Arama ve GEO Fırsatları · Yapay zeka yanıtlarında VitrA: ChatGPT, Gemini ve Google AI Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Sonraki Adımlar
-Kapsam: Aksiyonlar üç öncelik kademesinde verilmiştir; sıralama VitrA ekibinin stratejik tercihleri, pazaryeri ve GA4 verisiyle güncellenebilir. Öncelik 1 maddeleri mevcut altyapı ve mevcut talep üzerinde kısa vadede etki üretebilecek düzenlemelerdir.
-Sütun açıklamaları: Öncelik: Etki ve uygulanabilirlik birlikte değerlendirilerek verilen sıra. | Aksiyon: Önerilen düzenleme. | Dayanak: Öneriyi destekleyen bulgu ve kaynak. | Beklenen etki: Düzenlemenin hedeflediği sonuç.</t>
+          <t>Bölüm: AI Arama ve GEO Fırsatları · Yapay zeka yanıtlarında VitrA: ChatGPT, Gemini ve Google AI Overview
+Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek, soruyu doğrudan cevaplayan sayfaya, markanın tutarlı tanımlanmasına ve markadan site dışında söz edilmesine bağlıdır. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli marka kayıtlarına dayanmaktadır.
+Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 107 kelime, 29.09.2026 · Yapay zeka yanıt takibi, 125 soru, ChatGPT, Gemini ve Google AI Overview, 4 Eyl - 3 Eki 2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 41 , 52 , 53 , 54 , 55
+Sütun açıklamaları: Platform: Yanıtın alındığı yapay zeka platformu. | Yanıt: 4 Eyl - 3 Eki 2026 arasında marka adı geçmeyen 111 soruya alınan yanıt sayısı. | VitrA: VitrA'nın adıyla geçtiği yanıtların payı. | Kale: Kale adının geçtiği yanıtların payı (aynı yanıtlar). | Creavit: Creavit adının geçtiği yanıtların payı (aynı yanıtlar). | Geberit: Geberit adının geçtiği yanıtların payı (aynı yanıtlar). | Trendyol: Trendyol adının geçtiği yanıtların payı (aynı yanıtlar). | Hepsiburada: Hepsiburada adının geçtiği yanıtların payı (aynı yanıtlar). | Koçtaş: Koçtaş adının geçtiği yanıtların payı (aynı yanıtlar).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Öncelik</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Aksiyon</t>
+          <t>Yanıt</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Dayanak</t>
+          <t>VitrA</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Beklenen etki</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="69" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Yedek parça kategorisi ve ürün koduna göre parça bulucu; eski yedek parça adresinin bu kategoriye yönlendirilmesi</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>İç takım ve yedek parça aramaları aylık 113K; eski yedek parça sayfası Haziran - Kasım 2025'te Search Console'a göre ayda ~300 tık almış, bugün tek ürünlü kategoriye yönlenmektedir; Trendyol aramasında VitrA iç takımda ilk sıradadır 9 , 10 , 11 , 19 , 47 , 48</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Mevcut müşteriden tekrar satış ve marka savunması</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>"Banyo yenileme paketi": ürün seti + montaj + keşif tek teklifte; Banyo Asistanı paketin giriş kapısı</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Montaj, keşif, ücretsiz montajlı mobilya ve Banyo Asistanı mevcut ama ayrı sunuluyor; tasarım ve tadilat aramaları büyüyor; Koçtaş, Bauhaus ve Kohler proje satışına geçmiş 10 , 19 , 22 , 27 , 29</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Sepet büyüklüğü ve kanal farklılaşması</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Keşif ve montajın ölçüye bağlı ürün sayfalarına bağlanması; duşakabin, küvet ve duş teknesi için montaj kalemi</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Duşakabin talebi aylık 285K; duşakabin ürün sayfasında montaj ya da keşif seçeneği bulunmuyor 10 , 19</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Hacimli üründe karar öncesi belirsizliğin azalması</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Ürün sayfasına garanti süresi, yedek parça ve servis girişi; servis ücreti ve garanti reddi sürecinde standart metin</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 17 , 44</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Satış sonrası güven ve tekrar satın alma</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryeri fiyat ve satıcı izleme: aynı SKU'da resmi mağaza ile 3P farkının düzenli takibi, yetkili satıcı listesi ve hukuki değerlendirmeyle fiyat politikası çerçevesi</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>29 üründen 19'unda en ucuz kanal pazaryeri (medyan %24,7); Trendyol'da VitrA mağazasıyla birlikte bulunan 6 üründe 3P daha ucuz; Hepsiburada'da aynı ürün için birden fazla katalog kaydı 41 , 42</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Kanal başına tutarlı fiyat algısı</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="69" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Kategori sayfalarında stok görünürlüğü: stokta olmayan varyantların ürün sayısı ve fiyat aralığından ayrılması, "Gelince Haber Ver" kartlarının listenin sonuna alınması; "Sepette %N" etiketi yerine kartta net fiyat</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>55 kategori sayfasındaki 2.258 varyant kartının %71,1'i stoklu süzgeci dışında; 13 alt kategoride stoklu ürün yok; ilk sayfa kartlarının %89,9'unda "Sepette %N indirim" etiketi; aynı model kodunda pazaryeri fiyatı liste fiyatının medyan %14,4 altında, sepet fiyatına yakın 37</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Kategori sayfasından ürün sayfasına geçişte daha az "stokta yok" karşılaşması; kanallar arası fiyat algısının tekleşmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="56" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>AI aramada görünürlük için sorun çözen içerik: arıza, montaj, uyumluluk ve garanti konularında destek sayfaları; ölçü, seçim ve marka sorularında rehber içerik</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Rehber sayfalarında tıkların %35'i montaj, tamir ve temizlik yazılarından geliyor; destek bölümünde bu konularda sayfa yok; soru sorgularında site ilk sayfada ama CTR %0,93; VitrA 24 AI Overview'un 7'sinde kaynak 13 , 17 , 52</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>AI yanıtlarında kaynak gösterilme, tamir anında trafik ve satış sonrası başvurunun siteye dönmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="43" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Öncelik 1</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Marka ve entity tutarlılığı: Wikidata ve Wikipedia kayıtlarının VitrA ve Artema için güncel ve tutarlı hale getirilmesi</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Wikidata'da iki ayrı VitrA kaydı var ve ana kayıtta resmi web sitesi vitra.com.tr'yi göstermiyor; Artema'nın kaydı yok 53</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>AI yanıtlarında markanın doğru tanımlanması</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="56" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Taksit mesajının tüm temas noktalarında tekleştirilmesi</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Üst bantta "vade farksız 6 ay", Banyo Asistanı kampanya sayfasında "9 taksit", ürün sayfasındaki taksit tablosunda 12 taksite kadar; kullanıcı "vitra 9 taksit" ve "vitra taksit seçenekleri" arıyor 12 , 19</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Fiyat algısında netlik</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="56" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Kanal rolleri ve fiyat tutarlılığı; BM'de pazaryerinde fiyat yerine set, montaj ve garanti ile konumlanma</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>BM aramalarının %9,6'sı perakendeci adıyla yapılıyor; Trendyol'da banyo dolabı medyanı 3.249 TL, VitrA 14.462 TL; Hepsiburada'da VitrA ürünlerinin %69'u üçüncü taraf satıcıda 9 , 10 , 30 , 34 , 35</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Kanal başına net değer önerisi</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="82" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryeri ürün kartı standardı: kutu içeriği ("kapak ve rezervuar dahil değildir") başlık ve ilk görselde; klozet kodu ile uyumlu kapak ve iç takım eşleşme listesi; ölçü tablosu</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol iadelerinin %27,6'sında neden ölçü, %19,2'sinde yanlış sipariş; Eylül 2026'daki 352 ürün sorusunun 83'ü uyumluluk; ilan görselinde kapak ve rezervuar görünen klozetlerde "sadece klozet geldi" şikayeti; iki pazaryerindeki VitrA sorularının %31,9'u uyumluluk ve kullanım yeri, %18,3'ü kutu içeriği 38 , 40</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>İade ve soru yükünde azalma, düşük puanlı yorumlarda gerileme</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Kırılgan ürün paketleme standardı ve eksik parça kontrolü; hasarlı teslimde parça veya değişim akışı</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Kırık ve hasar temalı yorumların ortalama puanı 2,3 (36 yorum); cam aksesuar, lavabo ve klozet kapağı kırık teslim; vida, dübel, dolap ayağı, flex hortum eksikleri; satıcı değerlendirmesinde olumsuz etkilerin ilk üçü kusurlu, eksik ve yanlış ürün; pazaryeri yorumlarında VitrA ve Artema banyo dolabı olumsuz payı %17,9 (rakipler %7,5), bu yorumların %58,0'ı kırık veya hasarlı ürün 38 , 40</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Marka algısının korunması, iade maliyetinde azalma</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="43" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada'da VitrA ve Artema ürünlerine gelen soruların resmi mağaza tarafından takip edilmesi; sık sorulara ürün sayfasında hazır yanıt</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada'da VitrA ürünlerine gelen soruların %29,5'i resmi mağaza tarafından cevaplanmış, kalan sorular aynı ürünü satan diğer satıcılarca yanıtlanmıştır 40</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Ürün bilgisinin tek kaynaktan verilmesi, yanlış eşleşmeden kaynaklanan iadelerde azalma</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="56" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryerinde stok sürekliliği ve liste görünürlüğü: çok satanlarda stok takibi, mobilya, batarya, duş ve evye bataryası listelerine giriş ürünleri, conta ve iç takım parçalarının resmi mağazada listelenmesi</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>2026 Q3'te satılan ürünlerin 86'sında stok 0 (Q3 cirosunun %26,7'si); resmi mağaza 5 kategorinin Eylül listelerinde yok; rezervuar çok satan listesinin 2. sırası üçüncü taraftaki 71 TL'lik VitrA contası 38</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Resmi mağazanın kategori listelerinde yer alması, buybox ve yedek parça talebinin resmi kanala dönmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="56" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Google Merchant Center feed'inin tüm kategorileri kapsaması, başlıklarda kategori kelimesi; AI alışveriş yanıtları için zengin ürün bilgisi</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>VitrA sitesi Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 41 , 44</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Ücretsiz listelemelerde hazır olma</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="43" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Google Business Profile standardı: bayi profillerinde ad ve kategori, web sitesi alanı, yorum toplama ve yanıt akışı</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 44</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Banyo Asistanı mağaza adımına yerel görünürlük</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="56" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Kategori sayfalarında ilk 3 dışında kalan baş kelimeler için sayfa kurgusu; armatürde VitrA ve Artema görünürlüğü</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Banyo dolabı aylık 98.625 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; taharet musluğunda VitrA ilk sayfada yok, banyo ve lavabo bataryasında 3. sırada; baş kelimelerin çoğunda KD 0-2 13 , 32</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Mevcut kategori talebinden daha yüksek organik pay</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="43" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Katalog derinliği: hela taşı ve havlupanda ürün derinliği, çamaşır makinesi dolabının pazaryerinde listelenmesi</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Hela taşı 64,4K arama / 1 ürün, havlupan 50,7K arama / 2 ürün, çamaşır makinesi dolabı 103K arama / 29 ürün ama Trendyol ilk 40'ta yok 9 , 10 , 19</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Mevcut talebin karşılanması</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="82" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Kategori adlandırmasında pazaryeri karşılıkları ve sayfası olmayan kesitler: sıva üstü batarya, fotoselli batarya, jakuzi, duş sistemi, ayaklı lavabo eş anlamlıları; çocuk klozet, engelli klozet, köşe lavabo ve lavabo ayağı için ayrı sayfa; /c-online-ozel yönlendirme döngüsü</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>vitra.com.tr "Duvardan banyo bataryaları" ile pazaryerinde "sıva üstü banyo bataryası", "Temassız" ile "fotoselli" (Trendyol 994, Hepsiburada 588 sonuç); çocuk klozeti aramasında Trendyol 2.238, Hepsiburada 1.659 sonuç; engelli klozeti Trendyol'da 43 ürünlük ayrı kategori; dört başlığın sitede ayrı sayfası yok 13 , 37</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Kullanıcının aradığı adla eşleşen kategori sayfası; organik ve pazaryeri aramasında bulunabilirlik</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Erişilebilir banyo ve çocuk banyosu sayfaları (Conforma, tutunma barları, Sento çocuk)</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Yaşlı ve engelli ürünleri aylık 29,4K (YoY +%8,1 ); ürünler katalogda var ama tek sayfada toplanmıyor 10 , 19</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Niş ve büyüyen segmentte görünürlük</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="69" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>YouTube tamir serisi ve tesisatçı kanallarıyla iş birliği</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>En çok izlenen 14 tamir ve kurulum konusunun hiçbirinde VitrA kanal videosu yok (sifon ve iç takım 6,8M, batarya ve kartuş 7,0M izlenme); görünmelerin %43,7'si tesisatçı kanallarında; Macit Tesisat'ın VitrA tamir videosu 447K izlenme 14 , 15 , 16</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Tamir anında marka görünürlüğü</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="43" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Site dışı sinyaller: Şikayetvar yanıtları, YouTube tamir içerikleri ve rehber sitelerinde uzman içerik</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Şikayetvar puanı 18; en çok izlenen 14 tamir ve kurulum konusunda VitrA kanal videosu yok; AI Overview kaynakları arasında markadan bağımsız rehber siteleri var 13 , 16 , 17</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Markanın site dışında anılması ve AI yanıtlarında kaynak çeşitliliği</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="43" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Öncelik 2</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Banyo Asistanı'nın bayi ağına genişletilmesi ve adımlarının GA4'te ölçülmesi</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 1 Haziran 2025 - 25 Eylül 2026 döneminde 37.859 tık almıştır 11 , 19</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Lead'in satışa dönmesi</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="43" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Granit ve çelik evye + mutfak bataryası seti</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 9 , 10 , 21</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Mutfakta set satışı</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="43" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Arıtmalı batarya ve filtre aboneliği</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 554K; Trendyol'da arıtmalı batarya aramasının ilk 40 sonucunda armatür markası bulunmamaktadır 9 , 10 , 21</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Tekrarlı gelir</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="43" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Banyo planlayıcının (V-Design) yeniden devreye alınması ve Banyo Asistanı'na bağlanması</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Banyo tasarım ve planlama aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 10 , 19 , 45 , 46</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Ürün keşfinden lead'e geçiş</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Tamamlayıcı ürünlerde üçüncü taraf satıcı modelinin montaj malzemesi ve yapı kimyasalında test edilmesi</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Yapıştırıcı, derz ve su yalıtımı aramaları YoY +%12,8 ; montaj parçaları yapı marketten tamamlanıyor 10 , 12</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Sepet bütünlüğü</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Ledli ayna, aydınlatma ve koleksiyon uyumlu havlupan derinliği</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Ledli ayna ve aydınlatma aramaları üç yılda +%13,1 ; Trendyol'da ledli ayna medyanı 1.650 TL 9 , 10</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>BM setine bağlı ek satış</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="43" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Yenileme paketinde iş ortağı ürünleri (şofben, termosifon, tekstil, düzenleme)</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 10 , 22</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Tadilat sepetinin tamamlanması</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>V-Care için deneyim modeli ve universal akıllı kapağın izlenmesi</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 7 , 49</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Premium segmentte dönüşüm</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="43" customHeight="1">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Satın alan müşteriye ürün ömrüne göre yenileme ve yedek parça hatırlatması; olumsuz deneyim sonrası tekrar sipariş oranının izlenmesi</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Konut tamiratı niyeti yükselmekte, ipotekli konut satışları artmaktadır; mevcut müşteri tabanı yenileme adayı olarak değerlendirilebilir 3 , 4</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Yaşam boyu değer</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="56" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>Öncelik 3</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Karo, mutfak tezgahı ve yapı kimyasalında kategori genişlemesinin değerlendirilmesi</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 24.242 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 32</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Karo trafiğinden çapraz satış</t>
-        </is>
+          <t>Kale</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Creavit</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Geberit</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Trendyol</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Hepsiburada</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Koçtaş</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>527</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>614</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Google AI Overview</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>830</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>27.7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3888,637 +3316,404 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Yöntem ve Kapsam · Tablo 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="62" customHeight="1">
+          <t>AI Arama ve GEO Fırsatları · Yapay zeka yanıtlarında en çok kaynak gösterilen alan adları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="244" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Yöntem ve Kapsam
-Kapsam: Veri kaynaklarına, dönemlerine ve yöntem notlarına aşağıda yer verilmektedir.
-Sütun açıklamaları: Veri kaynağı: Kullanılan kaynak. | Kapsam: Dönem, coğrafya ve örneklem. | Kullanıldığı bölüm: Verinin işlendiği bölüm. | Not: Ölçüm sınırı veya yöntem notu.</t>
+          <t>Bölüm: AI Arama ve GEO Fırsatları · Yapay zeka yanıtlarında en çok kaynak gösterilen alan adları
+Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek, soruyu doğrudan cevaplayan sayfaya, markanın tutarlı tanımlanmasına ve markadan site dışında söz edilmesine bağlıdır. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli marka kayıtlarına dayanmaktadır.
+Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 107 kelime, 29.09.2026 · Yapay zeka yanıt takibi, 125 soru, ChatGPT, Gemini ve Google AI Overview, 4 Eyl - 3 Eki 2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 41 , 52 , 53 , 54 , 55
+Sütun açıklamaları: Alan adı: Yanıtta kaynak olarak bağlantı verilen alan adı; bağlantı siteyi açar. | Yanıt: Alan adının en az bir kez kaynak gösterildiği yanıt sayısı, markasız sorular, üç platform toplamı. | AI Overview: Google AI Overview yanıtlarında kaynak gösterildiği yanıt sayısı. | ChatGPT: ChatGPT yanıtlarında kaynak gösterildiği yanıt sayısı. | Gemini: Gemini yanıtlarında kaynak gösterildiği yanıt sayısı. | Satın alma soruları: "Nereden alınır", teslimat, iade ve montaj dahil satış gibi 14 markasız satın alma sorusunda (28.09 - 01.10.2026) kaynak gösterildiği yanıt sayısı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Veri kaynağı</t>
+          <t>Alan adı</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Kapsam</t>
+          <t>Yanıt</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Kullanıldığı bölüm</t>
+          <t>AI Overview</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="56" customHeight="1">
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Satın alma soruları</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Google Ads Keyword Planner</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2.342 tekil kelime · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026 (talep grafiğinde Oca 2023 - Ağu 2026)</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>03, 04, 05, 23</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Google Ads yakın yazım varyantlarına (çoğul, yazım farkı) aynı aylık seriyi döndürür; aynı seriye sahip kelimeler tek kelime olarak sayılmıştır (2.419 satırdan 2.342 tekil kelime)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>vitra.com.tr</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>882</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>372</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>422</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Google Search Console</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sorgu, cihaz, ülke</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>05, 06, 07, 08, 22, 23, 25</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Sayfa ve sorgu raporları ilk 25.000 satırla sınırlıdır; sayfa×gün tablosu 100.000 satır</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="43" customHeight="1">
+          <t>trendyol.com</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>699</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>257</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>391</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Google Autocomplete</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>66 kök ifade: "vitra" ile başlayan 14 (28.09.2026) ve kategori, hizmet, fiyat, rakip marka ve perakendeci için 52 (30.09.2026) · Türkiye, Türkçe, masaüstü Chrome</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>07, 23</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Öneriler tek günlük anlık görüntüdür; sıralama Google'ın sırasıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>koctas.com.tr</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>546</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>347</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>YouTube arama</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>30 ifade · Türkiye · ilk sayfa · 28.09.2026</t>
-        </is>
+          <t>hepsiburada.com</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>525</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>İzlenme sayıları video yayın tarihinden itibaren kümülatiftir</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+        <v>225</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>296</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Organik rakipler ve Batch Analysis · Türkiye · 27.09.2026</t>
-        </is>
+          <t>akakce.com</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>478</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek ziyaret sayısı değildir</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="56" customHeight="1">
+        <v>150</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>230</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Google Ads keyword ideas</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>10 kök ifade grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>04, 11, 12, 13</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Kelimeler 58 temalı sözlükle sınıflandırılmış, gürültü ifadeleri ayıklanmış, aynı aylık seriyi taşıyan yazım varyantları tek sayılmıştır; tema toplamları yaklaşık büyüklük gösterir</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>banyome.com</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>406</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>201</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>vitra.com.tr ürün sitemap'i ve site incelemesi</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · Banyo Asistanı · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>11, 13, 22, 23</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Ürün sayısı renk ve ölçü varyantlarını ayrı sayar; model sayısı renk ekleri ayıklanarak yaklaşık hesaplanmıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+          <t>kale.com.tr</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>286</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>186</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Rakip kategori sitemap'leri</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline · Koçtaş tarayıcı ile</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>12, 22</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Kategori varlığı gözlemidir; ürün derinliği ve satış hacmi ölçülmemiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="43" customHeight="1">
+          <t>yapilir.com</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>275</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>119</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>128</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Trendyol arama sonuçları</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>13 tema, ilk 40-45 ürün · 28.09.2026</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>04, 11, 12</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Değerlendirme sayısı satış hacmine yaklaşık gösterge olarak kullanılmıştır; sonuç sırası kişiselleştirmeye bağlı olarak değişebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="43" customHeight="1">
+          <t>youtube.com</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>265</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>106</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>103</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Rakip ve benzer oyuncuların siteleri</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Koçtaş, IKEA, Hepsiburada, Kale, Banyomarka, Bauhaus, Home Depot, Kohler, Villeroy &amp; Boch, Duravit, Hansgrohe, Grohe, Geberit, Victorian Plumbing</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>13, 22</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Hizmet ve kampanya koşulları erişim tarihindeki haliyle aktarılmıştır</t>
-        </is>
+          <t>bauhaus.com.tr</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>244</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Inbound sezonsallık ve rakip ürün analizi</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Haziran 2026 · Ahrefs content gap, 4.202 kelime, 7 rakip</t>
-        </is>
+          <t>cimri.com</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>225</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Dört ürün kümesi güncel veriyle yeniden ölçülmüştür</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+        <v>39</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>146</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Google arama sonuçları</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>109 kelime · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 29.09.2026</t>
-        </is>
+          <t>banyomarka.com</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>221</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Sıralamalar tek günlük gözlemdir ve gün içinde değişebilir; AI Overview içeriği 31 bloğun 24'ünde alınabilmiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+        <v>61</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>149</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>YouTube arama ve yorumlar (genişletilmiş)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>68 ifade · Türkiye · ilk 20 sonuç · 33 videonun 2.218 yorumu · 29.09.2026</t>
-        </is>
+          <t>creavit.com.tr</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>216</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Kanal türü ve yorum teması anahtar ifadelerle atanmıştır; bir yorum birden fazla temaya girebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="43" customHeight="1">
+        <v>105</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>107</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer ve Keywords Explorer (marka siteleri)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>24 marka ve uzman site top pages ve 69 baş kelimenin sıralama verisi · Türkiye · 28.09.2026; bu bölümdeki arama hacimleri Google Keyword Planner (Eyl 2024 - Ağu 2026)</t>
-        </is>
+          <t>shop.creavit.com.tr</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>174</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Sayfalar URL ve en iyi kelimeye göre temalara eşlenmiştir; listelenen sayfalar site toplamının %66-93'ünü kapsar</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+        <v>34</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs Site Explorer (pazaryeri ve yapı market)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>9 site, banyo kategori sayfaları ve kelimeleri · Türkiye · 28.09.2026</t>
-        </is>
+          <t>sikayetvar.com</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>77</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol ve Hepsiburada tarayıcı incelemesi</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Kategori ağacı, arama önerileri, marka filtreleri, mağaza ve çok satan listeleri · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Hepsiburada'da her listede ilk sayfa (36 ürün) okunmuştur; sıralama kişiselleştirmeye bağlı olarak değişebilir</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Şikayetvar</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>VitrA (978) ve Artema (544) marka sayfaları; son 24 ay 600 / 294 şikayetin tam metni · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Tema ataması anahtar ifadeyle; şikayetler tek taraflı beyandır, paylar yön gösterir; kişisel veriler çıkarılmıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Google Shopping</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>27 kategori + 3 marka kelimesi × 120 ilan; 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Mecra medyanı marka ve model karışımından etkilenir; aynı ürün kıyası yalnız satıcı listelerinde</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="43" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol ve Hepsiburada çok satan ve ürün sayfaları</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>14 kategori × 36 ürün × 2 kanal; 29 VitrA ve Artema ürününde 4 kanal liste fiyatı · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Çok satan sırası platform algoritmasıdır; fiyatlar tek günlük liste fiyatıdır, sepet indirimi ayrıca not edilmiştir; Hepsiburada'da ilk sayfa</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="43" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Akakçe ve Cimri</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>29 SKU arama ve ürün sayfası, 12 + 10 kategori sayfası, Cimri 19 ürün sayfası · 30.09.2026</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Akakçe satıcı listesi ilk 16 satıcıyla sınırlıdır; 10 SKU için Cimri kaydı bulunmamaktadır; paket ve set kayıtları fiyat kıyasına alınmamıştır</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="43" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryeri alt kategori taraması</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol 42, Hepsiburada 40, Akakçe 42 + 8, Cimri 30 kategori (ilk 2 sayfa); 6 rakip mağaza 110 kategori sayfası · 30.09.2026</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Çok satan sırası platform algoritmasıdır; aksesuar karışan listeler işaretlidir; mağazalarda Koçtaş dışında varsayılan sıralama; Kale ve IKEA kapsam dışı</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="82" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Resmi mağaza panel verisi</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol satıcı paneli: satış ve sipariş dağılımı (2025 Q4 - 2026 Q3), favori-görüntüleme (2025, 2026), 1.023 ürün ve 149 satıcı değerlendirmesi, 352 ürün sorusu, 44 Enleri listesi · Hepsiburada: hak ediş, görüntülenme, iptal, değerlendirme · 30.09.2026; ürün bazlı satış raporu, son 12 ay · 02.10.2026</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>18, 01, 25</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Yalnız resmi mağaza; ciro tutarı verilmez, pay ve oran kullanılır; temalar anahtar kelimeyle; Enleri ekran görüntüsünden okunmuştur</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="56" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Rehber içerik, soru sorguları ve marka kayıtları</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Search Console /ilham-veren-fikirler/ sayfaları ve "nasıl", "su kaçır" sorguları (1 Eki 2025 - 25 Eyl 2026); Wikidata ve Wikipedia VitrA ve Artema kayıtları; vitra.com.tr llms.txt ve site haritaları · 02.10.2026</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Rehber sayfaları adres yapısına göre konu gruplarına ayrılmıştır; en az 5 tık alan 93 sayfa değerlendirilmiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="56" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Alt kategori tamamlayıcı taraması</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>vitra.com.tr 55 kategori + 3 özel sayfa; Trendyol, Hepsiburada, Akakçe, Cimri aramaları (57 kesit); 6 rakip mağaza araması; 11.982 ürün satırı · 30.09.2026</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Kategori sayfası olmayan kesitlerde arama sırası; eşleşme ürün adında kesit anahtar sözcüğüyle; Cimri'de 17 kesitte veri bulunmamaktadır; stok sayımı süzgeç ve "Gelince Haber Ver" işaretine dayanır</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="43" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Site politika sayfaları, sosyal profiller, Google Maps ve SERP</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>13 site ve markanın ödeme, teslimat, iade, garanti ve servis sayfaları; 7 markanın sosyal hesapları; 103 Maps sorgusu; 15 + 10 kelime SERP · 29.09.2026</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Değerler 29-30.09.2026'da sitelerden okunmuştur; Instagram ve TikTok sayıları yaklaşıktır</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="43" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Similarweb site trafiği</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>31 alan adı: marka, uzman, yapı market, pazaryeri ve fiyat karşılaştırma siteleri; aylık ziyaret, kanal kırılımı, etkileşim · Haz - Ağu 2026 · 03.10.2026</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Ziyaretler tüm ülkeleri kapsayan tahminlerdir; aylık ziyareti ~35 binin altındaki 9 sitede kanal dağılımı modellendiği için gösterilmemiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="69" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Pazaryeri yorum ve soru-cevap kayıtları</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Trendyol ve Hepsiburada'da VitrA, Artema ve rakip markaların 665 ürün sayfası: 12.673 yorum (9.047 metinli), 4.912 soru-cevap; VitrA resmi mağaza Trendyol paneli dahil · 03.10.2026</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Duygu puandan türetilmiştir (4-5 olumlu, 1-2 olumsuz); temalar anahtar ifade kurallarıyla atanmıştır; rakip örneklemi çok satan ve en çok değerlendirilen ürünlerdir; ürün başına en fazla 50-100 yorum ve 20 soru; yorumcu adları kaydedilmemiştir</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="43" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>TCMB EVDS</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Kart harcamaları, kartlı ödeme endeksi, tüketici eğilimi, konut, banka kredileri, hane halkı beklentileri · 2024-2026</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Kart harcamaları nominaldir; reel karşılaştırma için kartlı ödeme endeksinin reel serisi kullanılmıştır</t>
-        </is>
+        <v>36</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5103,7 +4298,2444 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AI Arama ve GEO Fırsatları · Satın alma ve montaj sorularında VitrA ve vitra.com.tr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="230" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: AI Arama ve GEO Fırsatları · Satın alma ve montaj sorularında VitrA ve vitra.com.tr
+Kapsam: Google AI Overview, Gemini ve ChatGPT gibi yapay zeka yanıtları kullanıcının sorusunu birden fazla kaynaktan derlenen tek bir cevapla karşılamaktadır. Bu cevaplarda kaynak gösterilmek, soruyu doğrudan cevaplayan sayfaya, markanın tutarlı tanımlanmasına ve markadan site dışında söz edilmesine bağlıdır. Değerlendirme vitra.com.tr rehber içeriklerinin Search Console performansına (1 Eki 2025 - 25 Eyl 2026), 29.09.2026 AI Overview gözlemine ve 02.10.2026 tarihli marka kayıtlarına dayanmaktadır.
+Kaynak: Google Search Console · /ilham-veren-fikirler/ sayfaları ve soru sorguları, 1 Eki 2025 - 25 Eyl 2026 · Google arama sonuçları ve AI Overview, 107 kelime, 29.09.2026 · Yapay zeka yanıt takibi, 125 soru, ChatGPT, Gemini ve Google AI Overview, 4 Eyl - 3 Eki 2026 · Wikidata ve Wikipedia, 02.10.2026 · vitra.com.tr llms.txt ve site haritaları, 02.10.2026 · Şikayetvar, YouTube ve Google Shopping verileri ilgili bölümlerdeki kaynaklardandır 13 , 16 , 17 , 41 , 52 , 53 , 54 , 55
+Sütun açıklamaları: Soru metni: Yapay zeka platformlarına sorulan soru; kullanıcının yazdığı biçimde korunmuştur. | Grup: Satın alma ve teslimat soruları ile montaj soruları. | Markalı: Soruda VitrA adı geçiyor mu? | VitrA adı geçen: VitrA'nın adıyla geçtiği yanıt / toplam yanıt (ChatGPT, Gemini ve AI Overview birlikte). | vitra.com.tr kaynak: vitra.com.tr'nin kaynak gösterildiği yanıt / toplam yanıt. | Pazaryeri kaynak: Trendyol, Hepsiburada, Koçtaş, n11, Amazon, Bauhaus, Akakçe veya Cimri'nin kaynak gösterildiği yanıt / toplam yanıt.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Soru metni</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Grup</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Markalı</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>VitrA adı geçen</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>vitra.com.tr kaynak</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Pazaryeri kaynak</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>banyo ürünlerinde iade ve değişim nasıl yapılır online alışverişte</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>1 / 20</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0 / 20</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>8 / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı online mı mağazadan mı almak daha mantıklı</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>3 / 20</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>1 / 20</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>4 / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>online alınan klozet nasıl teslim edilir kargo hasarı olur mu</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>3 / 18</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2 / 18</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>3 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>banyo yenileme için montaj hizmeti de veren markalar</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>6 / 17</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>4 / 17</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>8 / 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>internetten banyo dolabı sipariş edenlerin yorumları</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>6 / 16</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>2 / 16</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>16 / 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>komple banyo takımı seti fiyatları ve nereden alınır</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>7 / 18</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>4 / 18</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>16 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı taksitle nereden alınır</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>9 / 20</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>6 / 20</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>17 / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>internetten klozet almak mantıklı mı</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>9 / 18</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>6 / 18</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>8 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>banyo mobilyası kargo ile gelir mi kurulum var mı</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>11 / 21</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>8 / 21</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>8 / 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>klozet nereden alınır en uygun fiyata</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>14 / 20</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>5 / 20</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>19 / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>klozet ve lavabo kampanyalı fiyat nereden bulunur</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>16 / 18</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>7 / 18</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>17 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>gömme rezervuar tamiri için kime başvurulur</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>17 / 18</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>4 / 18</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>0 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>klozet montajı dahil satış yapan siteler</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>20 / 21</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>17 / 21</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>19 / 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>banyo ürünleri alırken hangi siteye güvenilir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>20 / 20</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>8 / 20</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>12 / 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>vitra yetkili servis ve yedek parça nasıl bulunur</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>12 / 16</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>12 / 16</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>5 / 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>vitra ürünleri kendi sitesinden mi trendyol'dan mı alınır</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>16 / 18</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>10 / 18</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>14 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>vitra ürünlerini uygun fiyata nereden alabilirim</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>16 / 17</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>14 / 17</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>15 / 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>vitra bayi mi internet sitesi mi daha ucuz</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>16 / 16</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>15 / 16</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>11 / 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>vitra klozet garanti süresi ve garanti kapsamı</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>16 / 16</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>16 / 16</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>1 / 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>vitra klozet trendyol mu hepsiburada mı daha uygun</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Satın alma</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>18 / 18</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>1 / 18</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>18 / 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>banyo dolabı montajı</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>5 / 17</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0 / 17</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>4 / 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>klozet montajı nasıl yapılır</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>6 / 15</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>10 / 15</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>7 / 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>lavabo montajı nasıl yapılır</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>7 / 15</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>10 / 15</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>0 / 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>klozet kapağı montajı</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>10 / 15</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>9 / 15</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>3 / 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Banyo dolabı montajında teknik rehberliği en iyi olan mobilya markaları hangileri?</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>12 / 17</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>8 / 17</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>6 / 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>kumanda paneli montajı</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>11 / 15</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>3 / 15</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>2 / 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>lavabo bataryası montajı nasıl yapılır</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>13 / 17</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>12 / 17</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>3 / 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Kendi başına lavabo bataryası takmak isteyenler için en uygun markalar neler?</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>12 / 13</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>6 / 13</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>11 / 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Gömme rezervuar montajı için en güvenilir ve kolay kurulumlu markalar hangileridir?</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Montaj</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>14 / 14</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>9 / 14</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>6 / 14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet111.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sonraki Adımlar · Tablo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="104" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Sonraki Adımlar
+Kapsam: Aksiyonlar üç öncelik kademesinde verilmiştir; sıralama VitrA ekibinin stratejik tercihleri, pazaryeri ve GA4 verisiyle güncellenebilir. Öncelik 1 maddeleri mevcut altyapı ve mevcut talep üzerinde kısa vadede etki üretebilecek düzenlemelerdir.
+Sütun açıklamaları: Öncelik: Etki ve uygulanabilirlik birlikte değerlendirilerek verilen sıra. | Aksiyon: Önerilen düzenleme. | Dayanak: Öneriyi destekleyen bulgu ve kaynak. | Beklenen etki: Düzenlemenin hedeflediği sonuç.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Öncelik</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Aksiyon</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Dayanak</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Beklenen etki</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="69" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Yedek parça kategorisi ve ürün koduna göre parça bulucu; eski yedek parça adresinin bu kategoriye yönlendirilmesi</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>İç takım ve yedek parça aramaları aylık 113K; eski yedek parça sayfası Haziran - Kasım 2025'te Search Console'a göre ayda ~300 tık almış, bugün tek ürünlü kategoriye yönlenmektedir; Trendyol aramasında VitrA iç takımda ilk sıradadır 9 , 10 , 11 , 19 , 47 , 48</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Mevcut müşteriden tekrar satış ve marka savunması</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>"Banyo yenileme paketi": ürün seti + montaj + keşif tek teklifte; Banyo Asistanı paketin giriş kapısı</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Montaj, keşif, ücretsiz montajlı mobilya ve Banyo Asistanı mevcut ama ayrı sunuluyor; tasarım ve tadilat aramaları büyüyor; Koçtaş, Bauhaus ve Kohler proje satışına geçmiş 10 , 19 , 22 , 27 , 29</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sepet büyüklüğü ve kanal farklılaşması</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Keşif ve montajın ölçüye bağlı ürün sayfalarına bağlanması; duşakabin, küvet ve duş teknesi için montaj kalemi</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Duşakabin talebi aylık 285K; duşakabin ürün sayfasında montaj ya da keşif seçeneği bulunmuyor 10 , 19</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Hacimli üründe karar öncesi belirsizliğin azalması</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayfasına garanti süresi, yedek parça ve servis girişi; servis ücreti ve garanti reddi sürecinde standart metin</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Şikayetvar'da servis ve garanti teması %54,7, yedek parça %8,1'den %17,8'e; ürün sayfalarında garanti süresi yazmıyor, E.C.A. 20 yıl ve Grohe 48 saat parça teslimi yazıyor 17 , 44</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Satış sonrası güven ve tekrar satın alma</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri fiyat ve satıcı izleme: aynı SKU'da resmi mağaza ile 3P farkının düzenli takibi, yetkili satıcı listesi ve hukuki değerlendirmeyle fiyat politikası çerçevesi</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>29 üründen 19'unda en ucuz kanal pazaryeri (medyan %24,7); Trendyol'da VitrA mağazasıyla birlikte bulunan 6 üründe 3P daha ucuz; Hepsiburada'da aynı ürün için birden fazla katalog kaydı 41 , 42</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Kanal başına tutarlı fiyat algısı</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="69" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Kategori sayfalarında stok görünürlüğü: stokta olmayan varyantların ürün sayısı ve fiyat aralığından ayrılması, "Gelince Haber Ver" kartlarının listenin sonuna alınması; "Sepette %N" etiketi yerine kartta net fiyat</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>55 kategori sayfasındaki 2.258 varyant kartının %71,1'i stoklu süzgeci dışında; 13 alt kategoride stoklu ürün yok; ilk sayfa kartlarının %89,9'unda "Sepette %N indirim" etiketi; aynı model kodunda pazaryeri fiyatı liste fiyatının medyan %14,4 altında, sepet fiyatına yakın 37</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Kategori sayfasından ürün sayfasına geçişte daha az "stokta yok" karşılaşması; kanallar arası fiyat algısının tekleşmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>AI aramada görünürlük için sorun çözen içerik: arıza, montaj, uyumluluk ve garanti konularında destek sayfaları; ölçü, seçim ve marka sorularında rehber içerik</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Rehber sayfalarında tıkların %35'i montaj, tamir ve temizlik yazılarından geliyor; destek bölümünde bu konularda sayfa yok; soru sorgularında site ilk sayfada ama CTR %0,93; VitrA 23 AI Overview'un 7'sinde kaynak 13 , 17 , 52</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>AI yanıtlarında kaynak gösterilme, tamir anında trafik ve satış sonrası başvurunun siteye dönmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="43" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Öncelik 1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Marka ve entity tutarlılığı: Wikidata ve Wikipedia kayıtlarının VitrA ve Artema için güncel ve tutarlı hale getirilmesi</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Wikidata'da iki ayrı VitrA kaydı var ve ana kayıtta resmi web sitesi vitra.com.tr'yi göstermiyor; Artema'nın kaydı yok 54</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>AI yanıtlarında markanın doğru tanımlanması</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Taksit mesajının tüm temas noktalarında tekleştirilmesi</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Üst bantta "vade farksız 6 ay", Banyo Asistanı kampanya sayfasında "9 taksit", ürün sayfasındaki taksit tablosunda 12 taksite kadar; kullanıcı "vitra 9 taksit" ve "vitra taksit seçenekleri" arıyor 12 , 19</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Fiyat algısında netlik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Kanal rolleri ve fiyat tutarlılığı; BM'de pazaryerinde fiyat yerine set, montaj ve garanti ile konumlanma</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>BM aramalarının %9,6'sı perakendeci adıyla yapılıyor; Trendyol'da banyo dolabı medyanı 3.249 TL, VitrA 14.462 TL; Hepsiburada'da VitrA ürünlerinin %69'u üçüncü taraf satıcıda 9 , 10 , 30 , 34 , 35</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Kanal başına net değer önerisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="82" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri ürün kartı standardı: kutu içeriği ("kapak ve rezervuar dahil değildir") başlık ve ilk görselde; klozet kodu ile uyumlu kapak ve iç takım eşleşme listesi; ölçü tablosu</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol iadelerinin %27,6'sında neden ölçü, %19,2'sinde yanlış sipariş; Eylül 2026'daki 352 ürün sorusunun 83'ü uyumluluk; ilan görselinde kapak ve rezervuar görünen klozetlerde "sadece klozet geldi" şikayeti; iki pazaryerindeki VitrA sorularının %31,9'u uyumluluk ve kullanım yeri, %18,3'ü kutu içeriği 38 , 40</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>İade ve soru yükünde azalma, düşük puanlı yorumlarda gerileme</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Kırılgan ürün paketleme standardı ve eksik parça kontrolü; hasarlı teslimde parça veya değişim akışı</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Kırık ve hasar temalı yorumların ortalama puanı 2,3 (36 yorum); cam aksesuar, lavabo ve klozet kapağı kırık teslim; vida, dübel, dolap ayağı, flex hortum eksikleri; satıcı değerlendirmesinde olumsuz etkilerin ilk üçü kusurlu, eksik ve yanlış ürün; pazaryeri yorumlarında VitrA ve Artema banyo dolabı olumsuz payı %17,9 (rakipler %7,5), bu yorumların %58,0'ı kırık veya hasarlı ürün 38 , 40</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Marka algısının korunması, iade maliyetinde azalma</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="43" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada'da VitrA ve Artema ürünlerine gelen soruların resmi mağaza tarafından takip edilmesi; sık sorulara ürün sayfasında hazır yanıt</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada'da VitrA ürünlerine gelen soruların %29,5'i resmi mağaza tarafından cevaplanmış, kalan sorular aynı ürünü satan diğer satıcılarca yanıtlanmıştır 40</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Ürün bilgisinin tek kaynaktan verilmesi, yanlış eşleşmeden kaynaklanan iadelerde azalma</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryerinde stok sürekliliği ve liste görünürlüğü: çok satanlarda stok takibi, mobilya, batarya, duş ve evye bataryası listelerine giriş ürünleri, conta ve iç takım parçalarının resmi mağazada listelenmesi</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2026 Q3'te satılan ürünlerin 86'sında stok 0 (Q3 cirosunun %26,7'si); resmi mağaza 5 kategorinin Eylül listelerinde yok; rezervuar çok satan listesinin 2. sırası üçüncü taraftaki 71 TL'lik VitrA contası 38</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Resmi mağazanın kategori listelerinde yer alması, buybox ve yedek parça talebinin resmi kanala dönmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Google Merchant Center feed'inin tüm kategorileri kapsaması, başlıklarda kategori kelimesi; AI alışveriş yanıtları için zengin ürün bilgisi</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>VitrA sitesi Shopping listelemelerinin %0,7'si; klozet kapağı, duşakabin, duş seti, iç takım, havlupan ve evye dahil 15 kelimede hiç görünmüyor; SERP'te Shopping bloğu henüz çıkmıyor 41 , 44</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Ücretsiz listelemelerde hazır olma</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="43" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Google Business Profile standardı: bayi profillerinde ad ve kategori, web sitesi alanı, yorum toplama ve yanıt akışı</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Maps'te 262 VitrA etiketli profil, 123'ünde 10'dan az yorum, 18'inde puan 4,0 altı; 57 profilde web alanı başka adres 44</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Banyo Asistanı mağaza adımına yerel görünürlük</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Kategori sayfalarında ilk 3 dışında kalan baş kelimeler için sayfa kurgusu; armatürde VitrA ve Artema görünürlüğü</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Banyo dolabı aylık 98.625 arama ve VitrA 5. sırada, duşakabin 4., klozet kapağı 6.; taharet musluğunda VitrA ilk sayfada yok, banyo ve lavabo bataryasında 3. sırada; baş kelimelerin çoğunda KD 0-2 13 , 32</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Mevcut kategori talebinden daha yüksek organik pay</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="43" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Katalog derinliği: hela taşı ve havlupanda ürün derinliği, çamaşır makinesi dolabının pazaryerinde listelenmesi</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Hela taşı 64,4K arama / 1 ürün, havlupan 50,7K arama / 2 ürün, çamaşır makinesi dolabı 103K arama / 29 ürün ama Trendyol ilk 40'ta yok 9 , 10 , 19</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Mevcut talebin karşılanması</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="82" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Kategori adlandırmasında pazaryeri karşılıkları ve sayfası olmayan kesitler: sıva üstü batarya, fotoselli batarya, jakuzi, duş sistemi, ayaklı lavabo eş anlamlıları; çocuk klozet, engelli klozet, köşe lavabo ve lavabo ayağı için ayrı sayfa; /c-online-ozel yönlendirme döngüsü</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr "Duvardan banyo bataryaları" ile pazaryerinde "sıva üstü banyo bataryası", "Temassız" ile "fotoselli" (Trendyol 994, Hepsiburada 588 sonuç); çocuk klozeti aramasında Trendyol 2.238, Hepsiburada 1.659 sonuç; engelli klozeti Trendyol'da 43 ürünlük ayrı kategori; dört başlığın sitede ayrı sayfası yok 13 , 37</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Kullanıcının aradığı adla eşleşen kategori sayfası; organik ve pazaryeri aramasında bulunabilirlik</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Erişilebilir banyo ve çocuk banyosu sayfaları (Conforma, tutunma barları, Sento çocuk)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Yaşlı ve engelli ürünleri aylık 29,4K (YoY +%8,1 ); ürünler katalogda var ama tek sayfada toplanmıyor 10 , 19</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Niş ve büyüyen segmentte görünürlük</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="69" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>YouTube tamir serisi ve tesisatçı kanallarıyla iş birliği</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>En çok izlenen 14 tamir ve kurulum konusunun hiçbirinde VitrA kanal videosu yok (sifon ve iç takım 6,8M, batarya ve kartuş 7,0M izlenme); görünmelerin %43,7'si tesisatçı kanallarında; Macit Tesisat'ın VitrA tamir videosu 447K izlenme 14 , 15 , 16</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Tamir anında marka görünürlüğü</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="43" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Site dışı sinyaller: Şikayetvar yanıtları, YouTube tamir içerikleri ve rehber sitelerinde uzman içerik</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Şikayetvar puanı 18; en çok izlenen 14 tamir ve kurulum konusunda VitrA kanal videosu yok; AI Overview kaynakları arasında markadan bağımsız rehber siteleri var 13 , 16 , 17</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Markanın site dışında anılması ve AI yanıtlarında kaynak çeşitliliği</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="43" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Öncelik 2</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Banyo Asistanı'nın bayi ağına genişletilmesi ve adımlarının GA4'te ölçülmesi</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Mağaza seçeneğinde 5 VitrA mağazası listeleniyor; servisler ve satış noktaları sayfası 1 Haziran 2025 - 25 Eylül 2026 döneminde 37.859 tık almıştır 11 , 19</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Lead'in satışa dönmesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="43" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Granit ve çelik evye + mutfak bataryası seti</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Evye talebi aylık 225K; VitrA evye hattı seramikle sınırlı; Trendyol'da granit evye kategorisi olgunlaşmamış 9 , 10 , 21</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Mutfakta set satışı</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="43" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Arıtmalı batarya ve filtre aboneliği</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Arıtmalı batarya aramaları üç yılda +%10,7 ; su arıtma talebi aylık 554K; Trendyol'da arıtmalı batarya aramasının ilk 40 sonucunda armatür markası bulunmamaktadır 9 , 10 , 21</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Tekrarlı gelir</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="43" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Banyo planlayıcının (V-Design) yeniden devreye alınması ve Banyo Asistanı'na bağlanması</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Banyo tasarım ve planlama aramaları YoY +%22,8 ; /banyonu-tasarla adresi ana sayfaya yönleniyor; V&amp;B, Duravit ve IKEA planlayıcı sunuyor 10 , 19 , 45 , 46</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Ürün keşfinden lead'e geçiş</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Tamamlayıcı ürünlerde üçüncü taraf satıcı modelinin montaj malzemesi ve yapı kimyasalında test edilmesi</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Yapıştırıcı, derz ve su yalıtımı aramaları YoY +%12,8 ; montaj parçaları yapı marketten tamamlanıyor 10 , 12</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Sepet bütünlüğü</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Ledli ayna, aydınlatma ve koleksiyon uyumlu havlupan derinliği</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Ledli ayna ve aydınlatma aramaları üç yılda +%13,1 ; Trendyol'da ledli ayna medyanı 1.650 TL 9 , 10</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>BM setine bağlı ek satış</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="43" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Yenileme paketinde iş ortağı ürünleri (şofben, termosifon, tekstil, düzenleme)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Şofben ve termosifon aylık 540K, tekstil 338K, düzenleme 216K; Koçtaş bu ürünleri tadilat sayfasında topluyor 10 , 22</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Tadilat sepetinin tamamlanması</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>V-Care için deneyim modeli ve universal akıllı kapağın izlenmesi</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Akıllı klozet seti aramaları üç yılda +%103,8 ; Geberit AquaClean 4 hafta evde deneme sunuyor 7 , 49</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Premium segmentte dönüşüm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="43" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Satın alan müşteriye ürün ömrüne göre yenileme ve yedek parça hatırlatması; olumsuz deneyim sonrası tekrar sipariş oranının izlenmesi</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Konut tamiratı niyeti yükselmekte, ipotekli konut satışları artmaktadır; mevcut müşteri tabanı yenileme adayı olarak değerlendirilebilir 3 , 4</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Yaşam boyu değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Öncelik 3</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Karo, mutfak tezgahı ve yapı kimyasalında kategori genişlemesinin değerlendirilmesi</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Karoda Kale 59.089, VitrA 28.950 aylık organik ziyaret; "mutfak tezgahı" aylık 24.242 arama ve VitrA'da sayfa yok; Kalekim yapı kimyasalı sayfalarıyla 20.829 ziyaret alıyor 32</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Karo trafiğinden çapraz satış</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet112.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Yöntem ve Kapsam · Tablo 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="62" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bölüm: Yöntem ve Kapsam
+Kapsam: Veri kaynaklarına, dönemlerine ve yöntem notlarına aşağıda yer verilmektedir.
+Sütun açıklamaları: Veri kaynağı: Kullanılan kaynak. | Kapsam: Dönem, coğrafya ve örneklem. | Kullanıldığı bölüm: Verinin işlendiği bölüm. | Not: Ölçüm sınırı veya yöntem notu.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Veri kaynağı</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kapsam</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Kullanıldığı bölüm</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads Keyword Planner</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2.342 tekil kelime · Türkiye, Türkçe · aylık hacim Eyl 2022 - Ağu 2026 (talep grafiğinde Oca 2023 - Ağu 2026)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>03, 04, 05, 23</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads yakın yazım varyantlarına (çoğul, yazım farkı) aynı aylık seriyi döndürür; aynı seriye sahip kelimeler tek kelime olarak sayılmıştır (2.419 satırdan 2.342 tekil kelime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Google Search Console</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>sc-domain:vitra.com.tr · 1 Haz 2025 - 25 Eyl 2026 · sayfa, sorgu, cihaz, ülke</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>05, 06, 07, 08, 22, 23, 25</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sayfa ve sorgu raporları ilk 25.000 satırla sınırlıdır; sayfa×gün tablosu 100.000 satır</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="43" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Google Autocomplete</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>66 kök ifade: "vitra" ile başlayan 14 (28.09.2026) ve kategori, hizmet, fiyat, rakip marka ve perakendeci için 52 (30.09.2026) · Türkiye, Türkçe, masaüstü Chrome</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>07, 23</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Öneriler tek günlük anlık görüntüdür; sıralama Google'ın sırasıdır</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>30 ifade · Türkiye · ilk sayfa · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>İzlenme sayıları video yayın tarihinden itibaren kümülatiftir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Organik rakipler ve Batch Analysis · Türkiye · 27.09.2026</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Organik ve paid trafik değerleri Ahrefs tahminidir; gerçek ziyaret sayısı değildir</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Google Ads keyword ideas</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>10 kök ifade grubu, 52.973 kelime · 48 ay (Eyl 2022 - Ağu 2026)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>04, 11, 12, 13</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Kelimeler 58 temalı sözlükle sınıflandırılmış, gürültü ifadeleri ayıklanmış, aynı aylık seriyi taşıyan yazım varyantları tek sayılmıştır; tema toplamları yaklaşık büyüklük gösterir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr ürün sitemap'i ve site incelemesi</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>7.804 ürün adresi · hizmet, kategori ve ürün sayfaları · Banyo Asistanı · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>11, 13, 22, 23</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Ürün sayısı renk ve ölçü varyantlarını ayrı sayar; model sayısı renk ekleri ayıklanarak yaklaşık hesaplanmıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Rakip kategori sitemap'leri</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Bauhaus, IKEA, Tekzen, Evidea, Banyomarka, Kale, Banyoline · Koçtaş tarayıcı ile</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>12, 22</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Kategori varlığı gözlemidir; ürün derinliği ve satış hacmi ölçülmemiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol arama sonuçları</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>13 tema, ilk 40-45 ürün · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>04, 11, 12</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Değerlendirme sayısı satış hacmine yaklaşık gösterge olarak kullanılmıştır; sonuç sırası kişiselleştirmeye bağlı olarak değişebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="43" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Rakip ve benzer oyuncuların siteleri</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Koçtaş, IKEA, Hepsiburada, Kale, Banyomarka, Bauhaus, Home Depot, Kohler, Villeroy &amp; Boch, Duravit, Hansgrohe, Grohe, Geberit, Victorian Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>13, 22</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Hizmet ve kampanya koşulları erişim tarihindeki haliyle aktarılmıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Inbound sezonsallık ve rakip ürün analizi</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Haziran 2026 · Ahrefs content gap, 4.202 kelime, 7 rakip</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Dört ürün kümesi güncel veriyle yeniden ölçülmüştür</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="43" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Google arama sonuçları</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>107 kelime (dokuz temadan seçilen, Keyword Planner'da hacmi olan) · Türkiye, Türkçe, mobil · ilk 20 organik sonuç, AI Overview, PAA · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Sıralamalar tek günlük gözlemdir ve gün içinde değişebilir; AI Overview içeriği 30 bloğun 23'ünde alınabilmiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="43" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Yapay zeka yanıt takibi</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>125 soru (111 markasız, 14 VitrA adıyla) · ChatGPT, Gemini ve Google AI Overview · günlük koşu, 4 Eyl - 3 Eki 2026; satın alma ve montaj soruları 28.09.2026'dan itibaren</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Yanıtlar kişiselleştirilmemiş oturumlardan alınmıştır ve aynı soruya gün içinde farklı yanıt verilebilir; oranlar yön göstericidir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>YouTube arama ve yorumlar (genişletilmiş)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>68 ifade · Türkiye · ilk 20 sonuç · 33 videonun 2.218 yorumu · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Kanal türü ve yorum teması anahtar ifadelerle atanmıştır; bir yorum birden fazla temaya girebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="43" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer ve Keywords Explorer (marka siteleri)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>24 marka ve uzman site top pages ve 69 baş kelimenin sıralama verisi · Türkiye · 28.09.2026; bu bölümdeki arama hacimleri Google Keyword Planner (Eyl 2024 - Ağu 2026)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Sayfalar URL ve en iyi kelimeye göre temalara eşlenmiştir; listelenen sayfalar site toplamının %66-93'ünü kapsar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Ahrefs Site Explorer (pazaryeri ve yapı market)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>9 site, banyo kategori sayfaları ve kelimeleri · Türkiye · 28.09.2026</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Kategori trafiği listelenen sayfalarla sınırlıdır ve alt sınır olarak okunmalıdır</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol ve Hepsiburada tarayıcı incelemesi</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Kategori ağacı, arama önerileri, marka filtreleri, mağaza ve çok satan listeleri · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Hepsiburada'da her listede ilk sayfa (36 ürün) okunmuştur; sıralama kişiselleştirmeye bağlı olarak değişebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Şikayetvar</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>VitrA (978) ve Artema (544) marka sayfaları; son 24 ay 600 / 294 şikayetin tam metni · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Tema ataması anahtar ifadeyle; şikayetler tek taraflı beyandır, paylar yön gösterir; kişisel veriler çıkarılmıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Google Shopping</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>27 kategori + 3 marka kelimesi × 120 ilan; 24 satıcı listesi · Türkiye, masaüstü · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Mecra medyanı marka ve model karışımından etkilenir; aynı ürün kıyası yalnız satıcı listelerinde</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="43" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol ve Hepsiburada çok satan ve ürün sayfaları</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>14 kategori × 36 ürün × 2 kanal; 29 VitrA ve Artema ürününde 4 kanal liste fiyatı · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Çok satan sırası platform algoritmasıdır; fiyatlar tek günlük liste fiyatıdır, sepet indirimi ayrıca not edilmiştir; Hepsiburada'da ilk sayfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="43" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Akakçe ve Cimri</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>29 SKU arama ve ürün sayfası, 12 + 10 kategori sayfası, Cimri 19 ürün sayfası · 30.09.2026</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Akakçe satıcı listesi ilk 16 satıcıyla sınırlıdır; 10 SKU için Cimri kaydı bulunmamaktadır; paket ve set kayıtları fiyat kıyasına alınmamıştır</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="43" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri alt kategori taraması</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol 42, Hepsiburada 40, Akakçe 42 + 8, Cimri 30 kategori (ilk 2 sayfa); 6 rakip mağaza 110 kategori sayfası · 30.09.2026</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Çok satan sırası platform algoritmasıdır; aksesuar karışan listeler işaretlidir; mağazalarda Koçtaş dışında varsayılan sıralama; Kale ve IKEA kapsam dışı</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="82" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Resmi mağaza panel verisi</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol satıcı paneli: satış ve sipariş dağılımı (2025 Q4 - 2026 Q3), favori-görüntüleme (2025, 2026), 1.023 ürün ve 149 satıcı değerlendirmesi, 352 ürün sorusu, 44 Enleri listesi · Hepsiburada: hak ediş, görüntülenme, iptal, değerlendirme · 30.09.2026; ürün bazlı satış raporu, son 12 ay · 02.10.2026</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>18, 01, 25</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Yalnız resmi mağaza; ciro tutarı verilmez, pay ve oran kullanılır; temalar anahtar kelimeyle; Enleri ekran görüntüsünden okunmuştur</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Rehber içerik, soru sorguları ve marka kayıtları</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Search Console /ilham-veren-fikirler/ sayfaları ve "nasıl", "su kaçır" sorguları (1 Eki 2025 - 25 Eyl 2026); Wikidata ve Wikipedia VitrA ve Artema kayıtları; vitra.com.tr llms.txt ve site haritaları · 02.10.2026</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Rehber sayfaları adres yapısına göre konu gruplarına ayrılmıştır; en az 5 tık alan 93 sayfa değerlendirilmiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Alt kategori tamamlayıcı taraması</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>vitra.com.tr 55 kategori + 3 özel sayfa; Trendyol, Hepsiburada, Akakçe, Cimri aramaları (57 kesit); 6 rakip mağaza araması; 11.982 ürün satırı · 30.09.2026</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Kategori sayfası olmayan kesitlerde arama sırası; eşleşme ürün adında kesit anahtar sözcüğüyle; Cimri'de 17 kesitte veri bulunmamaktadır; stok sayımı süzgeç ve "Gelince Haber Ver" işaretine dayanır</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="43" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Site politika sayfaları, sosyal profiller, Google Maps ve SERP</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>13 site ve markanın ödeme, teslimat, iade, garanti ve servis sayfaları; 7 markanın sosyal hesapları; 103 Maps sorgusu; 15 + 10 kelime SERP · 29.09.2026</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Değerler 29-30.09.2026'da sitelerden okunmuştur; Instagram ve TikTok sayıları yaklaşıktır</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="43" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Similarweb site trafiği</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>31 alan adı: marka, uzman, yapı market, pazaryeri ve fiyat karşılaştırma siteleri; aylık ziyaret, kanal kırılımı, etkileşim · Haz - Ağu 2026 · 03.10.2026</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Ziyaretler tüm ülkeleri kapsayan tahminlerdir; aylık ziyareti ~35 binin altındaki 9 sitede kanal dağılımı modellendiği için gösterilmemiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="69" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Pazaryeri yorum ve soru-cevap kayıtları</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Trendyol ve Hepsiburada'da VitrA, Artema ve rakip markaların 665 ürün sayfası: 12.673 yorum (9.047 metinli), 4.912 soru-cevap; VitrA resmi mağaza Trendyol paneli dahil · 03.10.2026</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Duygu puandan türetilmiştir (4-5 olumlu, 1-2 olumsuz); temalar anahtar ifade kurallarıyla atanmıştır; rakip örneklemi çok satan ve en çok değerlendirilen ürünlerdir; ürün başına en fazla 50-100 yorum ve 20 soru; yorumcu adları kaydedilmemiştir</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="43" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>TCMB EVDS</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Kart harcamaları, kartlı ödeme endeksi, tüketici eğilimi, konut, banka kredileri, hane halkı beklentileri · 2024-2026</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Kart harcamaları nominaldir; reel karşılaştırma için kartlı ödeme endeksinin reel serisi kullanılmıştır</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet113.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5393,7 +7025,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Google arama sonuçları · 109 kelime, ilk 20 organik sonuç, AI Overview ve SERP özellikleri · Türkiye, Türkçe, mobil · 29.09.2026</t>
+          <t>Google arama sonuçları · 107 kelime, ilk 20 organik sonuç, AI Overview ve SERP özellikleri · Türkiye, Türkçe, mobil · 29.09.2026</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -6189,17 +7821,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Wikidata ve Wikipedia · VitrA (Q7937213, Q127325081), Türkçe ve İngilizce VitrA maddeleri, Artema araması · 02.10.2026</t>
+          <t>Yapay zeka yanıt takibi · 125 banyo ve satın alma sorusu (14'ü VitrA adıyla) · ChatGPT, Gemini ve Google AI Overview yanıtları, adı geçen markalar ve kaynak gösterilen alan adları · 4 Eyl - 3 Eki 2026</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>https://www.wikidata.org/wiki/Q7937213 · https://www.wikidata.org/wiki/Q127325081 · https://tr.wikipedia.org/wiki/VitrA · https://en.wikipedia.org/wiki/VitrA_(sanitaryware)</t>
+          <t>https://chatgpt.com · https://gemini.google.com · https://www.google.com.tr</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Erişim 02.10.2026</t>
+          <t>Erişim 28.09.2026</t>
         </is>
       </c>
     </row>
@@ -6209,15 +7841,35 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
+          <t>Wikidata ve Wikipedia · VitrA (Q7937213, Q127325081), Türkçe ve İngilizce VitrA maddeleri, Artema araması · 02.10.2026</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q7937213 · https://www.wikidata.org/wiki/Q127325081 · https://tr.wikipedia.org/wiki/VitrA · https://en.wikipedia.org/wiki/VitrA_(sanitaryware)</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Erişim 02.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="43" customHeight="1">
+      <c r="A59" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
           <t>vitra.com.tr · llms.txt, robots.txt, site haritaları (ilham, destek) · 02.10.2026</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>https://www.vitra.com.tr/llms.txt · https://www.vitra.com.tr/sitemaps/sitemap-ilham.xml · https://www.vitra.com.tr/sitemaps/sitemap-support.xml</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Erişim 02.10.2026</t>
         </is>
@@ -8656,15 +10308,15 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Makro Ortam ve Ödeme Gücü · Konut hareketliliği ve kredi koşulları</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="132" customHeight="1">
+          <t>Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Konut hareketliliği ve kredi koşulları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Makro Ortam ve Ödeme Gücü · Konut hareketliliği ve kredi koşulları
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
+          <t>Bölüm: Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Konut hareketliliği ve kredi koşulları
+Kapsam: Bu bölüm, banyo ürünlerine olan talebi etkileyen genel ekonomik koşulları özetlemektedir: insanların kartla ne kadar harcadığı, ekonomiye güvenleri ve evlerini tamir ettirme niyetleri, konut alım-satımı ve bankaların kredi verme koşulları. Banyo yenilemesi ertelenebilen bir harcama olduğu için bu göstergeler, kategori aramalarındaki daralmanın (Bölüm 03) arka planını açıklamaya yardımcı olur. Veriler Türkiye Cumhuriyet Merkez Bankası'nın veri sisteminden (TCMB EVDS) alınmıştır.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Gösterge: TCMB EVDS'den alınan seri. | Değer: Belirtilen dönem için değer. | Karşılaştırma: Bir önceki dönem veya bir yıl önceki değer. | Okuma: Banyo kategorisi açısından kısa yorum.</t>
         </is>
@@ -10402,13 +12054,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="160" customHeight="1">
+    <row r="2" ht="202" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · Kim sıralanıyor?
-Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
-Kaynak: Google TR mobil sonuç sayfası · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
-Sütun açıklamaları: Alan adı: Google TR mobil ilk 10 organik sonuçta görünen alan adı. | İlk 10 (kelime): 109 kelimeden kaçında ilk 10'da. | İlk 3 (kelime): Kaç kelimede ilk 3'te. | Ort. sıra: Görüldüğü kelimelerdeki en iyi sıranın ortalaması. | SSG / BM / Armatür / Bitişik: Tema bazında ilk 10'da görüldüğü kelime sayısı (tema büyüklükleri 16 / 15 / 13 / 24).</t>
+Kapsam: Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri 107 kelime için incelenmiştir. Kelimeler sabit bir hacim sıralamasıyla değil, VitrA'nın kategori ağacını ve fırsat alanlarını temsil edecek biçimde dokuz temadan seçilmiştir: SSG, banyo mobilyası, armatür ve duş, yıkanma alanları, bitişik ürünler, hizmet ve ilham, karo, soru ve marka. Her temada ana kelime, fiyat ifadeli biçimi ve önemli alt tipler alınmış; Google Keyword Planner'da arama hacmi olmayan kelimeler analizden çıkarılmıştır. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
+Kaynak: Google TR mobil sonuç sayfası · %d kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Sütun açıklamaları: Alan adı: Google TR mobil ilk 10 organik sonuçta görünen alan adı. | İlk 10 (kelime): 107 kelimeden kaçında ilk 10'da. | İlk 3 (kelime): Kaç kelimede ilk 3'te. | Ort. sıra: Görüldüğü kelimelerdeki en iyi sıranın ortalaması. | SSG / BM / Armatür / Bitişik: Tema bazında ilk 10'da görüldüğü kelime sayısı (tema büyüklükleri 16 / 14 / 13 / 24).</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -10450,17 +12102,17 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>2.3</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>14 / 14 / 12 / 21</t>
+          <t>14 / 13 / 12 / 21</t>
         </is>
       </c>
     </row>
@@ -10471,59 +12123,59 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>30</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>9 / 13 / 8 / 15</t>
+          <t>9 / 12 / 8 / 15</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>vitra.com.tr</t>
+          <t>hepsiburada.com</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
         <v>54</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>3.1</v>
+        <v>5.2</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>14 / 11 / 5 / 3</t>
+          <t>8 / 11 / 8 / 18</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>hepsiburada.com</t>
+          <t>vitra.com.tr</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>5.2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>8 / 11 / 8 / 18</t>
+          <t>14 / 10 / 5 / 3</t>
         </is>
       </c>
     </row>
@@ -10555,17 +12207,17 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>13 / 9 / 4 / 1</t>
+          <t>13 / 8 / 4 / 1</t>
         </is>
       </c>
     </row>
@@ -10576,17 +12228,17 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>1 / 11 / - / 4</t>
+          <t>1 / 10 / - / 4</t>
         </is>
       </c>
     </row>
@@ -10597,13 +12249,13 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>10</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
@@ -10618,13 +12270,13 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -10639,7 +12291,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>5</v>
@@ -10681,7 +12333,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>6</v>
@@ -10691,35 +12343,35 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>7 / 2 / 2 / 1</t>
+          <t>7 / 1 / 2 / 1</t>
         </is>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>ikea.com.tr</t>
+          <t>amazon.com.tr</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>6.3</v>
+        <v>5.2</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>1 / 8 / 2 / 3</t>
+          <t>1 / 2 / 3 / 8</t>
         </is>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>amazon.com.tr</t>
+          <t>ikea.com.tr</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
@@ -10729,11 +12381,11 @@
         <v>5</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>5.2</v>
+        <v>6.5</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1 / 2 / 3 / 8</t>
+          <t>1 / 7 / 2 / 3</t>
         </is>
       </c>
     </row>
@@ -10744,17 +12396,17 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>6 / 4 / 4 / 2</t>
+          <t>6 / 3 / 4 / 2</t>
         </is>
       </c>
     </row>
@@ -10790,12 +12442,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="174" customHeight="1">
+    <row r="2" ht="216" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · VitrA nerede?
-Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
-Kaynak: Google TR mobil sonuç sayfası · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Kapsam: Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri 107 kelime için incelenmiştir. Kelimeler sabit bir hacim sıralamasıyla değil, VitrA'nın kategori ağacını ve fırsat alanlarını temsil edecek biçimde dokuz temadan seçilmiştir: SSG, banyo mobilyası, armatür ve duş, yıkanma alanları, bitişik ürünler, hizmet ve ilham, karo, soru ve marka. Her temada ana kelime, fiyat ifadeli biçimi ve önemli alt tipler alınmış; Google Keyword Planner'da arama hacmi olmayan kelimeler analizden çıkarılmıştır. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
+Kaynak: Google TR mobil sonuç sayfası · %d kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
 Sütun açıklamaları: Tema: Kelime grubu; ok simgesi temadaki kelimeleri ve metriklerini açar. | Kelime: Temadaki kelime sayısı. | VitrA ilk 3 (SERP): 29.09.2026 mobil gözlemde vitra.com.tr'nin ilk 3'te olduğu kelime sayısı. | VitrA ilk 10 (SERP): Aynı gözlemde ilk 10'da olduğu kelime sayısı. | VitrA ilk 10 (Search Console): Search Console'da 26.06 - 25.09.2026 ortalama sırası 10 ve altında olan kelime sayısı; tüm cihazlar. | SERP'te ilk 20'de yok: Tek günlük gözlemde vitra.com.tr'nin ilk 20'de görünmediği kelime sayısı.</t>
         </is>
       </c>
@@ -10866,16 +12518,16 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>4</v>
@@ -10998,7 +12650,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>5</v>
@@ -11068,12 +12720,12 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="216" customHeight="1">
+    <row r="2" ht="258" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · Tek günlük gözlemde VitrA'nın ilk 20'de görünmediği kelimeler: SERP, Search Console ve Google kontrolü
-Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
-Kaynak: Google TR mobil sonuç sayfası · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Kapsam: Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri 107 kelime için incelenmiştir. Kelimeler sabit bir hacim sıralamasıyla değil, VitrA'nın kategori ağacını ve fırsat alanlarını temsil edecek biçimde dokuz temadan seçilmiştir: SSG, banyo mobilyası, armatür ve duş, yıkanma alanları, bitişik ürünler, hizmet ve ilham, karo, soru ve marka. Her temada ana kelime, fiyat ifadeli biçimi ve önemli alt tipler alınmış; Google Keyword Planner'da arama hacmi olmayan kelimeler analizden çıkarılmıştır. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
+Kaynak: Google TR mobil sonuç sayfası · %d kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
 Sütun açıklamaları: Arama kelimesi: 29.09.2026 mobil SERP gözleminde vitra.com.tr'nin ilk 20'de görünmediği kelime. | Aylık hacim: Google Keyword Planner, Eylül 2025 - Ağustos 2026 aylık ortalama arama hacmi. | Search Console ort. sıra: vitra.com.tr'nin bu sorgudaki 26.06 - 25.09.2026 ortalama sırası (sorgu düzeyinde, tüm cihazlar); "-" sorgu raporda yok. | Search Console click: Aynı dönemde bu kelimeden gelen click. | Google sırası (30.09): google.com.tr, oturumsuz arama, 30.09.2026; ilk sayfadaki organik sonuçlar arasında vitra.com.tr'nin sırası; "-" ilk sayfada yok. | İlk 5 sonuç (30.09): Aynı Google kontrolünde ilk beş organik sonucun alan adı, sırasıyla; "-" alan adı okunamayan sonuç. | Durum: VitrA'nın 30.09.2026 Google ilk sayfasındaki varlığı.</t>
         </is>
       </c>
@@ -11891,7 +13543,7 @@
     <col width="49" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -11901,13 +13553,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="146" customHeight="1">
+    <row r="2" ht="188" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Google Arama Sonuçları ve AI Overview · SERP özellikleri ve AI Overview
-Kapsam: Kategori, ürün, bitişik ürün, hizmet, soru ve marka kelimelerinden oluşan 109 kelime için Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri incelenmiştir. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
-Kaynak: Google TR mobil sonuç sayfası · 109 kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
-Sütun açıklamaları: SERP özelliği: Arama sonuç sayfasında organik sonuç dışındaki blok. | Kelime (pay): 109 kelimeden kaçında görüldüğü. | SSG / BM / Armatür / Bitişik: Tema bazında görüldüğü kelime sayısı. | En yoğun olduğu temalar: En yüksek görülme oranı.</t>
+Kapsam: Google Türkiye mobil arama sonuçlarının ilk 20 organik sonucu ve SERP özellikleri 107 kelime için incelenmiştir. Kelimeler sabit bir hacim sıralamasıyla değil, VitrA'nın kategori ağacını ve fırsat alanlarını temsil edecek biçimde dokuz temadan seçilmiştir: SSG, banyo mobilyası, armatür ve duş, yıkanma alanları, bitişik ürünler, hizmet ve ilham, karo, soru ve marka. Her temada ana kelime, fiyat ifadeli biçimi ve önemli alt tipler alınmış; Google Keyword Planner'da arama hacmi olmayan kelimeler analizden çıkarılmıştır. Sonuçlar 29 Eylül 2026 tarihli tek gözlemdir.
+Kaynak: Google TR mobil sonuç sayfası · %d kelime · ilk 20 organik sonuç · 29.09.2026 · Search Console sc-domain:vitra.com.tr, 26.06 - 25.09.2026 · google.com.tr oturumsuz kontrol, 24 kelime, 30.09.2026 · hacim Keyword Planner 10 , 11 , 13
+Sütun açıklamaları: SERP özelliği: Arama sonuç sayfasında organik sonuç dışındaki blok. | Kelime (pay): 107 kelimeden kaçında görüldüğü. | SSG / BM / Armatür / Bitişik: Tema bazında görüldüğü kelime sayısı. | En yoğun olduğu temalar: En yüksek görülme oranı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -11944,7 +13596,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>31 (%28)</t>
+          <t>30 (%28)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -11954,7 +13606,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Soru 5/7, karo 3/5</t>
+          <t>Soru 4/6, karo 3/5, bitişik 8/24</t>
         </is>
       </c>
     </row>
@@ -11966,7 +13618,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>84 (%77)</t>
+          <t>83 (%78)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -11976,7 +13628,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Yıkanma 6/6, karo 5/5, soru 7/7, marka 9/9</t>
+          <t>Marka 9/9, yıkanma 6/6, soru 6/6</t>
         </is>
       </c>
     </row>
@@ -11998,7 +13650,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Hizmet 10/14, soru 5/7</t>
+          <t>Soru 5/6, hizmet 10/14, SSG 7/16</t>
         </is>
       </c>
     </row>
@@ -12020,7 +13672,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Yıkanma 5/6, marka 6/9</t>
+          <t>Yıkanma 5/6, marka 6/9, hizmet 8/14</t>
         </is>
       </c>
     </row>
@@ -12042,7 +13694,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Banyo dolabı, duşakabin, tesisatçı</t>
+          <t>Yıkanma 3/6, BM 5/14, bitişik 3/24</t>
         </is>
       </c>
     </row>
@@ -13474,15 +15126,15 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="174" customHeight="1">
+          <t>Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Yıllık banyo yenileme ve yeni konut banyosu tahmini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="202" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
+          <t>Bölüm: Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Yıllık banyo yenileme ve yeni konut banyosu tahmini
+Kapsam: Bu bölüm, banyo ürünlerine olan talebi etkileyen genel ekonomik koşulları özetlemektedir: insanların kartla ne kadar harcadığı, ekonomiye güvenleri ve evlerini tamir ettirme niyetleri, konut alım-satımı ve bankaların kredi verme koşulları. Banyo yenilemesi ertelenebilen bir harcama olduğu için bu göstergeler, kategori aramalarındaki daralmanın (Bölüm 03) arka planını açıklamaya yardımcı olur. Veriler Türkiye Cumhuriyet Merkez Bankası'nın veri sisteminden (TCMB EVDS) alınmıştır.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Yıllık yenileme oranı: Konutların yılda yüzde kaçında banyonun yenilendiği varsayımı; Türkiye için ölçülmüş bir oran bulunmadığından senaryo olarak verilmiştir. | Karşılığı: Oranın ima ettiği ortalama yenileme döngüsü; Almanya'da yenilenmemiş banyoların ortalama yaşı 19,5 yıldır (VDS, 2017). | Yenilenen banyo (milyon): 26,6 milyon hane × oran × konut başına 1,1-1,3 banyo. | Yeni konut banyosu (milyon): Yılda 0,4-0,6 milyon iskanlı daire × 1,1-1,3 banyo. | Toplam (milyon banyo / yıl): Yenileme ve yeni konut toplamı.</t>
         </is>
@@ -16983,15 +18635,15 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="132" customHeight="1">
+          <t>Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Yıllık banyo yenileme ve yeni konut banyosu tahmini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bölüm: Makro Ortam ve Ödeme Gücü · Yıllık banyo yenileme ve yeni konut banyosu tahmini
-Kapsam: Banyo yenilemesi, dayanıklı mal harcamaları ve konut hareketliliğiyle birlikte hareket etmektedir: kart harcamaları, tüketici eğilimi, konut satışları ve banka kredi koşulları (TCMB EVDS), kategori talebindeki daralmanın (Bölüm 03) arka planını göstermektedir.
+          <t>Bölüm: Ekonomik Ortam: Harcama, Güven ve Konut Piyasası · Yıllık banyo yenileme ve yeni konut banyosu tahmini
+Kapsam: Bu bölüm, banyo ürünlerine olan talebi etkileyen genel ekonomik koşulları özetlemektedir: insanların kartla ne kadar harcadığı, ekonomiye güvenleri ve evlerini tamir ettirme niyetleri, konut alım-satımı ve bankaların kredi verme koşulları. Banyo yenilemesi ertelenebilen bir harcama olduğu için bu göstergeler, kategori aramalarındaki daralmanın (Bölüm 03) arka planını açıklamaya yardımcı olur. Veriler Türkiye Cumhuriyet Merkez Bankası'nın veri sisteminden (TCMB EVDS) alınmıştır.
 Kaynak: TCMB EVDS · kart harcamaları BKM haftalık akım (KT1, KT17, KT23, KT50, KT8, KT16); kartlı ödeme endeksi; Tüketici Eğilim Anketi; konut satış ve fiyat istatistikleri; Banka Kredileri Eğilim Anketi; hane halkı beklentileri · erişim 28.09.2026 1 , 2 , 3 , 4 , 5
 Sütun açıklamaları: Gösterge: Tahminde kullanılan girdi. | Değer: Kaynaktaki değer. | Kaynak ve not: Kaynak ve ölçüm türü.</t>
         </is>
@@ -31007,13 +32659,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="328" customHeight="1">
+    <row r="2" ht="454" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · Alt kesitler: vitra.com.tr, pazaryeri ve fiyat karşılaştırma siteleri
 Kapsam: Trendyol (42 kategori), Hepsiburada (40), Akakçe (42 sayfa ve 8 VitrA marka sayfası) ve Cimri'de (30) çok satan ya da popülerlik sıralamasının ilk iki sayfası ile Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağazasının kategori sayfaları okunmuştur; toplam 9.000'den fazla pazaryeri ve 2.500'den fazla mağaza ürün satırı. Kategoriler VitrA'nın hedef gamı (SSG, rezervuar, mobilya, armatür, yıkanma) ve hedef dışı bitişik kesitler olarak ayrılmıştır. Değerlendirme sayısı satış hacminin yaklaşık göstergesidir; fiyatlar 30.09.2026 tarihli liste fiyatlarıdır. Kale fiyat göstermediği, IKEA TR ürün listesi vermediği için kapsam dışıdır.
 Kaynak: Trendyol, Hepsiburada, Akakçe ve Cimri kategori listeleri (ilk 2 sayfa) · Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağaza kategori sayfaları · 30.09.2026 36
-Sütun açıklamaları: Ana &gt; alt kategori: VitrA'nın ana kategorisi ve vitra.com.tr alt kategori adı; arama ifadesi pazaryerinde kullanılan karşılıktır. | vitra.com.tr ürün / stokta yok: Kategori sayfasındaki renk ve varyant kartı sayısı / "Gelince Haber Ver" işaretli kart sayısı; 30.09.2026. | vitra.com.tr fiyat aralığı (TL): Kategori sayfasındaki liste fiyatı aralığı; 30.09.2026. | Trendyol toplam: Trendyol arama sonucu toplamı. | Trendyol medyan (TL): Çok satan sıralı ilk 36 üründe kesitle eşleşen ürünlerin medyan fiyatı. | Hepsiburada toplam: Hepsiburada arama sonucu toplamı (10.000 üst sınır). | Hepsiburada medyan (TL): Çok satan sıralı ilk 36 üründe eşleşen ürünlerin medyan fiyatı. | Akakçe medyan (TL): Eşleşen ürünlerin en düşük fiyat medyanı. | Akakçe satıcı: Ürün başına satıcı sayısı medyanı. | Cimri medyan (TL): Eşleşen ürünlerin en düşük fiyat medyanı; "-" veri yok. | Cimri satıcı: Ürün başına satıcı sayısı medyanı; "-" veri yok. | VitrA / Artema adet (TY / HB / Ak / Ci): Eşleşen ürünler içinde VitrA ya da Artema markalı ürün sayısı; sırasıyla Trendyol, Hepsiburada, Akakçe, Cimri. | En çok değerlendirilen marka: Trendyol (yoksa Hepsiburada) eşleşen ürünlerinde değerlendirme sayısı en yüksek marka ve kesitteki değerlendirme payı.</t>
+Sütun açıklamaları: Ana &gt; alt kategori: VitrA'nın ana kategorisi ve vitra.com.tr'deki alt kategori adı (ör. Armatürler &gt; Sürgülü el duşu takımı). Pazaryerlerinde bu alt kategorinin adıyla arama yapılmıştır. | vitra.com.tr ürün / stokta yok: vitra.com.tr'de bu alt kategorinin sayfasında listelenen ürün kartı sayısı (her renk ve ölçü ayrı kart sayılır) / bunlardan stokta olmayan, "Gelince Haber Ver" düğmesi taşıyan kart sayısı (30.09.2026). | vitra.com.tr fiyat aralığı (TL): vitra.com.tr'nin bu alt kategori sayfasındaki en ucuz ve en pahalı ürünün liste fiyatı (sepette uygulanan indirim öncesi). | Trendyol toplam: Trendyol'da alt kategori adıyla (ör. "sürgülü el duşu") arama yapıldığında listelenen toplam ürün sayısı; Trendyol'da bu alt kategoride ne kadar ürün olduğunu gösterir. | Trendyol medyan (TL): Aynı Trendyol aramasında çok satana göre sıralanan ilk 36 ürün içinden, adında alt kategori kelimesi geçen ürünlerin ortanca (medyan) fiyatı. | Hepsiburada toplam: Hepsiburada'da alt kategori adıyla arama yapıldığında listelenen toplam ürün sayısı; Hepsiburada 10.000'in üzerini göstermediği için en fazla 10.000. | Hepsiburada medyan (TL): Aynı Hepsiburada aramasında çok satana göre sıralanan ilk 36 ürün içinden, adında alt kategori kelimesi geçenlerin ortanca fiyatı. | Akakçe medyan (TL): Akakçe'de alt kategori adıyla yapılan aramada eşleşen her ürün için en düşük satıcı fiyatı alınmış, bu fiyatların ortanca değeri verilmiştir. | Akakçe satıcı: Akakçe'de eşleşen ürünlerde ürün başına fiyat veren satıcı sayısının ortanca değeri; rekabetin ne kadar yoğun olduğunu gösterir. | Cimri medyan (TL): Cimri'de aynı yöntemle bulunan ortanca en düşük fiyat; "-" Cimri'de bu alt kategori için sonuç bulunamadı. | Cimri satıcı: Cimri'de ürün başına satıcı sayısının ortanca değeri; "-" sonuç yok. | VitrA / Artema adet (TY / HB / Ak / Ci): Her kanalda alt kategoriyle eşleşen ürünler arasında VitrA veya Artema markalı ürün sayısı; sırasıyla Trendyol, Hepsiburada, Akakçe, Cimri. VitrA'nın pazaryeri listelerinde ne kadar yer aldığını gösterir. | En çok değerlendirilen marka: Trendyol'da (Trendyol'da sonuç yoksa Hepsiburada'da) eşleşen ürünler içinde en çok kullanıcı değerlendirmesi alan marka ve alt kategorideki değerlendirmelerin yüzde kaçını aldığı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -34150,10 +35802,10 @@
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
@@ -34165,13 +35817,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="258" customHeight="1">
+    <row r="2" ht="300" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Bölüm: Pazaryeri Alt Kategori Derinliği: Çok Satanlar ve Rakip Mağazalar · vitra.com.tr kategori sayfaları: ürün, fiyat aralığı ve stok
 Kapsam: Trendyol (42 kategori), Hepsiburada (40), Akakçe (42 sayfa ve 8 VitrA marka sayfası) ve Cimri'de (30) çok satan ya da popülerlik sıralamasının ilk iki sayfası ile Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağazasının kategori sayfaları okunmuştur; toplam 9.000'den fazla pazaryeri ve 2.500'den fazla mağaza ürün satırı. Kategoriler VitrA'nın hedef gamı (SSG, rezervuar, mobilya, armatür, yıkanma) ve hedef dışı bitişik kesitler olarak ayrılmıştır. Değerlendirme sayısı satış hacminin yaklaşık göstergesidir; fiyatlar 30.09.2026 tarihli liste fiyatlarıdır. Kale fiyat göstermediği, IKEA TR ürün listesi vermediği için kapsam dışıdır.
 Kaynak: Trendyol, Hepsiburada, Akakçe ve Cimri kategori listeleri (ilk 2 sayfa) · Koçtaş, Bauhaus, Banyomarka, Banyomega, Banyoline ve Creavit e-mağaza kategori sayfaları · 30.09.2026 36
-Sütun açıklamaları: Alt kategori: vitra.com.tr kategori sayfası. | Sayfa yolu: Kategori sayfasının yolu; yeni sekmede açılır. | Ürün (varyant): Sayfadaki "N sonuç listeleniyor" değeri; renk ve varyant kartları ayrı sayılır. | Fiyat aralığı (TL): Liste fiyatı; fiyata göre artan ve azalan sıralamanın ilk kartları. | Stoklu: "Sadece stoklu ürünleri göster" süzgeciyle listelenen kart sayısı; 0 olan sayfalarda ilk sayfadaki tüm kartlar "Gelince Haber Ver" işaretlidir. | Stokta yok: Sayfa toplamı ile stoklu kart sayısı arasındaki fark. | İlk sayfada "Sepette indirim": İlk sayfadaki kartların kaçında "Sepette %N indirim" etiketi bulunduğu / ilk sayfadaki kart sayısı. | Ücretsiz montaj (liste): /c-ucretsiz-montaj listesinde bu kategoriden yer alan ürün sayısı.</t>
+Sütun açıklamaları: Alt kategori: vitra.com.tr'deki kategori sayfasının adı. | Sayfa yolu: Kategori sayfasının adresi; yeni sekmede açılır. | Ürün kartı: Sayfanın üstündeki "N sonuç listeleniyor" değeri. Aynı ürünün her rengi ve ölçüsü ayrı kart olarak sayılır. | Fiyat aralığı (TL): Sayfadaki en ucuz ve en pahalı kartın liste fiyatı (sepet indirimi öncesi); sayfa fiyata göre artan ve azalan sıralanarak okunmuştur. | Stokta olan: Sayfadaki "Sadece stoklu ürünleri göster" süzgeci açıldığında kalan kart sayısı; 0 ise sayfadaki hiçbir ürün stokta değildir. | Stokta olmayan: Toplam kart sayısından stokta olan kartlar çıkarılarak bulunmuştur; bu kartlar fiyatıyla birlikte listelenmeye devam eder. | İlk sayfada "Sepette indirim": Sayfanın ilk ekranındaki kartlardan kaçında "Sepette %N indirim" etiketi olduğu / ilk ekrandaki toplam kart. Bu kartlarda gösterilen fiyat, sepette ödenecek fiyattan yüksektir. | Ücretsiz montaj (liste): vitra.com.tr'nin ücretsiz montaj sayfasında (/c-ucretsiz-montaj) bu kategoriden yer alan ürün sayısı.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -34195,7 +35847,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Ürün (varyant)</t>
+          <t>Ürün kartı</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -34205,12 +35857,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Stoklu</t>
+          <t>Stokta olan</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Stokta yok</t>
+          <t>Stokta olmayan</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">

</xml_diff>